<commit_message>
Auto update 2026-03-10 17:22:13
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,462 +436,462 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1111-05-32</t>
+          <t>1282_1_1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1111-05-32/001.jpg,https://oleks-netizen.github.io/product-images/1111-05-32/003.jpg,https://oleks-netizen.github.io/product-images/1111-05-32/004.jpg,https://oleks-netizen.github.io/product-images/1111-05-32/005.jpg,https://oleks-netizen.github.io/product-images/1111-05-32/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/1282_1_1/001.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1313-05-38</t>
+          <t>1282_1_2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1313-05-38/001.jpg,https://oleks-netizen.github.io/product-images/1313-05-38/002.jpg,https://oleks-netizen.github.io/product-images/1313-05-38/003.jpg,https://oleks-netizen.github.io/product-images/1313-05-38/004.jpg,https://oleks-netizen.github.io/product-images/1313-05-38/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/1282_1_2/001.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1313-18-38</t>
+          <t>1282_1_4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1313-18-38/001.jpg,https://oleks-netizen.github.io/product-images/1313-18-38/002.jpg,https://oleks-netizen.github.io/product-images/1313-18-38/003.jpg,https://oleks-netizen.github.io/product-images/1313-18-38/005.jpg,https://oleks-netizen.github.io/product-images/1313-18-38/006.jpg,https://oleks-netizen.github.io/product-images/1313-18-38/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/1282_1_4/001.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1314-05-38</t>
+          <t>1282_1_5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1314-05-38/001.jpg,https://oleks-netizen.github.io/product-images/1314-05-38/002.jpg,https://oleks-netizen.github.io/product-images/1314-05-38/004.jpg,https://oleks-netizen.github.io/product-images/1314-05-38/005.jpg,https://oleks-netizen.github.io/product-images/1314-05-38/006.jpg,https://oleks-netizen.github.io/product-images/1314-05-38/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/1282_1_5/001.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1314-06-38</t>
+          <t>1793_1_100</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1314-06-38/001.jpg,https://oleks-netizen.github.io/product-images/1314-06-38/002.jpg,https://oleks-netizen.github.io/product-images/1314-06-38/004.jpg,https://oleks-netizen.github.io/product-images/1314-06-38/005.jpg,https://oleks-netizen.github.io/product-images/1314-06-38/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/1793_1_100/001.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1665-09-32</t>
+          <t>1892_1_2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1665-09-32/001.jpg,https://oleks-netizen.github.io/product-images/1665-09-32/002.jpg,https://oleks-netizen.github.io/product-images/1665-09-32/003.jpg,https://oleks-netizen.github.io/product-images/1665-09-32/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/1892_1_2/001.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2210-05-31</t>
+          <t>2212-05-31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/2210-05-31/001.jpg,https://oleks-netizen.github.io/product-images/2210-05-31/002.jpg,https://oleks-netizen.github.io/product-images/2210-05-31/003.jpg,https://oleks-netizen.github.io/product-images/2210-05-31/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/2212-05-31/001.jpg,https://oleks-netizen.github.io/product-images/2212-05-31/002.jpg,https://oleks-netizen.github.io/product-images/2212-05-31/003.jpg,https://oleks-netizen.github.io/product-images/2212-05-31/004.jpg,https://oleks-netizen.github.io/product-images/2212-05-31/005.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2210-45-31</t>
+          <t>2212-45-31</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/2210-45-31/001.jpg,https://oleks-netizen.github.io/product-images/2210-45-31/002.jpg,https://oleks-netizen.github.io/product-images/2210-45-31/004.jpg,https://oleks-netizen.github.io/product-images/2210-45-31/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/2212-45-31/001.jpg,https://oleks-netizen.github.io/product-images/2212-45-31/002.jpg,https://oleks-netizen.github.io/product-images/2212-45-31/003.jpg,https://oleks-netizen.github.io/product-images/2212-45-31/004.jpg,https://oleks-netizen.github.io/product-images/2212-45-31/005.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2210-56-31</t>
+          <t>2212-56-31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/2210-56-31/001.jpg,https://oleks-netizen.github.io/product-images/2210-56-31/002.jpg,https://oleks-netizen.github.io/product-images/2210-56-31/004.jpg,https://oleks-netizen.github.io/product-images/2210-56-31/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/2212-56-31/001.jpg,https://oleks-netizen.github.io/product-images/2212-56-31/002.jpg,https://oleks-netizen.github.io/product-images/2212-56-31/003.jpg,https://oleks-netizen.github.io/product-images/2212-56-31/004.jpg,https://oleks-netizen.github.io/product-images/2212-56-31/005.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2213-06-31</t>
+          <t>5192301</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/2213-06-31/001.jpg,https://oleks-netizen.github.io/product-images/2213-06-31/002.jpg,https://oleks-netizen.github.io/product-images/2213-06-31/003.jpg,https://oleks-netizen.github.io/product-images/2213-06-31/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5192301/001.jpg,https://oleks-netizen.github.io/product-images/5192301/002.jpg,https://oleks-netizen.github.io/product-images/5192301/003.jpg,https://oleks-netizen.github.io/product-images/5192301/005.jpg,https://oleks-netizen.github.io/product-images/5192301/006.jpg,https://oleks-netizen.github.io/product-images/5192301/007.jpg,https://oleks-netizen.github.io/product-images/5192301/008.jpg,https://oleks-netizen.github.io/product-images/5192301/009.jpg,https://oleks-netizen.github.io/product-images/5192301/010.jpg,https://oleks-netizen.github.io/product-images/5192301/011.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2213-56-32</t>
+          <t>5215901</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/2213-56-32/001.jpg,https://oleks-netizen.github.io/product-images/2213-56-32/002.jpg,https://oleks-netizen.github.io/product-images/2213-56-32/003.jpg,https://oleks-netizen.github.io/product-images/2213-56-32/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5215901/001.jpg,https://oleks-netizen.github.io/product-images/5215901/002.jpg,https://oleks-netizen.github.io/product-images/5215901/003.jpg,https://oleks-netizen.github.io/product-images/5215901/004.jpg,https://oleks-netizen.github.io/product-images/5215901/005.jpg,https://oleks-netizen.github.io/product-images/5215901/006.jpg,https://oleks-netizen.github.io/product-images/5215901/007.jpg,https://oleks-netizen.github.io/product-images/5215901/008.jpg,https://oleks-netizen.github.io/product-images/5215901/009.jpg,https://oleks-netizen.github.io/product-images/5215901/010.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2222-06-31</t>
+          <t>5218401</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/2222-06-31/001.jpg,https://oleks-netizen.github.io/product-images/2222-06-31/002.jpg,https://oleks-netizen.github.io/product-images/2222-06-31/003.jpg,https://oleks-netizen.github.io/product-images/2222-06-31/004.jpg,https://oleks-netizen.github.io/product-images/2222-06-31/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5218401/001.jpg,https://oleks-netizen.github.io/product-images/5218401/003.jpg,https://oleks-netizen.github.io/product-images/5218401/004.jpg,https://oleks-netizen.github.io/product-images/5218401/005.jpg,https://oleks-netizen.github.io/product-images/5218401/006.jpg,https://oleks-netizen.github.io/product-images/5218401/007.jpg,https://oleks-netizen.github.io/product-images/5218401/008.jpg,https://oleks-netizen.github.io/product-images/5218401/009.jpg,https://oleks-netizen.github.io/product-images/5218401/010.jpg,https://oleks-netizen.github.io/product-images/5218401/011.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2222-56-31</t>
+          <t>5231601</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/2222-56-31/001.jpg,https://oleks-netizen.github.io/product-images/2222-56-31/002.jpg,https://oleks-netizen.github.io/product-images/2222-56-31/003.jpg,https://oleks-netizen.github.io/product-images/2222-56-31/004.jpg,https://oleks-netizen.github.io/product-images/2222-56-31/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5231601/001.jpg,https://oleks-netizen.github.io/product-images/5231601/002.jpg,https://oleks-netizen.github.io/product-images/5231601/003.jpg,https://oleks-netizen.github.io/product-images/5231601/005.jpg,https://oleks-netizen.github.io/product-images/5231601/006.jpg,https://oleks-netizen.github.io/product-images/5231601/007.jpg,https://oleks-netizen.github.io/product-images/5231601/008.jpg,https://oleks-netizen.github.io/product-images/5231601/009.jpg,https://oleks-netizen.github.io/product-images/5231601/010.jpg,https://oleks-netizen.github.io/product-images/5231601/011.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>53100020</t>
+          <t>5231701</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53100020/001.jpg,https://oleks-netizen.github.io/product-images/53100020/002.jpg,https://oleks-netizen.github.io/product-images/53100020/003.jpg,https://oleks-netizen.github.io/product-images/53100020/004.jpg,https://oleks-netizen.github.io/product-images/53100020/005.jpg,https://oleks-netizen.github.io/product-images/53100020/006.jpg,https://oleks-netizen.github.io/product-images/53100020/007.jpg,https://oleks-netizen.github.io/product-images/53100020/009.jpg,https://oleks-netizen.github.io/product-images/53100020/010.jpg,https://oleks-netizen.github.io/product-images/53100020/011.jpg,https://oleks-netizen.github.io/product-images/53100020/012.jpg,https://oleks-netizen.github.io/product-images/53100020/013.jpg,https://oleks-netizen.github.io/product-images/53100020/014.jpg,https://oleks-netizen.github.io/product-images/53100020/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5231701/001.jpg,https://oleks-netizen.github.io/product-images/5231701/002.jpg,https://oleks-netizen.github.io/product-images/5231701/003.jpg,https://oleks-netizen.github.io/product-images/5231701/004.jpg,https://oleks-netizen.github.io/product-images/5231701/005.jpg,https://oleks-netizen.github.io/product-images/5231701/006.jpg,https://oleks-netizen.github.io/product-images/5231701/007.jpg,https://oleks-netizen.github.io/product-images/5231701/009.jpg,https://oleks-netizen.github.io/product-images/5231701/010.jpg,https://oleks-netizen.github.io/product-images/5231701/011.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>53100067</t>
+          <t>5240601</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53100067/001.jpg,https://oleks-netizen.github.io/product-images/53100067/002.jpg,https://oleks-netizen.github.io/product-images/53100067/003.jpg,https://oleks-netizen.github.io/product-images/53100067/004.jpg,https://oleks-netizen.github.io/product-images/53100067/005.jpg,https://oleks-netizen.github.io/product-images/53100067/006.jpg,https://oleks-netizen.github.io/product-images/53100067/007.jpg,https://oleks-netizen.github.io/product-images/53100067/008.jpg,https://oleks-netizen.github.io/product-images/53100067/009.jpg,https://oleks-netizen.github.io/product-images/53100067/010.jpg,https://oleks-netizen.github.io/product-images/53100067/012.jpg,https://oleks-netizen.github.io/product-images/53100067/013.jpg,https://oleks-netizen.github.io/product-images/53100067/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5240601/001.jpg,https://oleks-netizen.github.io/product-images/5240601/002.jpg,https://oleks-netizen.github.io/product-images/5240601/003.jpg,https://oleks-netizen.github.io/product-images/5240601/004.jpg,https://oleks-netizen.github.io/product-images/5240601/005.jpg,https://oleks-netizen.github.io/product-images/5240601/006.jpg,https://oleks-netizen.github.io/product-images/5240601/007.jpg,https://oleks-netizen.github.io/product-images/5240601/008.jpg,https://oleks-netizen.github.io/product-images/5240601/009.jpg,https://oleks-netizen.github.io/product-images/5240601/010.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>53100068</t>
+          <t>5240801</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53100068/001.jpg,https://oleks-netizen.github.io/product-images/53100068/002.jpg,https://oleks-netizen.github.io/product-images/53100068/003.jpg,https://oleks-netizen.github.io/product-images/53100068/004.jpg,https://oleks-netizen.github.io/product-images/53100068/005.jpg,https://oleks-netizen.github.io/product-images/53100068/007.jpg,https://oleks-netizen.github.io/product-images/53100068/008.jpg,https://oleks-netizen.github.io/product-images/53100068/009.jpg,https://oleks-netizen.github.io/product-images/53100068/010.jpg,https://oleks-netizen.github.io/product-images/53100068/011.jpg,https://oleks-netizen.github.io/product-images/53100068/012.jpg,https://oleks-netizen.github.io/product-images/53100068/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5240801/001.jpg,https://oleks-netizen.github.io/product-images/5240801/002.jpg,https://oleks-netizen.github.io/product-images/5240801/003.jpg,https://oleks-netizen.github.io/product-images/5240801/004.jpg,https://oleks-netizen.github.io/product-images/5240801/005.jpg,https://oleks-netizen.github.io/product-images/5240801/006.jpg,https://oleks-netizen.github.io/product-images/5240801/007.jpg,https://oleks-netizen.github.io/product-images/5240801/008.jpg,https://oleks-netizen.github.io/product-images/5240801/009.jpg</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>53200013</t>
+          <t>5246601W</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53200013/001.jpg,https://oleks-netizen.github.io/product-images/53200013/002.jpg,https://oleks-netizen.github.io/product-images/53200013/003.jpg,https://oleks-netizen.github.io/product-images/53200013/004.jpg,https://oleks-netizen.github.io/product-images/53200013/005.jpg,https://oleks-netizen.github.io/product-images/53200013/006.jpg,https://oleks-netizen.github.io/product-images/53200013/007.jpg,https://oleks-netizen.github.io/product-images/53200013/008.jpg,https://oleks-netizen.github.io/product-images/53200013/009.jpg,https://oleks-netizen.github.io/product-images/53200013/010.jpg,https://oleks-netizen.github.io/product-images/53200013/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5246601W/001.jpg,https://oleks-netizen.github.io/product-images/5246601W/002.jpg,https://oleks-netizen.github.io/product-images/5246601W/003.jpg,https://oleks-netizen.github.io/product-images/5246601W/005.jpg,https://oleks-netizen.github.io/product-images/5246601W/006.jpg,https://oleks-netizen.github.io/product-images/5246601W/007.jpg</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>53300061</t>
+          <t>5246701W</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53300061/001.jpg,https://oleks-netizen.github.io/product-images/53300061/002.jpg,https://oleks-netizen.github.io/product-images/53300061/003.jpg,https://oleks-netizen.github.io/product-images/53300061/004.jpg,https://oleks-netizen.github.io/product-images/53300061/005.jpg,https://oleks-netizen.github.io/product-images/53300061/006.jpg,https://oleks-netizen.github.io/product-images/53300061/008.jpg,https://oleks-netizen.github.io/product-images/53300061/009.jpg,https://oleks-netizen.github.io/product-images/53300061/010.jpg,https://oleks-netizen.github.io/product-images/53300061/011.jpg,https://oleks-netizen.github.io/product-images/53300061/012.jpg,https://oleks-netizen.github.io/product-images/53300061/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5246701W/001.jpg,https://oleks-netizen.github.io/product-images/5246701W/002.jpg,https://oleks-netizen.github.io/product-images/5246701W/003.jpg,https://oleks-netizen.github.io/product-images/5246701W/005.jpg,https://oleks-netizen.github.io/product-images/5246701W/006.jpg,https://oleks-netizen.github.io/product-images/5246701W/007.jpg</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>53300070</t>
+          <t>BN-BV-1-choko</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53300070/001.jpg,https://oleks-netizen.github.io/product-images/53300070/002.jpg,https://oleks-netizen.github.io/product-images/53300070/003.jpg,https://oleks-netizen.github.io/product-images/53300070/004.jpg,https://oleks-netizen.github.io/product-images/53300070/005.jpg,https://oleks-netizen.github.io/product-images/53300070/006.jpg,https://oleks-netizen.github.io/product-images/53300070/007.jpg,https://oleks-netizen.github.io/product-images/53300070/008.jpg,https://oleks-netizen.github.io/product-images/53300070/009.jpg,https://oleks-netizen.github.io/product-images/53300070/010.jpg,https://oleks-netizen.github.io/product-images/53300070/012.jpg,https://oleks-netizen.github.io/product-images/53300070/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-choko/005.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-choko/006.jpg</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>53300519</t>
+          <t>BN-BV-1-g</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53300519/001.jpg,https://oleks-netizen.github.io/product-images/53300519/002.jpg,https://oleks-netizen.github.io/product-images/53300519/003.jpg,https://oleks-netizen.github.io/product-images/53300519/004.jpg,https://oleks-netizen.github.io/product-images/53300519/005.jpg,https://oleks-netizen.github.io/product-images/53300519/006.jpg,https://oleks-netizen.github.io/product-images/53300519/008.jpg,https://oleks-netizen.github.io/product-images/53300519/009.jpg,https://oleks-netizen.github.io/product-images/53300519/010.jpg,https://oleks-netizen.github.io/product-images/53300519/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-g/004.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-g/005.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-g/006.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-g/007.jpg</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>53330506</t>
+          <t>BN-BV-1-g-kr</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330506/001.jpg,https://oleks-netizen.github.io/product-images/53330506/002.jpg,https://oleks-netizen.github.io/product-images/53330506/003.jpg,https://oleks-netizen.github.io/product-images/53330506/005.jpg,https://oleks-netizen.github.io/product-images/53330506/006.jpg,https://oleks-netizen.github.io/product-images/53330506/007.jpg,https://oleks-netizen.github.io/product-images/53330506/008.jpg,https://oleks-netizen.github.io/product-images/53330506/009.jpg,https://oleks-netizen.github.io/product-images/53330506/010.jpg,https://oleks-netizen.github.io/product-images/53330506/011.jpg,https://oleks-netizen.github.io/product-images/53330506/012.jpg,https://oleks-netizen.github.io/product-images/53330506/013.jpg,https://oleks-netizen.github.io/product-images/53330506/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-g-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-g-kr/002.jpg</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>80411003</t>
+          <t>BN-BV-1-iz</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80411003/001.jpg,https://oleks-netizen.github.io/product-images/80411003/002.jpg,https://oleks-netizen.github.io/product-images/80411003/003.jpg,https://oleks-netizen.github.io/product-images/80411003/004.jpg,https://oleks-netizen.github.io/product-images/80411003/005.jpg,https://oleks-netizen.github.io/product-images/80411003/006.jpg,https://oleks-netizen.github.io/product-images/80411003/007.jpg,https://oleks-netizen.github.io/product-images/80411003/009.jpg,https://oleks-netizen.github.io/product-images/80411003/010.jpg,https://oleks-netizen.github.io/product-images/80411003/011.jpg,https://oleks-netizen.github.io/product-images/80411003/012.jpg,https://oleks-netizen.github.io/product-images/80411003/013.jpg,https://oleks-netizen.github.io/product-images/80411003/014.jpg,https://oleks-netizen.github.io/product-images/80411003/015.jpg,https://oleks-netizen.github.io/product-images/80411003/016.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-iz/003.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-iz/004.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-iz/005.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-iz/006.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-iz/007.jpg</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>80411506</t>
+          <t>BN-BV-1-k</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80411506/001.jpg,https://oleks-netizen.github.io/product-images/80411506/002.jpg,https://oleks-netizen.github.io/product-images/80411506/003.jpg,https://oleks-netizen.github.io/product-images/80411506/004.jpg,https://oleks-netizen.github.io/product-images/80411506/005.jpg,https://oleks-netizen.github.io/product-images/80411506/006.jpg,https://oleks-netizen.github.io/product-images/80411506/007.jpg,https://oleks-netizen.github.io/product-images/80411506/008.jpg,https://oleks-netizen.github.io/product-images/80411506/009.jpg,https://oleks-netizen.github.io/product-images/80411506/010.jpg,https://oleks-netizen.github.io/product-images/80411506/011.jpg,https://oleks-netizen.github.io/product-images/80411506/012.jpg,https://oleks-netizen.github.io/product-images/80411506/014.jpg,https://oleks-netizen.github.io/product-images/80411506/015.jpg,https://oleks-netizen.github.io/product-images/80411506/016.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-k/005.jpg</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>80411514</t>
+          <t>BN-BV-1-k-kr</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80411514/001.jpg,https://oleks-netizen.github.io/product-images/80411514/002.jpg,https://oleks-netizen.github.io/product-images/80411514/003.jpg,https://oleks-netizen.github.io/product-images/80411514/004.jpg,https://oleks-netizen.github.io/product-images/80411514/005.jpg,https://oleks-netizen.github.io/product-images/80411514/006.jpg,https://oleks-netizen.github.io/product-images/80411514/007.jpg,https://oleks-netizen.github.io/product-images/80411514/008.jpg,https://oleks-netizen.github.io/product-images/80411514/009.jpg,https://oleks-netizen.github.io/product-images/80411514/010.jpg,https://oleks-netizen.github.io/product-images/80411514/011.jpg,https://oleks-netizen.github.io/product-images/80411514/012.jpg,https://oleks-netizen.github.io/product-images/80411514/013.jpg,https://oleks-netizen.github.io/product-images/80411514/015.jpg,https://oleks-netizen.github.io/product-images/80411514/016.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-k-kr/005.jpg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>80411515</t>
+          <t>BN-BV-1-navy-blue</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80411515/001.jpg,https://oleks-netizen.github.io/product-images/80411515/002.jpg,https://oleks-netizen.github.io/product-images/80411515/003.jpg,https://oleks-netizen.github.io/product-images/80411515/004.jpg,https://oleks-netizen.github.io/product-images/80411515/005.jpg,https://oleks-netizen.github.io/product-images/80411515/006.jpg,https://oleks-netizen.github.io/product-images/80411515/007.jpg,https://oleks-netizen.github.io/product-images/80411515/008.jpg,https://oleks-netizen.github.io/product-images/80411515/010.jpg,https://oleks-netizen.github.io/product-images/80411515/011.jpg,https://oleks-netizen.github.io/product-images/80411515/012.jpg,https://oleks-netizen.github.io/product-images/80411515/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-navy-blue/006.jpg</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>80460061</t>
+          <t>BN-BV-1-nn</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80460061/001.jpg,https://oleks-netizen.github.io/product-images/80460061/002.jpg,https://oleks-netizen.github.io/product-images/80460061/003.jpg,https://oleks-netizen.github.io/product-images/80460061/004.jpg,https://oleks-netizen.github.io/product-images/80460061/005.jpg,https://oleks-netizen.github.io/product-images/80460061/006.jpg,https://oleks-netizen.github.io/product-images/80460061/007.jpg,https://oleks-netizen.github.io/product-images/80460061/008.jpg,https://oleks-netizen.github.io/product-images/80460061/010.jpg,https://oleks-netizen.github.io/product-images/80460061/011.jpg,https://oleks-netizen.github.io/product-images/80460061/012.jpg,https://oleks-netizen.github.io/product-images/80460061/013.jpg,https://oleks-netizen.github.io/product-images/80460061/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-nn/003.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-nn/004.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-nn/005.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-nn/006.jpg</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>80460101</t>
+          <t>BN-BV-1-o</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80460101/001.jpg,https://oleks-netizen.github.io/product-images/80460101/002.jpg,https://oleks-netizen.github.io/product-images/80460101/003.jpg,https://oleks-netizen.github.io/product-images/80460101/004.jpg,https://oleks-netizen.github.io/product-images/80460101/005.jpg,https://oleks-netizen.github.io/product-images/80460101/007.jpg,https://oleks-netizen.github.io/product-images/80460101/008.jpg,https://oleks-netizen.github.io/product-images/80460101/009.jpg,https://oleks-netizen.github.io/product-images/80460101/010.jpg,https://oleks-netizen.github.io/product-images/80460101/011.jpg,https://oleks-netizen.github.io/product-images/80460101/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-o/003.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-o/004.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-o/005.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-o/006.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-o/007.jpg</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>85515006</t>
+          <t>BN-BV-1-vin</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/85515006/001.jpg,https://oleks-netizen.github.io/product-images/85515006/002.jpg,https://oleks-netizen.github.io/product-images/85515006/004.jpg,https://oleks-netizen.github.io/product-images/85515006/005.jpg,https://oleks-netizen.github.io/product-images/85515006/006.jpg,https://oleks-netizen.github.io/product-images/85515006/007.jpg,https://oleks-netizen.github.io/product-images/85515006/008.jpg,https://oleks-netizen.github.io/product-images/85515006/009.jpg,https://oleks-netizen.github.io/product-images/85515006/010.jpg,https://oleks-netizen.github.io/product-images/85515006/011.jpg,https://oleks-netizen.github.io/product-images/85515006/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-vin/002.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-vin/003.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-vin/005.jpg</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>85515106</t>
+          <t>BN-BV-1-vin-kr</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/85515106/001.jpg,https://oleks-netizen.github.io/product-images/85515106/002.jpg,https://oleks-netizen.github.io/product-images/85515106/003.jpg,https://oleks-netizen.github.io/product-images/85515106/004.jpg,https://oleks-netizen.github.io/product-images/85515106/005.jpg,https://oleks-netizen.github.io/product-images/85515106/006.jpg,https://oleks-netizen.github.io/product-images/85515106/008.jpg,https://oleks-netizen.github.io/product-images/85515106/009.jpg,https://oleks-netizen.github.io/product-images/85515106/010.jpg,https://oleks-netizen.github.io/product-images/85515106/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-vin-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-vin-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-vin-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-vin-kr/005.jpg</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>93220021</t>
+          <t>BN-CB-4-choko</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/93220021/001.jpg,https://oleks-netizen.github.io/product-images/93220021/002.jpg,https://oleks-netizen.github.io/product-images/93220021/003.jpg,https://oleks-netizen.github.io/product-images/93220021/004.jpg,https://oleks-netizen.github.io/product-images/93220021/005.jpg,https://oleks-netizen.github.io/product-images/93220021/007.jpg,https://oleks-netizen.github.io/product-images/93220021/008.jpg,https://oleks-netizen.github.io/product-images/93220021/009.jpg,https://oleks-netizen.github.io/product-images/93220021/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-4-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-choko/004.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-choko/006.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-choko/007.jpg</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>fz379334_chok</t>
+          <t>BN-CB-4-g</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/fz379334_chok/001.jpg,https://oleks-netizen.github.io/product-images/fz379334_chok/002.jpg,https://oleks-netizen.github.io/product-images/fz379334_chok/003.jpg,https://oleks-netizen.github.io/product-images/fz379334_chok/004.jpg,https://oleks-netizen.github.io/product-images/fz379334_chok/006.jpg,https://oleks-netizen.github.io/product-images/fz379334_chok/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-4-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g/005.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g/006.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g/007.jpg</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -901,12 +901,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GA-1304-4lx</t>
+          <t>BN-CB-4-g-kr</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/GA-1304-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GA-1304-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GA-1304-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GA-1304-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GA-1304-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GA-1304-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GA-1304-4lx/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-4-g-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g-kr/006.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-g-kr/008.jpg</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -916,46 +916,781 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RA-wall-005</t>
+          <t>BN-CB-4-iz</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RA-wall-005/001.jpg,https://oleks-netizen.github.io/product-images/RA-wall-005/002.jpg,https://oleks-netizen.github.io/product-images/RA-wall-005/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-4-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-iz/004.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-iz/005.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-iz/006.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-iz/007.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-iz/008.jpg</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>RY-6002-3md</t>
+          <t>BN-CB-4-k-kr</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RY-6002-3md/001.jpg,https://oleks-netizen.github.io/product-images/RY-6002-3md/002.jpg,https://oleks-netizen.github.io/product-images/RY-6002-3md/003.jpg,https://oleks-netizen.github.io/product-images/RY-6002-3md/004.jpg,https://oleks-netizen.github.io/product-images/RY-6002-3md/005.jpg,https://oleks-netizen.github.io/product-images/RY-6002-3md/006.jpg,https://oleks-netizen.github.io/product-images/RY-6002-3md/008.jpg,https://oleks-netizen.github.io/product-images/RY-6002-3md/009.jpg,https://oleks-netizen.github.io/product-images/RY-6002-3md/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-4-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-k-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-k-kr/006.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-k-kr/007.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-k-kr/008.jpg</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>VC02807ltaup</t>
+          <t>BN-CB-4-navy-blue</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/VC02807ltaup/001.jpg,https://oleks-netizen.github.io/product-images/VC02807ltaup/002.jpg,https://oleks-netizen.github.io/product-images/VC02807ltaup/003.jpg,https://oleks-netizen.github.io/product-images/VC02807ltaup/004.jpg,https://oleks-netizen.github.io/product-images/VC02807ltaup/005.jpg,https://oleks-netizen.github.io/product-images/VC02807ltaup/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-4-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-navy-blue/004.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-navy-blue/005.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-navy-blue/007.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-navy-blue/008.jpg</t>
         </is>
       </c>
       <c r="C36" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BN-CB-4-nn</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-4-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-nn/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-nn/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-nn/004.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-nn/005.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-nn/007.jpg</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BN-CB-4-o</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-4-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-o/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-o/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-o/004.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-o/006.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-o/007.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-o/008.jpg</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BN-CB-4-vin</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-4-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-vin/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-vin/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-vin/004.jpg,https://oleks-netizen.github.io/product-images/BN-CB-4-vin/005.jpg</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BN-GC-23-beige-kr</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-beige-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-beige-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-beige-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-beige-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-beige-kr/006.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-beige-kr/007.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-beige-kr/008.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-beige-kr/009.jpg</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>BN-GC-23-choko</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-choko/004.jpg</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>BN-GC-23-g</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-g/004.jpg</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BN-GC-23-g-kr</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-g-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-g-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-g-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-g-kr/005.jpg</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BN-GC-23-iz</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-iz/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-iz/005.jpg</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BN-GC-23-k</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-k/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-k/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-k/006.jpg</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BN-GC-23-k-kr</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-k-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-k-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-k-kr/006.jpg</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BN-GC-23-malachite</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-malachite/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-malachite/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-malachite/006.jpg</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BN-GC-23-navy-blue</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-navy-blue/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-navy-blue/006.jpg</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BN-GC-23-nn</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-nn/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-nn/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-nn/005.jpg</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BN-GC-23-o</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-o/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-o/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-o/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-o/006.jpg</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>BN-GC-23-red</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-23-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-red/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-red/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-23-red/006.jpg</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BN-GC-24-1-g-kr</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-1-g-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-g-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-g-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-g-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-g-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-g-kr/006.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-g-kr/007.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-g-kr/009.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-g-kr/010.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-g-kr/011.jpg</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BN-GC-24-1-iz</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-1-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-iz/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-iz/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-iz/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-iz/006.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-iz/007.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-iz/009.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-iz/010.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-iz/011.jpg</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BN-GC-24-1-k-kr</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-1-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-k-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-k-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-k-kr/006.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-k-kr/007.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-k-kr/009.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-k-kr/010.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-k-kr/011.jpg</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>BN-GC-24-1-o</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-1-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-o/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-o/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-o/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-o/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-o/006.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-o/007.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-o/009.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-o/010.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-o/011.jpg</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>BN-GC-24-1-vin-kr</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-1-vin-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-vin-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-vin-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-vin-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-vin-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-vin-kr/006.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-vin-kr/007.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-vin-kr/009.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-vin-kr/010.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-1-vin-kr/011.jpg</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>BN-GC-24-choko</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-choko/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-choko/006.jpg</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BN-GC-24-g</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-g/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-g/005.jpg</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>BN-GC-24-g-kr</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-g-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-g-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-g-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-g-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-g-kr/005.jpg</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>BN-GC-24-iz</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-iz/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-iz/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-iz/005.jpg</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>BN-GC-24-k</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-k/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-k/005.jpg</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>BN-GC-24-k-kr</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-k-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-k-kr/005.jpg</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BN-GC-24-malachite</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-malachite/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-malachite/005.jpg</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>BN-GC-24-navy-blue</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-navy-blue/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-navy-blue/005.jpg</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>BN-GC-24-nn</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-nn/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-nn/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-nn/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-nn/005.jpg</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>BN-GC-24-o</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-o/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-o/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-o/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-o/005.jpg</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>BN-GC-24-red</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-24-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-red/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-red/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-24-red/005.jpg</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>BV38416-160</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38416-160/001.jpg,https://oleks-netizen.github.io/product-images/BV38416-160/002.jpg,https://oleks-netizen.github.io/product-images/BV38416-160/003.jpg,https://oleks-netizen.github.io/product-images/BV38416-160/005.jpg,https://oleks-netizen.github.io/product-images/BV38416-160/006.jpg,https://oleks-netizen.github.io/product-images/BV38416-160/007.jpg,https://oleks-netizen.github.io/product-images/BV38416-160/008.jpg,https://oleks-netizen.github.io/product-images/BV38416-160/009.jpg</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>BV38416-2924</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38416-2924/001.jpg,https://oleks-netizen.github.io/product-images/BV38416-2924/002.jpg,https://oleks-netizen.github.io/product-images/BV38416-2924/004.jpg,https://oleks-netizen.github.io/product-images/BV38416-2924/005.jpg,https://oleks-netizen.github.io/product-images/BV38416-2924/006.jpg,https://oleks-netizen.github.io/product-images/BV38416-2924/007.jpg,https://oleks-netizen.github.io/product-images/BV38416-2924/008.jpg,https://oleks-netizen.github.io/product-images/BV38416-2924/009.jpg</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>BV38525-2802</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38525-2802/001.jpg,https://oleks-netizen.github.io/product-images/BV38525-2802/002.jpg,https://oleks-netizen.github.io/product-images/BV38525-2802/004.jpg,https://oleks-netizen.github.io/product-images/BV38525-2802/005.jpg,https://oleks-netizen.github.io/product-images/BV38525-2802/006.jpg,https://oleks-netizen.github.io/product-images/BV38525-2802/007.jpg,https://oleks-netizen.github.io/product-images/BV38525-2802/008.jpg</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>BV38525-446</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38525-446/001.jpg,https://oleks-netizen.github.io/product-images/BV38525-446/002.jpg,https://oleks-netizen.github.io/product-images/BV38525-446/004.jpg,https://oleks-netizen.github.io/product-images/BV38525-446/005.jpg,https://oleks-netizen.github.io/product-images/BV38525-446/006.jpg,https://oleks-netizen.github.io/product-images/BV38525-446/007.jpg,https://oleks-netizen.github.io/product-images/BV38525-446/008.jpg</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>BV38601-2802</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38601-2802/001.jpg,https://oleks-netizen.github.io/product-images/BV38601-2802/002.jpg,https://oleks-netizen.github.io/product-images/BV38601-2802/004.jpg,https://oleks-netizen.github.io/product-images/BV38601-2802/005.jpg,https://oleks-netizen.github.io/product-images/BV38601-2802/006.jpg,https://oleks-netizen.github.io/product-images/BV38601-2802/007.jpg,https://oleks-netizen.github.io/product-images/BV38601-2802/008.jpg</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>BV38648-2807</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38648-2807/001.jpg,https://oleks-netizen.github.io/product-images/BV38648-2807/002.jpg,https://oleks-netizen.github.io/product-images/BV38648-2807/004.jpg,https://oleks-netizen.github.io/product-images/BV38648-2807/005.jpg,https://oleks-netizen.github.io/product-images/BV38648-2807/006.jpg,https://oleks-netizen.github.io/product-images/BV38648-2807/007.jpg,https://oleks-netizen.github.io/product-images/BV38648-2807/008.jpg</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>BV38648-306</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38648-306/001.jpg,https://oleks-netizen.github.io/product-images/BV38648-306/002.jpg,https://oleks-netizen.github.io/product-images/BV38648-306/003.jpg,https://oleks-netizen.github.io/product-images/BV38648-306/005.jpg,https://oleks-netizen.github.io/product-images/BV38648-306/006.jpg,https://oleks-netizen.github.io/product-images/BV38648-306/007.jpg</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>BV38655-2802</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38655-2802/001.jpg,https://oleks-netizen.github.io/product-images/BV38655-2802/002.jpg,https://oleks-netizen.github.io/product-images/BV38655-2802/004.jpg,https://oleks-netizen.github.io/product-images/BV38655-2802/005.jpg,https://oleks-netizen.github.io/product-images/BV38655-2802/006.jpg,https://oleks-netizen.github.io/product-images/BV38655-2802/007.jpg,https://oleks-netizen.github.io/product-images/BV38655-2802/008.jpg,https://oleks-netizen.github.io/product-images/BV38655-2802/009.jpg</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>BV38753-2924</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38753-2924/001.jpg,https://oleks-netizen.github.io/product-images/BV38753-2924/002.jpg,https://oleks-netizen.github.io/product-images/BV38753-2924/004.jpg,https://oleks-netizen.github.io/product-images/BV38753-2924/005.jpg,https://oleks-netizen.github.io/product-images/BV38753-2924/006.jpg,https://oleks-netizen.github.io/product-images/BV38753-2924/007.jpg,https://oleks-netizen.github.io/product-images/BV38753-2924/008.jpg</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>BV38755-160</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38755-160/001.jpg,https://oleks-netizen.github.io/product-images/BV38755-160/002.jpg,https://oleks-netizen.github.io/product-images/BV38755-160/004.jpg,https://oleks-netizen.github.io/product-images/BV38755-160/005.jpg,https://oleks-netizen.github.io/product-images/BV38755-160/006.jpg,https://oleks-netizen.github.io/product-images/BV38755-160/007.jpg,https://oleks-netizen.github.io/product-images/BV38755-160/008.jpg,https://oleks-netizen.github.io/product-images/BV38755-160/009.jpg</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>BV38755-191</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38755-191/001.jpg,https://oleks-netizen.github.io/product-images/BV38755-191/002.jpg,https://oleks-netizen.github.io/product-images/BV38755-191/004.jpg,https://oleks-netizen.github.io/product-images/BV38755-191/005.jpg,https://oleks-netizen.github.io/product-images/BV38755-191/006.jpg,https://oleks-netizen.github.io/product-images/BV38755-191/007.jpg,https://oleks-netizen.github.io/product-images/BV38755-191/008.jpg,https://oleks-netizen.github.io/product-images/BV38755-191/009.jpg</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>BV38755-2802</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38755-2802/001.jpg,https://oleks-netizen.github.io/product-images/BV38755-2802/002.jpg,https://oleks-netizen.github.io/product-images/BV38755-2802/004.jpg,https://oleks-netizen.github.io/product-images/BV38755-2802/005.jpg,https://oleks-netizen.github.io/product-images/BV38755-2802/006.jpg,https://oleks-netizen.github.io/product-images/BV38755-2802/007.jpg,https://oleks-netizen.github.io/product-images/BV38755-2802/008.jpg,https://oleks-netizen.github.io/product-images/BV38755-2802/009.jpg</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>BV38792-1</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38792-1/001.jpg,https://oleks-netizen.github.io/product-images/BV38792-1/002.jpg,https://oleks-netizen.github.io/product-images/BV38792-1/004.jpg,https://oleks-netizen.github.io/product-images/BV38792-1/005.jpg,https://oleks-netizen.github.io/product-images/BV38792-1/006.jpg,https://oleks-netizen.github.io/product-images/BV38792-1/007.jpg,https://oleks-netizen.github.io/product-images/BV38792-1/008.jpg,https://oleks-netizen.github.io/product-images/BV38792-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>BV38792-160</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38792-160/001.jpg,https://oleks-netizen.github.io/product-images/BV38792-160/002.jpg,https://oleks-netizen.github.io/product-images/BV38792-160/004.jpg,https://oleks-netizen.github.io/product-images/BV38792-160/005.jpg,https://oleks-netizen.github.io/product-images/BV38792-160/006.jpg,https://oleks-netizen.github.io/product-images/BV38792-160/007.jpg,https://oleks-netizen.github.io/product-images/BV38792-160/008.jpg</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>BV38800-2924</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38800-2924/001.jpg,https://oleks-netizen.github.io/product-images/BV38800-2924/002.jpg,https://oleks-netizen.github.io/product-images/BV38800-2924/004.jpg,https://oleks-netizen.github.io/product-images/BV38800-2924/005.jpg,https://oleks-netizen.github.io/product-images/BV38800-2924/006.jpg,https://oleks-netizen.github.io/product-images/BV38800-2924/007.jpg,https://oleks-netizen.github.io/product-images/BV38800-2924/008.jpg,https://oleks-netizen.github.io/product-images/BV38800-2924/009.jpg,https://oleks-netizen.github.io/product-images/BV38800-2924/010.jpg,https://oleks-netizen.github.io/product-images/BV38800-2924/011.jpg</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Y4309 CATCB 1</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/Y4309 CATCB 1/001.jpg,https://oleks-netizen.github.io/product-images/Y4309 CATCB 1/002.jpg,https://oleks-netizen.github.io/product-images/Y4309 CATCB 1/003.jpg,https://oleks-netizen.github.io/product-images/Y4309 CATCB 1/005.jpg,https://oleks-netizen.github.io/product-images/Y4309 CATCB 1/006.jpg</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>BN-BV-1-malachite</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-BV-1-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-BV-1-malachite/006.jpg</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>BV38792-160 (1)</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BV38792-160 (1)/004.jpg</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-03-30 16:28:02
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,507 +436,507 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BN-KL-6-choko</t>
+          <t>18228066</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-KL-6-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-KL-6-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-KL-6-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-KL-6-choko/004.jpg,https://oleks-netizen.github.io/product-images/BN-KL-6-choko/006.jpg,https://oleks-netizen.github.io/product-images/BN-KL-6-choko/007.jpg,https://oleks-netizen.github.io/product-images/BN-KL-6-choko/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/18228066/001.jpg,https://oleks-netizen.github.io/product-images/18228066/002.jpg,https://oleks-netizen.github.io/product-images/18228066/003.jpg,https://oleks-netizen.github.io/product-images/18228066/004.jpg,https://oleks-netizen.github.io/product-images/18228066/005.jpg,https://oleks-netizen.github.io/product-images/18228066/006.jpg,https://oleks-netizen.github.io/product-images/18228066/007.jpg,https://oleks-netizen.github.io/product-images/18228066/008.jpg,https://oleks-netizen.github.io/product-images/18228066/009.jpg,https://oleks-netizen.github.io/product-images/18228066/011.jpg,https://oleks-netizen.github.io/product-images/18228066/012.jpg,https://oleks-netizen.github.io/product-images/18228066/013.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BN-OP-33-beige</t>
+          <t>18228067</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-33-beige/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-beige/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-beige/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-beige/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-beige/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-beige/006.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-beige/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/18228067/001.jpg,https://oleks-netizen.github.io/product-images/18228067/002.jpg,https://oleks-netizen.github.io/product-images/18228067/003.jpg,https://oleks-netizen.github.io/product-images/18228067/005.jpg,https://oleks-netizen.github.io/product-images/18228067/006.jpg,https://oleks-netizen.github.io/product-images/18228067/007.jpg,https://oleks-netizen.github.io/product-images/18228067/008.jpg,https://oleks-netizen.github.io/product-images/18228067/009.jpg,https://oleks-netizen.github.io/product-images/18228067/010.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BN-OP-33-choko</t>
+          <t>18228068</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-33-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-choko/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-choko/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-choko/006.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-choko/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/18228068/001.jpg,https://oleks-netizen.github.io/product-images/18228068/002.jpg,https://oleks-netizen.github.io/product-images/18228068/003.jpg,https://oleks-netizen.github.io/product-images/18228068/004.jpg,https://oleks-netizen.github.io/product-images/18228068/005.jpg,https://oleks-netizen.github.io/product-images/18228068/007.jpg,https://oleks-netizen.github.io/product-images/18228068/008.jpg,https://oleks-netizen.github.io/product-images/18228068/009.jpg,https://oleks-netizen.github.io/product-images/18228068/010.jpg,https://oleks-netizen.github.io/product-images/18228068/011.jpg,https://oleks-netizen.github.io/product-images/18228068/012.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BN-OP-33-malachite</t>
+          <t>25000506</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-33-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-malachite/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-malachite/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-malachite/006.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-malachite/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000506/001.jpg,https://oleks-netizen.github.io/product-images/25000506/002.jpg,https://oleks-netizen.github.io/product-images/25000506/003.jpg,https://oleks-netizen.github.io/product-images/25000506/004.jpg,https://oleks-netizen.github.io/product-images/25000506/005.jpg,https://oleks-netizen.github.io/product-images/25000506/006.jpg,https://oleks-netizen.github.io/product-images/25000506/007.jpg,https://oleks-netizen.github.io/product-images/25000506/009.jpg,https://oleks-netizen.github.io/product-images/25000506/010.jpg,https://oleks-netizen.github.io/product-images/25000506/011.jpg,https://oleks-netizen.github.io/product-images/25000506/012.jpg,https://oleks-netizen.github.io/product-images/25000506/013.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BN-OP-33-navy-blue</t>
+          <t>25000514</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-33-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-navy-blue/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-navy-blue/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-navy-blue/006.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-navy-blue/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000514/001.jpg,https://oleks-netizen.github.io/product-images/25000514/002.jpg,https://oleks-netizen.github.io/product-images/25000514/003.jpg,https://oleks-netizen.github.io/product-images/25000514/004.jpg,https://oleks-netizen.github.io/product-images/25000514/005.jpg,https://oleks-netizen.github.io/product-images/25000514/006.jpg,https://oleks-netizen.github.io/product-images/25000514/007.jpg,https://oleks-netizen.github.io/product-images/25000514/008.jpg,https://oleks-netizen.github.io/product-images/25000514/009.jpg,https://oleks-netizen.github.io/product-images/25000514/011.jpg,https://oleks-netizen.github.io/product-images/25000514/012.jpg,https://oleks-netizen.github.io/product-images/25000514/013.jpg,https://oleks-netizen.github.io/product-images/25000514/014.jpg,https://oleks-netizen.github.io/product-images/25000514/015.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BN-OP-33-vin</t>
+          <t>25000514m</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-33-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-vin/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-vin/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-vin/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-vin/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-vin/006.jpg,https://oleks-netizen.github.io/product-images/BN-OP-33-vin/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000514m/001.jpg,https://oleks-netizen.github.io/product-images/25000514m/002.jpg,https://oleks-netizen.github.io/product-images/25000514m/004.jpg,https://oleks-netizen.github.io/product-images/25000514m/005.jpg,https://oleks-netizen.github.io/product-images/25000514m/006.jpg,https://oleks-netizen.github.io/product-images/25000514m/007.jpg,https://oleks-netizen.github.io/product-images/25000514m/008.jpg,https://oleks-netizen.github.io/product-images/25000514m/009.jpg,https://oleks-netizen.github.io/product-images/25000514m/010.jpg,https://oleks-netizen.github.io/product-images/25000514m/011.jpg,https://oleks-netizen.github.io/product-images/25000514m/012.jpg,https://oleks-netizen.github.io/product-images/25000514m/013.jpg,https://oleks-netizen.github.io/product-images/25000514m/014.jpg,https://oleks-netizen.github.io/product-images/25000514m/015.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BN-OP-34-g</t>
+          <t>25000515</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-34-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-34-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-34-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-34-g/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-34-g/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000515/001.jpg,https://oleks-netizen.github.io/product-images/25000515/002.jpg,https://oleks-netizen.github.io/product-images/25000515/003.jpg,https://oleks-netizen.github.io/product-images/25000515/005.jpg,https://oleks-netizen.github.io/product-images/25000515/006.jpg,https://oleks-netizen.github.io/product-images/25000515/007.jpg,https://oleks-netizen.github.io/product-images/25000515/008.jpg,https://oleks-netizen.github.io/product-images/25000515/009.jpg,https://oleks-netizen.github.io/product-images/25000515/010.jpg,https://oleks-netizen.github.io/product-images/25000515/011.jpg,https://oleks-netizen.github.io/product-images/25000515/012.jpg,https://oleks-netizen.github.io/product-images/25000515/013.jpg,https://oleks-netizen.github.io/product-images/25000515/014.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BN-OP-35-k</t>
+          <t>25000515m</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-35-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-k/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000515m/001.jpg,https://oleks-netizen.github.io/product-images/25000515m/002.jpg,https://oleks-netizen.github.io/product-images/25000515m/003.jpg,https://oleks-netizen.github.io/product-images/25000515m/004.jpg,https://oleks-netizen.github.io/product-images/25000515m/005.jpg,https://oleks-netizen.github.io/product-images/25000515m/007.jpg,https://oleks-netizen.github.io/product-images/25000515m/008.jpg,https://oleks-netizen.github.io/product-images/25000515m/009.jpg,https://oleks-netizen.github.io/product-images/25000515m/010.jpg,https://oleks-netizen.github.io/product-images/25000515m/011.jpg,https://oleks-netizen.github.io/product-images/25000515m/012.jpg,https://oleks-netizen.github.io/product-images/25000515m/013.jpg,https://oleks-netizen.github.io/product-images/25000515m/014.jpg,https://oleks-netizen.github.io/product-images/25000515m/015.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BN-OP-35-light</t>
+          <t>51311506</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-35-light/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-light/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-light/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-light/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51311506/001.jpg,https://oleks-netizen.github.io/product-images/51311506/002.jpg,https://oleks-netizen.github.io/product-images/51311506/003.jpg,https://oleks-netizen.github.io/product-images/51311506/004.jpg,https://oleks-netizen.github.io/product-images/51311506/005.jpg,https://oleks-netizen.github.io/product-images/51311506/006.jpg,https://oleks-netizen.github.io/product-images/51311506/008.jpg,https://oleks-netizen.github.io/product-images/51311506/009.jpg,https://oleks-netizen.github.io/product-images/51311506/010.jpg,https://oleks-netizen.github.io/product-images/51311506/011.jpg,https://oleks-netizen.github.io/product-images/51311506/012.jpg,https://oleks-netizen.github.io/product-images/51311506/013.jpg,https://oleks-netizen.github.io/product-images/51311506/014.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BN-OP-35-light-beige</t>
+          <t>51411006</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-35-light-beige/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-light-beige/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-light-beige/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-light-beige/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411006/001.jpg,https://oleks-netizen.github.io/product-images/51411006/002.jpg,https://oleks-netizen.github.io/product-images/51411006/003.jpg,https://oleks-netizen.github.io/product-images/51411006/004.jpg,https://oleks-netizen.github.io/product-images/51411006/005.jpg,https://oleks-netizen.github.io/product-images/51411006/006.jpg,https://oleks-netizen.github.io/product-images/51411006/008.jpg,https://oleks-netizen.github.io/product-images/51411006/009.jpg,https://oleks-netizen.github.io/product-images/51411006/010.jpg,https://oleks-netizen.github.io/product-images/51411006/011.jpg,https://oleks-netizen.github.io/product-images/51411006/012.jpg,https://oleks-netizen.github.io/product-images/51411006/013.jpg,https://oleks-netizen.github.io/product-images/51411006/014.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BN-OP-35-malachite</t>
+          <t>51411506</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-35-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-malachite/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411506/001.jpg,https://oleks-netizen.github.io/product-images/51411506/002.jpg,https://oleks-netizen.github.io/product-images/51411506/003.jpg,https://oleks-netizen.github.io/product-images/51411506/004.jpg,https://oleks-netizen.github.io/product-images/51411506/005.jpg,https://oleks-netizen.github.io/product-images/51411506/006.jpg,https://oleks-netizen.github.io/product-images/51411506/007.jpg,https://oleks-netizen.github.io/product-images/51411506/009.jpg,https://oleks-netizen.github.io/product-images/51411506/010.jpg,https://oleks-netizen.github.io/product-images/51411506/011.jpg,https://oleks-netizen.github.io/product-images/51411506/012.jpg,https://oleks-netizen.github.io/product-images/51411506/013.jpg,https://oleks-netizen.github.io/product-images/51411506/014.jpg,https://oleks-netizen.github.io/product-images/51411506/015.jpg,https://oleks-netizen.github.io/product-images/51411506/016.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BN-OP-35-navy-blue</t>
+          <t>53100066</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-35-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-navy-blue/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53100066/001.jpg,https://oleks-netizen.github.io/product-images/53100066/002.jpg,https://oleks-netizen.github.io/product-images/53100066/003.jpg,https://oleks-netizen.github.io/product-images/53100066/004.jpg,https://oleks-netizen.github.io/product-images/53100066/005.jpg,https://oleks-netizen.github.io/product-images/53100066/006.jpg,https://oleks-netizen.github.io/product-images/53100066/007.jpg,https://oleks-netizen.github.io/product-images/53100066/009.jpg,https://oleks-netizen.github.io/product-images/53100066/010.jpg,https://oleks-netizen.github.io/product-images/53100066/011.jpg,https://oleks-netizen.github.io/product-images/53100066/012.jpg,https://oleks-netizen.github.io/product-images/53100066/013.jpg,https://oleks-netizen.github.io/product-images/53100066/014.jpg,https://oleks-netizen.github.io/product-images/53100066/015.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BN-OP-35-pink-peach</t>
+          <t>53100106</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-35-pink-peach/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-pink-peach/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-pink-peach/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-pink-peach/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53100106/001.jpg,https://oleks-netizen.github.io/product-images/53100106/002.jpg,https://oleks-netizen.github.io/product-images/53100106/003.jpg,https://oleks-netizen.github.io/product-images/53100106/004.jpg,https://oleks-netizen.github.io/product-images/53100106/005.jpg,https://oleks-netizen.github.io/product-images/53100106/007.jpg,https://oleks-netizen.github.io/product-images/53100106/008.jpg,https://oleks-netizen.github.io/product-images/53100106/009.jpg,https://oleks-netizen.github.io/product-images/53100106/010.jpg,https://oleks-netizen.github.io/product-images/53100106/011.jpg,https://oleks-netizen.github.io/product-images/53100106/012.jpg,https://oleks-netizen.github.io/product-images/53100106/013.jpg,https://oleks-netizen.github.io/product-images/53100106/014.jpg,https://oleks-netizen.github.io/product-images/53100106/015.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BN-OP-35-tiffany</t>
+          <t>53300066</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-35-tiffany/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-tiffany/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-tiffany/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-35-tiffany/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53300066/001.jpg,https://oleks-netizen.github.io/product-images/53300066/002.jpg,https://oleks-netizen.github.io/product-images/53300066/003.jpg,https://oleks-netizen.github.io/product-images/53300066/004.jpg,https://oleks-netizen.github.io/product-images/53300066/005.jpg,https://oleks-netizen.github.io/product-images/53300066/006.jpg,https://oleks-netizen.github.io/product-images/53300066/007.jpg,https://oleks-netizen.github.io/product-images/53300066/009.jpg,https://oleks-netizen.github.io/product-images/53300066/010.jpg,https://oleks-netizen.github.io/product-images/53300066/011.jpg,https://oleks-netizen.github.io/product-images/53300066/012.jpg,https://oleks-netizen.github.io/product-images/53300066/013.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BN-SB-16-1-choko</t>
+          <t>53330029</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-1-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-choko/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53330029/001.jpg,https://oleks-netizen.github.io/product-images/53330029/002.jpg,https://oleks-netizen.github.io/product-images/53330029/003.jpg,https://oleks-netizen.github.io/product-images/53330029/004.jpg,https://oleks-netizen.github.io/product-images/53330029/005.jpg,https://oleks-netizen.github.io/product-images/53330029/006.jpg,https://oleks-netizen.github.io/product-images/53330029/008.jpg,https://oleks-netizen.github.io/product-images/53330029/009.jpg,https://oleks-netizen.github.io/product-images/53330029/010.jpg,https://oleks-netizen.github.io/product-images/53330029/011.jpg,https://oleks-netizen.github.io/product-images/53330029/012.jpg,https://oleks-netizen.github.io/product-images/53330029/013.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BN-SB-16-1-g</t>
+          <t>53330029m</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-1-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-g/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53330029m/001.jpg,https://oleks-netizen.github.io/product-images/53330029m/002.jpg,https://oleks-netizen.github.io/product-images/53330029m/003.jpg,https://oleks-netizen.github.io/product-images/53330029m/004.jpg,https://oleks-netizen.github.io/product-images/53330029m/005.jpg,https://oleks-netizen.github.io/product-images/53330029m/006.jpg,https://oleks-netizen.github.io/product-images/53330029m/008.jpg,https://oleks-netizen.github.io/product-images/53330029m/009.jpg,https://oleks-netizen.github.io/product-images/53330029m/010.jpg,https://oleks-netizen.github.io/product-images/53330029m/011.jpg</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BN-SB-16-1-k</t>
+          <t>53330064</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-1-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-k/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53330064/001.jpg,https://oleks-netizen.github.io/product-images/53330064/002.jpg,https://oleks-netizen.github.io/product-images/53330064/003.jpg,https://oleks-netizen.github.io/product-images/53330064/004.jpg,https://oleks-netizen.github.io/product-images/53330064/005.jpg,https://oleks-netizen.github.io/product-images/53330064/006.jpg,https://oleks-netizen.github.io/product-images/53330064/007.jpg,https://oleks-netizen.github.io/product-images/53330064/008.jpg,https://oleks-netizen.github.io/product-images/53330064/009.jpg,https://oleks-netizen.github.io/product-images/53330064/010.jpg,https://oleks-netizen.github.io/product-images/53330064/011.jpg,https://oleks-netizen.github.io/product-images/53330064/013.jpg,https://oleks-netizen.github.io/product-images/53330064/014.jpg</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BN-SB-16-1-k-kr</t>
+          <t>53330064m</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-1-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-k-kr/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53330064m/001.jpg,https://oleks-netizen.github.io/product-images/53330064m/002.jpg,https://oleks-netizen.github.io/product-images/53330064m/003.jpg,https://oleks-netizen.github.io/product-images/53330064m/004.jpg,https://oleks-netizen.github.io/product-images/53330064m/006.jpg,https://oleks-netizen.github.io/product-images/53330064m/007.jpg,https://oleks-netizen.github.io/product-images/53330064m/008.jpg,https://oleks-netizen.github.io/product-images/53330064m/009.jpg,https://oleks-netizen.github.io/product-images/53330064m/010.jpg,https://oleks-netizen.github.io/product-images/53330064m/011.jpg,https://oleks-netizen.github.io/product-images/53330064m/012.jpg</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BN-SB-16-1-navy-blue</t>
+          <t>53330066</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-1-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-navy-blue/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53330066/001.jpg,https://oleks-netizen.github.io/product-images/53330066/002.jpg,https://oleks-netizen.github.io/product-images/53330066/003.jpg,https://oleks-netizen.github.io/product-images/53330066/004.jpg,https://oleks-netizen.github.io/product-images/53330066/005.jpg,https://oleks-netizen.github.io/product-images/53330066/007.jpg,https://oleks-netizen.github.io/product-images/53330066/008.jpg,https://oleks-netizen.github.io/product-images/53330066/009.jpg,https://oleks-netizen.github.io/product-images/53330066/010.jpg,https://oleks-netizen.github.io/product-images/53330066/011.jpg,https://oleks-netizen.github.io/product-images/53330066/012.jpg</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BN-SB-16-1-o</t>
+          <t>53330068</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-1-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-o/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-o/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-1-o/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53330068/001.jpg,https://oleks-netizen.github.io/product-images/53330068/002.jpg,https://oleks-netizen.github.io/product-images/53330068/003.jpg,https://oleks-netizen.github.io/product-images/53330068/004.jpg,https://oleks-netizen.github.io/product-images/53330068/005.jpg,https://oleks-netizen.github.io/product-images/53330068/006.jpg,https://oleks-netizen.github.io/product-images/53330068/007.jpg,https://oleks-netizen.github.io/product-images/53330068/009.jpg,https://oleks-netizen.github.io/product-images/53330068/010.jpg,https://oleks-netizen.github.io/product-images/53330068/011.jpg,https://oleks-netizen.github.io/product-images/53330068/012.jpg,https://oleks-netizen.github.io/product-images/53330068/013.jpg,https://oleks-netizen.github.io/product-images/53330068/014.jpg</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BN-SB-16-choko</t>
+          <t>53330514</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-choko/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53330514/001.jpg,https://oleks-netizen.github.io/product-images/53330514/002.jpg,https://oleks-netizen.github.io/product-images/53330514/003.jpg,https://oleks-netizen.github.io/product-images/53330514/004.jpg,https://oleks-netizen.github.io/product-images/53330514/005.jpg,https://oleks-netizen.github.io/product-images/53330514/006.jpg,https://oleks-netizen.github.io/product-images/53330514/008.jpg,https://oleks-netizen.github.io/product-images/53330514/009.jpg,https://oleks-netizen.github.io/product-images/53330514/010.jpg,https://oleks-netizen.github.io/product-images/53330514/011.jpg,https://oleks-netizen.github.io/product-images/53330514/012.jpg,https://oleks-netizen.github.io/product-images/53330514/013.jpg,https://oleks-netizen.github.io/product-images/53330514/014.jpg,https://oleks-netizen.github.io/product-images/53330514/015.jpg,https://oleks-netizen.github.io/product-images/53330514/016.jpg</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BN-SB-16-g</t>
+          <t>53330514m</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-g/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53330514m/001.jpg,https://oleks-netizen.github.io/product-images/53330514m/002.jpg,https://oleks-netizen.github.io/product-images/53330514m/003.jpg,https://oleks-netizen.github.io/product-images/53330514m/004.jpg,https://oleks-netizen.github.io/product-images/53330514m/005.jpg,https://oleks-netizen.github.io/product-images/53330514m/006.jpg,https://oleks-netizen.github.io/product-images/53330514m/007.jpg,https://oleks-netizen.github.io/product-images/53330514m/008.jpg,https://oleks-netizen.github.io/product-images/53330514m/010.jpg,https://oleks-netizen.github.io/product-images/53330514m/011.jpg,https://oleks-netizen.github.io/product-images/53330514m/012.jpg,https://oleks-netizen.github.io/product-images/53330514m/013.jpg</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BN-SB-16-k</t>
+          <t>53330530</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-k/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53330530/001.jpg,https://oleks-netizen.github.io/product-images/53330530/002.jpg,https://oleks-netizen.github.io/product-images/53330530/003.jpg,https://oleks-netizen.github.io/product-images/53330530/004.jpg,https://oleks-netizen.github.io/product-images/53330530/005.jpg,https://oleks-netizen.github.io/product-images/53330530/006.jpg,https://oleks-netizen.github.io/product-images/53330530/007.jpg,https://oleks-netizen.github.io/product-images/53330530/008.jpg,https://oleks-netizen.github.io/product-images/53330530/009.jpg,https://oleks-netizen.github.io/product-images/53330530/010.jpg,https://oleks-netizen.github.io/product-images/53330530/011.jpg,https://oleks-netizen.github.io/product-images/53330530/013.jpg,https://oleks-netizen.github.io/product-images/53330530/014.jpg,https://oleks-netizen.github.io/product-images/53330530/015.jpg</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BN-SB-16-k-kr</t>
+          <t>53330530m</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-k-kr/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53330530m/001.jpg,https://oleks-netizen.github.io/product-images/53330530m/002.jpg,https://oleks-netizen.github.io/product-images/53330530m/003.jpg,https://oleks-netizen.github.io/product-images/53330530m/004.jpg,https://oleks-netizen.github.io/product-images/53330530m/005.jpg,https://oleks-netizen.github.io/product-images/53330530m/006.jpg,https://oleks-netizen.github.io/product-images/53330530m/008.jpg,https://oleks-netizen.github.io/product-images/53330530m/009.jpg,https://oleks-netizen.github.io/product-images/53330530m/010.jpg,https://oleks-netizen.github.io/product-images/53330530m/011.jpg,https://oleks-netizen.github.io/product-images/53330530m/012.jpg,https://oleks-netizen.github.io/product-images/53330530m/013.jpg,https://oleks-netizen.github.io/product-images/53330530m/014.jpg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BN-SB-16-navy-blue</t>
+          <t>53400506</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-navy-blue/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400506/001.jpg,https://oleks-netizen.github.io/product-images/53400506/002.jpg,https://oleks-netizen.github.io/product-images/53400506/003.jpg,https://oleks-netizen.github.io/product-images/53400506/004.jpg,https://oleks-netizen.github.io/product-images/53400506/005.jpg,https://oleks-netizen.github.io/product-images/53400506/006.jpg,https://oleks-netizen.github.io/product-images/53400506/007.jpg,https://oleks-netizen.github.io/product-images/53400506/008.jpg,https://oleks-netizen.github.io/product-images/53400506/009.jpg,https://oleks-netizen.github.io/product-images/53400506/010.jpg,https://oleks-netizen.github.io/product-images/53400506/012.jpg,https://oleks-netizen.github.io/product-images/53400506/013.jpg,https://oleks-netizen.github.io/product-images/53400506/014.jpg,https://oleks-netizen.github.io/product-images/53400506/015.jpg</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BN-SB-16-o</t>
+          <t>53400514</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-16-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-o/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-o/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-16-o/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400514/001.jpg,https://oleks-netizen.github.io/product-images/53400514/002.jpg,https://oleks-netizen.github.io/product-images/53400514/003.jpg,https://oleks-netizen.github.io/product-images/53400514/005.jpg,https://oleks-netizen.github.io/product-images/53400514/006.jpg,https://oleks-netizen.github.io/product-images/53400514/007.jpg,https://oleks-netizen.github.io/product-images/53400514/008.jpg,https://oleks-netizen.github.io/product-images/53400514/009.jpg,https://oleks-netizen.github.io/product-images/53400514/010.jpg,https://oleks-netizen.github.io/product-images/53400514/011.jpg,https://oleks-netizen.github.io/product-images/53400514/012.jpg,https://oleks-netizen.github.io/product-images/53400514/013.jpg</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GC-8086-3md</t>
+          <t>53400514m</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/GC-8086-3md/001.jpg,https://oleks-netizen.github.io/product-images/GC-8086-3md/002.jpg,https://oleks-netizen.github.io/product-images/GC-8086-3md/003.jpg,https://oleks-netizen.github.io/product-images/GC-8086-3md/004.jpg,https://oleks-netizen.github.io/product-images/GC-8086-3md/006.jpg,https://oleks-netizen.github.io/product-images/GC-8086-3md/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400514m/001.jpg,https://oleks-netizen.github.io/product-images/53400514m/002.jpg,https://oleks-netizen.github.io/product-images/53400514m/003.jpg,https://oleks-netizen.github.io/product-images/53400514m/004.jpg,https://oleks-netizen.github.io/product-images/53400514m/005.jpg,https://oleks-netizen.github.io/product-images/53400514m/006.jpg,https://oleks-netizen.github.io/product-images/53400514m/007.jpg,https://oleks-netizen.github.io/product-images/53400514m/009.jpg,https://oleks-netizen.github.io/product-images/53400514m/010.jpg,https://oleks-netizen.github.io/product-images/53400514m/011.jpg,https://oleks-netizen.github.io/product-images/53400514m/012.jpg,https://oleks-netizen.github.io/product-images/53400514m/013.jpg,https://oleks-netizen.github.io/product-images/53400514m/014.jpg,https://oleks-netizen.github.io/product-images/53400514m/015.jpg</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RA-3025-3md-</t>
+          <t>6936686411318</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RA-3025-3md-/001.jpg,https://oleks-netizen.github.io/product-images/RA-3025-3md-/002.jpg,https://oleks-netizen.github.io/product-images/RA-3025-3md-/004.jpg,https://oleks-netizen.github.io/product-images/RA-3025-3md-/005.jpg,https://oleks-netizen.github.io/product-images/RA-3025-3md-/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6936686411318/001.jpg,https://oleks-netizen.github.io/product-images/6936686411318/002.jpg,https://oleks-netizen.github.io/product-images/6936686411318/003.jpg,https://oleks-netizen.github.io/product-images/6936686411318/004.jpg,https://oleks-netizen.github.io/product-images/6936686411318/005.jpg,https://oleks-netizen.github.io/product-images/6936686411318/006.jpg,https://oleks-netizen.github.io/product-images/6936686411318/007.jpg,https://oleks-netizen.github.io/product-images/6936686411318/008.jpg</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RB112 BERRY M</t>
+          <t>6976195091748</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RB112 BERRY M/001.jpg,https://oleks-netizen.github.io/product-images/RB112 BERRY M/002.jpg,https://oleks-netizen.github.io/product-images/RB112 BERRY M/004.jpg,https://oleks-netizen.github.io/product-images/RB112 BERRY M/005.jpg,https://oleks-netizen.github.io/product-images/RB112 BERRY M/006.jpg,https://oleks-netizen.github.io/product-images/RB112 BERRY M/007.jpg,https://oleks-netizen.github.io/product-images/RB112 BERRY M/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976195091748/001.jpg,https://oleks-netizen.github.io/product-images/6976195091748/002.jpg,https://oleks-netizen.github.io/product-images/6976195091748/003.jpg,https://oleks-netizen.github.io/product-images/6976195091748/004.jpg,https://oleks-netizen.github.io/product-images/6976195091748/005.jpg,https://oleks-netizen.github.io/product-images/6976195091748/007.jpg,https://oleks-netizen.github.io/product-images/6976195091748/008.jpg,https://oleks-netizen.github.io/product-images/6976195091748/009.jpg,https://oleks-netizen.github.io/product-images/6976195091748/010.jpg</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RB112 BLK_RHUMBA</t>
+          <t>6976195091755</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RB112 BLK_RHUMBA/001.jpg,https://oleks-netizen.github.io/product-images/RB112 BLK_RHUMBA/002.jpg,https://oleks-netizen.github.io/product-images/RB112 BLK_RHUMBA/003.jpg,https://oleks-netizen.github.io/product-images/RB112 BLK_RHUMBA/005.jpg,https://oleks-netizen.github.io/product-images/RB112 BLK_RHUMBA/006.jpg,https://oleks-netizen.github.io/product-images/RB112 BLK_RHUMBA/007.jpg,https://oleks-netizen.github.io/product-images/RB112 BLK_RHUMBA/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976195091755/001.jpg,https://oleks-netizen.github.io/product-images/6976195091755/002.jpg,https://oleks-netizen.github.io/product-images/6976195091755/003.jpg,https://oleks-netizen.github.io/product-images/6976195091755/004.jpg,https://oleks-netizen.github.io/product-images/6976195091755/005.jpg,https://oleks-netizen.github.io/product-images/6976195091755/007.jpg,https://oleks-netizen.github.io/product-images/6976195091755/008.jpg,https://oleks-netizen.github.io/product-images/6976195091755/009.jpg,https://oleks-netizen.github.io/product-images/6976195091755/010.jpg</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RB112 BLUE M</t>
+          <t>6976195091779</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RB112 BLUE M/001.jpg,https://oleks-netizen.github.io/product-images/RB112 BLUE M/002.jpg,https://oleks-netizen.github.io/product-images/RB112 BLUE M/003.jpg,https://oleks-netizen.github.io/product-images/RB112 BLUE M/004.jpg,https://oleks-netizen.github.io/product-images/RB112 BLUE M/006.jpg,https://oleks-netizen.github.io/product-images/RB112 BLUE M/007.jpg,https://oleks-netizen.github.io/product-images/RB112 BLUE M/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976195091779/001.jpg,https://oleks-netizen.github.io/product-images/6976195091779/002.jpg,https://oleks-netizen.github.io/product-images/6976195091779/003.jpg,https://oleks-netizen.github.io/product-images/6976195091779/004.jpg,https://oleks-netizen.github.io/product-images/6976195091779/005.jpg,https://oleks-netizen.github.io/product-images/6976195091779/007.jpg,https://oleks-netizen.github.io/product-images/6976195091779/008.jpg,https://oleks-netizen.github.io/product-images/6976195091779/009.jpg</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>RB112 LIME M</t>
+          <t>6976195091786</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RB112 LIME M/001.jpg,https://oleks-netizen.github.io/product-images/RB112 LIME M/002.jpg,https://oleks-netizen.github.io/product-images/RB112 LIME M/004.jpg,https://oleks-netizen.github.io/product-images/RB112 LIME M/005.jpg,https://oleks-netizen.github.io/product-images/RB112 LIME M/006.jpg,https://oleks-netizen.github.io/product-images/RB112 LIME M/007.jpg,https://oleks-netizen.github.io/product-images/RB112 LIME M/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976195091786/001.jpg,https://oleks-netizen.github.io/product-images/6976195091786/002.jpg,https://oleks-netizen.github.io/product-images/6976195091786/003.jpg,https://oleks-netizen.github.io/product-images/6976195091786/004.jpg,https://oleks-netizen.github.io/product-images/6976195091786/006.jpg,https://oleks-netizen.github.io/product-images/6976195091786/007.jpg</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RB112 PLUM M</t>
+          <t>6976195091793</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RB112 PLUM M/001.jpg,https://oleks-netizen.github.io/product-images/RB112 PLUM M/002.jpg,https://oleks-netizen.github.io/product-images/RB112 PLUM M/004.jpg,https://oleks-netizen.github.io/product-images/RB112 PLUM M/005.jpg,https://oleks-netizen.github.io/product-images/RB112 PLUM M/006.jpg,https://oleks-netizen.github.io/product-images/RB112 PLUM M/007.jpg,https://oleks-netizen.github.io/product-images/RB112 PLUM M/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976195091793/001.jpg,https://oleks-netizen.github.io/product-images/6976195091793/002.jpg,https://oleks-netizen.github.io/product-images/6976195091793/004.jpg,https://oleks-netizen.github.io/product-images/6976195091793/005.jpg,https://oleks-netizen.github.io/product-images/6976195091793/006.jpg,https://oleks-netizen.github.io/product-images/6976195091793/007.jpg</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>RB112 RED M</t>
+          <t>6976195094718</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RB112 RED M/001.jpg,https://oleks-netizen.github.io/product-images/RB112 RED M/002.jpg,https://oleks-netizen.github.io/product-images/RB112 RED M/004.jpg,https://oleks-netizen.github.io/product-images/RB112 RED M/005.jpg,https://oleks-netizen.github.io/product-images/RB112 RED M/006.jpg,https://oleks-netizen.github.io/product-images/RB112 RED M/007.jpg,https://oleks-netizen.github.io/product-images/RB112 RED M/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976195094718/001.jpg,https://oleks-netizen.github.io/product-images/6976195094718/002.jpg,https://oleks-netizen.github.io/product-images/6976195094718/003.jpg,https://oleks-netizen.github.io/product-images/6976195094718/004.jpg,https://oleks-netizen.github.io/product-images/6976195094718/005.jpg,https://oleks-netizen.github.io/product-images/6976195094718/006.jpg,https://oleks-netizen.github.io/product-images/6976195094718/008.jpg</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -946,76 +946,886 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>RE-3025-3md-</t>
+          <t>6976195095838</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RE-3025-3md-/001.jpg,https://oleks-netizen.github.io/product-images/RE-3025-3md-/002.jpg,https://oleks-netizen.github.io/product-images/RE-3025-3md-/004.jpg,https://oleks-netizen.github.io/product-images/RE-3025-3md-/005.jpg,https://oleks-netizen.github.io/product-images/RE-3025-3md-/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976195095838/001.jpg,https://oleks-netizen.github.io/product-images/6976195095838/002.jpg,https://oleks-netizen.github.io/product-images/6976195095838/004.jpg</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>RK-3025-3md-</t>
+          <t>6976195095845</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RK-3025-3md-/001.jpg,https://oleks-netizen.github.io/product-images/RK-3025-3md-/002.jpg,https://oleks-netizen.github.io/product-images/RK-3025-3md-/004.jpg,https://oleks-netizen.github.io/product-images/RK-3025-3md-/005.jpg,https://oleks-netizen.github.io/product-images/RK-3025-3md-/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976195095845/001.jpg,https://oleks-netizen.github.io/product-images/6976195095845/002.jpg</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>S5 BLUE M</t>
+          <t>6976195096064</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S5 BLUE M/001.jpg,https://oleks-netizen.github.io/product-images/S5 BLUE M/002.jpg,https://oleks-netizen.github.io/product-images/S5 BLUE M/004.jpg,https://oleks-netizen.github.io/product-images/S5 BLUE M/005.jpg,https://oleks-netizen.github.io/product-images/S5 BLUE M/006.jpg,https://oleks-netizen.github.io/product-images/S5 BLUE M/007.jpg,https://oleks-netizen.github.io/product-images/S5 BLUE M/008.jpg,https://oleks-netizen.github.io/product-images/S5 BLUE M/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976195096064/001.jpg,https://oleks-netizen.github.io/product-images/6976195096064/002.jpg,https://oleks-netizen.github.io/product-images/6976195096064/004.jpg,https://oleks-netizen.github.io/product-images/6976195096064/005.jpg,https://oleks-netizen.github.io/product-images/6976195096064/006.jpg,https://oleks-netizen.github.io/product-images/6976195096064/007.jpg</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>S5 OIL TAN</t>
+          <t>6976195096989</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S5 OIL TAN/001.jpg,https://oleks-netizen.github.io/product-images/S5 OIL TAN/002.jpg,https://oleks-netizen.github.io/product-images/S5 OIL TAN/004.jpg,https://oleks-netizen.github.io/product-images/S5 OIL TAN/005.jpg,https://oleks-netizen.github.io/product-images/S5 OIL TAN/006.jpg,https://oleks-netizen.github.io/product-images/S5 OIL TAN/007.jpg,https://oleks-netizen.github.io/product-images/S5 OIL TAN/008.jpg,https://oleks-netizen.github.io/product-images/S5 OIL TAN/009.jpg,https://oleks-netizen.github.io/product-images/S5 OIL TAN/010.jpg,https://oleks-netizen.github.io/product-images/S5 OIL TAN/011.jpg,https://oleks-netizen.github.io/product-images/S5 OIL TAN/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976195096989/001.jpg,https://oleks-netizen.github.io/product-images/6976195096989/002.jpg,https://oleks-netizen.github.io/product-images/6976195096989/003.jpg,https://oleks-netizen.github.io/product-images/6976195096989/004.jpg,https://oleks-netizen.github.io/product-images/6976195096989/006.jpg</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TW-Camilla-brown-zam</t>
+          <t>6976975615294</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/TW-Camilla-brown-zam/001.jpg,https://oleks-netizen.github.io/product-images/TW-Camilla-brown-zam/002.jpg,https://oleks-netizen.github.io/product-images/TW-Camilla-brown-zam/003.jpg,https://oleks-netizen.github.io/product-images/TW-Camilla-brown-zam/005.jpg,https://oleks-netizen.github.io/product-images/TW-Camilla-brown-zam/006.jpg,https://oleks-netizen.github.io/product-images/TW-Camilla-brown-zam/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/6976975615294/001.jpg,https://oleks-netizen.github.io/product-images/6976975615294/002.jpg</t>
         </is>
       </c>
       <c r="C40" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>6976975615324</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/6976975615324/001.jpg,https://oleks-netizen.github.io/product-images/6976975615324/003.jpg,https://oleks-netizen.github.io/product-images/6976975615324/004.jpg</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>6977703651690</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/6977703651690/001.jpg,https://oleks-netizen.github.io/product-images/6977703651690/002.jpg,https://oleks-netizen.github.io/product-images/6977703651690/003.jpg,https://oleks-netizen.github.io/product-images/6977703651690/005.jpg</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>6977703651713</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/6977703651713/001.jpg,https://oleks-netizen.github.io/product-images/6977703651713/002.jpg,https://oleks-netizen.github.io/product-images/6977703651713/003.jpg</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>80411514m</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/80411514m/001.jpg,https://oleks-netizen.github.io/product-images/80411514m/002.jpg,https://oleks-netizen.github.io/product-images/80411514m/004.jpg,https://oleks-netizen.github.io/product-images/80411514m/005.jpg,https://oleks-netizen.github.io/product-images/80411514m/006.jpg,https://oleks-netizen.github.io/product-images/80411514m/007.jpg,https://oleks-netizen.github.io/product-images/80411514m/008.jpg,https://oleks-netizen.github.io/product-images/80411514m/009.jpg,https://oleks-netizen.github.io/product-images/80411514m/010.jpg,https://oleks-netizen.github.io/product-images/80411514m/011.jpg,https://oleks-netizen.github.io/product-images/80411514m/012.jpg,https://oleks-netizen.github.io/product-images/80411514m/013.jpg</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>80411515m</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/80411515m/001.jpg,https://oleks-netizen.github.io/product-images/80411515m/002.jpg,https://oleks-netizen.github.io/product-images/80411515m/003.jpg,https://oleks-netizen.github.io/product-images/80411515m/005.jpg,https://oleks-netizen.github.io/product-images/80411515m/006.jpg,https://oleks-netizen.github.io/product-images/80411515m/007.jpg,https://oleks-netizen.github.io/product-images/80411515m/008.jpg,https://oleks-netizen.github.io/product-images/80411515m/009.jpg,https://oleks-netizen.github.io/product-images/80411515m/010.jpg,https://oleks-netizen.github.io/product-images/80411515m/011.jpg,https://oleks-netizen.github.io/product-images/80411515m/012.jpg,https://oleks-netizen.github.io/product-images/80411515m/013.jpg,https://oleks-netizen.github.io/product-images/80411515m/014.jpg,https://oleks-netizen.github.io/product-images/80411515m/015.jpg</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>80411530m</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/80411530m/001.jpg,https://oleks-netizen.github.io/product-images/80411530m/002.jpg,https://oleks-netizen.github.io/product-images/80411530m/003.jpg,https://oleks-netizen.github.io/product-images/80411530m/004.jpg,https://oleks-netizen.github.io/product-images/80411530m/005.jpg,https://oleks-netizen.github.io/product-images/80411530m/006.jpg,https://oleks-netizen.github.io/product-images/80411530m/007.jpg,https://oleks-netizen.github.io/product-images/80411530m/009.jpg,https://oleks-netizen.github.io/product-images/80411530m/010.jpg,https://oleks-netizen.github.io/product-images/80411530m/011.jpg,https://oleks-netizen.github.io/product-images/80411530m/012.jpg,https://oleks-netizen.github.io/product-images/80411530m/013.jpg,https://oleks-netizen.github.io/product-images/80411530m/014.jpg</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>80411714</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/80411714/001.jpg,https://oleks-netizen.github.io/product-images/80411714/002.jpg,https://oleks-netizen.github.io/product-images/80411714/003.jpg,https://oleks-netizen.github.io/product-images/80411714/004.jpg,https://oleks-netizen.github.io/product-images/80411714/006.jpg,https://oleks-netizen.github.io/product-images/80411714/007.jpg,https://oleks-netizen.github.io/product-images/80411714/008.jpg,https://oleks-netizen.github.io/product-images/80411714/009.jpg,https://oleks-netizen.github.io/product-images/80411714/010.jpg,https://oleks-netizen.github.io/product-images/80411714/011.jpg,https://oleks-netizen.github.io/product-images/80411714/012.jpg,https://oleks-netizen.github.io/product-images/80411714/013.jpg,https://oleks-netizen.github.io/product-images/80411714/014.jpg</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>804600410</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/804600410/001.jpg,https://oleks-netizen.github.io/product-images/804600410/002.jpg,https://oleks-netizen.github.io/product-images/804600410/003.jpg,https://oleks-netizen.github.io/product-images/804600410/005.jpg,https://oleks-netizen.github.io/product-images/804600410/006.jpg,https://oleks-netizen.github.io/product-images/804600410/007.jpg,https://oleks-netizen.github.io/product-images/804600410/008.jpg,https://oleks-netizen.github.io/product-images/804600410/009.jpg,https://oleks-netizen.github.io/product-images/804600410/010.jpg,https://oleks-netizen.github.io/product-images/804600410/011.jpg,https://oleks-netizen.github.io/product-images/804600410/012.jpg,https://oleks-netizen.github.io/product-images/804600410/013.jpg,https://oleks-netizen.github.io/product-images/804600410/014.jpg,https://oleks-netizen.github.io/product-images/804600410/015.jpg,https://oleks-netizen.github.io/product-images/804600410/016.jpg</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>80460060</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/80460060/001.jpg,https://oleks-netizen.github.io/product-images/80460060/002.jpg,https://oleks-netizen.github.io/product-images/80460060/003.jpg,https://oleks-netizen.github.io/product-images/80460060/005.jpg,https://oleks-netizen.github.io/product-images/80460060/006.jpg,https://oleks-netizen.github.io/product-images/80460060/007.jpg,https://oleks-netizen.github.io/product-images/80460060/008.jpg,https://oleks-netizen.github.io/product-images/80460060/009.jpg,https://oleks-netizen.github.io/product-images/80460060/010.jpg,https://oleks-netizen.github.io/product-images/80460060/011.jpg,https://oleks-netizen.github.io/product-images/80460060/012.jpg,https://oleks-netizen.github.io/product-images/80460060/013.jpg,https://oleks-netizen.github.io/product-images/80460060/014.jpg,https://oleks-netizen.github.io/product-images/80460060/015.jpg,https://oleks-netizen.github.io/product-images/80460060/016.jpg</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>80460401</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/80460401/001.jpg,https://oleks-netizen.github.io/product-images/80460401/002.jpg,https://oleks-netizen.github.io/product-images/80460401/003.jpg,https://oleks-netizen.github.io/product-images/80460401/005.jpg,https://oleks-netizen.github.io/product-images/80460401/006.jpg,https://oleks-netizen.github.io/product-images/80460401/007.jpg,https://oleks-netizen.github.io/product-images/80460401/008.jpg,https://oleks-netizen.github.io/product-images/80460401/009.jpg,https://oleks-netizen.github.io/product-images/80460401/010.jpg,https://oleks-netizen.github.io/product-images/80460401/011.jpg,https://oleks-netizen.github.io/product-images/80460401/012.jpg,https://oleks-netizen.github.io/product-images/80460401/013.jpg,https://oleks-netizen.github.io/product-images/80460401/014.jpg,https://oleks-netizen.github.io/product-images/80460401/015.jpg,https://oleks-netizen.github.io/product-images/80460401/016.jpg</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>85151020</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/85151020/001.jpg,https://oleks-netizen.github.io/product-images/85151020/002.jpg,https://oleks-netizen.github.io/product-images/85151020/003.jpg,https://oleks-netizen.github.io/product-images/85151020/004.jpg,https://oleks-netizen.github.io/product-images/85151020/005.jpg,https://oleks-netizen.github.io/product-images/85151020/006.jpg,https://oleks-netizen.github.io/product-images/85151020/007.jpg,https://oleks-netizen.github.io/product-images/85151020/009.jpg</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>85451064</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/85451064/001.jpg,https://oleks-netizen.github.io/product-images/85451064/002.jpg,https://oleks-netizen.github.io/product-images/85451064/004.jpg,https://oleks-netizen.github.io/product-images/85451064/005.jpg,https://oleks-netizen.github.io/product-images/85451064/006.jpg,https://oleks-netizen.github.io/product-images/85451064/007.jpg,https://oleks-netizen.github.io/product-images/85451064/008.jpg,https://oleks-netizen.github.io/product-images/85451064/009.jpg,https://oleks-netizen.github.io/product-images/85451064/010.jpg,https://oleks-netizen.github.io/product-images/85451064/011.jpg,https://oleks-netizen.github.io/product-images/85451064/012.jpg,https://oleks-netizen.github.io/product-images/85451064/013.jpg,https://oleks-netizen.github.io/product-images/85451064/014.jpg</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>85451064m</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/85451064m/001.jpg,https://oleks-netizen.github.io/product-images/85451064m/002.jpg,https://oleks-netizen.github.io/product-images/85451064m/003.jpg,https://oleks-netizen.github.io/product-images/85451064m/004.jpg,https://oleks-netizen.github.io/product-images/85451064m/005.jpg,https://oleks-netizen.github.io/product-images/85451064m/006.jpg,https://oleks-netizen.github.io/product-images/85451064m/007.jpg,https://oleks-netizen.github.io/product-images/85451064m/009.jpg,https://oleks-netizen.github.io/product-images/85451064m/010.jpg,https://oleks-netizen.github.io/product-images/85451064m/011.jpg,https://oleks-netizen.github.io/product-images/85451064m/012.jpg,https://oleks-netizen.github.io/product-images/85451064m/013.jpg,https://oleks-netizen.github.io/product-images/85451064m/014.jpg</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>85451506</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/85451506/001.jpg,https://oleks-netizen.github.io/product-images/85451506/002.jpg,https://oleks-netizen.github.io/product-images/85451506/003.jpg,https://oleks-netizen.github.io/product-images/85451506/004.jpg,https://oleks-netizen.github.io/product-images/85451506/005.jpg,https://oleks-netizen.github.io/product-images/85451506/007.jpg,https://oleks-netizen.github.io/product-images/85451506/008.jpg,https://oleks-netizen.github.io/product-images/85451506/009.jpg,https://oleks-netizen.github.io/product-images/85451506/010.jpg,https://oleks-netizen.github.io/product-images/85451506/011.jpg,https://oleks-netizen.github.io/product-images/85451506/012.jpg,https://oleks-netizen.github.io/product-images/85451506/013.jpg,https://oleks-netizen.github.io/product-images/85451506/014.jpg</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>B085</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/B085/001.jpg,https://oleks-netizen.github.io/product-images/B085/002.jpg,https://oleks-netizen.github.io/product-images/B085/004.jpg,https://oleks-netizen.github.io/product-images/B085/005.jpg,https://oleks-netizen.github.io/product-images/B085/006.jpg</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>B158</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/B158/001.jpg,https://oleks-netizen.github.io/product-images/B158/002.jpg,https://oleks-netizen.github.io/product-images/B158/003.jpg,https://oleks-netizen.github.io/product-images/B158/004.jpg,https://oleks-netizen.github.io/product-images/B158/005.jpg,https://oleks-netizen.github.io/product-images/B158/006.jpg,https://oleks-netizen.github.io/product-images/B158/007.jpg,https://oleks-netizen.github.io/product-images/B158/009.jpg,https://oleks-netizen.github.io/product-images/B158/010.jpg,https://oleks-netizen.github.io/product-images/B158/011.jpg,https://oleks-netizen.github.io/product-images/B158/012.jpg,https://oleks-netizen.github.io/product-images/B158/013.jpg,https://oleks-netizen.github.io/product-images/B158/014.jpg,https://oleks-netizen.github.io/product-images/B158/015.jpg,https://oleks-netizen.github.io/product-images/B158/016.jpg,https://oleks-netizen.github.io/product-images/B158/017.jpg,https://oleks-netizen.github.io/product-images/B158/018.jpg,https://oleks-netizen.github.io/product-images/B158/019.jpg</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>BN-BAG-62-g</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-62-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/008.jpg</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BN-DC-7-k-kr</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/006.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/007.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/008.jpg</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>CC602_SN_BLK</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/CC602_SN_BLK/001.jpg,https://oleks-netizen.github.io/product-images/CC602_SN_BLK/002.jpg,https://oleks-netizen.github.io/product-images/CC602_SN_BLK/003.jpg,https://oleks-netizen.github.io/product-images/CC602_SN_BLK/005.jpg,https://oleks-netizen.github.io/product-images/CC602_SN_BLK/006.jpg,https://oleks-netizen.github.io/product-images/CC602_SN_BLK/007.jpg</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>L21360-010</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21360-010/001.jpg,https://oleks-netizen.github.io/product-images/L21360-010/002.jpg,https://oleks-netizen.github.io/product-images/L21360-010/004.jpg,https://oleks-netizen.github.io/product-images/L21360-010/005.jpg,https://oleks-netizen.github.io/product-images/L21360-010/006.jpg,https://oleks-netizen.github.io/product-images/L21360-010/007.jpg,https://oleks-netizen.github.io/product-images/L21360-010/008.jpg</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>L21360-021</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21360-021/001.jpg,https://oleks-netizen.github.io/product-images/L21360-021/002.jpg,https://oleks-netizen.github.io/product-images/L21360-021/004.jpg,https://oleks-netizen.github.io/product-images/L21360-021/005.jpg,https://oleks-netizen.github.io/product-images/L21360-021/006.jpg,https://oleks-netizen.github.io/product-images/L21360-021/007.jpg,https://oleks-netizen.github.io/product-images/L21360-021/008.jpg</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>L21360-025</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21360-025/001.jpg,https://oleks-netizen.github.io/product-images/L21360-025/002.jpg,https://oleks-netizen.github.io/product-images/L21360-025/003.jpg,https://oleks-netizen.github.io/product-images/L21360-025/005.jpg,https://oleks-netizen.github.io/product-images/L21360-025/006.jpg,https://oleks-netizen.github.io/product-images/L21360-025/007.jpg</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>L21563-010</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21563-010/001.jpg,https://oleks-netizen.github.io/product-images/L21563-010/002.jpg,https://oleks-netizen.github.io/product-images/L21563-010/003.jpg,https://oleks-netizen.github.io/product-images/L21563-010/005.jpg,https://oleks-netizen.github.io/product-images/L21563-010/006.jpg,https://oleks-netizen.github.io/product-images/L21563-010/007.jpg,https://oleks-netizen.github.io/product-images/L21563-010/008.jpg</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>L21563-038</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21563-038/001.jpg,https://oleks-netizen.github.io/product-images/L21563-038/002.jpg,https://oleks-netizen.github.io/product-images/L21563-038/003.jpg,https://oleks-netizen.github.io/product-images/L21563-038/005.jpg,https://oleks-netizen.github.io/product-images/L21563-038/006.jpg,https://oleks-netizen.github.io/product-images/L21563-038/007.jpg,https://oleks-netizen.github.io/product-images/L21563-038/008.jpg</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>L21563-045</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21563-045/001.jpg,https://oleks-netizen.github.io/product-images/L21563-045/002.jpg,https://oleks-netizen.github.io/product-images/L21563-045/003.jpg,https://oleks-netizen.github.io/product-images/L21563-045/005.jpg,https://oleks-netizen.github.io/product-images/L21563-045/006.jpg,https://oleks-netizen.github.io/product-images/L21563-045/007.jpg,https://oleks-netizen.github.io/product-images/L21563-045/008.jpg</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>L21564-010</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21564-010/001.jpg,https://oleks-netizen.github.io/product-images/L21564-010/002.jpg,https://oleks-netizen.github.io/product-images/L21564-010/003.jpg,https://oleks-netizen.github.io/product-images/L21564-010/005.jpg,https://oleks-netizen.github.io/product-images/L21564-010/006.jpg,https://oleks-netizen.github.io/product-images/L21564-010/007.jpg,https://oleks-netizen.github.io/product-images/L21564-010/008.jpg</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>L21564-025</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21564-025/001.jpg,https://oleks-netizen.github.io/product-images/L21564-025/002.jpg,https://oleks-netizen.github.io/product-images/L21564-025/003.jpg,https://oleks-netizen.github.io/product-images/L21564-025/005.jpg,https://oleks-netizen.github.io/product-images/L21564-025/006.jpg,https://oleks-netizen.github.io/product-images/L21564-025/007.jpg,https://oleks-netizen.github.io/product-images/L21564-025/008.jpg</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>L21564-066</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21564-066/001.jpg,https://oleks-netizen.github.io/product-images/L21564-066/002.jpg,https://oleks-netizen.github.io/product-images/L21564-066/003.jpg,https://oleks-netizen.github.io/product-images/L21564-066/005.jpg,https://oleks-netizen.github.io/product-images/L21564-066/006.jpg,https://oleks-netizen.github.io/product-images/L21564-066/007.jpg,https://oleks-netizen.github.io/product-images/L21564-066/008.jpg</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>L21580-1</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21580-1/001.jpg,https://oleks-netizen.github.io/product-images/L21580-1/002.jpg,https://oleks-netizen.github.io/product-images/L21580-1/003.jpg,https://oleks-netizen.github.io/product-images/L21580-1/005.jpg,https://oleks-netizen.github.io/product-images/L21580-1/006.jpg,https://oleks-netizen.github.io/product-images/L21580-1/007.jpg,https://oleks-netizen.github.io/product-images/L21580-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>L21580-175</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21580-175/001.jpg,https://oleks-netizen.github.io/product-images/L21580-175/002.jpg,https://oleks-netizen.github.io/product-images/L21580-175/003.jpg,https://oleks-netizen.github.io/product-images/L21580-175/005.jpg,https://oleks-netizen.github.io/product-images/L21580-175/006.jpg,https://oleks-netizen.github.io/product-images/L21580-175/007.jpg,https://oleks-netizen.github.io/product-images/L21580-175/008.jpg</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>L21580-49</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21580-49/001.jpg,https://oleks-netizen.github.io/product-images/L21580-49/002.jpg,https://oleks-netizen.github.io/product-images/L21580-49/003.jpg,https://oleks-netizen.github.io/product-images/L21580-49/005.jpg,https://oleks-netizen.github.io/product-images/L21580-49/006.jpg,https://oleks-netizen.github.io/product-images/L21580-49/007.jpg,https://oleks-netizen.github.io/product-images/L21580-49/008.jpg</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>L87025-01</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87025-01/001.jpg,https://oleks-netizen.github.io/product-images/L87025-01/002.jpg,https://oleks-netizen.github.io/product-images/L87025-01/003.jpg,https://oleks-netizen.github.io/product-images/L87025-01/005.jpg,https://oleks-netizen.github.io/product-images/L87025-01/006.jpg,https://oleks-netizen.github.io/product-images/L87025-01/007.jpg,https://oleks-netizen.github.io/product-images/L87025-01/008.jpg</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>L87025-13</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87025-13/001.jpg,https://oleks-netizen.github.io/product-images/L87025-13/002.jpg,https://oleks-netizen.github.io/product-images/L87025-13/003.jpg,https://oleks-netizen.github.io/product-images/L87025-13/005.jpg,https://oleks-netizen.github.io/product-images/L87025-13/006.jpg,https://oleks-netizen.github.io/product-images/L87025-13/007.jpg,https://oleks-netizen.github.io/product-images/L87025-13/008.jpg</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>L87025-23</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87025-23/001.jpg,https://oleks-netizen.github.io/product-images/L87025-23/002.jpg,https://oleks-netizen.github.io/product-images/L87025-23/003.jpg,https://oleks-netizen.github.io/product-images/L87025-23/005.jpg,https://oleks-netizen.github.io/product-images/L87025-23/006.jpg,https://oleks-netizen.github.io/product-images/L87025-23/007.jpg,https://oleks-netizen.github.io/product-images/L87025-23/008.jpg</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>L87025-26</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87025-26/001.jpg,https://oleks-netizen.github.io/product-images/L87025-26/002.jpg,https://oleks-netizen.github.io/product-images/L87025-26/003.jpg,https://oleks-netizen.github.io/product-images/L87025-26/005.jpg,https://oleks-netizen.github.io/product-images/L87025-26/006.jpg,https://oleks-netizen.github.io/product-images/L87025-26/007.jpg,https://oleks-netizen.github.io/product-images/L87025-26/008.jpg</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>L87093-01</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87093-01/001.jpg,https://oleks-netizen.github.io/product-images/L87093-01/002.jpg,https://oleks-netizen.github.io/product-images/L87093-01/004.jpg,https://oleks-netizen.github.io/product-images/L87093-01/005.jpg,https://oleks-netizen.github.io/product-images/L87093-01/006.jpg,https://oleks-netizen.github.io/product-images/L87093-01/007.jpg,https://oleks-netizen.github.io/product-images/L87093-01/008.jpg</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>L87093-108</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87093-108/001.jpg,https://oleks-netizen.github.io/product-images/L87093-108/003.jpg,https://oleks-netizen.github.io/product-images/L87093-108/004.jpg,https://oleks-netizen.github.io/product-images/L87093-108/005.jpg,https://oleks-netizen.github.io/product-images/L87093-108/006.jpg,https://oleks-netizen.github.io/product-images/L87093-108/007.jpg,https://oleks-netizen.github.io/product-images/L87093-108/008.jpg</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>L87093-245</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87093-245/001.jpg,https://oleks-netizen.github.io/product-images/L87093-245/003.jpg,https://oleks-netizen.github.io/product-images/L87093-245/004.jpg,https://oleks-netizen.github.io/product-images/L87093-245/005.jpg,https://oleks-netizen.github.io/product-images/L87093-245/006.jpg,https://oleks-netizen.github.io/product-images/L87093-245/007.jpg,https://oleks-netizen.github.io/product-images/L87093-245/008.jpg</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>L87093-246</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87093-246/001.jpg,https://oleks-netizen.github.io/product-images/L87093-246/002.jpg,https://oleks-netizen.github.io/product-images/L87093-246/004.jpg,https://oleks-netizen.github.io/product-images/L87093-246/005.jpg,https://oleks-netizen.github.io/product-images/L87093-246/006.jpg,https://oleks-netizen.github.io/product-images/L87093-246/007.jpg,https://oleks-netizen.github.io/product-images/L87093-246/008.jpg</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>L87114-01</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87114-01/001.jpg,https://oleks-netizen.github.io/product-images/L87114-01/002.jpg,https://oleks-netizen.github.io/product-images/L87114-01/003.jpg,https://oleks-netizen.github.io/product-images/L87114-01/005.jpg,https://oleks-netizen.github.io/product-images/L87114-01/006.jpg,https://oleks-netizen.github.io/product-images/L87114-01/007.jpg,https://oleks-netizen.github.io/product-images/L87114-01/008.jpg</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>L87114-108</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87114-108/001.jpg,https://oleks-netizen.github.io/product-images/L87114-108/002.jpg,https://oleks-netizen.github.io/product-images/L87114-108/003.jpg,https://oleks-netizen.github.io/product-images/L87114-108/005.jpg,https://oleks-netizen.github.io/product-images/L87114-108/006.jpg,https://oleks-netizen.github.io/product-images/L87114-108/007.jpg</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>L87114-246</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87114-246/001.jpg,https://oleks-netizen.github.io/product-images/L87114-246/002.jpg,https://oleks-netizen.github.io/product-images/L87114-246/003.jpg,https://oleks-netizen.github.io/product-images/L87114-246/005.jpg,https://oleks-netizen.github.io/product-images/L87114-246/006.jpg,https://oleks-netizen.github.io/product-images/L87114-246/007.jpg,https://oleks-netizen.github.io/product-images/L87114-246/008.jpg</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>L87169-01</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87169-01/001.jpg,https://oleks-netizen.github.io/product-images/L87169-01/002.jpg,https://oleks-netizen.github.io/product-images/L87169-01/003.jpg,https://oleks-netizen.github.io/product-images/L87169-01/005.jpg,https://oleks-netizen.github.io/product-images/L87169-01/006.jpg,https://oleks-netizen.github.io/product-images/L87169-01/007.jpg,https://oleks-netizen.github.io/product-images/L87169-01/008.jpg</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>L87169-113</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87169-113/001.jpg,https://oleks-netizen.github.io/product-images/L87169-113/002.jpg,https://oleks-netizen.github.io/product-images/L87169-113/003.jpg,https://oleks-netizen.github.io/product-images/L87169-113/005.jpg,https://oleks-netizen.github.io/product-images/L87169-113/006.jpg,https://oleks-netizen.github.io/product-images/L87169-113/007.jpg,https://oleks-netizen.github.io/product-images/L87169-113/008.jpg</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>L87169-175</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87169-175/001.jpg,https://oleks-netizen.github.io/product-images/L87169-175/002.jpg,https://oleks-netizen.github.io/product-images/L87169-175/003.jpg,https://oleks-netizen.github.io/product-images/L87169-175/005.jpg,https://oleks-netizen.github.io/product-images/L87169-175/006.jpg,https://oleks-netizen.github.io/product-images/L87169-175/007.jpg,https://oleks-netizen.github.io/product-images/L87169-175/008.jpg</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>L87169-81</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87169-81/001.jpg,https://oleks-netizen.github.io/product-images/L87169-81/002.jpg,https://oleks-netizen.github.io/product-images/L87169-81/003.jpg,https://oleks-netizen.github.io/product-images/L87169-81/005.jpg,https://oleks-netizen.github.io/product-images/L87169-81/006.jpg,https://oleks-netizen.github.io/product-images/L87169-81/007.jpg,https://oleks-netizen.github.io/product-images/L87169-81/008.jpg</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>L87518-01</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87518-01/001.jpg,https://oleks-netizen.github.io/product-images/L87518-01/002.jpg,https://oleks-netizen.github.io/product-images/L87518-01/003.jpg,https://oleks-netizen.github.io/product-images/L87518-01/005.jpg,https://oleks-netizen.github.io/product-images/L87518-01/006.jpg,https://oleks-netizen.github.io/product-images/L87518-01/007.jpg,https://oleks-netizen.github.io/product-images/L87518-01/008.jpg</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>L87518-56</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87518-56/001.jpg,https://oleks-netizen.github.io/product-images/L87518-56/002.jpg,https://oleks-netizen.github.io/product-images/L87518-56/004.jpg,https://oleks-netizen.github.io/product-images/L87518-56/005.jpg,https://oleks-netizen.github.io/product-images/L87518-56/006.jpg,https://oleks-netizen.github.io/product-images/L87518-56/007.jpg,https://oleks-netizen.github.io/product-images/L87518-56/008.jpg</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>L87518-79</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87518-79/001.jpg,https://oleks-netizen.github.io/product-images/L87518-79/002.jpg,https://oleks-netizen.github.io/product-images/L87518-79/004.jpg,https://oleks-netizen.github.io/product-images/L87518-79/005.jpg,https://oleks-netizen.github.io/product-images/L87518-79/006.jpg,https://oleks-netizen.github.io/product-images/L87518-79/007.jpg,https://oleks-netizen.github.io/product-images/L87518-79/008.jpg</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>L87713-01</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87713-01/001.jpg,https://oleks-netizen.github.io/product-images/L87713-01/002.jpg,https://oleks-netizen.github.io/product-images/L87713-01/003.jpg,https://oleks-netizen.github.io/product-images/L87713-01/005.jpg,https://oleks-netizen.github.io/product-images/L87713-01/006.jpg,https://oleks-netizen.github.io/product-images/L87713-01/007.jpg,https://oleks-netizen.github.io/product-images/L87713-01/008.jpg</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>L87713-107</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87713-107/001.jpg,https://oleks-netizen.github.io/product-images/L87713-107/002.jpg,https://oleks-netizen.github.io/product-images/L87713-107/003.jpg,https://oleks-netizen.github.io/product-images/L87713-107/005.jpg,https://oleks-netizen.github.io/product-images/L87713-107/006.jpg,https://oleks-netizen.github.io/product-images/L87713-107/007.jpg,https://oleks-netizen.github.io/product-images/L87713-107/008.jpg</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>L87713-221</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87713-221/001.jpg,https://oleks-netizen.github.io/product-images/L87713-221/002.jpg,https://oleks-netizen.github.io/product-images/L87713-221/003.jpg,https://oleks-netizen.github.io/product-images/L87713-221/005.jpg,https://oleks-netizen.github.io/product-images/L87713-221/006.jpg,https://oleks-netizen.github.io/product-images/L87713-221/007.jpg,https://oleks-netizen.github.io/product-images/L87713-221/008.jpg</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>L87713-97</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87713-97/001.jpg,https://oleks-netizen.github.io/product-images/L87713-97/002.jpg,https://oleks-netizen.github.io/product-images/L87713-97/003.jpg,https://oleks-netizen.github.io/product-images/L87713-97/005.jpg,https://oleks-netizen.github.io/product-images/L87713-97/006.jpg,https://oleks-netizen.github.io/product-images/L87713-97/007.jpg,https://oleks-netizen.github.io/product-images/L87713-97/008.jpg</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>TW-Vivian-mokko</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Vivian-mokko/001.jpg,https://oleks-netizen.github.io/product-images/TW-Vivian-mokko/002.jpg,https://oleks-netizen.github.io/product-images/TW-Vivian-mokko/004.jpg,https://oleks-netizen.github.io/product-images/TW-Vivian-mokko/005.jpg,https://oleks-netizen.github.io/product-images/TW-Vivian-mokko/006.jpg</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-04-03 19:50:42
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,252 +436,252 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18228066</t>
+          <t>1733_1_1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/18228066/001.jpg,https://oleks-netizen.github.io/product-images/18228066/002.jpg,https://oleks-netizen.github.io/product-images/18228066/003.jpg,https://oleks-netizen.github.io/product-images/18228066/004.jpg,https://oleks-netizen.github.io/product-images/18228066/005.jpg,https://oleks-netizen.github.io/product-images/18228066/006.jpg,https://oleks-netizen.github.io/product-images/18228066/007.jpg,https://oleks-netizen.github.io/product-images/18228066/008.jpg,https://oleks-netizen.github.io/product-images/18228066/009.jpg,https://oleks-netizen.github.io/product-images/18228066/011.jpg,https://oleks-netizen.github.io/product-images/18228066/012.jpg,https://oleks-netizen.github.io/product-images/18228066/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/1733_1_1/001.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18228067</t>
+          <t>206120</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/18228067/001.jpg,https://oleks-netizen.github.io/product-images/18228067/002.jpg,https://oleks-netizen.github.io/product-images/18228067/003.jpg,https://oleks-netizen.github.io/product-images/18228067/005.jpg,https://oleks-netizen.github.io/product-images/18228067/006.jpg,https://oleks-netizen.github.io/product-images/18228067/007.jpg,https://oleks-netizen.github.io/product-images/18228067/008.jpg,https://oleks-netizen.github.io/product-images/18228067/009.jpg,https://oleks-netizen.github.io/product-images/18228067/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/206120/001.jpg,https://oleks-netizen.github.io/product-images/206120/002.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18228068</t>
+          <t>20906_1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/18228068/001.jpg,https://oleks-netizen.github.io/product-images/18228068/002.jpg,https://oleks-netizen.github.io/product-images/18228068/003.jpg,https://oleks-netizen.github.io/product-images/18228068/004.jpg,https://oleks-netizen.github.io/product-images/18228068/005.jpg,https://oleks-netizen.github.io/product-images/18228068/007.jpg,https://oleks-netizen.github.io/product-images/18228068/008.jpg,https://oleks-netizen.github.io/product-images/18228068/009.jpg,https://oleks-netizen.github.io/product-images/18228068/010.jpg,https://oleks-netizen.github.io/product-images/18228068/011.jpg,https://oleks-netizen.github.io/product-images/18228068/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/20906_1/001.jpg,https://oleks-netizen.github.io/product-images/20906_1/003.jpg,https://oleks-netizen.github.io/product-images/20906_1/004.jpg,https://oleks-netizen.github.io/product-images/20906_1/005.jpg,https://oleks-netizen.github.io/product-images/20906_1/007.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25000506</t>
+          <t>2140_1_1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/25000506/001.jpg,https://oleks-netizen.github.io/product-images/25000506/002.jpg,https://oleks-netizen.github.io/product-images/25000506/003.jpg,https://oleks-netizen.github.io/product-images/25000506/004.jpg,https://oleks-netizen.github.io/product-images/25000506/005.jpg,https://oleks-netizen.github.io/product-images/25000506/006.jpg,https://oleks-netizen.github.io/product-images/25000506/007.jpg,https://oleks-netizen.github.io/product-images/25000506/009.jpg,https://oleks-netizen.github.io/product-images/25000506/010.jpg,https://oleks-netizen.github.io/product-images/25000506/011.jpg,https://oleks-netizen.github.io/product-images/25000506/012.jpg,https://oleks-netizen.github.io/product-images/25000506/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/2140_1_1/001.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>25000514</t>
+          <t>224420</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/25000514/001.jpg,https://oleks-netizen.github.io/product-images/25000514/002.jpg,https://oleks-netizen.github.io/product-images/25000514/003.jpg,https://oleks-netizen.github.io/product-images/25000514/004.jpg,https://oleks-netizen.github.io/product-images/25000514/005.jpg,https://oleks-netizen.github.io/product-images/25000514/006.jpg,https://oleks-netizen.github.io/product-images/25000514/007.jpg,https://oleks-netizen.github.io/product-images/25000514/008.jpg,https://oleks-netizen.github.io/product-images/25000514/009.jpg,https://oleks-netizen.github.io/product-images/25000514/011.jpg,https://oleks-netizen.github.io/product-images/25000514/012.jpg,https://oleks-netizen.github.io/product-images/25000514/013.jpg,https://oleks-netizen.github.io/product-images/25000514/014.jpg,https://oleks-netizen.github.io/product-images/25000514/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/224420/001.jpg,https://oleks-netizen.github.io/product-images/224420/002.jpg,https://oleks-netizen.github.io/product-images/224420/003.jpg,https://oleks-netizen.github.io/product-images/224420/004.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>25000514m</t>
+          <t>2338_1_5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/25000514m/001.jpg,https://oleks-netizen.github.io/product-images/25000514m/002.jpg,https://oleks-netizen.github.io/product-images/25000514m/004.jpg,https://oleks-netizen.github.io/product-images/25000514m/005.jpg,https://oleks-netizen.github.io/product-images/25000514m/006.jpg,https://oleks-netizen.github.io/product-images/25000514m/007.jpg,https://oleks-netizen.github.io/product-images/25000514m/008.jpg,https://oleks-netizen.github.io/product-images/25000514m/009.jpg,https://oleks-netizen.github.io/product-images/25000514m/010.jpg,https://oleks-netizen.github.io/product-images/25000514m/011.jpg,https://oleks-netizen.github.io/product-images/25000514m/012.jpg,https://oleks-netizen.github.io/product-images/25000514m/013.jpg,https://oleks-netizen.github.io/product-images/25000514m/014.jpg,https://oleks-netizen.github.io/product-images/25000514m/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/2338_1_5/001.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>25000515</t>
+          <t>2421_1_2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/25000515/001.jpg,https://oleks-netizen.github.io/product-images/25000515/002.jpg,https://oleks-netizen.github.io/product-images/25000515/003.jpg,https://oleks-netizen.github.io/product-images/25000515/005.jpg,https://oleks-netizen.github.io/product-images/25000515/006.jpg,https://oleks-netizen.github.io/product-images/25000515/007.jpg,https://oleks-netizen.github.io/product-images/25000515/008.jpg,https://oleks-netizen.github.io/product-images/25000515/009.jpg,https://oleks-netizen.github.io/product-images/25000515/010.jpg,https://oleks-netizen.github.io/product-images/25000515/011.jpg,https://oleks-netizen.github.io/product-images/25000515/012.jpg,https://oleks-netizen.github.io/product-images/25000515/013.jpg,https://oleks-netizen.github.io/product-images/25000515/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/2421_1_2/001.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>25000515m</t>
+          <t>2423_1_100</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/25000515m/001.jpg,https://oleks-netizen.github.io/product-images/25000515m/002.jpg,https://oleks-netizen.github.io/product-images/25000515m/003.jpg,https://oleks-netizen.github.io/product-images/25000515m/004.jpg,https://oleks-netizen.github.io/product-images/25000515m/005.jpg,https://oleks-netizen.github.io/product-images/25000515m/007.jpg,https://oleks-netizen.github.io/product-images/25000515m/008.jpg,https://oleks-netizen.github.io/product-images/25000515m/009.jpg,https://oleks-netizen.github.io/product-images/25000515m/010.jpg,https://oleks-netizen.github.io/product-images/25000515m/011.jpg,https://oleks-netizen.github.io/product-images/25000515m/012.jpg,https://oleks-netizen.github.io/product-images/25000515m/013.jpg,https://oleks-netizen.github.io/product-images/25000515m/014.jpg,https://oleks-netizen.github.io/product-images/25000515m/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/2423_1_100/001.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>51311506</t>
+          <t>2459_1_6</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/51311506/001.jpg,https://oleks-netizen.github.io/product-images/51311506/002.jpg,https://oleks-netizen.github.io/product-images/51311506/003.jpg,https://oleks-netizen.github.io/product-images/51311506/004.jpg,https://oleks-netizen.github.io/product-images/51311506/005.jpg,https://oleks-netizen.github.io/product-images/51311506/006.jpg,https://oleks-netizen.github.io/product-images/51311506/008.jpg,https://oleks-netizen.github.io/product-images/51311506/009.jpg,https://oleks-netizen.github.io/product-images/51311506/010.jpg,https://oleks-netizen.github.io/product-images/51311506/011.jpg,https://oleks-netizen.github.io/product-images/51311506/012.jpg,https://oleks-netizen.github.io/product-images/51311506/013.jpg,https://oleks-netizen.github.io/product-images/51311506/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/2459_1_6/001.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>51411006</t>
+          <t>25000010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/51411006/001.jpg,https://oleks-netizen.github.io/product-images/51411006/002.jpg,https://oleks-netizen.github.io/product-images/51411006/003.jpg,https://oleks-netizen.github.io/product-images/51411006/004.jpg,https://oleks-netizen.github.io/product-images/51411006/005.jpg,https://oleks-netizen.github.io/product-images/51411006/006.jpg,https://oleks-netizen.github.io/product-images/51411006/008.jpg,https://oleks-netizen.github.io/product-images/51411006/009.jpg,https://oleks-netizen.github.io/product-images/51411006/010.jpg,https://oleks-netizen.github.io/product-images/51411006/011.jpg,https://oleks-netizen.github.io/product-images/51411006/012.jpg,https://oleks-netizen.github.io/product-images/51411006/013.jpg,https://oleks-netizen.github.io/product-images/51411006/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000010/001.jpg,https://oleks-netizen.github.io/product-images/25000010/002.jpg,https://oleks-netizen.github.io/product-images/25000010/003.jpg,https://oleks-netizen.github.io/product-images/25000010/005.jpg,https://oleks-netizen.github.io/product-images/25000010/006.jpg,https://oleks-netizen.github.io/product-images/25000010/007.jpg,https://oleks-netizen.github.io/product-images/25000010/008.jpg,https://oleks-netizen.github.io/product-images/25000010/009.jpg,https://oleks-netizen.github.io/product-images/25000010/010.jpg,https://oleks-netizen.github.io/product-images/25000010/011.jpg,https://oleks-netizen.github.io/product-images/25000010/012.jpg,https://oleks-netizen.github.io/product-images/25000010/013.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>51411506</t>
+          <t>25000010m</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/51411506/001.jpg,https://oleks-netizen.github.io/product-images/51411506/002.jpg,https://oleks-netizen.github.io/product-images/51411506/003.jpg,https://oleks-netizen.github.io/product-images/51411506/004.jpg,https://oleks-netizen.github.io/product-images/51411506/005.jpg,https://oleks-netizen.github.io/product-images/51411506/006.jpg,https://oleks-netizen.github.io/product-images/51411506/007.jpg,https://oleks-netizen.github.io/product-images/51411506/009.jpg,https://oleks-netizen.github.io/product-images/51411506/010.jpg,https://oleks-netizen.github.io/product-images/51411506/011.jpg,https://oleks-netizen.github.io/product-images/51411506/012.jpg,https://oleks-netizen.github.io/product-images/51411506/013.jpg,https://oleks-netizen.github.io/product-images/51411506/014.jpg,https://oleks-netizen.github.io/product-images/51411506/015.jpg,https://oleks-netizen.github.io/product-images/51411506/016.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000010m/001.jpg,https://oleks-netizen.github.io/product-images/25000010m/002.jpg,https://oleks-netizen.github.io/product-images/25000010m/004.jpg,https://oleks-netizen.github.io/product-images/25000010m/005.jpg,https://oleks-netizen.github.io/product-images/25000010m/006.jpg,https://oleks-netizen.github.io/product-images/25000010m/007.jpg,https://oleks-netizen.github.io/product-images/25000010m/008.jpg,https://oleks-netizen.github.io/product-images/25000010m/009.jpg,https://oleks-netizen.github.io/product-images/25000010m/010.jpg,https://oleks-netizen.github.io/product-images/25000010m/011.jpg,https://oleks-netizen.github.io/product-images/25000010m/012.jpg,https://oleks-netizen.github.io/product-images/25000010m/013.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>53100066</t>
+          <t>25000064</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53100066/001.jpg,https://oleks-netizen.github.io/product-images/53100066/002.jpg,https://oleks-netizen.github.io/product-images/53100066/003.jpg,https://oleks-netizen.github.io/product-images/53100066/004.jpg,https://oleks-netizen.github.io/product-images/53100066/005.jpg,https://oleks-netizen.github.io/product-images/53100066/006.jpg,https://oleks-netizen.github.io/product-images/53100066/007.jpg,https://oleks-netizen.github.io/product-images/53100066/009.jpg,https://oleks-netizen.github.io/product-images/53100066/010.jpg,https://oleks-netizen.github.io/product-images/53100066/011.jpg,https://oleks-netizen.github.io/product-images/53100066/012.jpg,https://oleks-netizen.github.io/product-images/53100066/013.jpg,https://oleks-netizen.github.io/product-images/53100066/014.jpg,https://oleks-netizen.github.io/product-images/53100066/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000064/001.jpg,https://oleks-netizen.github.io/product-images/25000064/002.jpg,https://oleks-netizen.github.io/product-images/25000064/003.jpg,https://oleks-netizen.github.io/product-images/25000064/005.jpg,https://oleks-netizen.github.io/product-images/25000064/006.jpg,https://oleks-netizen.github.io/product-images/25000064/007.jpg,https://oleks-netizen.github.io/product-images/25000064/008.jpg,https://oleks-netizen.github.io/product-images/25000064/009.jpg,https://oleks-netizen.github.io/product-images/25000064/010.jpg,https://oleks-netizen.github.io/product-images/25000064/011.jpg,https://oleks-netizen.github.io/product-images/25000064/012.jpg,https://oleks-netizen.github.io/product-images/25000064/013.jpg,https://oleks-netizen.github.io/product-images/25000064/014.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>53100106</t>
+          <t>25000064m</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53100106/001.jpg,https://oleks-netizen.github.io/product-images/53100106/002.jpg,https://oleks-netizen.github.io/product-images/53100106/003.jpg,https://oleks-netizen.github.io/product-images/53100106/004.jpg,https://oleks-netizen.github.io/product-images/53100106/005.jpg,https://oleks-netizen.github.io/product-images/53100106/007.jpg,https://oleks-netizen.github.io/product-images/53100106/008.jpg,https://oleks-netizen.github.io/product-images/53100106/009.jpg,https://oleks-netizen.github.io/product-images/53100106/010.jpg,https://oleks-netizen.github.io/product-images/53100106/011.jpg,https://oleks-netizen.github.io/product-images/53100106/012.jpg,https://oleks-netizen.github.io/product-images/53100106/013.jpg,https://oleks-netizen.github.io/product-images/53100106/014.jpg,https://oleks-netizen.github.io/product-images/53100106/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000064m/001.jpg,https://oleks-netizen.github.io/product-images/25000064m/003.jpg,https://oleks-netizen.github.io/product-images/25000064m/004.jpg,https://oleks-netizen.github.io/product-images/25000064m/005.jpg,https://oleks-netizen.github.io/product-images/25000064m/006.jpg,https://oleks-netizen.github.io/product-images/25000064m/007.jpg,https://oleks-netizen.github.io/product-images/25000064m/008.jpg,https://oleks-netizen.github.io/product-images/25000064m/009.jpg,https://oleks-netizen.github.io/product-images/25000064m/010.jpg,https://oleks-netizen.github.io/product-images/25000064m/011.jpg,https://oleks-netizen.github.io/product-images/25000064m/012.jpg,https://oleks-netizen.github.io/product-images/25000064m/013.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>53300066</t>
+          <t>25000264</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53300066/001.jpg,https://oleks-netizen.github.io/product-images/53300066/002.jpg,https://oleks-netizen.github.io/product-images/53300066/003.jpg,https://oleks-netizen.github.io/product-images/53300066/004.jpg,https://oleks-netizen.github.io/product-images/53300066/005.jpg,https://oleks-netizen.github.io/product-images/53300066/006.jpg,https://oleks-netizen.github.io/product-images/53300066/007.jpg,https://oleks-netizen.github.io/product-images/53300066/009.jpg,https://oleks-netizen.github.io/product-images/53300066/010.jpg,https://oleks-netizen.github.io/product-images/53300066/011.jpg,https://oleks-netizen.github.io/product-images/53300066/012.jpg,https://oleks-netizen.github.io/product-images/53300066/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000264/001.jpg,https://oleks-netizen.github.io/product-images/25000264/002.jpg,https://oleks-netizen.github.io/product-images/25000264/003.jpg,https://oleks-netizen.github.io/product-images/25000264/004.jpg,https://oleks-netizen.github.io/product-images/25000264/005.jpg,https://oleks-netizen.github.io/product-images/25000264/007.jpg,https://oleks-netizen.github.io/product-images/25000264/008.jpg,https://oleks-netizen.github.io/product-images/25000264/009.jpg,https://oleks-netizen.github.io/product-images/25000264/010.jpg,https://oleks-netizen.github.io/product-images/25000264/011.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>53330029</t>
+          <t>25000264m</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330029/001.jpg,https://oleks-netizen.github.io/product-images/53330029/002.jpg,https://oleks-netizen.github.io/product-images/53330029/003.jpg,https://oleks-netizen.github.io/product-images/53330029/004.jpg,https://oleks-netizen.github.io/product-images/53330029/005.jpg,https://oleks-netizen.github.io/product-images/53330029/006.jpg,https://oleks-netizen.github.io/product-images/53330029/008.jpg,https://oleks-netizen.github.io/product-images/53330029/009.jpg,https://oleks-netizen.github.io/product-images/53330029/010.jpg,https://oleks-netizen.github.io/product-images/53330029/011.jpg,https://oleks-netizen.github.io/product-images/53330029/012.jpg,https://oleks-netizen.github.io/product-images/53330029/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25000264m/001.jpg,https://oleks-netizen.github.io/product-images/25000264m/002.jpg,https://oleks-netizen.github.io/product-images/25000264m/003.jpg,https://oleks-netizen.github.io/product-images/25000264m/004.jpg,https://oleks-netizen.github.io/product-images/25000264m/005.jpg,https://oleks-netizen.github.io/product-images/25000264m/006.jpg,https://oleks-netizen.github.io/product-images/25000264m/007.jpg,https://oleks-netizen.github.io/product-images/25000264m/008.jpg,https://oleks-netizen.github.io/product-images/25000264m/010.jpg,https://oleks-netizen.github.io/product-images/25000264m/011.jpg,https://oleks-netizen.github.io/product-images/25000264m/012.jpg,https://oleks-netizen.github.io/product-images/25000264m/013.jpg,https://oleks-netizen.github.io/product-images/25000264m/014.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>53330029m</t>
+          <t>25428164</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330029m/001.jpg,https://oleks-netizen.github.io/product-images/53330029m/002.jpg,https://oleks-netizen.github.io/product-images/53330029m/003.jpg,https://oleks-netizen.github.io/product-images/53330029m/004.jpg,https://oleks-netizen.github.io/product-images/53330029m/005.jpg,https://oleks-netizen.github.io/product-images/53330029m/006.jpg,https://oleks-netizen.github.io/product-images/53330029m/008.jpg,https://oleks-netizen.github.io/product-images/53330029m/009.jpg,https://oleks-netizen.github.io/product-images/53330029m/010.jpg,https://oleks-netizen.github.io/product-images/53330029m/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25428164/001.jpg,https://oleks-netizen.github.io/product-images/25428164/002.jpg,https://oleks-netizen.github.io/product-images/25428164/003.jpg,https://oleks-netizen.github.io/product-images/25428164/004.jpg,https://oleks-netizen.github.io/product-images/25428164/005.jpg,https://oleks-netizen.github.io/product-images/25428164/007.jpg,https://oleks-netizen.github.io/product-images/25428164/008.jpg,https://oleks-netizen.github.io/product-images/25428164/009.jpg,https://oleks-netizen.github.io/product-images/25428164/010.jpg,https://oleks-netizen.github.io/product-images/25428164/011.jpg,https://oleks-netizen.github.io/product-images/25428164/012.jpg,https://oleks-netizen.github.io/product-images/25428164/013.jpg,https://oleks-netizen.github.io/product-images/25428164/014.jpg</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>53330064</t>
+          <t>25428164m</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330064/001.jpg,https://oleks-netizen.github.io/product-images/53330064/002.jpg,https://oleks-netizen.github.io/product-images/53330064/003.jpg,https://oleks-netizen.github.io/product-images/53330064/004.jpg,https://oleks-netizen.github.io/product-images/53330064/005.jpg,https://oleks-netizen.github.io/product-images/53330064/006.jpg,https://oleks-netizen.github.io/product-images/53330064/007.jpg,https://oleks-netizen.github.io/product-images/53330064/008.jpg,https://oleks-netizen.github.io/product-images/53330064/009.jpg,https://oleks-netizen.github.io/product-images/53330064/010.jpg,https://oleks-netizen.github.io/product-images/53330064/011.jpg,https://oleks-netizen.github.io/product-images/53330064/013.jpg,https://oleks-netizen.github.io/product-images/53330064/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25428164m/001.jpg,https://oleks-netizen.github.io/product-images/25428164m/002.jpg,https://oleks-netizen.github.io/product-images/25428164m/004.jpg,https://oleks-netizen.github.io/product-images/25428164m/005.jpg,https://oleks-netizen.github.io/product-images/25428164m/006.jpg,https://oleks-netizen.github.io/product-images/25428164m/007.jpg,https://oleks-netizen.github.io/product-images/25428164m/008.jpg,https://oleks-netizen.github.io/product-images/25428164m/009.jpg,https://oleks-netizen.github.io/product-images/25428164m/010.jpg,https://oleks-netizen.github.io/product-images/25428164m/011.jpg,https://oleks-netizen.github.io/product-images/25428164m/012.jpg,https://oleks-netizen.github.io/product-images/25428164m/013.jpg,https://oleks-netizen.github.io/product-images/25428164m/014.jpg</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -691,27 +691,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>53330064m</t>
+          <t>25438115</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330064m/001.jpg,https://oleks-netizen.github.io/product-images/53330064m/002.jpg,https://oleks-netizen.github.io/product-images/53330064m/003.jpg,https://oleks-netizen.github.io/product-images/53330064m/004.jpg,https://oleks-netizen.github.io/product-images/53330064m/006.jpg,https://oleks-netizen.github.io/product-images/53330064m/007.jpg,https://oleks-netizen.github.io/product-images/53330064m/008.jpg,https://oleks-netizen.github.io/product-images/53330064m/009.jpg,https://oleks-netizen.github.io/product-images/53330064m/010.jpg,https://oleks-netizen.github.io/product-images/53330064m/011.jpg,https://oleks-netizen.github.io/product-images/53330064m/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25438115/001.jpg,https://oleks-netizen.github.io/product-images/25438115/002.jpg,https://oleks-netizen.github.io/product-images/25438115/003.jpg,https://oleks-netizen.github.io/product-images/25438115/004.jpg,https://oleks-netizen.github.io/product-images/25438115/006.jpg,https://oleks-netizen.github.io/product-images/25438115/007.jpg,https://oleks-netizen.github.io/product-images/25438115/008.jpg,https://oleks-netizen.github.io/product-images/25438115/009.jpg,https://oleks-netizen.github.io/product-images/25438115/010.jpg,https://oleks-netizen.github.io/product-images/25438115/011.jpg,https://oleks-netizen.github.io/product-images/25438115/012.jpg,https://oleks-netizen.github.io/product-images/25438115/013.jpg,https://oleks-netizen.github.io/product-images/25438115/014.jpg,https://oleks-netizen.github.io/product-images/25438115/015.jpg</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>53330066</t>
+          <t>25438115m</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330066/001.jpg,https://oleks-netizen.github.io/product-images/53330066/002.jpg,https://oleks-netizen.github.io/product-images/53330066/003.jpg,https://oleks-netizen.github.io/product-images/53330066/004.jpg,https://oleks-netizen.github.io/product-images/53330066/005.jpg,https://oleks-netizen.github.io/product-images/53330066/007.jpg,https://oleks-netizen.github.io/product-images/53330066/008.jpg,https://oleks-netizen.github.io/product-images/53330066/009.jpg,https://oleks-netizen.github.io/product-images/53330066/010.jpg,https://oleks-netizen.github.io/product-images/53330066/011.jpg,https://oleks-netizen.github.io/product-images/53330066/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25438115m/001.jpg,https://oleks-netizen.github.io/product-images/25438115m/002.jpg,https://oleks-netizen.github.io/product-images/25438115m/004.jpg,https://oleks-netizen.github.io/product-images/25438115m/005.jpg,https://oleks-netizen.github.io/product-images/25438115m/006.jpg,https://oleks-netizen.github.io/product-images/25438115m/007.jpg,https://oleks-netizen.github.io/product-images/25438115m/008.jpg,https://oleks-netizen.github.io/product-images/25438115m/009.jpg,https://oleks-netizen.github.io/product-images/25438115m/010.jpg,https://oleks-netizen.github.io/product-images/25438115m/011.jpg,https://oleks-netizen.github.io/product-images/25438115m/012.jpg</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -721,12 +721,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>53330068</t>
+          <t>25438164</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330068/001.jpg,https://oleks-netizen.github.io/product-images/53330068/002.jpg,https://oleks-netizen.github.io/product-images/53330068/003.jpg,https://oleks-netizen.github.io/product-images/53330068/004.jpg,https://oleks-netizen.github.io/product-images/53330068/005.jpg,https://oleks-netizen.github.io/product-images/53330068/006.jpg,https://oleks-netizen.github.io/product-images/53330068/007.jpg,https://oleks-netizen.github.io/product-images/53330068/009.jpg,https://oleks-netizen.github.io/product-images/53330068/010.jpg,https://oleks-netizen.github.io/product-images/53330068/011.jpg,https://oleks-netizen.github.io/product-images/53330068/012.jpg,https://oleks-netizen.github.io/product-images/53330068/013.jpg,https://oleks-netizen.github.io/product-images/53330068/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25438164/001.jpg,https://oleks-netizen.github.io/product-images/25438164/002.jpg,https://oleks-netizen.github.io/product-images/25438164/003.jpg,https://oleks-netizen.github.io/product-images/25438164/004.jpg,https://oleks-netizen.github.io/product-images/25438164/005.jpg,https://oleks-netizen.github.io/product-images/25438164/006.jpg,https://oleks-netizen.github.io/product-images/25438164/007.jpg,https://oleks-netizen.github.io/product-images/25438164/008.jpg,https://oleks-netizen.github.io/product-images/25438164/009.jpg,https://oleks-netizen.github.io/product-images/25438164/010.jpg,https://oleks-netizen.github.io/product-images/25438164/011.jpg,https://oleks-netizen.github.io/product-images/25438164/012.jpg,https://oleks-netizen.github.io/product-images/25438164/014.jpg</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -736,552 +736,552 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>53330514</t>
+          <t>25438164m</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330514/001.jpg,https://oleks-netizen.github.io/product-images/53330514/002.jpg,https://oleks-netizen.github.io/product-images/53330514/003.jpg,https://oleks-netizen.github.io/product-images/53330514/004.jpg,https://oleks-netizen.github.io/product-images/53330514/005.jpg,https://oleks-netizen.github.io/product-images/53330514/006.jpg,https://oleks-netizen.github.io/product-images/53330514/008.jpg,https://oleks-netizen.github.io/product-images/53330514/009.jpg,https://oleks-netizen.github.io/product-images/53330514/010.jpg,https://oleks-netizen.github.io/product-images/53330514/011.jpg,https://oleks-netizen.github.io/product-images/53330514/012.jpg,https://oleks-netizen.github.io/product-images/53330514/013.jpg,https://oleks-netizen.github.io/product-images/53330514/014.jpg,https://oleks-netizen.github.io/product-images/53330514/015.jpg,https://oleks-netizen.github.io/product-images/53330514/016.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/25438164m/001.jpg,https://oleks-netizen.github.io/product-images/25438164m/002.jpg,https://oleks-netizen.github.io/product-images/25438164m/003.jpg,https://oleks-netizen.github.io/product-images/25438164m/004.jpg,https://oleks-netizen.github.io/product-images/25438164m/005.jpg,https://oleks-netizen.github.io/product-images/25438164m/006.jpg,https://oleks-netizen.github.io/product-images/25438164m/007.jpg,https://oleks-netizen.github.io/product-images/25438164m/008.jpg,https://oleks-netizen.github.io/product-images/25438164m/009.jpg,https://oleks-netizen.github.io/product-images/25438164m/010.jpg,https://oleks-netizen.github.io/product-images/25438164m/011.jpg,https://oleks-netizen.github.io/product-images/25438164m/012.jpg,https://oleks-netizen.github.io/product-images/25438164m/013.jpg</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>53330514m</t>
+          <t>30127445</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330514m/001.jpg,https://oleks-netizen.github.io/product-images/53330514m/002.jpg,https://oleks-netizen.github.io/product-images/53330514m/003.jpg,https://oleks-netizen.github.io/product-images/53330514m/004.jpg,https://oleks-netizen.github.io/product-images/53330514m/005.jpg,https://oleks-netizen.github.io/product-images/53330514m/006.jpg,https://oleks-netizen.github.io/product-images/53330514m/007.jpg,https://oleks-netizen.github.io/product-images/53330514m/008.jpg,https://oleks-netizen.github.io/product-images/53330514m/010.jpg,https://oleks-netizen.github.io/product-images/53330514m/011.jpg,https://oleks-netizen.github.io/product-images/53330514m/012.jpg,https://oleks-netizen.github.io/product-images/53330514m/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/30127445/001.jpg,https://oleks-netizen.github.io/product-images/30127445/002.jpg,https://oleks-netizen.github.io/product-images/30127445/003.jpg,https://oleks-netizen.github.io/product-images/30127445/004.jpg,https://oleks-netizen.github.io/product-images/30127445/005.jpg</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>53330530</t>
+          <t>303660</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330530/001.jpg,https://oleks-netizen.github.io/product-images/53330530/002.jpg,https://oleks-netizen.github.io/product-images/53330530/003.jpg,https://oleks-netizen.github.io/product-images/53330530/004.jpg,https://oleks-netizen.github.io/product-images/53330530/005.jpg,https://oleks-netizen.github.io/product-images/53330530/006.jpg,https://oleks-netizen.github.io/product-images/53330530/007.jpg,https://oleks-netizen.github.io/product-images/53330530/008.jpg,https://oleks-netizen.github.io/product-images/53330530/009.jpg,https://oleks-netizen.github.io/product-images/53330530/010.jpg,https://oleks-netizen.github.io/product-images/53330530/011.jpg,https://oleks-netizen.github.io/product-images/53330530/013.jpg,https://oleks-netizen.github.io/product-images/53330530/014.jpg,https://oleks-netizen.github.io/product-images/53330530/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/303660/001.jpg,https://oleks-netizen.github.io/product-images/303660/003.jpg,https://oleks-netizen.github.io/product-images/303660/004.jpg</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>53330530m</t>
+          <t>51411010</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53330530m/001.jpg,https://oleks-netizen.github.io/product-images/53330530m/002.jpg,https://oleks-netizen.github.io/product-images/53330530m/003.jpg,https://oleks-netizen.github.io/product-images/53330530m/004.jpg,https://oleks-netizen.github.io/product-images/53330530m/005.jpg,https://oleks-netizen.github.io/product-images/53330530m/006.jpg,https://oleks-netizen.github.io/product-images/53330530m/008.jpg,https://oleks-netizen.github.io/product-images/53330530m/009.jpg,https://oleks-netizen.github.io/product-images/53330530m/010.jpg,https://oleks-netizen.github.io/product-images/53330530m/011.jpg,https://oleks-netizen.github.io/product-images/53330530m/012.jpg,https://oleks-netizen.github.io/product-images/53330530m/013.jpg,https://oleks-netizen.github.io/product-images/53330530m/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411010/001.jpg,https://oleks-netizen.github.io/product-images/51411010/002.jpg,https://oleks-netizen.github.io/product-images/51411010/003.jpg,https://oleks-netizen.github.io/product-images/51411010/005.jpg,https://oleks-netizen.github.io/product-images/51411010/006.jpg,https://oleks-netizen.github.io/product-images/51411010/007.jpg,https://oleks-netizen.github.io/product-images/51411010/008.jpg,https://oleks-netizen.github.io/product-images/51411010/009.jpg,https://oleks-netizen.github.io/product-images/51411010/010.jpg,https://oleks-netizen.github.io/product-images/51411010/011.jpg,https://oleks-netizen.github.io/product-images/51411010/012.jpg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>53400506</t>
+          <t>51411064</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53400506/001.jpg,https://oleks-netizen.github.io/product-images/53400506/002.jpg,https://oleks-netizen.github.io/product-images/53400506/003.jpg,https://oleks-netizen.github.io/product-images/53400506/004.jpg,https://oleks-netizen.github.io/product-images/53400506/005.jpg,https://oleks-netizen.github.io/product-images/53400506/006.jpg,https://oleks-netizen.github.io/product-images/53400506/007.jpg,https://oleks-netizen.github.io/product-images/53400506/008.jpg,https://oleks-netizen.github.io/product-images/53400506/009.jpg,https://oleks-netizen.github.io/product-images/53400506/010.jpg,https://oleks-netizen.github.io/product-images/53400506/012.jpg,https://oleks-netizen.github.io/product-images/53400506/013.jpg,https://oleks-netizen.github.io/product-images/53400506/014.jpg,https://oleks-netizen.github.io/product-images/53400506/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411064/001.jpg,https://oleks-netizen.github.io/product-images/51411064/002.jpg,https://oleks-netizen.github.io/product-images/51411064/003.jpg,https://oleks-netizen.github.io/product-images/51411064/004.jpg,https://oleks-netizen.github.io/product-images/51411064/005.jpg,https://oleks-netizen.github.io/product-images/51411064/006.jpg,https://oleks-netizen.github.io/product-images/51411064/008.jpg,https://oleks-netizen.github.io/product-images/51411064/009.jpg,https://oleks-netizen.github.io/product-images/51411064/010.jpg,https://oleks-netizen.github.io/product-images/51411064/011.jpg</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>53400514</t>
+          <t>51411064m</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53400514/001.jpg,https://oleks-netizen.github.io/product-images/53400514/002.jpg,https://oleks-netizen.github.io/product-images/53400514/003.jpg,https://oleks-netizen.github.io/product-images/53400514/005.jpg,https://oleks-netizen.github.io/product-images/53400514/006.jpg,https://oleks-netizen.github.io/product-images/53400514/007.jpg,https://oleks-netizen.github.io/product-images/53400514/008.jpg,https://oleks-netizen.github.io/product-images/53400514/009.jpg,https://oleks-netizen.github.io/product-images/53400514/010.jpg,https://oleks-netizen.github.io/product-images/53400514/011.jpg,https://oleks-netizen.github.io/product-images/53400514/012.jpg,https://oleks-netizen.github.io/product-images/53400514/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411064m/001.jpg,https://oleks-netizen.github.io/product-images/51411064m/002.jpg,https://oleks-netizen.github.io/product-images/51411064m/003.jpg,https://oleks-netizen.github.io/product-images/51411064m/004.jpg,https://oleks-netizen.github.io/product-images/51411064m/005.jpg,https://oleks-netizen.github.io/product-images/51411064m/007.jpg,https://oleks-netizen.github.io/product-images/51411064m/008.jpg,https://oleks-netizen.github.io/product-images/51411064m/009.jpg,https://oleks-netizen.github.io/product-images/51411064m/010.jpg,https://oleks-netizen.github.io/product-images/51411064m/011.jpg,https://oleks-netizen.github.io/product-images/51411064m/012.jpg,https://oleks-netizen.github.io/product-images/51411064m/013.jpg,https://oleks-netizen.github.io/product-images/51411064m/014.jpg,https://oleks-netizen.github.io/product-images/51411064m/015.jpg</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>53400514m</t>
+          <t>51411120</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53400514m/001.jpg,https://oleks-netizen.github.io/product-images/53400514m/002.jpg,https://oleks-netizen.github.io/product-images/53400514m/003.jpg,https://oleks-netizen.github.io/product-images/53400514m/004.jpg,https://oleks-netizen.github.io/product-images/53400514m/005.jpg,https://oleks-netizen.github.io/product-images/53400514m/006.jpg,https://oleks-netizen.github.io/product-images/53400514m/007.jpg,https://oleks-netizen.github.io/product-images/53400514m/009.jpg,https://oleks-netizen.github.io/product-images/53400514m/010.jpg,https://oleks-netizen.github.io/product-images/53400514m/011.jpg,https://oleks-netizen.github.io/product-images/53400514m/012.jpg,https://oleks-netizen.github.io/product-images/53400514m/013.jpg,https://oleks-netizen.github.io/product-images/53400514m/014.jpg,https://oleks-netizen.github.io/product-images/53400514m/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411120/001.jpg,https://oleks-netizen.github.io/product-images/51411120/002.jpg,https://oleks-netizen.github.io/product-images/51411120/003.jpg,https://oleks-netizen.github.io/product-images/51411120/004.jpg,https://oleks-netizen.github.io/product-images/51411120/005.jpg,https://oleks-netizen.github.io/product-images/51411120/007.jpg,https://oleks-netizen.github.io/product-images/51411120/008.jpg,https://oleks-netizen.github.io/product-images/51411120/009.jpg,https://oleks-netizen.github.io/product-images/51411120/010.jpg,https://oleks-netizen.github.io/product-images/51411120/011.jpg,https://oleks-netizen.github.io/product-images/51411120/012.jpg,https://oleks-netizen.github.io/product-images/51411120/013.jpg,https://oleks-netizen.github.io/product-images/51411120/014.jpg</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6936686411318</t>
+          <t>51411129</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6936686411318/001.jpg,https://oleks-netizen.github.io/product-images/6936686411318/002.jpg,https://oleks-netizen.github.io/product-images/6936686411318/003.jpg,https://oleks-netizen.github.io/product-images/6936686411318/004.jpg,https://oleks-netizen.github.io/product-images/6936686411318/005.jpg,https://oleks-netizen.github.io/product-images/6936686411318/006.jpg,https://oleks-netizen.github.io/product-images/6936686411318/007.jpg,https://oleks-netizen.github.io/product-images/6936686411318/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411129/001.jpg,https://oleks-netizen.github.io/product-images/51411129/002.jpg,https://oleks-netizen.github.io/product-images/51411129/003.jpg,https://oleks-netizen.github.io/product-images/51411129/004.jpg,https://oleks-netizen.github.io/product-images/51411129/005.jpg,https://oleks-netizen.github.io/product-images/51411129/007.jpg,https://oleks-netizen.github.io/product-images/51411129/008.jpg,https://oleks-netizen.github.io/product-images/51411129/009.jpg,https://oleks-netizen.github.io/product-images/51411129/010.jpg,https://oleks-netizen.github.io/product-images/51411129/011.jpg,https://oleks-netizen.github.io/product-images/51411129/012.jpg,https://oleks-netizen.github.io/product-images/51411129/013.jpg</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6976195091748</t>
+          <t>51411210</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976195091748/001.jpg,https://oleks-netizen.github.io/product-images/6976195091748/002.jpg,https://oleks-netizen.github.io/product-images/6976195091748/003.jpg,https://oleks-netizen.github.io/product-images/6976195091748/004.jpg,https://oleks-netizen.github.io/product-images/6976195091748/005.jpg,https://oleks-netizen.github.io/product-images/6976195091748/007.jpg,https://oleks-netizen.github.io/product-images/6976195091748/008.jpg,https://oleks-netizen.github.io/product-images/6976195091748/009.jpg,https://oleks-netizen.github.io/product-images/6976195091748/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411210/001.jpg,https://oleks-netizen.github.io/product-images/51411210/002.jpg,https://oleks-netizen.github.io/product-images/51411210/003.jpg,https://oleks-netizen.github.io/product-images/51411210/004.jpg,https://oleks-netizen.github.io/product-images/51411210/005.jpg,https://oleks-netizen.github.io/product-images/51411210/006.jpg,https://oleks-netizen.github.io/product-images/51411210/008.jpg,https://oleks-netizen.github.io/product-images/51411210/009.jpg,https://oleks-netizen.github.io/product-images/51411210/010.jpg,https://oleks-netizen.github.io/product-images/51411210/011.jpg,https://oleks-netizen.github.io/product-images/51411210/012.jpg,https://oleks-netizen.github.io/product-images/51411210/013.jpg</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>6976195091755</t>
+          <t>51411210m</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976195091755/001.jpg,https://oleks-netizen.github.io/product-images/6976195091755/002.jpg,https://oleks-netizen.github.io/product-images/6976195091755/003.jpg,https://oleks-netizen.github.io/product-images/6976195091755/004.jpg,https://oleks-netizen.github.io/product-images/6976195091755/005.jpg,https://oleks-netizen.github.io/product-images/6976195091755/007.jpg,https://oleks-netizen.github.io/product-images/6976195091755/008.jpg,https://oleks-netizen.github.io/product-images/6976195091755/009.jpg,https://oleks-netizen.github.io/product-images/6976195091755/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411210m/001.jpg,https://oleks-netizen.github.io/product-images/51411210m/002.jpg,https://oleks-netizen.github.io/product-images/51411210m/004.jpg,https://oleks-netizen.github.io/product-images/51411210m/005.jpg,https://oleks-netizen.github.io/product-images/51411210m/006.jpg,https://oleks-netizen.github.io/product-images/51411210m/007.jpg,https://oleks-netizen.github.io/product-images/51411210m/008.jpg,https://oleks-netizen.github.io/product-images/51411210m/009.jpg,https://oleks-netizen.github.io/product-images/51411210m/010.jpg,https://oleks-netizen.github.io/product-images/51411210m/011.jpg,https://oleks-netizen.github.io/product-images/51411210m/012.jpg,https://oleks-netizen.github.io/product-images/51411210m/013.jpg,https://oleks-netizen.github.io/product-images/51411210m/014.jpg,https://oleks-netizen.github.io/product-images/51411210m/015.jpg</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6976195091779</t>
+          <t>51411215</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976195091779/001.jpg,https://oleks-netizen.github.io/product-images/6976195091779/002.jpg,https://oleks-netizen.github.io/product-images/6976195091779/003.jpg,https://oleks-netizen.github.io/product-images/6976195091779/004.jpg,https://oleks-netizen.github.io/product-images/6976195091779/005.jpg,https://oleks-netizen.github.io/product-images/6976195091779/007.jpg,https://oleks-netizen.github.io/product-images/6976195091779/008.jpg,https://oleks-netizen.github.io/product-images/6976195091779/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411215/001.jpg,https://oleks-netizen.github.io/product-images/51411215/002.jpg,https://oleks-netizen.github.io/product-images/51411215/003.jpg,https://oleks-netizen.github.io/product-images/51411215/004.jpg,https://oleks-netizen.github.io/product-images/51411215/005.jpg,https://oleks-netizen.github.io/product-images/51411215/006.jpg,https://oleks-netizen.github.io/product-images/51411215/008.jpg,https://oleks-netizen.github.io/product-images/51411215/009.jpg,https://oleks-netizen.github.io/product-images/51411215/010.jpg,https://oleks-netizen.github.io/product-images/51411215/011.jpg,https://oleks-netizen.github.io/product-images/51411215/012.jpg</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>6976195091786</t>
+          <t>51411215m</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976195091786/001.jpg,https://oleks-netizen.github.io/product-images/6976195091786/002.jpg,https://oleks-netizen.github.io/product-images/6976195091786/003.jpg,https://oleks-netizen.github.io/product-images/6976195091786/004.jpg,https://oleks-netizen.github.io/product-images/6976195091786/006.jpg,https://oleks-netizen.github.io/product-images/6976195091786/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411215m/001.jpg,https://oleks-netizen.github.io/product-images/51411215m/002.jpg,https://oleks-netizen.github.io/product-images/51411215m/004.jpg,https://oleks-netizen.github.io/product-images/51411215m/005.jpg,https://oleks-netizen.github.io/product-images/51411215m/006.jpg,https://oleks-netizen.github.io/product-images/51411215m/007.jpg,https://oleks-netizen.github.io/product-images/51411215m/008.jpg,https://oleks-netizen.github.io/product-images/51411215m/009.jpg,https://oleks-netizen.github.io/product-images/51411215m/010.jpg,https://oleks-netizen.github.io/product-images/51411215m/011.jpg,https://oleks-netizen.github.io/product-images/51411215m/012.jpg,https://oleks-netizen.github.io/product-images/51411215m/013.jpg,https://oleks-netizen.github.io/product-images/51411215m/014.jpg,https://oleks-netizen.github.io/product-images/51411215m/015.jpg</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6976195091793</t>
+          <t>51411264</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976195091793/001.jpg,https://oleks-netizen.github.io/product-images/6976195091793/002.jpg,https://oleks-netizen.github.io/product-images/6976195091793/004.jpg,https://oleks-netizen.github.io/product-images/6976195091793/005.jpg,https://oleks-netizen.github.io/product-images/6976195091793/006.jpg,https://oleks-netizen.github.io/product-images/6976195091793/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411264/001.jpg,https://oleks-netizen.github.io/product-images/51411264/002.jpg,https://oleks-netizen.github.io/product-images/51411264/003.jpg,https://oleks-netizen.github.io/product-images/51411264/005.jpg,https://oleks-netizen.github.io/product-images/51411264/006.jpg,https://oleks-netizen.github.io/product-images/51411264/007.jpg,https://oleks-netizen.github.io/product-images/51411264/008.jpg,https://oleks-netizen.github.io/product-images/51411264/009.jpg,https://oleks-netizen.github.io/product-images/51411264/010.jpg,https://oleks-netizen.github.io/product-images/51411264/011.jpg,https://oleks-netizen.github.io/product-images/51411264/012.jpg</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>6976195094718</t>
+          <t>51411264m</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976195094718/001.jpg,https://oleks-netizen.github.io/product-images/6976195094718/002.jpg,https://oleks-netizen.github.io/product-images/6976195094718/003.jpg,https://oleks-netizen.github.io/product-images/6976195094718/004.jpg,https://oleks-netizen.github.io/product-images/6976195094718/005.jpg,https://oleks-netizen.github.io/product-images/6976195094718/006.jpg,https://oleks-netizen.github.io/product-images/6976195094718/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411264m/001.jpg,https://oleks-netizen.github.io/product-images/51411264m/002.jpg,https://oleks-netizen.github.io/product-images/51411264m/003.jpg,https://oleks-netizen.github.io/product-images/51411264m/004.jpg,https://oleks-netizen.github.io/product-images/51411264m/005.jpg,https://oleks-netizen.github.io/product-images/51411264m/006.jpg,https://oleks-netizen.github.io/product-images/51411264m/007.jpg,https://oleks-netizen.github.io/product-images/51411264m/009.jpg,https://oleks-netizen.github.io/product-images/51411264m/010.jpg,https://oleks-netizen.github.io/product-images/51411264m/011.jpg,https://oleks-netizen.github.io/product-images/51411264m/012.jpg,https://oleks-netizen.github.io/product-images/51411264m/013.jpg,https://oleks-netizen.github.io/product-images/51411264m/014.jpg,https://oleks-netizen.github.io/product-images/51411264m/015.jpg</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>6976195095838</t>
+          <t>5193401</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976195095838/001.jpg,https://oleks-netizen.github.io/product-images/6976195095838/002.jpg,https://oleks-netizen.github.io/product-images/6976195095838/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5193401/001.jpg,https://oleks-netizen.github.io/product-images/5193401/002.jpg,https://oleks-netizen.github.io/product-images/5193401/003.jpg,https://oleks-netizen.github.io/product-images/5193401/004.jpg,https://oleks-netizen.github.io/product-images/5193401/005.jpg,https://oleks-netizen.github.io/product-images/5193401/006.jpg,https://oleks-netizen.github.io/product-images/5193401/007.jpg,https://oleks-netizen.github.io/product-images/5193401/009.jpg,https://oleks-netizen.github.io/product-images/5193401/010.jpg</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>6976195095845</t>
+          <t>5202801</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976195095845/001.jpg,https://oleks-netizen.github.io/product-images/6976195095845/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5202801/001.jpg,https://oleks-netizen.github.io/product-images/5202801/002.jpg,https://oleks-netizen.github.io/product-images/5202801/004.jpg,https://oleks-netizen.github.io/product-images/5202801/005.jpg,https://oleks-netizen.github.io/product-images/5202801/006.jpg,https://oleks-netizen.github.io/product-images/5202801/007.jpg,https://oleks-netizen.github.io/product-images/5202801/008.jpg,https://oleks-netizen.github.io/product-images/5202801/009.jpg,https://oleks-netizen.github.io/product-images/5202801/010.jpg,https://oleks-netizen.github.io/product-images/5202801/011.jpg</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>6976195096064</t>
+          <t>5204101</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976195096064/001.jpg,https://oleks-netizen.github.io/product-images/6976195096064/002.jpg,https://oleks-netizen.github.io/product-images/6976195096064/004.jpg,https://oleks-netizen.github.io/product-images/6976195096064/005.jpg,https://oleks-netizen.github.io/product-images/6976195096064/006.jpg,https://oleks-netizen.github.io/product-images/6976195096064/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5204101/001.jpg,https://oleks-netizen.github.io/product-images/5204101/002.jpg,https://oleks-netizen.github.io/product-images/5204101/003.jpg,https://oleks-netizen.github.io/product-images/5204101/004.jpg,https://oleks-netizen.github.io/product-images/5204101/005.jpg,https://oleks-netizen.github.io/product-images/5204101/006.jpg,https://oleks-netizen.github.io/product-images/5204101/007.jpg,https://oleks-netizen.github.io/product-images/5204101/008.jpg,https://oleks-netizen.github.io/product-images/5204101/009.jpg,https://oleks-netizen.github.io/product-images/5204101/010.jpg</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>6976195096989</t>
+          <t>5205701</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976195096989/001.jpg,https://oleks-netizen.github.io/product-images/6976195096989/002.jpg,https://oleks-netizen.github.io/product-images/6976195096989/003.jpg,https://oleks-netizen.github.io/product-images/6976195096989/004.jpg,https://oleks-netizen.github.io/product-images/6976195096989/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5205701/001.jpg,https://oleks-netizen.github.io/product-images/5205701/002.jpg,https://oleks-netizen.github.io/product-images/5205701/004.jpg,https://oleks-netizen.github.io/product-images/5205701/005.jpg,https://oleks-netizen.github.io/product-images/5205701/006.jpg,https://oleks-netizen.github.io/product-images/5205701/007.jpg,https://oleks-netizen.github.io/product-images/5205701/008.jpg,https://oleks-netizen.github.io/product-images/5205701/009.jpg,https://oleks-netizen.github.io/product-images/5205701/010.jpg</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>6976975615294</t>
+          <t>5205801</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976975615294/001.jpg,https://oleks-netizen.github.io/product-images/6976975615294/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5205801/001.jpg,https://oleks-netizen.github.io/product-images/5205801/002.jpg,https://oleks-netizen.github.io/product-images/5205801/004.jpg,https://oleks-netizen.github.io/product-images/5205801/005.jpg,https://oleks-netizen.github.io/product-images/5205801/006.jpg,https://oleks-netizen.github.io/product-images/5205801/007.jpg,https://oleks-netizen.github.io/product-images/5205801/008.jpg,https://oleks-netizen.github.io/product-images/5205801/009.jpg,https://oleks-netizen.github.io/product-images/5205801/010.jpg,https://oleks-netizen.github.io/product-images/5205801/011.jpg</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>6976975615324</t>
+          <t>5210401</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6976975615324/001.jpg,https://oleks-netizen.github.io/product-images/6976975615324/003.jpg,https://oleks-netizen.github.io/product-images/6976975615324/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5210401/001.jpg,https://oleks-netizen.github.io/product-images/5210401/002.jpg,https://oleks-netizen.github.io/product-images/5210401/004.jpg,https://oleks-netizen.github.io/product-images/5210401/005.jpg,https://oleks-netizen.github.io/product-images/5210401/006.jpg,https://oleks-netizen.github.io/product-images/5210401/007.jpg,https://oleks-netizen.github.io/product-images/5210401/008.jpg,https://oleks-netizen.github.io/product-images/5210401/009.jpg,https://oleks-netizen.github.io/product-images/5210401/010.jpg,https://oleks-netizen.github.io/product-images/5210401/011.jpg</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>6977703651690</t>
+          <t>5218101</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6977703651690/001.jpg,https://oleks-netizen.github.io/product-images/6977703651690/002.jpg,https://oleks-netizen.github.io/product-images/6977703651690/003.jpg,https://oleks-netizen.github.io/product-images/6977703651690/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5218101/001.jpg,https://oleks-netizen.github.io/product-images/5218101/002.jpg,https://oleks-netizen.github.io/product-images/5218101/003.jpg,https://oleks-netizen.github.io/product-images/5218101/004.jpg,https://oleks-netizen.github.io/product-images/5218101/005.jpg,https://oleks-netizen.github.io/product-images/5218101/006.jpg,https://oleks-netizen.github.io/product-images/5218101/007.jpg,https://oleks-netizen.github.io/product-images/5218101/008.jpg,https://oleks-netizen.github.io/product-images/5218101/009.jpg,https://oleks-netizen.github.io/product-images/5218101/010.jpg</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>6977703651713</t>
+          <t>5221401</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/6977703651713/001.jpg,https://oleks-netizen.github.io/product-images/6977703651713/002.jpg,https://oleks-netizen.github.io/product-images/6977703651713/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5221401/001.jpg,https://oleks-netizen.github.io/product-images/5221401/003.jpg,https://oleks-netizen.github.io/product-images/5221401/004.jpg,https://oleks-netizen.github.io/product-images/5221401/005.jpg,https://oleks-netizen.github.io/product-images/5221401/006.jpg,https://oleks-netizen.github.io/product-images/5221401/007.jpg,https://oleks-netizen.github.io/product-images/5221401/008.jpg,https://oleks-netizen.github.io/product-images/5221401/009.jpg,https://oleks-netizen.github.io/product-images/5221401/010.jpg,https://oleks-netizen.github.io/product-images/5221401/011.jpg</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>80411514m</t>
+          <t>5225501</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80411514m/001.jpg,https://oleks-netizen.github.io/product-images/80411514m/002.jpg,https://oleks-netizen.github.io/product-images/80411514m/004.jpg,https://oleks-netizen.github.io/product-images/80411514m/005.jpg,https://oleks-netizen.github.io/product-images/80411514m/006.jpg,https://oleks-netizen.github.io/product-images/80411514m/007.jpg,https://oleks-netizen.github.io/product-images/80411514m/008.jpg,https://oleks-netizen.github.io/product-images/80411514m/009.jpg,https://oleks-netizen.github.io/product-images/80411514m/010.jpg,https://oleks-netizen.github.io/product-images/80411514m/011.jpg,https://oleks-netizen.github.io/product-images/80411514m/012.jpg,https://oleks-netizen.github.io/product-images/80411514m/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5225501/001.jpg,https://oleks-netizen.github.io/product-images/5225501/003.jpg,https://oleks-netizen.github.io/product-images/5225501/004.jpg,https://oleks-netizen.github.io/product-images/5225501/005.jpg,https://oleks-netizen.github.io/product-images/5225501/006.jpg,https://oleks-netizen.github.io/product-images/5225501/007.jpg,https://oleks-netizen.github.io/product-images/5225501/008.jpg,https://oleks-netizen.github.io/product-images/5225501/009.jpg,https://oleks-netizen.github.io/product-images/5225501/010.jpg,https://oleks-netizen.github.io/product-images/5225501/011.jpg</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>80411515m</t>
+          <t>522623</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80411515m/001.jpg,https://oleks-netizen.github.io/product-images/80411515m/002.jpg,https://oleks-netizen.github.io/product-images/80411515m/003.jpg,https://oleks-netizen.github.io/product-images/80411515m/005.jpg,https://oleks-netizen.github.io/product-images/80411515m/006.jpg,https://oleks-netizen.github.io/product-images/80411515m/007.jpg,https://oleks-netizen.github.io/product-images/80411515m/008.jpg,https://oleks-netizen.github.io/product-images/80411515m/009.jpg,https://oleks-netizen.github.io/product-images/80411515m/010.jpg,https://oleks-netizen.github.io/product-images/80411515m/011.jpg,https://oleks-netizen.github.io/product-images/80411515m/012.jpg,https://oleks-netizen.github.io/product-images/80411515m/013.jpg,https://oleks-netizen.github.io/product-images/80411515m/014.jpg,https://oleks-netizen.github.io/product-images/80411515m/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/522623/001.jpg,https://oleks-netizen.github.io/product-images/522623/002.jpg</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>80411530m</t>
+          <t>522660</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80411530m/001.jpg,https://oleks-netizen.github.io/product-images/80411530m/002.jpg,https://oleks-netizen.github.io/product-images/80411530m/003.jpg,https://oleks-netizen.github.io/product-images/80411530m/004.jpg,https://oleks-netizen.github.io/product-images/80411530m/005.jpg,https://oleks-netizen.github.io/product-images/80411530m/006.jpg,https://oleks-netizen.github.io/product-images/80411530m/007.jpg,https://oleks-netizen.github.io/product-images/80411530m/009.jpg,https://oleks-netizen.github.io/product-images/80411530m/010.jpg,https://oleks-netizen.github.io/product-images/80411530m/011.jpg,https://oleks-netizen.github.io/product-images/80411530m/012.jpg,https://oleks-netizen.github.io/product-images/80411530m/013.jpg,https://oleks-netizen.github.io/product-images/80411530m/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/522660/001.jpg,https://oleks-netizen.github.io/product-images/522660/002.jpg</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>80411714</t>
+          <t>5230401</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80411714/001.jpg,https://oleks-netizen.github.io/product-images/80411714/002.jpg,https://oleks-netizen.github.io/product-images/80411714/003.jpg,https://oleks-netizen.github.io/product-images/80411714/004.jpg,https://oleks-netizen.github.io/product-images/80411714/006.jpg,https://oleks-netizen.github.io/product-images/80411714/007.jpg,https://oleks-netizen.github.io/product-images/80411714/008.jpg,https://oleks-netizen.github.io/product-images/80411714/009.jpg,https://oleks-netizen.github.io/product-images/80411714/010.jpg,https://oleks-netizen.github.io/product-images/80411714/011.jpg,https://oleks-netizen.github.io/product-images/80411714/012.jpg,https://oleks-netizen.github.io/product-images/80411714/013.jpg,https://oleks-netizen.github.io/product-images/80411714/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5230401/001.jpg,https://oleks-netizen.github.io/product-images/5230401/002.jpg,https://oleks-netizen.github.io/product-images/5230401/003.jpg,https://oleks-netizen.github.io/product-images/5230401/005.jpg,https://oleks-netizen.github.io/product-images/5230401/006.jpg,https://oleks-netizen.github.io/product-images/5230401/007.jpg,https://oleks-netizen.github.io/product-images/5230401/008.jpg,https://oleks-netizen.github.io/product-images/5230401/009.jpg,https://oleks-netizen.github.io/product-images/5230401/010.jpg,https://oleks-netizen.github.io/product-images/5230401/011.jpg</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>804600410</t>
+          <t>5231101</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/804600410/001.jpg,https://oleks-netizen.github.io/product-images/804600410/002.jpg,https://oleks-netizen.github.io/product-images/804600410/003.jpg,https://oleks-netizen.github.io/product-images/804600410/005.jpg,https://oleks-netizen.github.io/product-images/804600410/006.jpg,https://oleks-netizen.github.io/product-images/804600410/007.jpg,https://oleks-netizen.github.io/product-images/804600410/008.jpg,https://oleks-netizen.github.io/product-images/804600410/009.jpg,https://oleks-netizen.github.io/product-images/804600410/010.jpg,https://oleks-netizen.github.io/product-images/804600410/011.jpg,https://oleks-netizen.github.io/product-images/804600410/012.jpg,https://oleks-netizen.github.io/product-images/804600410/013.jpg,https://oleks-netizen.github.io/product-images/804600410/014.jpg,https://oleks-netizen.github.io/product-images/804600410/015.jpg,https://oleks-netizen.github.io/product-images/804600410/016.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5231101/001.jpg,https://oleks-netizen.github.io/product-images/5231101/002.jpg,https://oleks-netizen.github.io/product-images/5231101/003.jpg,https://oleks-netizen.github.io/product-images/5231101/004.jpg,https://oleks-netizen.github.io/product-images/5231101/005.jpg,https://oleks-netizen.github.io/product-images/5231101/006.jpg,https://oleks-netizen.github.io/product-images/5231101/007.jpg,https://oleks-netizen.github.io/product-images/5231101/008.jpg,https://oleks-netizen.github.io/product-images/5231101/009.jpg,https://oleks-netizen.github.io/product-images/5231101/010.jpg</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>80460060</t>
+          <t>5233301</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80460060/001.jpg,https://oleks-netizen.github.io/product-images/80460060/002.jpg,https://oleks-netizen.github.io/product-images/80460060/003.jpg,https://oleks-netizen.github.io/product-images/80460060/005.jpg,https://oleks-netizen.github.io/product-images/80460060/006.jpg,https://oleks-netizen.github.io/product-images/80460060/007.jpg,https://oleks-netizen.github.io/product-images/80460060/008.jpg,https://oleks-netizen.github.io/product-images/80460060/009.jpg,https://oleks-netizen.github.io/product-images/80460060/010.jpg,https://oleks-netizen.github.io/product-images/80460060/011.jpg,https://oleks-netizen.github.io/product-images/80460060/012.jpg,https://oleks-netizen.github.io/product-images/80460060/013.jpg,https://oleks-netizen.github.io/product-images/80460060/014.jpg,https://oleks-netizen.github.io/product-images/80460060/015.jpg,https://oleks-netizen.github.io/product-images/80460060/016.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5233301/001.jpg,https://oleks-netizen.github.io/product-images/5233301/002.jpg,https://oleks-netizen.github.io/product-images/5233301/003.jpg,https://oleks-netizen.github.io/product-images/5233301/004.jpg,https://oleks-netizen.github.io/product-images/5233301/006.jpg,https://oleks-netizen.github.io/product-images/5233301/007.jpg,https://oleks-netizen.github.io/product-images/5233301/008.jpg,https://oleks-netizen.github.io/product-images/5233301/009.jpg,https://oleks-netizen.github.io/product-images/5233301/010.jpg,https://oleks-netizen.github.io/product-images/5233301/011.jpg</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>80460401</t>
+          <t>5241901</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80460401/001.jpg,https://oleks-netizen.github.io/product-images/80460401/002.jpg,https://oleks-netizen.github.io/product-images/80460401/003.jpg,https://oleks-netizen.github.io/product-images/80460401/005.jpg,https://oleks-netizen.github.io/product-images/80460401/006.jpg,https://oleks-netizen.github.io/product-images/80460401/007.jpg,https://oleks-netizen.github.io/product-images/80460401/008.jpg,https://oleks-netizen.github.io/product-images/80460401/009.jpg,https://oleks-netizen.github.io/product-images/80460401/010.jpg,https://oleks-netizen.github.io/product-images/80460401/011.jpg,https://oleks-netizen.github.io/product-images/80460401/012.jpg,https://oleks-netizen.github.io/product-images/80460401/013.jpg,https://oleks-netizen.github.io/product-images/80460401/014.jpg,https://oleks-netizen.github.io/product-images/80460401/015.jpg,https://oleks-netizen.github.io/product-images/80460401/016.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5241901/001.jpg,https://oleks-netizen.github.io/product-images/5241901/002.jpg,https://oleks-netizen.github.io/product-images/5241901/004.jpg,https://oleks-netizen.github.io/product-images/5241901/005.jpg,https://oleks-netizen.github.io/product-images/5241901/006.jpg,https://oleks-netizen.github.io/product-images/5241901/007.jpg,https://oleks-netizen.github.io/product-images/5241901/008.jpg,https://oleks-netizen.github.io/product-images/5241901/009.jpg,https://oleks-netizen.github.io/product-images/5241901/010.jpg,https://oleks-netizen.github.io/product-images/5241901/011.jpg</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>85151020</t>
+          <t>5244701</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/85151020/001.jpg,https://oleks-netizen.github.io/product-images/85151020/002.jpg,https://oleks-netizen.github.io/product-images/85151020/003.jpg,https://oleks-netizen.github.io/product-images/85151020/004.jpg,https://oleks-netizen.github.io/product-images/85151020/005.jpg,https://oleks-netizen.github.io/product-images/85151020/006.jpg,https://oleks-netizen.github.io/product-images/85151020/007.jpg,https://oleks-netizen.github.io/product-images/85151020/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5244701/001.jpg,https://oleks-netizen.github.io/product-images/5244701/002.jpg,https://oleks-netizen.github.io/product-images/5244701/003.jpg,https://oleks-netizen.github.io/product-images/5244701/004.jpg,https://oleks-netizen.github.io/product-images/5244701/005.jpg,https://oleks-netizen.github.io/product-images/5244701/006.jpg,https://oleks-netizen.github.io/product-images/5244701/007.jpg,https://oleks-netizen.github.io/product-images/5244701/008.jpg,https://oleks-netizen.github.io/product-images/5244701/009.jpg,https://oleks-netizen.github.io/product-images/5244701/010.jpg</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>85451064</t>
+          <t>5246401</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/85451064/001.jpg,https://oleks-netizen.github.io/product-images/85451064/002.jpg,https://oleks-netizen.github.io/product-images/85451064/004.jpg,https://oleks-netizen.github.io/product-images/85451064/005.jpg,https://oleks-netizen.github.io/product-images/85451064/006.jpg,https://oleks-netizen.github.io/product-images/85451064/007.jpg,https://oleks-netizen.github.io/product-images/85451064/008.jpg,https://oleks-netizen.github.io/product-images/85451064/009.jpg,https://oleks-netizen.github.io/product-images/85451064/010.jpg,https://oleks-netizen.github.io/product-images/85451064/011.jpg,https://oleks-netizen.github.io/product-images/85451064/012.jpg,https://oleks-netizen.github.io/product-images/85451064/013.jpg,https://oleks-netizen.github.io/product-images/85451064/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5246401/001.jpg,https://oleks-netizen.github.io/product-images/5246401/002.jpg,https://oleks-netizen.github.io/product-images/5246401/003.jpg,https://oleks-netizen.github.io/product-images/5246401/004.jpg,https://oleks-netizen.github.io/product-images/5246401/005.jpg,https://oleks-netizen.github.io/product-images/5246401/006.jpg,https://oleks-netizen.github.io/product-images/5246401/007.jpg,https://oleks-netizen.github.io/product-images/5246401/008.jpg,https://oleks-netizen.github.io/product-images/5246401/009.jpg,https://oleks-netizen.github.io/product-images/5246401/010.jpg</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>85451064m</t>
+          <t>5248401</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/85451064m/001.jpg,https://oleks-netizen.github.io/product-images/85451064m/002.jpg,https://oleks-netizen.github.io/product-images/85451064m/003.jpg,https://oleks-netizen.github.io/product-images/85451064m/004.jpg,https://oleks-netizen.github.io/product-images/85451064m/005.jpg,https://oleks-netizen.github.io/product-images/85451064m/006.jpg,https://oleks-netizen.github.io/product-images/85451064m/007.jpg,https://oleks-netizen.github.io/product-images/85451064m/009.jpg,https://oleks-netizen.github.io/product-images/85451064m/010.jpg,https://oleks-netizen.github.io/product-images/85451064m/011.jpg,https://oleks-netizen.github.io/product-images/85451064m/012.jpg,https://oleks-netizen.github.io/product-images/85451064m/013.jpg,https://oleks-netizen.github.io/product-images/85451064m/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5248401/001.jpg,https://oleks-netizen.github.io/product-images/5248401/002.jpg,https://oleks-netizen.github.io/product-images/5248401/003.jpg,https://oleks-netizen.github.io/product-images/5248401/004.jpg,https://oleks-netizen.github.io/product-images/5248401/005.jpg,https://oleks-netizen.github.io/product-images/5248401/006.jpg,https://oleks-netizen.github.io/product-images/5248401/007.jpg,https://oleks-netizen.github.io/product-images/5248401/008.jpg,https://oleks-netizen.github.io/product-images/5248401/009.jpg,https://oleks-netizen.github.io/product-images/5248401/010.jpg</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>85451506</t>
+          <t>53100013</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/85451506/001.jpg,https://oleks-netizen.github.io/product-images/85451506/002.jpg,https://oleks-netizen.github.io/product-images/85451506/003.jpg,https://oleks-netizen.github.io/product-images/85451506/004.jpg,https://oleks-netizen.github.io/product-images/85451506/005.jpg,https://oleks-netizen.github.io/product-images/85451506/007.jpg,https://oleks-netizen.github.io/product-images/85451506/008.jpg,https://oleks-netizen.github.io/product-images/85451506/009.jpg,https://oleks-netizen.github.io/product-images/85451506/010.jpg,https://oleks-netizen.github.io/product-images/85451506/011.jpg,https://oleks-netizen.github.io/product-images/85451506/012.jpg,https://oleks-netizen.github.io/product-images/85451506/013.jpg,https://oleks-netizen.github.io/product-images/85451506/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53100013/001.jpg,https://oleks-netizen.github.io/product-images/53100013/002.jpg,https://oleks-netizen.github.io/product-images/53100013/003.jpg,https://oleks-netizen.github.io/product-images/53100013/005.jpg,https://oleks-netizen.github.io/product-images/53100013/006.jpg,https://oleks-netizen.github.io/product-images/53100013/007.jpg,https://oleks-netizen.github.io/product-images/53100013/008.jpg,https://oleks-netizen.github.io/product-images/53100013/009.jpg,https://oleks-netizen.github.io/product-images/53100013/010.jpg,https://oleks-netizen.github.io/product-images/53100013/011.jpg,https://oleks-netizen.github.io/product-images/53100013/012.jpg</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>B085</t>
+          <t>53300039</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/B085/001.jpg,https://oleks-netizen.github.io/product-images/B085/002.jpg,https://oleks-netizen.github.io/product-images/B085/004.jpg,https://oleks-netizen.github.io/product-images/B085/005.jpg,https://oleks-netizen.github.io/product-images/B085/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53300039/001.jpg,https://oleks-netizen.github.io/product-images/53300039/002.jpg,https://oleks-netizen.github.io/product-images/53300039/003.jpg,https://oleks-netizen.github.io/product-images/53300039/004.jpg,https://oleks-netizen.github.io/product-images/53300039/005.jpg,https://oleks-netizen.github.io/product-images/53300039/007.jpg,https://oleks-netizen.github.io/product-images/53300039/008.jpg,https://oleks-netizen.github.io/product-images/53300039/009.jpg,https://oleks-netizen.github.io/product-images/53300039/010.jpg,https://oleks-netizen.github.io/product-images/53300039/011.jpg,https://oleks-netizen.github.io/product-images/53300039/012.jpg</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>B158</t>
+          <t>53400013</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/B158/001.jpg,https://oleks-netizen.github.io/product-images/B158/002.jpg,https://oleks-netizen.github.io/product-images/B158/003.jpg,https://oleks-netizen.github.io/product-images/B158/004.jpg,https://oleks-netizen.github.io/product-images/B158/005.jpg,https://oleks-netizen.github.io/product-images/B158/006.jpg,https://oleks-netizen.github.io/product-images/B158/007.jpg,https://oleks-netizen.github.io/product-images/B158/009.jpg,https://oleks-netizen.github.io/product-images/B158/010.jpg,https://oleks-netizen.github.io/product-images/B158/011.jpg,https://oleks-netizen.github.io/product-images/B158/012.jpg,https://oleks-netizen.github.io/product-images/B158/013.jpg,https://oleks-netizen.github.io/product-images/B158/014.jpg,https://oleks-netizen.github.io/product-images/B158/015.jpg,https://oleks-netizen.github.io/product-images/B158/016.jpg,https://oleks-netizen.github.io/product-images/B158/017.jpg,https://oleks-netizen.github.io/product-images/B158/018.jpg,https://oleks-netizen.github.io/product-images/B158/019.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400013/001.jpg,https://oleks-netizen.github.io/product-images/53400013/002.jpg,https://oleks-netizen.github.io/product-images/53400013/004.jpg,https://oleks-netizen.github.io/product-images/53400013/005.jpg,https://oleks-netizen.github.io/product-images/53400013/006.jpg,https://oleks-netizen.github.io/product-images/53400013/007.jpg,https://oleks-netizen.github.io/product-images/53400013/008.jpg,https://oleks-netizen.github.io/product-images/53400013/009.jpg,https://oleks-netizen.github.io/product-images/53400013/010.jpg,https://oleks-netizen.github.io/product-images/53400013/011.jpg,https://oleks-netizen.github.io/product-images/53400013/012.jpg,https://oleks-netizen.github.io/product-images/53400013/013.jpg</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BN-BAG-62-g</t>
+          <t>53400020</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BAG-62-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-g/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400020/001.jpg,https://oleks-netizen.github.io/product-images/53400020/002.jpg,https://oleks-netizen.github.io/product-images/53400020/004.jpg,https://oleks-netizen.github.io/product-images/53400020/005.jpg,https://oleks-netizen.github.io/product-images/53400020/006.jpg,https://oleks-netizen.github.io/product-images/53400020/007.jpg,https://oleks-netizen.github.io/product-images/53400020/008.jpg,https://oleks-netizen.github.io/product-images/53400020/009.jpg,https://oleks-netizen.github.io/product-images/53400020/010.jpg,https://oleks-netizen.github.io/product-images/53400020/011.jpg,https://oleks-netizen.github.io/product-images/53400020/012.jpg,https://oleks-netizen.github.io/product-images/53400020/013.jpg,https://oleks-netizen.github.io/product-images/53400020/014.jpg</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>BN-DC-7-k-kr</t>
+          <t>62725</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/006.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/007.jpg,https://oleks-netizen.github.io/product-images/BN-DC-7-k-kr/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/62725/001.jpg,https://oleks-netizen.github.io/product-images/62725/002.jpg,https://oleks-netizen.github.io/product-images/62725/003.jpg,https://oleks-netizen.github.io/product-images/62725/004.jpg,https://oleks-netizen.github.io/product-images/62725/005.jpg,https://oleks-netizen.github.io/product-images/62725/006.jpg,https://oleks-netizen.github.io/product-images/62725/007.jpg</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -1291,27 +1291,27 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CC602_SN_BLK</t>
+          <t>62726</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/CC602_SN_BLK/001.jpg,https://oleks-netizen.github.io/product-images/CC602_SN_BLK/002.jpg,https://oleks-netizen.github.io/product-images/CC602_SN_BLK/003.jpg,https://oleks-netizen.github.io/product-images/CC602_SN_BLK/005.jpg,https://oleks-netizen.github.io/product-images/CC602_SN_BLK/006.jpg,https://oleks-netizen.github.io/product-images/CC602_SN_BLK/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/62726/001.jpg,https://oleks-netizen.github.io/product-images/62726/002.jpg,https://oleks-netizen.github.io/product-images/62726/003.jpg,https://oleks-netizen.github.io/product-images/62726/004.jpg,https://oleks-netizen.github.io/product-images/62726/005.jpg,https://oleks-netizen.github.io/product-images/62726/006.jpg,https://oleks-netizen.github.io/product-images/62726/007.jpg</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>L21360-010</t>
+          <t>62727</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21360-010/001.jpg,https://oleks-netizen.github.io/product-images/L21360-010/002.jpg,https://oleks-netizen.github.io/product-images/L21360-010/004.jpg,https://oleks-netizen.github.io/product-images/L21360-010/005.jpg,https://oleks-netizen.github.io/product-images/L21360-010/006.jpg,https://oleks-netizen.github.io/product-images/L21360-010/007.jpg,https://oleks-netizen.github.io/product-images/L21360-010/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/62727/001.jpg,https://oleks-netizen.github.io/product-images/62727/002.jpg,https://oleks-netizen.github.io/product-images/62727/004.jpg,https://oleks-netizen.github.io/product-images/62727/005.jpg,https://oleks-netizen.github.io/product-images/62727/006.jpg,https://oleks-netizen.github.io/product-images/62727/007.jpg,https://oleks-netizen.github.io/product-images/62727/008.jpg</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -1321,72 +1321,72 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>L21360-021</t>
+          <t>701661</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21360-021/001.jpg,https://oleks-netizen.github.io/product-images/L21360-021/002.jpg,https://oleks-netizen.github.io/product-images/L21360-021/004.jpg,https://oleks-netizen.github.io/product-images/L21360-021/005.jpg,https://oleks-netizen.github.io/product-images/L21360-021/006.jpg,https://oleks-netizen.github.io/product-images/L21360-021/007.jpg,https://oleks-netizen.github.io/product-images/L21360-021/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/701661/001.jpg,https://oleks-netizen.github.io/product-images/701661/002.jpg,https://oleks-netizen.github.io/product-images/701661/003.jpg,https://oleks-netizen.github.io/product-images/701661/004.jpg</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>L21360-025</t>
+          <t>746710</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21360-025/001.jpg,https://oleks-netizen.github.io/product-images/L21360-025/002.jpg,https://oleks-netizen.github.io/product-images/L21360-025/003.jpg,https://oleks-netizen.github.io/product-images/L21360-025/005.jpg,https://oleks-netizen.github.io/product-images/L21360-025/006.jpg,https://oleks-netizen.github.io/product-images/L21360-025/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/746710/001.jpg,https://oleks-netizen.github.io/product-images/746710/002.jpg,https://oleks-netizen.github.io/product-images/746710/003.jpg,https://oleks-netizen.github.io/product-images/746710/004.jpg,https://oleks-netizen.github.io/product-images/746710/005.jpg</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>L21563-010</t>
+          <t>746743</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21563-010/001.jpg,https://oleks-netizen.github.io/product-images/L21563-010/002.jpg,https://oleks-netizen.github.io/product-images/L21563-010/003.jpg,https://oleks-netizen.github.io/product-images/L21563-010/005.jpg,https://oleks-netizen.github.io/product-images/L21563-010/006.jpg,https://oleks-netizen.github.io/product-images/L21563-010/007.jpg,https://oleks-netizen.github.io/product-images/L21563-010/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/746743/001.jpg,https://oleks-netizen.github.io/product-images/746743/002.jpg,https://oleks-netizen.github.io/product-images/746743/003.jpg,https://oleks-netizen.github.io/product-images/746743/004.jpg,https://oleks-netizen.github.io/product-images/746743/005.jpg</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>L21563-038</t>
+          <t>75_1_1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21563-038/001.jpg,https://oleks-netizen.github.io/product-images/L21563-038/002.jpg,https://oleks-netizen.github.io/product-images/L21563-038/003.jpg,https://oleks-netizen.github.io/product-images/L21563-038/005.jpg,https://oleks-netizen.github.io/product-images/L21563-038/006.jpg,https://oleks-netizen.github.io/product-images/L21563-038/007.jpg,https://oleks-netizen.github.io/product-images/L21563-038/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/75_1_1/001.jpg</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>L21563-045</t>
+          <t>77266101</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21563-045/001.jpg,https://oleks-netizen.github.io/product-images/L21563-045/002.jpg,https://oleks-netizen.github.io/product-images/L21563-045/003.jpg,https://oleks-netizen.github.io/product-images/L21563-045/005.jpg,https://oleks-netizen.github.io/product-images/L21563-045/006.jpg,https://oleks-netizen.github.io/product-images/L21563-045/007.jpg,https://oleks-netizen.github.io/product-images/L21563-045/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/77266101/001.jpg,https://oleks-netizen.github.io/product-images/77266101/002.jpg,https://oleks-netizen.github.io/product-images/77266101/003.jpg,https://oleks-netizen.github.io/product-images/77266101/004.jpg,https://oleks-netizen.github.io/product-images/77266101/005.jpg,https://oleks-netizen.github.io/product-images/77266101/006.jpg,https://oleks-netizen.github.io/product-images/77266101/007.jpg</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -1396,192 +1396,192 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>L21564-010</t>
+          <t>96193001</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21564-010/001.jpg,https://oleks-netizen.github.io/product-images/L21564-010/002.jpg,https://oleks-netizen.github.io/product-images/L21564-010/003.jpg,https://oleks-netizen.github.io/product-images/L21564-010/005.jpg,https://oleks-netizen.github.io/product-images/L21564-010/006.jpg,https://oleks-netizen.github.io/product-images/L21564-010/007.jpg,https://oleks-netizen.github.io/product-images/L21564-010/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/96193001/001.jpg,https://oleks-netizen.github.io/product-images/96193001/002.jpg,https://oleks-netizen.github.io/product-images/96193001/003.jpg,https://oleks-netizen.github.io/product-images/96193001/004.jpg,https://oleks-netizen.github.io/product-images/96193001/005.jpg,https://oleks-netizen.github.io/product-images/96193001/007.jpg,https://oleks-netizen.github.io/product-images/96193001/008.jpg,https://oleks-netizen.github.io/product-images/96193001/009.jpg,https://oleks-netizen.github.io/product-images/96193001/010.jpg,https://oleks-netizen.github.io/product-images/96193001/011.jpg,https://oleks-netizen.github.io/product-images/96193001/012.jpg,https://oleks-netizen.github.io/product-images/96193001/013.jpg,https://oleks-netizen.github.io/product-images/96193001/014.jpg</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>L21564-025</t>
+          <t>96193008</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21564-025/001.jpg,https://oleks-netizen.github.io/product-images/L21564-025/002.jpg,https://oleks-netizen.github.io/product-images/L21564-025/003.jpg,https://oleks-netizen.github.io/product-images/L21564-025/005.jpg,https://oleks-netizen.github.io/product-images/L21564-025/006.jpg,https://oleks-netizen.github.io/product-images/L21564-025/007.jpg,https://oleks-netizen.github.io/product-images/L21564-025/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/96193008/001.jpg,https://oleks-netizen.github.io/product-images/96193008/002.jpg,https://oleks-netizen.github.io/product-images/96193008/003.jpg,https://oleks-netizen.github.io/product-images/96193008/004.jpg,https://oleks-netizen.github.io/product-images/96193008/006.jpg,https://oleks-netizen.github.io/product-images/96193008/007.jpg,https://oleks-netizen.github.io/product-images/96193008/008.jpg,https://oleks-netizen.github.io/product-images/96193008/009.jpg,https://oleks-netizen.github.io/product-images/96193008/010.jpg,https://oleks-netizen.github.io/product-images/96193008/011.jpg,https://oleks-netizen.github.io/product-images/96193008/012.jpg,https://oleks-netizen.github.io/product-images/96193008/013.jpg,https://oleks-netizen.github.io/product-images/96193008/014.jpg</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>L21564-066</t>
+          <t>96193070</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21564-066/001.jpg,https://oleks-netizen.github.io/product-images/L21564-066/002.jpg,https://oleks-netizen.github.io/product-images/L21564-066/003.jpg,https://oleks-netizen.github.io/product-images/L21564-066/005.jpg,https://oleks-netizen.github.io/product-images/L21564-066/006.jpg,https://oleks-netizen.github.io/product-images/L21564-066/007.jpg,https://oleks-netizen.github.io/product-images/L21564-066/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/96193070/001.jpg,https://oleks-netizen.github.io/product-images/96193070/002.jpg,https://oleks-netizen.github.io/product-images/96193070/003.jpg,https://oleks-netizen.github.io/product-images/96193070/004.jpg,https://oleks-netizen.github.io/product-images/96193070/005.jpg,https://oleks-netizen.github.io/product-images/96193070/006.jpg,https://oleks-netizen.github.io/product-images/96193070/007.jpg,https://oleks-netizen.github.io/product-images/96193070/009.jpg,https://oleks-netizen.github.io/product-images/96193070/010.jpg,https://oleks-netizen.github.io/product-images/96193070/011.jpg,https://oleks-netizen.github.io/product-images/96193070/012.jpg</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>L21580-1</t>
+          <t>96199170</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21580-1/001.jpg,https://oleks-netizen.github.io/product-images/L21580-1/002.jpg,https://oleks-netizen.github.io/product-images/L21580-1/003.jpg,https://oleks-netizen.github.io/product-images/L21580-1/005.jpg,https://oleks-netizen.github.io/product-images/L21580-1/006.jpg,https://oleks-netizen.github.io/product-images/L21580-1/007.jpg,https://oleks-netizen.github.io/product-images/L21580-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/96199170/001.jpg,https://oleks-netizen.github.io/product-images/96199170/002.jpg,https://oleks-netizen.github.io/product-images/96199170/003.jpg,https://oleks-netizen.github.io/product-images/96199170/004.jpg,https://oleks-netizen.github.io/product-images/96199170/005.jpg,https://oleks-netizen.github.io/product-images/96199170/006.jpg,https://oleks-netizen.github.io/product-images/96199170/007.jpg,https://oleks-netizen.github.io/product-images/96199170/008.jpg,https://oleks-netizen.github.io/product-images/96199170/009.jpg,https://oleks-netizen.github.io/product-images/96199170/010.jpg,https://oleks-netizen.github.io/product-images/96199170/011.jpg,https://oleks-netizen.github.io/product-images/96199170/013.jpg</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>L21580-175</t>
+          <t>B10-434A</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21580-175/001.jpg,https://oleks-netizen.github.io/product-images/L21580-175/002.jpg,https://oleks-netizen.github.io/product-images/L21580-175/003.jpg,https://oleks-netizen.github.io/product-images/L21580-175/005.jpg,https://oleks-netizen.github.io/product-images/L21580-175/006.jpg,https://oleks-netizen.github.io/product-images/L21580-175/007.jpg,https://oleks-netizen.github.io/product-images/L21580-175/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/B10-434A/001.jpg,https://oleks-netizen.github.io/product-images/B10-434A/002.jpg,https://oleks-netizen.github.io/product-images/B10-434A/003.jpg,https://oleks-netizen.github.io/product-images/B10-434A/004.jpg,https://oleks-netizen.github.io/product-images/B10-434A/005.jpg</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>L21580-49</t>
+          <t>BB80701-50</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21580-49/001.jpg,https://oleks-netizen.github.io/product-images/L21580-49/002.jpg,https://oleks-netizen.github.io/product-images/L21580-49/003.jpg,https://oleks-netizen.github.io/product-images/L21580-49/005.jpg,https://oleks-netizen.github.io/product-images/L21580-49/006.jpg,https://oleks-netizen.github.io/product-images/L21580-49/007.jpg,https://oleks-netizen.github.io/product-images/L21580-49/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BB80701-50/001.jpg,https://oleks-netizen.github.io/product-images/BB80701-50/002.jpg,https://oleks-netizen.github.io/product-images/BB80701-50/003.jpg,https://oleks-netizen.github.io/product-images/BB80701-50/005.jpg,https://oleks-netizen.github.io/product-images/BB80701-50/006.jpg,https://oleks-netizen.github.io/product-images/BB80701-50/007.jpg</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>L87025-01</t>
+          <t>BB81251-02</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87025-01/001.jpg,https://oleks-netizen.github.io/product-images/L87025-01/002.jpg,https://oleks-netizen.github.io/product-images/L87025-01/003.jpg,https://oleks-netizen.github.io/product-images/L87025-01/005.jpg,https://oleks-netizen.github.io/product-images/L87025-01/006.jpg,https://oleks-netizen.github.io/product-images/L87025-01/007.jpg,https://oleks-netizen.github.io/product-images/L87025-01/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BB81251-02/001.jpg,https://oleks-netizen.github.io/product-images/BB81251-02/002.jpg,https://oleks-netizen.github.io/product-images/BB81251-02/003.jpg,https://oleks-netizen.github.io/product-images/BB81251-02/005.jpg,https://oleks-netizen.github.io/product-images/BB81251-02/006.jpg,https://oleks-netizen.github.io/product-images/BB81251-02/007.jpg</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>L87025-13</t>
+          <t>BN-KK-4-k-kr-karbon</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87025-13/001.jpg,https://oleks-netizen.github.io/product-images/L87025-13/002.jpg,https://oleks-netizen.github.io/product-images/L87025-13/003.jpg,https://oleks-netizen.github.io/product-images/L87025-13/005.jpg,https://oleks-netizen.github.io/product-images/L87025-13/006.jpg,https://oleks-netizen.github.io/product-images/L87025-13/007.jpg,https://oleks-netizen.github.io/product-images/L87025-13/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-KK-4-k-kr-karbon/001.jpg,https://oleks-netizen.github.io/product-images/BN-KK-4-k-kr-karbon/002.jpg,https://oleks-netizen.github.io/product-images/BN-KK-4-k-kr-karbon/003.jpg,https://oleks-netizen.github.io/product-images/BN-KK-4-k-kr-karbon/004.jpg,https://oleks-netizen.github.io/product-images/BN-KK-4-k-kr-karbon/006.jpg</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>L87025-23</t>
+          <t>BN-KK-4-vin-kr</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87025-23/001.jpg,https://oleks-netizen.github.io/product-images/L87025-23/002.jpg,https://oleks-netizen.github.io/product-images/L87025-23/003.jpg,https://oleks-netizen.github.io/product-images/L87025-23/005.jpg,https://oleks-netizen.github.io/product-images/L87025-23/006.jpg,https://oleks-netizen.github.io/product-images/L87025-23/007.jpg,https://oleks-netizen.github.io/product-images/L87025-23/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-KK-4-vin-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-KK-4-vin-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-KK-4-vin-kr/003.jpg</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>L87025-26</t>
+          <t>BN-SB-2-st-red</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87025-26/001.jpg,https://oleks-netizen.github.io/product-images/L87025-26/002.jpg,https://oleks-netizen.github.io/product-images/L87025-26/003.jpg,https://oleks-netizen.github.io/product-images/L87025-26/005.jpg,https://oleks-netizen.github.io/product-images/L87025-26/006.jpg,https://oleks-netizen.github.io/product-images/L87025-26/007.jpg,https://oleks-netizen.github.io/product-images/L87025-26/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-SB-2-st-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-2-st-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-2-st-red/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-2-st-red/005.jpg</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>L87093-01</t>
+          <t>BS70106-01</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87093-01/001.jpg,https://oleks-netizen.github.io/product-images/L87093-01/002.jpg,https://oleks-netizen.github.io/product-images/L87093-01/004.jpg,https://oleks-netizen.github.io/product-images/L87093-01/005.jpg,https://oleks-netizen.github.io/product-images/L87093-01/006.jpg,https://oleks-netizen.github.io/product-images/L87093-01/007.jpg,https://oleks-netizen.github.io/product-images/L87093-01/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BS70106-01/001.jpg,https://oleks-netizen.github.io/product-images/BS70106-01/002.jpg,https://oleks-netizen.github.io/product-images/BS70106-01/003.jpg,https://oleks-netizen.github.io/product-images/BS70106-01/005.jpg,https://oleks-netizen.github.io/product-images/BS70106-01/006.jpg,https://oleks-netizen.github.io/product-images/BS70106-01/007.jpg</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>L87093-108</t>
+          <t>BS80401-01</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87093-108/001.jpg,https://oleks-netizen.github.io/product-images/L87093-108/003.jpg,https://oleks-netizen.github.io/product-images/L87093-108/004.jpg,https://oleks-netizen.github.io/product-images/L87093-108/005.jpg,https://oleks-netizen.github.io/product-images/L87093-108/006.jpg,https://oleks-netizen.github.io/product-images/L87093-108/007.jpg,https://oleks-netizen.github.io/product-images/L87093-108/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BS80401-01/001.jpg,https://oleks-netizen.github.io/product-images/BS80401-01/002.jpg,https://oleks-netizen.github.io/product-images/BS80401-01/003.jpg,https://oleks-netizen.github.io/product-images/BS80401-01/005.jpg,https://oleks-netizen.github.io/product-images/BS80401-01/006.jpg,https://oleks-netizen.github.io/product-images/BS80401-01/007.jpg</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>L87093-245</t>
+          <t>BV39032-1</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87093-245/001.jpg,https://oleks-netizen.github.io/product-images/L87093-245/003.jpg,https://oleks-netizen.github.io/product-images/L87093-245/004.jpg,https://oleks-netizen.github.io/product-images/L87093-245/005.jpg,https://oleks-netizen.github.io/product-images/L87093-245/006.jpg,https://oleks-netizen.github.io/product-images/L87093-245/007.jpg,https://oleks-netizen.github.io/product-images/L87093-245/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39032-1/001.jpg,https://oleks-netizen.github.io/product-images/BV39032-1/002.jpg,https://oleks-netizen.github.io/product-images/BV39032-1/004.jpg,https://oleks-netizen.github.io/product-images/BV39032-1/005.jpg,https://oleks-netizen.github.io/product-images/BV39032-1/006.jpg,https://oleks-netizen.github.io/product-images/BV39032-1/007.jpg,https://oleks-netizen.github.io/product-images/BV39032-1/008.jpg</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -1591,12 +1591,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>L87093-246</t>
+          <t>BV39032-191</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87093-246/001.jpg,https://oleks-netizen.github.io/product-images/L87093-246/002.jpg,https://oleks-netizen.github.io/product-images/L87093-246/004.jpg,https://oleks-netizen.github.io/product-images/L87093-246/005.jpg,https://oleks-netizen.github.io/product-images/L87093-246/006.jpg,https://oleks-netizen.github.io/product-images/L87093-246/007.jpg,https://oleks-netizen.github.io/product-images/L87093-246/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39032-191/001.jpg,https://oleks-netizen.github.io/product-images/BV39032-191/002.jpg,https://oleks-netizen.github.io/product-images/BV39032-191/003.jpg,https://oleks-netizen.github.io/product-images/BV39032-191/004.jpg,https://oleks-netizen.github.io/product-images/BV39032-191/005.jpg,https://oleks-netizen.github.io/product-images/BV39032-191/006.jpg,https://oleks-netizen.github.io/product-images/BV39032-191/007.jpg</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -1606,12 +1606,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>L87114-01</t>
+          <t>BV39139-1</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87114-01/001.jpg,https://oleks-netizen.github.io/product-images/L87114-01/002.jpg,https://oleks-netizen.github.io/product-images/L87114-01/003.jpg,https://oleks-netizen.github.io/product-images/L87114-01/005.jpg,https://oleks-netizen.github.io/product-images/L87114-01/006.jpg,https://oleks-netizen.github.io/product-images/L87114-01/007.jpg,https://oleks-netizen.github.io/product-images/L87114-01/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39139-1/001.jpg,https://oleks-netizen.github.io/product-images/BV39139-1/002.jpg,https://oleks-netizen.github.io/product-images/BV39139-1/004.jpg,https://oleks-netizen.github.io/product-images/BV39139-1/005.jpg,https://oleks-netizen.github.io/product-images/BV39139-1/006.jpg,https://oleks-netizen.github.io/product-images/BV39139-1/007.jpg,https://oleks-netizen.github.io/product-images/BV39139-1/008.jpg</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -1621,27 +1621,27 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>L87114-108</t>
+          <t>BV39218-1</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87114-108/001.jpg,https://oleks-netizen.github.io/product-images/L87114-108/002.jpg,https://oleks-netizen.github.io/product-images/L87114-108/003.jpg,https://oleks-netizen.github.io/product-images/L87114-108/005.jpg,https://oleks-netizen.github.io/product-images/L87114-108/006.jpg,https://oleks-netizen.github.io/product-images/L87114-108/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39218-1/001.jpg,https://oleks-netizen.github.io/product-images/BV39218-1/002.jpg,https://oleks-netizen.github.io/product-images/BV39218-1/004.jpg,https://oleks-netizen.github.io/product-images/BV39218-1/005.jpg,https://oleks-netizen.github.io/product-images/BV39218-1/006.jpg,https://oleks-netizen.github.io/product-images/BV39218-1/007.jpg,https://oleks-netizen.github.io/product-images/BV39218-1/008.jpg</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>L87114-246</t>
+          <t>BV39218-153</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87114-246/001.jpg,https://oleks-netizen.github.io/product-images/L87114-246/002.jpg,https://oleks-netizen.github.io/product-images/L87114-246/003.jpg,https://oleks-netizen.github.io/product-images/L87114-246/005.jpg,https://oleks-netizen.github.io/product-images/L87114-246/006.jpg,https://oleks-netizen.github.io/product-images/L87114-246/007.jpg,https://oleks-netizen.github.io/product-images/L87114-246/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39218-153/001.jpg,https://oleks-netizen.github.io/product-images/BV39218-153/002.jpg,https://oleks-netizen.github.io/product-images/BV39218-153/004.jpg,https://oleks-netizen.github.io/product-images/BV39218-153/005.jpg,https://oleks-netizen.github.io/product-images/BV39218-153/006.jpg,https://oleks-netizen.github.io/product-images/BV39218-153/007.jpg,https://oleks-netizen.github.io/product-images/BV39218-153/008.jpg</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -1651,12 +1651,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>L87169-01</t>
+          <t>BV39223-1</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87169-01/001.jpg,https://oleks-netizen.github.io/product-images/L87169-01/002.jpg,https://oleks-netizen.github.io/product-images/L87169-01/003.jpg,https://oleks-netizen.github.io/product-images/L87169-01/005.jpg,https://oleks-netizen.github.io/product-images/L87169-01/006.jpg,https://oleks-netizen.github.io/product-images/L87169-01/007.jpg,https://oleks-netizen.github.io/product-images/L87169-01/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39223-1/001.jpg,https://oleks-netizen.github.io/product-images/BV39223-1/002.jpg,https://oleks-netizen.github.io/product-images/BV39223-1/003.jpg,https://oleks-netizen.github.io/product-images/BV39223-1/004.jpg,https://oleks-netizen.github.io/product-images/BV39223-1/005.jpg,https://oleks-netizen.github.io/product-images/BV39223-1/006.jpg,https://oleks-netizen.github.io/product-images/BV39223-1/007.jpg</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -1666,12 +1666,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>L87169-113</t>
+          <t>BV39223-1-small</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87169-113/001.jpg,https://oleks-netizen.github.io/product-images/L87169-113/002.jpg,https://oleks-netizen.github.io/product-images/L87169-113/003.jpg,https://oleks-netizen.github.io/product-images/L87169-113/005.jpg,https://oleks-netizen.github.io/product-images/L87169-113/006.jpg,https://oleks-netizen.github.io/product-images/L87169-113/007.jpg,https://oleks-netizen.github.io/product-images/L87169-113/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39223-1-small/001.jpg,https://oleks-netizen.github.io/product-images/BV39223-1-small/002.jpg,https://oleks-netizen.github.io/product-images/BV39223-1-small/003.jpg,https://oleks-netizen.github.io/product-images/BV39223-1-small/004.jpg,https://oleks-netizen.github.io/product-images/BV39223-1-small/005.jpg,https://oleks-netizen.github.io/product-images/BV39223-1-small/006.jpg,https://oleks-netizen.github.io/product-images/BV39223-1-small/007.jpg</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -1681,12 +1681,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>L87169-175</t>
+          <t>BV39223-145</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87169-175/001.jpg,https://oleks-netizen.github.io/product-images/L87169-175/002.jpg,https://oleks-netizen.github.io/product-images/L87169-175/003.jpg,https://oleks-netizen.github.io/product-images/L87169-175/005.jpg,https://oleks-netizen.github.io/product-images/L87169-175/006.jpg,https://oleks-netizen.github.io/product-images/L87169-175/007.jpg,https://oleks-netizen.github.io/product-images/L87169-175/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39223-145/001.jpg,https://oleks-netizen.github.io/product-images/BV39223-145/002.jpg,https://oleks-netizen.github.io/product-images/BV39223-145/004.jpg,https://oleks-netizen.github.io/product-images/BV39223-145/005.jpg,https://oleks-netizen.github.io/product-images/BV39223-145/006.jpg,https://oleks-netizen.github.io/product-images/BV39223-145/007.jpg,https://oleks-netizen.github.io/product-images/BV39223-145/008.jpg</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -1696,42 +1696,42 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>L87169-81</t>
+          <t>BV39311-1</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87169-81/001.jpg,https://oleks-netizen.github.io/product-images/L87169-81/002.jpg,https://oleks-netizen.github.io/product-images/L87169-81/003.jpg,https://oleks-netizen.github.io/product-images/L87169-81/005.jpg,https://oleks-netizen.github.io/product-images/L87169-81/006.jpg,https://oleks-netizen.github.io/product-images/L87169-81/007.jpg,https://oleks-netizen.github.io/product-images/L87169-81/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39311-1/001.jpg,https://oleks-netizen.github.io/product-images/BV39311-1/002.jpg,https://oleks-netizen.github.io/product-images/BV39311-1/004.jpg,https://oleks-netizen.github.io/product-images/BV39311-1/005.jpg,https://oleks-netizen.github.io/product-images/BV39311-1/006.jpg,https://oleks-netizen.github.io/product-images/BV39311-1/007.jpg,https://oleks-netizen.github.io/product-images/BV39311-1/008.jpg,https://oleks-netizen.github.io/product-images/BV39311-1/009.jpg,https://oleks-netizen.github.io/product-images/BV39311-1/010.jpg</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>L87518-01</t>
+          <t>BV39311-153</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87518-01/001.jpg,https://oleks-netizen.github.io/product-images/L87518-01/002.jpg,https://oleks-netizen.github.io/product-images/L87518-01/003.jpg,https://oleks-netizen.github.io/product-images/L87518-01/005.jpg,https://oleks-netizen.github.io/product-images/L87518-01/006.jpg,https://oleks-netizen.github.io/product-images/L87518-01/007.jpg,https://oleks-netizen.github.io/product-images/L87518-01/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39311-153/001.jpg,https://oleks-netizen.github.io/product-images/BV39311-153/002.jpg,https://oleks-netizen.github.io/product-images/BV39311-153/004.jpg,https://oleks-netizen.github.io/product-images/BV39311-153/005.jpg,https://oleks-netizen.github.io/product-images/BV39311-153/006.jpg,https://oleks-netizen.github.io/product-images/BV39311-153/007.jpg,https://oleks-netizen.github.io/product-images/BV39311-153/008.jpg,https://oleks-netizen.github.io/product-images/BV39311-153/009.jpg,https://oleks-netizen.github.io/product-images/BV39311-153/010.jpg,https://oleks-netizen.github.io/product-images/BV39311-153/011.jpg</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>L87518-56</t>
+          <t>BV39318-1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87518-56/001.jpg,https://oleks-netizen.github.io/product-images/L87518-56/002.jpg,https://oleks-netizen.github.io/product-images/L87518-56/004.jpg,https://oleks-netizen.github.io/product-images/L87518-56/005.jpg,https://oleks-netizen.github.io/product-images/L87518-56/006.jpg,https://oleks-netizen.github.io/product-images/L87518-56/007.jpg,https://oleks-netizen.github.io/product-images/L87518-56/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39318-1/001.jpg,https://oleks-netizen.github.io/product-images/BV39318-1/002.jpg,https://oleks-netizen.github.io/product-images/BV39318-1/003.jpg,https://oleks-netizen.github.io/product-images/BV39318-1/004.jpg,https://oleks-netizen.github.io/product-images/BV39318-1/005.jpg,https://oleks-netizen.github.io/product-images/BV39318-1/006.jpg,https://oleks-netizen.github.io/product-images/BV39318-1/007.jpg</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -1741,12 +1741,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>L87518-79</t>
+          <t>BV39318-232</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87518-79/001.jpg,https://oleks-netizen.github.io/product-images/L87518-79/002.jpg,https://oleks-netizen.github.io/product-images/L87518-79/004.jpg,https://oleks-netizen.github.io/product-images/L87518-79/005.jpg,https://oleks-netizen.github.io/product-images/L87518-79/006.jpg,https://oleks-netizen.github.io/product-images/L87518-79/007.jpg,https://oleks-netizen.github.io/product-images/L87518-79/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39318-232/001.jpg,https://oleks-netizen.github.io/product-images/BV39318-232/002.jpg,https://oleks-netizen.github.io/product-images/BV39318-232/003.jpg,https://oleks-netizen.github.io/product-images/BV39318-232/004.jpg,https://oleks-netizen.github.io/product-images/BV39318-232/005.jpg,https://oleks-netizen.github.io/product-images/BV39318-232/006.jpg,https://oleks-netizen.github.io/product-images/BV39318-232/007.jpg</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -1756,12 +1756,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>L87713-01</t>
+          <t>BV39318-76A</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87713-01/001.jpg,https://oleks-netizen.github.io/product-images/L87713-01/002.jpg,https://oleks-netizen.github.io/product-images/L87713-01/003.jpg,https://oleks-netizen.github.io/product-images/L87713-01/005.jpg,https://oleks-netizen.github.io/product-images/L87713-01/006.jpg,https://oleks-netizen.github.io/product-images/L87713-01/007.jpg,https://oleks-netizen.github.io/product-images/L87713-01/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39318-76A/001.jpg,https://oleks-netizen.github.io/product-images/BV39318-76A/002.jpg,https://oleks-netizen.github.io/product-images/BV39318-76A/003.jpg,https://oleks-netizen.github.io/product-images/BV39318-76A/004.jpg,https://oleks-netizen.github.io/product-images/BV39318-76A/005.jpg,https://oleks-netizen.github.io/product-images/BV39318-76A/006.jpg,https://oleks-netizen.github.io/product-images/BV39318-76A/007.jpg</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -1771,12 +1771,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>L87713-107</t>
+          <t>BV39351-1</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87713-107/001.jpg,https://oleks-netizen.github.io/product-images/L87713-107/002.jpg,https://oleks-netizen.github.io/product-images/L87713-107/003.jpg,https://oleks-netizen.github.io/product-images/L87713-107/005.jpg,https://oleks-netizen.github.io/product-images/L87713-107/006.jpg,https://oleks-netizen.github.io/product-images/L87713-107/007.jpg,https://oleks-netizen.github.io/product-images/L87713-107/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39351-1/001.jpg,https://oleks-netizen.github.io/product-images/BV39351-1/002.jpg,https://oleks-netizen.github.io/product-images/BV39351-1/003.jpg,https://oleks-netizen.github.io/product-images/BV39351-1/004.jpg,https://oleks-netizen.github.io/product-images/BV39351-1/005.jpg,https://oleks-netizen.github.io/product-images/BV39351-1/006.jpg,https://oleks-netizen.github.io/product-images/BV39351-1/007.jpg</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -1786,12 +1786,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>L87713-221</t>
+          <t>BV39529-1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87713-221/001.jpg,https://oleks-netizen.github.io/product-images/L87713-221/002.jpg,https://oleks-netizen.github.io/product-images/L87713-221/003.jpg,https://oleks-netizen.github.io/product-images/L87713-221/005.jpg,https://oleks-netizen.github.io/product-images/L87713-221/006.jpg,https://oleks-netizen.github.io/product-images/L87713-221/007.jpg,https://oleks-netizen.github.io/product-images/L87713-221/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39529-1/001.jpg,https://oleks-netizen.github.io/product-images/BV39529-1/002.jpg,https://oleks-netizen.github.io/product-images/BV39529-1/003.jpg,https://oleks-netizen.github.io/product-images/BV39529-1/004.jpg,https://oleks-netizen.github.io/product-images/BV39529-1/005.jpg,https://oleks-netizen.github.io/product-images/BV39529-1/006.jpg,https://oleks-netizen.github.io/product-images/BV39529-1/007.jpg</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -1801,12 +1801,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>L87713-97</t>
+          <t>BV39529-145</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87713-97/001.jpg,https://oleks-netizen.github.io/product-images/L87713-97/002.jpg,https://oleks-netizen.github.io/product-images/L87713-97/003.jpg,https://oleks-netizen.github.io/product-images/L87713-97/005.jpg,https://oleks-netizen.github.io/product-images/L87713-97/006.jpg,https://oleks-netizen.github.io/product-images/L87713-97/007.jpg,https://oleks-netizen.github.io/product-images/L87713-97/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV39529-145/001.jpg,https://oleks-netizen.github.io/product-images/BV39529-145/002.jpg,https://oleks-netizen.github.io/product-images/BV39529-145/004.jpg,https://oleks-netizen.github.io/product-images/BV39529-145/005.jpg,https://oleks-netizen.github.io/product-images/BV39529-145/006.jpg,https://oleks-netizen.github.io/product-images/BV39529-145/007.jpg,https://oleks-netizen.github.io/product-images/BV39529-145/008.jpg</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -1816,16 +1816,3031 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>TW-Vivian-mokko</t>
+          <t>bx050a</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/TW-Vivian-mokko/001.jpg,https://oleks-netizen.github.io/product-images/TW-Vivian-mokko/002.jpg,https://oleks-netizen.github.io/product-images/TW-Vivian-mokko/004.jpg,https://oleks-netizen.github.io/product-images/TW-Vivian-mokko/005.jpg,https://oleks-netizen.github.io/product-images/TW-Vivian-mokko/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/bx050a/001.jpg,https://oleks-netizen.github.io/product-images/bx050a/002.jpg,https://oleks-netizen.github.io/product-images/bx050a/003.jpg,https://oleks-netizen.github.io/product-images/bx050a/004.jpg,https://oleks-netizen.github.io/product-images/bx050a/005.jpg,https://oleks-netizen.github.io/product-images/bx050a/006.jpg</t>
         </is>
       </c>
       <c r="C94" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>bx050c</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/bx050c/001.jpg,https://oleks-netizen.github.io/product-images/bx050c/002.jpg,https://oleks-netizen.github.io/product-images/bx050c/003.jpg,https://oleks-netizen.github.io/product-images/bx050c/005.jpg,https://oleks-netizen.github.io/product-images/bx050c/006.jpg</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>bx9020</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/bx9020/001.jpg,https://oleks-netizen.github.io/product-images/bx9020/002.jpg,https://oleks-netizen.github.io/product-images/bx9020/003.jpg,https://oleks-netizen.github.io/product-images/bx9020/004.jpg,https://oleks-netizen.github.io/product-images/bx9020/005.jpg,https://oleks-netizen.github.io/product-images/bx9020/006.jpg,https://oleks-netizen.github.io/product-images/bx9020/007.jpg,https://oleks-netizen.github.io/product-images/bx9020/008.jpg</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>CC605_BN</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/CC605_BN/001.jpg,https://oleks-netizen.github.io/product-images/CC605_BN/002.jpg,https://oleks-netizen.github.io/product-images/CC605_BN/004.jpg,https://oleks-netizen.github.io/product-images/CC605_BN/005.jpg,https://oleks-netizen.github.io/product-images/CC605_BN/006.jpg,https://oleks-netizen.github.io/product-images/CC605_BN/007.jpg</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>CrH-1294-4lx</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/CrH-1294-4lx/001.jpg,https://oleks-netizen.github.io/product-images/CrH-1294-4lx/002.jpg,https://oleks-netizen.github.io/product-images/CrH-1294-4lx/003.jpg,https://oleks-netizen.github.io/product-images/CrH-1294-4lx/005.jpg,https://oleks-netizen.github.io/product-images/CrH-1294-4lx/006.jpg,https://oleks-netizen.github.io/product-images/CrH-1294-4lx/007.jpg,https://oleks-netizen.github.io/product-images/CrH-1294-4lx/008.jpg,https://oleks-netizen.github.io/product-images/CrH-1294-4lx/009.jpg,https://oleks-netizen.github.io/product-images/CrH-1294-4lx/010.jpg,https://oleks-netizen.github.io/product-images/CrH-1294-4lx/011.jpg</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>DRL19031-3</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19031-3/001.jpg,https://oleks-netizen.github.io/product-images/DRL19031-3/002.jpg,https://oleks-netizen.github.io/product-images/DRL19031-3/004.jpg,https://oleks-netizen.github.io/product-images/DRL19031-3/005.jpg,https://oleks-netizen.github.io/product-images/DRL19031-3/006.jpg,https://oleks-netizen.github.io/product-images/DRL19031-3/007.jpg</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>DRL19086-1</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19086-1/001.jpg,https://oleks-netizen.github.io/product-images/DRL19086-1/002.jpg,https://oleks-netizen.github.io/product-images/DRL19086-1/004.jpg,https://oleks-netizen.github.io/product-images/DRL19086-1/005.jpg,https://oleks-netizen.github.io/product-images/DRL19086-1/006.jpg,https://oleks-netizen.github.io/product-images/DRL19086-1/007.jpg,https://oleks-netizen.github.io/product-images/DRL19086-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>DRL19101-1</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19101-1/001.jpg,https://oleks-netizen.github.io/product-images/DRL19101-1/002.jpg,https://oleks-netizen.github.io/product-images/DRL19101-1/004.jpg,https://oleks-netizen.github.io/product-images/DRL19101-1/005.jpg,https://oleks-netizen.github.io/product-images/DRL19101-1/006.jpg,https://oleks-netizen.github.io/product-images/DRL19101-1/007.jpg,https://oleks-netizen.github.io/product-images/DRL19101-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>DRL19158-2</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19158-2/001.jpg,https://oleks-netizen.github.io/product-images/DRL19158-2/002.jpg,https://oleks-netizen.github.io/product-images/DRL19158-2/003.jpg,https://oleks-netizen.github.io/product-images/DRL19158-2/004.jpg,https://oleks-netizen.github.io/product-images/DRL19158-2/005.jpg,https://oleks-netizen.github.io/product-images/DRL19158-2/006.jpg</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>DRL1925-1</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL1925-1/001.jpg,https://oleks-netizen.github.io/product-images/DRL1925-1/002.jpg,https://oleks-netizen.github.io/product-images/DRL1925-1/004.jpg,https://oleks-netizen.github.io/product-images/DRL1925-1/005.jpg,https://oleks-netizen.github.io/product-images/DRL1925-1/006.jpg,https://oleks-netizen.github.io/product-images/DRL1925-1/007.jpg,https://oleks-netizen.github.io/product-images/DRL1925-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>DRL19286-6</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19286-6/001.jpg,https://oleks-netizen.github.io/product-images/DRL19286-6/002.jpg,https://oleks-netizen.github.io/product-images/DRL19286-6/004.jpg,https://oleks-netizen.github.io/product-images/DRL19286-6/005.jpg,https://oleks-netizen.github.io/product-images/DRL19286-6/006.jpg,https://oleks-netizen.github.io/product-images/DRL19286-6/007.jpg,https://oleks-netizen.github.io/product-images/DRL19286-6/008.jpg</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>DRL19333-1</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19333-1/001.jpg,https://oleks-netizen.github.io/product-images/DRL19333-1/002.jpg,https://oleks-netizen.github.io/product-images/DRL19333-1/004.jpg,https://oleks-netizen.github.io/product-images/DRL19333-1/005.jpg,https://oleks-netizen.github.io/product-images/DRL19333-1/006.jpg,https://oleks-netizen.github.io/product-images/DRL19333-1/007.jpg,https://oleks-netizen.github.io/product-images/DRL19333-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>DRL19377-1</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19377-1/001.jpg,https://oleks-netizen.github.io/product-images/DRL19377-1/002.jpg,https://oleks-netizen.github.io/product-images/DRL19377-1/004.jpg,https://oleks-netizen.github.io/product-images/DRL19377-1/005.jpg,https://oleks-netizen.github.io/product-images/DRL19377-1/006.jpg,https://oleks-netizen.github.io/product-images/DRL19377-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>DRL19389-6</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19389-6/001.jpg,https://oleks-netizen.github.io/product-images/DRL19389-6/002.jpg,https://oleks-netizen.github.io/product-images/DRL19389-6/004.jpg,https://oleks-netizen.github.io/product-images/DRL19389-6/005.jpg,https://oleks-netizen.github.io/product-images/DRL19389-6/006.jpg,https://oleks-netizen.github.io/product-images/DRL19389-6/007.jpg,https://oleks-netizen.github.io/product-images/DRL19389-6/008.jpg</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>DRL19393-6</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19393-6/001.jpg,https://oleks-netizen.github.io/product-images/DRL19393-6/002.jpg,https://oleks-netizen.github.io/product-images/DRL19393-6/004.jpg,https://oleks-netizen.github.io/product-images/DRL19393-6/005.jpg,https://oleks-netizen.github.io/product-images/DRL19393-6/006.jpg,https://oleks-netizen.github.io/product-images/DRL19393-6/007.jpg,https://oleks-netizen.github.io/product-images/DRL19393-6/008.jpg</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>DRL19429-1</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19429-1/001.jpg,https://oleks-netizen.github.io/product-images/DRL19429-1/002.jpg,https://oleks-netizen.github.io/product-images/DRL19429-1/004.jpg,https://oleks-netizen.github.io/product-images/DRL19429-1/005.jpg,https://oleks-netizen.github.io/product-images/DRL19429-1/006.jpg,https://oleks-netizen.github.io/product-images/DRL19429-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>DRL19460-1</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19460-1/001.jpg,https://oleks-netizen.github.io/product-images/DRL19460-1/002.jpg,https://oleks-netizen.github.io/product-images/DRL19460-1/004.jpg,https://oleks-netizen.github.io/product-images/DRL19460-1/005.jpg,https://oleks-netizen.github.io/product-images/DRL19460-1/006.jpg,https://oleks-netizen.github.io/product-images/DRL19460-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>DRL19608-1</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19608-1/001.jpg,https://oleks-netizen.github.io/product-images/DRL19608-1/002.jpg,https://oleks-netizen.github.io/product-images/DRL19608-1/004.jpg,https://oleks-netizen.github.io/product-images/DRL19608-1/005.jpg,https://oleks-netizen.github.io/product-images/DRL19608-1/006.jpg,https://oleks-netizen.github.io/product-images/DRL19608-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>DRL19710-1</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19710-1/001.jpg,https://oleks-netizen.github.io/product-images/DRL19710-1/002.jpg,https://oleks-netizen.github.io/product-images/DRL19710-1/004.jpg,https://oleks-netizen.github.io/product-images/DRL19710-1/005.jpg,https://oleks-netizen.github.io/product-images/DRL19710-1/006.jpg,https://oleks-netizen.github.io/product-images/DRL19710-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>DRL19946-1</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRL19946-1/001.jpg,https://oleks-netizen.github.io/product-images/DRL19946-1/002.jpg,https://oleks-netizen.github.io/product-images/DRL19946-1/004.jpg,https://oleks-netizen.github.io/product-images/DRL19946-1/005.jpg,https://oleks-netizen.github.io/product-images/DRL19946-1/006.jpg,https://oleks-netizen.github.io/product-images/DRL19946-1/007.jpg,https://oleks-netizen.github.io/product-images/DRL19946-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Elit-2020-4lx</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/Elit-2020-4lx/001.jpg,https://oleks-netizen.github.io/product-images/Elit-2020-4lx/002.jpg,https://oleks-netizen.github.io/product-images/Elit-2020-4lx/003.jpg,https://oleks-netizen.github.io/product-images/Elit-2020-4lx/004.jpg,https://oleks-netizen.github.io/product-images/Elit-2020-4lx/005.jpg,https://oleks-netizen.github.io/product-images/Elit-2020-4lx/006.jpg,https://oleks-netizen.github.io/product-images/Elit-2020-4lx/007.jpg,https://oleks-netizen.github.io/product-images/Elit-2020-4lx/009.jpg,https://oleks-netizen.github.io/product-images/Elit-2020-4lx/010.jpg,https://oleks-netizen.github.io/product-images/Elit-2020-4lx/011.jpg</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Elit-2022-4lx</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/Elit-2022-4lx/001.jpg,https://oleks-netizen.github.io/product-images/Elit-2022-4lx/002.jpg,https://oleks-netizen.github.io/product-images/Elit-2022-4lx/003.jpg,https://oleks-netizen.github.io/product-images/Elit-2022-4lx/004.jpg,https://oleks-netizen.github.io/product-images/Elit-2022-4lx/005.jpg,https://oleks-netizen.github.io/product-images/Elit-2022-4lx/006.jpg,https://oleks-netizen.github.io/product-images/Elit-2022-4lx/007.jpg,https://oleks-netizen.github.io/product-images/Elit-2022-4lx/008.jpg,https://oleks-netizen.github.io/product-images/Elit-2022-4lx/009.jpg,https://oleks-netizen.github.io/product-images/Elit-2022-4lx/010.jpg</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Elit-2023-4lx</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/Elit-2023-4lx/001.jpg,https://oleks-netizen.github.io/product-images/Elit-2023-4lx/002.jpg,https://oleks-netizen.github.io/product-images/Elit-2023-4lx/003.jpg,https://oleks-netizen.github.io/product-images/Elit-2023-4lx/004.jpg,https://oleks-netizen.github.io/product-images/Elit-2023-4lx/005.jpg,https://oleks-netizen.github.io/product-images/Elit-2023-4lx/006.jpg,https://oleks-netizen.github.io/product-images/Elit-2023-4lx/007.jpg,https://oleks-netizen.github.io/product-images/Elit-2023-4lx/008.jpg,https://oleks-netizen.github.io/product-images/Elit-2023-4lx/009.jpg</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>FA-1501-3md</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/FA-1501-3md/001.jpg,https://oleks-netizen.github.io/product-images/FA-1501-3md/002.jpg,https://oleks-netizen.github.io/product-images/FA-1501-3md/003.jpg,https://oleks-netizen.github.io/product-images/FA-1501-3md/004.jpg,https://oleks-netizen.github.io/product-images/FA-1501-3md/005.jpg,https://oleks-netizen.github.io/product-images/FA-1501-3md/006.jpg,https://oleks-netizen.github.io/product-images/FA-1501-3md/007.jpg</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>FCream-8077-3md</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/FCream-8077-3md/001.jpg,https://oleks-netizen.github.io/product-images/FCream-8077-3md/002.jpg,https://oleks-netizen.github.io/product-images/FCream-8077-3md/003.jpg,https://oleks-netizen.github.io/product-images/FCream-8077-3md/005.jpg,https://oleks-netizen.github.io/product-images/FCream-8077-3md/006.jpg,https://oleks-netizen.github.io/product-images/FCream-8077-3md/007.jpg</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>FR7007K</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/FR7007K/001.jpg,https://oleks-netizen.github.io/product-images/FR7007K/002.jpg,https://oleks-netizen.github.io/product-images/FR7007K/003.jpg,https://oleks-netizen.github.io/product-images/FR7007K/004.jpg</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>FR7007O</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/FR7007O/001.jpg,https://oleks-netizen.github.io/product-images/FR7007O/002.jpg,https://oleks-netizen.github.io/product-images/FR7007O/003.jpg,https://oleks-netizen.github.io/product-images/FR7007O/004.jpg</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>FR7007P</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/FR7007P/001.jpg,https://oleks-netizen.github.io/product-images/FR7007P/002.jpg,https://oleks-netizen.github.io/product-images/FR7007P/003.jpg,https://oleks-netizen.github.io/product-images/FR7007P/004.jpg,https://oleks-netizen.github.io/product-images/FR7007P/005.jpg</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>fz118545</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/fz118545/001.jpg,https://oleks-netizen.github.io/product-images/fz118545/002.jpg,https://oleks-netizen.github.io/product-images/fz118545/003.jpg,https://oleks-netizen.github.io/product-images/fz118545/004.jpg,https://oleks-netizen.github.io/product-images/fz118545/005.jpg,https://oleks-netizen.github.io/product-images/fz118545/006.jpg,https://oleks-netizen.github.io/product-images/fz118545/007.jpg,https://oleks-netizen.github.io/product-images/fz118545/008.jpg</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>fz189606</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/fz189606/001.jpg,https://oleks-netizen.github.io/product-images/fz189606/002.jpg,https://oleks-netizen.github.io/product-images/fz189606/003.jpg,https://oleks-netizen.github.io/product-images/fz189606/004.jpg,https://oleks-netizen.github.io/product-images/fz189606/006.jpg,https://oleks-netizen.github.io/product-images/fz189606/007.jpg,https://oleks-netizen.github.io/product-images/fz189606/008.jpg</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>fz1896103</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/fz1896103/001.jpg,https://oleks-netizen.github.io/product-images/fz1896103/002.jpg,https://oleks-netizen.github.io/product-images/fz1896103/004.jpg,https://oleks-netizen.github.io/product-images/fz1896103/005.jpg,https://oleks-netizen.github.io/product-images/fz1896103/006.jpg,https://oleks-netizen.github.io/product-images/fz1896103/007.jpg,https://oleks-netizen.github.io/product-images/fz1896103/008.jpg,https://oleks-netizen.github.io/product-images/fz1896103/009.jpg,https://oleks-netizen.github.io/product-images/fz1896103/010.jpg,https://oleks-netizen.github.io/product-images/fz1896103/011.jpg</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>fz189645</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/fz189645/001.jpg,https://oleks-netizen.github.io/product-images/fz189645/002.jpg,https://oleks-netizen.github.io/product-images/fz189645/003.jpg,https://oleks-netizen.github.io/product-images/fz189645/004.jpg,https://oleks-netizen.github.io/product-images/fz189645/005.jpg,https://oleks-netizen.github.io/product-images/fz189645/006.jpg,https://oleks-netizen.github.io/product-images/fz189645/007.jpg,https://oleks-netizen.github.io/product-images/fz189645/008.jpg,https://oleks-netizen.github.io/product-images/fz189645/009.jpg,https://oleks-netizen.github.io/product-images/fz189645/010.jpg</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>GA-0307-4lx</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GA-0307-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GA-0307-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GA-0307-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GA-0307-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GA-0307-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GA-0307-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GA-0307-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GA-0307-4lx/009.jpg,https://oleks-netizen.github.io/product-images/GA-0307-4lx/010.jpg</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>GA-0324-4lx</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GA-0324-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GA-0324-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GA-0324-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GA-0324-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GA-0324-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GA-0324-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GA-0324-4lx/008.jpg,https://oleks-netizen.github.io/product-images/GA-0324-4lx/009.jpg,https://oleks-netizen.github.io/product-images/GA-0324-4lx/010.jpg,https://oleks-netizen.github.io/product-images/GA-0324-4lx/011.jpg</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>GA-1402-4lx</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GA-1402-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GA-1402-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GA-1402-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GA-1402-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GA-1402-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GA-1402-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GA-1402-4lx/008.jpg,https://oleks-netizen.github.io/product-images/GA-1402-4lx/009.jpg,https://oleks-netizen.github.io/product-images/GA-1402-4lx/010.jpg</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>GA-7281-3md</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GA-7281-3md/001.jpg,https://oleks-netizen.github.io/product-images/GA-7281-3md/002.jpg,https://oleks-netizen.github.io/product-images/GA-7281-3md/004.jpg,https://oleks-netizen.github.io/product-images/GA-7281-3md/005.jpg,https://oleks-netizen.github.io/product-images/GA-7281-3md/006.jpg,https://oleks-netizen.github.io/product-images/GA-7281-3md/007.jpg,https://oleks-netizen.github.io/product-images/GA-7281-3md/008.jpg,https://oleks-netizen.github.io/product-images/GA-7281-3md/009.jpg</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>GB-7107-3md</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GB-7107-3md/001.jpg,https://oleks-netizen.github.io/product-images/GB-7107-3md/002.jpg,https://oleks-netizen.github.io/product-images/GB-7107-3md/004.jpg,https://oleks-netizen.github.io/product-images/GB-7107-3md/005.jpg,https://oleks-netizen.github.io/product-images/GB-7107-3md/006.jpg</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>GBalc-2067-4lx</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GBalc-2067-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GBalc-2067-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GBalc-2067-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GBalc-2067-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GBalc-2067-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GBalc-2067-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GBalc-2067-4lx/008.jpg,https://oleks-netizen.github.io/product-images/GBalc-2067-4lx/009.jpg</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>GBord-2067-4lx</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GBord-2067-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GBord-2067-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GBord-2067-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GBord-2067-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GBord-2067-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GBord-2067-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GBord-2067-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GBord-2067-4lx/008.jpg,https://oleks-netizen.github.io/product-images/GBord-2067-4lx/009.jpg,https://oleks-netizen.github.io/product-images/GBord-2067-4lx/010.jpg</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>GC-0060-4lx</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GC-0060-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GC-0060-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GC-0060-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GC-0060-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GC-0060-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GC-0060-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GC-0060-4lx/008.jpg</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>GC-1239-4lx</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GC-1239-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GC-1239-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GC-1239-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GC-1239-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GC-1239-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GC-1239-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GC-1239-4lx/008.jpg</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>GC-1402-4lx</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GC-1402-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GC-1402-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GC-1402-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GC-1402-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GC-1402-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GC-1402-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GC-1402-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GC-1402-4lx/008.jpg,https://oleks-netizen.github.io/product-images/GC-1402-4lx/009.jpg</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>GC-2067-4lx</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GC-2067-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GC-2067-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GC-2067-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GC-2067-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GC-2067-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GC-2067-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GC-2067-4lx/008.jpg,https://oleks-netizen.github.io/product-images/GC-2067-4lx/009.jpg,https://oleks-netizen.github.io/product-images/GC-2067-4lx/010.jpg</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>GC-8033-4lx</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GC-8033-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GC-8033-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GC-8033-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GC-8033-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GC-8033-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GC-8033-4lx/006.jpg</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>GYalc-5565-4lx</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/GYalc-5565-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GYalc-5565-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GYalc-5565-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GYalc-5565-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GYalc-5565-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GYalc-5565-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GYalc-5565-4lx/007.jpg</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>HB0502</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HB0502/001.jpg,https://oleks-netizen.github.io/product-images/HB0502/002.jpg,https://oleks-netizen.github.io/product-images/HB0502/003.jpg,https://oleks-netizen.github.io/product-images/HB0502/005.jpg,https://oleks-netizen.github.io/product-images/HB0502/006.jpg,https://oleks-netizen.github.io/product-images/HB0502/007.jpg</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>HB0502Blu</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HB0502Blu/001.jpg,https://oleks-netizen.github.io/product-images/HB0502Blu/003.jpg,https://oleks-netizen.github.io/product-images/HB0502Blu/004.jpg,https://oleks-netizen.github.io/product-images/HB0502Blu/005.jpg,https://oleks-netizen.github.io/product-images/HB0502Blu/006.jpg,https://oleks-netizen.github.io/product-images/HB0502Blu/007.jpg,https://oleks-netizen.github.io/product-images/HB0502Blu/008.jpg</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>HB19153A</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HB19153A/001.jpg,https://oleks-netizen.github.io/product-images/HB19153A/002.jpg,https://oleks-netizen.github.io/product-images/HB19153A/003.jpg,https://oleks-netizen.github.io/product-images/HB19153A/004.jpg,https://oleks-netizen.github.io/product-images/HB19153A/005.jpg</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>HB3069Asmall</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HB3069Asmall/001.jpg,https://oleks-netizen.github.io/product-images/HB3069Asmall/002.jpg,https://oleks-netizen.github.io/product-images/HB3069Asmall/003.jpg,https://oleks-netizen.github.io/product-images/HB3069Asmall/005.jpg,https://oleks-netizen.github.io/product-images/HB3069Asmall/006.jpg</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>HB3095</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HB3095/001.jpg,https://oleks-netizen.github.io/product-images/HB3095/002.jpg,https://oleks-netizen.github.io/product-images/HB3095/003.jpg,https://oleks-netizen.github.io/product-images/HB3095/004.jpg</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>HB3193A</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HB3193A/001.jpg,https://oleks-netizen.github.io/product-images/HB3193A/002.jpg,https://oleks-netizen.github.io/product-images/HB3193A/004.jpg,https://oleks-netizen.github.io/product-images/HB3193A/005.jpg,https://oleks-netizen.github.io/product-images/HB3193A/006.jpg,https://oleks-netizen.github.io/product-images/HB3193A/007.jpg,https://oleks-netizen.github.io/product-images/HB3193A/008.jpg,https://oleks-netizen.github.io/product-images/HB3193A/009.jpg</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>HB3237B</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HB3237B/001.jpg,https://oleks-netizen.github.io/product-images/HB3237B/002.jpg,https://oleks-netizen.github.io/product-images/HB3237B/003.jpg,https://oleks-netizen.github.io/product-images/HB3237B/004.jpg,https://oleks-netizen.github.io/product-images/HB3237B/005.jpg,https://oleks-netizen.github.io/product-images/HB3237B/006.jpg,https://oleks-netizen.github.io/product-images/HB3237B/007.jpg,https://oleks-netizen.github.io/product-images/HB3237B/008.jpg,https://oleks-netizen.github.io/product-images/HB3237B/009.jpg,https://oleks-netizen.github.io/product-images/HB3237B/010.jpg</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>HB3628R</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HB3628R/001.jpg,https://oleks-netizen.github.io/product-images/HB3628R/002.jpg,https://oleks-netizen.github.io/product-images/HB3628R/004.jpg,https://oleks-netizen.github.io/product-images/HB3628R/005.jpg,https://oleks-netizen.github.io/product-images/HB3628R/006.jpg,https://oleks-netizen.github.io/product-images/HB3628R/007.jpg,https://oleks-netizen.github.io/product-images/HB3628R/008.jpg</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>HF502LN_BR</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF502LN_BR/001.jpg,https://oleks-netizen.github.io/product-images/HF502LN_BR/002.jpg,https://oleks-netizen.github.io/product-images/HF502LN_BR/003.jpg,https://oleks-netizen.github.io/product-images/HF502LN_BR/004.jpg,https://oleks-netizen.github.io/product-images/HF502LN_BR/005.jpg,https://oleks-netizen.github.io/product-images/HF502LN_BR/006.jpg</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>HF502_BU</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF502_BU/001.jpg,https://oleks-netizen.github.io/product-images/HF502_BU/002.jpg,https://oleks-netizen.github.io/product-images/HF502_BU/003.jpg,https://oleks-netizen.github.io/product-images/HF502_BU/004.jpg,https://oleks-netizen.github.io/product-images/HF502_BU/005.jpg,https://oleks-netizen.github.io/product-images/HF502_BU/006.jpg,https://oleks-netizen.github.io/product-images/HF502_BU/007.jpg</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>HF502_CROC-PLN_BRN</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BRN/001.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BRN/002.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BRN/003.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BRN/004.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BRN/005.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BRN/006.jpg</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>HF502_CROC-PLN_BU</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BU/001.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BU/002.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BU/003.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BU/004.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BU/005.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BU/006.jpg,https://oleks-netizen.github.io/product-images/HF502_CROC-PLN_BU/007.jpg</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>HF502_GRN</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF502_GRN/001.jpg,https://oleks-netizen.github.io/product-images/HF502_GRN/002.jpg,https://oleks-netizen.github.io/product-images/HF502_GRN/003.jpg,https://oleks-netizen.github.io/product-images/HF502_GRN/005.jpg,https://oleks-netizen.github.io/product-images/HF502_GRN/006.jpg,https://oleks-netizen.github.io/product-images/HF502_GRN/007.jpg</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>HF577BLL</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF577BLL/001.jpg,https://oleks-netizen.github.io/product-images/HF577BLL/002.jpg,https://oleks-netizen.github.io/product-images/HF577BLL/003.jpg,https://oleks-netizen.github.io/product-images/HF577BLL/004.jpg,https://oleks-netizen.github.io/product-images/HF577BLL/005.jpg,https://oleks-netizen.github.io/product-images/HF577BLL/006.jpg,https://oleks-netizen.github.io/product-images/HF577BLL/007.jpg</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>HF577BN</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF577BN/001.jpg,https://oleks-netizen.github.io/product-images/HF577BN/002.jpg,https://oleks-netizen.github.io/product-images/HF577BN/003.jpg,https://oleks-netizen.github.io/product-images/HF577BN/004.jpg,https://oleks-netizen.github.io/product-images/HF577BN/005.jpg,https://oleks-netizen.github.io/product-images/HF577BN/006.jpg</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>HF577LN_BR</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF577LN_BR/001.jpg,https://oleks-netizen.github.io/product-images/HF577LN_BR/002.jpg,https://oleks-netizen.github.io/product-images/HF577LN_BR/003.jpg,https://oleks-netizen.github.io/product-images/HF577LN_BR/004.jpg,https://oleks-netizen.github.io/product-images/HF577LN_BR/005.jpg,https://oleks-netizen.github.io/product-images/HF577LN_BR/006.jpg</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>HF577_CROC-PLN_BRN</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BRN/001.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BRN/002.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BRN/003.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BRN/004.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BRN/005.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BRN/006.jpg</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>HF577_CROC-PLN_BU</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BU/001.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BU/002.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BU/003.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BU/004.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BU/005.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BU/006.jpg,https://oleks-netizen.github.io/product-images/HF577_CROC-PLN_BU/007.jpg</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>HF577_GRN</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF577_GRN/001.jpg,https://oleks-netizen.github.io/product-images/HF577_GRN/002.jpg,https://oleks-netizen.github.io/product-images/HF577_GRN/003.jpg,https://oleks-netizen.github.io/product-images/HF577_GRN/004.jpg,https://oleks-netizen.github.io/product-images/HF577_GRN/005.jpg,https://oleks-netizen.github.io/product-images/HF577_GRN/006.jpg,https://oleks-netizen.github.io/product-images/HF577_GRN/007.jpg</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>HF592BLK</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF592BLK/001.jpg,https://oleks-netizen.github.io/product-images/HF592BLK/002.jpg,https://oleks-netizen.github.io/product-images/HF592BLK/003.jpg,https://oleks-netizen.github.io/product-images/HF592BLK/004.jpg,https://oleks-netizen.github.io/product-images/HF592BLK/005.jpg</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>HF592BNL</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF592BNL/001.jpg,https://oleks-netizen.github.io/product-images/HF592BNL/002.jpg,https://oleks-netizen.github.io/product-images/HF592BNL/003.jpg,https://oleks-netizen.github.io/product-images/HF592BNL/004.jpg,https://oleks-netizen.github.io/product-images/HF592BNL/005.jpg,https://oleks-netizen.github.io/product-images/HF592BNL/006.jpg</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>HF592LNBR</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF592LNBR/001.jpg,https://oleks-netizen.github.io/product-images/HF592LNBR/002.jpg,https://oleks-netizen.github.io/product-images/HF592LNBR/003.jpg,https://oleks-netizen.github.io/product-images/HF592LNBR/004.jpg,https://oleks-netizen.github.io/product-images/HF592LNBR/005.jpg</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>HF594BL</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF594BL/001.jpg,https://oleks-netizen.github.io/product-images/HF594BL/002.jpg,https://oleks-netizen.github.io/product-images/HF594BL/003.jpg,https://oleks-netizen.github.io/product-images/HF594BL/004.jpg,https://oleks-netizen.github.io/product-images/HF594BL/005.jpg</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>HF594MH</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF594MH/001.jpg,https://oleks-netizen.github.io/product-images/HF594MH/002.jpg,https://oleks-netizen.github.io/product-images/HF594MH/003.jpg,https://oleks-netizen.github.io/product-images/HF594MH/004.jpg,https://oleks-netizen.github.io/product-images/HF594MH/005.jpg</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>HF594_BNL</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF594_BNL/001.jpg,https://oleks-netizen.github.io/product-images/HF594_BNL/002.jpg,https://oleks-netizen.github.io/product-images/HF594_BNL/003.jpg,https://oleks-netizen.github.io/product-images/HF594_BNL/004.jpg,https://oleks-netizen.github.io/product-images/HF594_BNL/005.jpg</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>HF594_GRN</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF594_GRN/001.jpg,https://oleks-netizen.github.io/product-images/HF594_GRN/002.jpg,https://oleks-netizen.github.io/product-images/HF594_GRN/003.jpg,https://oleks-netizen.github.io/product-images/HF594_GRN/004.jpg,https://oleks-netizen.github.io/product-images/HF594_GRN/005.jpg</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>HF595_MTN_BLK</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF595_MTN_BLK/001.jpg,https://oleks-netizen.github.io/product-images/HF595_MTN_BLK/002.jpg,https://oleks-netizen.github.io/product-images/HF595_MTN_BLK/003.jpg,https://oleks-netizen.github.io/product-images/HF595_MTN_BLK/004.jpg,https://oleks-netizen.github.io/product-images/HF595_MTN_BLK/005.jpg,https://oleks-netizen.github.io/product-images/HF595_MTN_BLK/006.jpg</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>HF597_LNBR</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/HF597_LNBR/001.jpg,https://oleks-netizen.github.io/product-images/HF597_LNBR/002.jpg,https://oleks-netizen.github.io/product-images/HF597_LNBR/003.jpg,https://oleks-netizen.github.io/product-images/HF597_LNBR/004.jpg,https://oleks-netizen.github.io/product-images/HF597_LNBR/005.jpg,https://oleks-netizen.github.io/product-images/HF597_LNBR/006.jpg</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>JD6020B</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/JD6020B/001.jpg,https://oleks-netizen.github.io/product-images/JD6020B/002.jpg,https://oleks-netizen.github.io/product-images/JD6020B/003.jpg,https://oleks-netizen.github.io/product-images/JD6020B/004.jpg,https://oleks-netizen.github.io/product-images/JD6020B/005.jpg,https://oleks-netizen.github.io/product-images/JD6020B/006.jpg,https://oleks-netizen.github.io/product-images/JD6020B/007.jpg</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>JD7289A</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/JD7289A/001.jpg,https://oleks-netizen.github.io/product-images/JD7289A/002.jpg,https://oleks-netizen.github.io/product-images/JD7289A/003.jpg,https://oleks-netizen.github.io/product-images/JD7289A/005.jpg,https://oleks-netizen.github.io/product-images/JD7289A/006.jpg,https://oleks-netizen.github.io/product-images/JD7289A/007.jpg,https://oleks-netizen.github.io/product-images/JD7289A/008.jpg,https://oleks-netizen.github.io/product-images/JD7289A/009.jpg,https://oleks-netizen.github.io/product-images/JD7289A/010.jpg,https://oleks-netizen.github.io/product-images/JD7289A/011.jpg</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>K1617f-black</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K1617f-black/001.jpg,https://oleks-netizen.github.io/product-images/K1617f-black/002.jpg,https://oleks-netizen.github.io/product-images/K1617f-black/004.jpg,https://oleks-netizen.github.io/product-images/K1617f-black/005.jpg,https://oleks-netizen.github.io/product-images/K1617f-black/006.jpg</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>L28001-1</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28001-1/001.jpg,https://oleks-netizen.github.io/product-images/L28001-1/003.jpg,https://oleks-netizen.github.io/product-images/L28001-1/004.jpg,https://oleks-netizen.github.io/product-images/L28001-1/005.jpg,https://oleks-netizen.github.io/product-images/L28001-1/006.jpg,https://oleks-netizen.github.io/product-images/L28001-1/007.jpg,https://oleks-netizen.github.io/product-images/L28001-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>L28001-2</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28001-2/001.jpg,https://oleks-netizen.github.io/product-images/L28001-2/003.jpg,https://oleks-netizen.github.io/product-images/L28001-2/004.jpg,https://oleks-netizen.github.io/product-images/L28001-2/005.jpg,https://oleks-netizen.github.io/product-images/L28001-2/006.jpg,https://oleks-netizen.github.io/product-images/L28001-2/007.jpg</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>L28001-3</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28001-3/001.jpg,https://oleks-netizen.github.io/product-images/L28001-3/003.jpg,https://oleks-netizen.github.io/product-images/L28001-3/004.jpg,https://oleks-netizen.github.io/product-images/L28001-3/005.jpg,https://oleks-netizen.github.io/product-images/L28001-3/006.jpg,https://oleks-netizen.github.io/product-images/L28001-3/007.jpg</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>L28001-4</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28001-4/001.jpg,https://oleks-netizen.github.io/product-images/L28001-4/003.jpg,https://oleks-netizen.github.io/product-images/L28001-4/004.jpg,https://oleks-netizen.github.io/product-images/L28001-4/005.jpg,https://oleks-netizen.github.io/product-images/L28001-4/006.jpg,https://oleks-netizen.github.io/product-images/L28001-4/007.jpg,https://oleks-netizen.github.io/product-images/L28001-4/008.jpg</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>L28028-1</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28028-1/001.jpg,https://oleks-netizen.github.io/product-images/L28028-1/003.jpg,https://oleks-netizen.github.io/product-images/L28028-1/004.jpg,https://oleks-netizen.github.io/product-images/L28028-1/005.jpg,https://oleks-netizen.github.io/product-images/L28028-1/006.jpg,https://oleks-netizen.github.io/product-images/L28028-1/007.jpg,https://oleks-netizen.github.io/product-images/L28028-1/008.jpg,https://oleks-netizen.github.io/product-images/L28028-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>L28028-2</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28028-2/001.jpg,https://oleks-netizen.github.io/product-images/L28028-2/003.jpg,https://oleks-netizen.github.io/product-images/L28028-2/004.jpg,https://oleks-netizen.github.io/product-images/L28028-2/005.jpg,https://oleks-netizen.github.io/product-images/L28028-2/006.jpg,https://oleks-netizen.github.io/product-images/L28028-2/007.jpg,https://oleks-netizen.github.io/product-images/L28028-2/008.jpg,https://oleks-netizen.github.io/product-images/L28028-2/009.jpg</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>L28028-3</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28028-3/001.jpg,https://oleks-netizen.github.io/product-images/L28028-3/003.jpg,https://oleks-netizen.github.io/product-images/L28028-3/004.jpg,https://oleks-netizen.github.io/product-images/L28028-3/005.jpg,https://oleks-netizen.github.io/product-images/L28028-3/006.jpg,https://oleks-netizen.github.io/product-images/L28028-3/007.jpg,https://oleks-netizen.github.io/product-images/L28028-3/008.jpg,https://oleks-netizen.github.io/product-images/L28028-3/009.jpg</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>L28029-1</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28029-1/001.jpg,https://oleks-netizen.github.io/product-images/L28029-1/003.jpg,https://oleks-netizen.github.io/product-images/L28029-1/004.jpg,https://oleks-netizen.github.io/product-images/L28029-1/005.jpg,https://oleks-netizen.github.io/product-images/L28029-1/006.jpg,https://oleks-netizen.github.io/product-images/L28029-1/007.jpg,https://oleks-netizen.github.io/product-images/L28029-1/008.jpg,https://oleks-netizen.github.io/product-images/L28029-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>L28029-2</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28029-2/001.jpg,https://oleks-netizen.github.io/product-images/L28029-2/003.jpg,https://oleks-netizen.github.io/product-images/L28029-2/004.jpg,https://oleks-netizen.github.io/product-images/L28029-2/005.jpg,https://oleks-netizen.github.io/product-images/L28029-2/006.jpg,https://oleks-netizen.github.io/product-images/L28029-2/007.jpg,https://oleks-netizen.github.io/product-images/L28029-2/008.jpg,https://oleks-netizen.github.io/product-images/L28029-2/009.jpg</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>L28029-3</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28029-3/001.jpg,https://oleks-netizen.github.io/product-images/L28029-3/003.jpg,https://oleks-netizen.github.io/product-images/L28029-3/004.jpg,https://oleks-netizen.github.io/product-images/L28029-3/005.jpg,https://oleks-netizen.github.io/product-images/L28029-3/006.jpg,https://oleks-netizen.github.io/product-images/L28029-3/007.jpg,https://oleks-netizen.github.io/product-images/L28029-3/008.jpg,https://oleks-netizen.github.io/product-images/L28029-3/009.jpg</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>L28029-4</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28029-4/001.jpg,https://oleks-netizen.github.io/product-images/L28029-4/002.jpg,https://oleks-netizen.github.io/product-images/L28029-4/004.jpg,https://oleks-netizen.github.io/product-images/L28029-4/005.jpg,https://oleks-netizen.github.io/product-images/L28029-4/006.jpg,https://oleks-netizen.github.io/product-images/L28029-4/007.jpg,https://oleks-netizen.github.io/product-images/L28029-4/008.jpg,https://oleks-netizen.github.io/product-images/L28029-4/009.jpg</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>L501-041857</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L501-041857/001.jpg,https://oleks-netizen.github.io/product-images/L501-041857/002.jpg,https://oleks-netizen.github.io/product-images/L501-041857/003.jpg,https://oleks-netizen.github.io/product-images/L501-041857/004.jpg,https://oleks-netizen.github.io/product-images/L501-041857/005.jpg</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>L501-042014</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L501-042014/001.jpg,https://oleks-netizen.github.io/product-images/L501-042014/002.jpg,https://oleks-netizen.github.io/product-images/L501-042014/003.jpg,https://oleks-netizen.github.io/product-images/L501-042014/004.jpg,https://oleks-netizen.github.io/product-images/L501-042014/005.jpg,https://oleks-netizen.github.io/product-images/L501-042014/006.jpg,https://oleks-netizen.github.io/product-images/L501-042014/007.jpg</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>L501-042021</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L501-042021/001.jpg,https://oleks-netizen.github.io/product-images/L501-042021/002.jpg,https://oleks-netizen.github.io/product-images/L501-042021/003.jpg,https://oleks-netizen.github.io/product-images/L501-042021/004.jpg,https://oleks-netizen.github.io/product-images/L501-042021/005.jpg,https://oleks-netizen.github.io/product-images/L501-042021/006.jpg,https://oleks-netizen.github.io/product-images/L501-042021/007.jpg,https://oleks-netizen.github.io/product-images/L501-042021/008.jpg</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>L501-042038</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L501-042038/001.jpg,https://oleks-netizen.github.io/product-images/L501-042038/002.jpg,https://oleks-netizen.github.io/product-images/L501-042038/003.jpg,https://oleks-netizen.github.io/product-images/L501-042038/004.jpg,https://oleks-netizen.github.io/product-images/L501-042038/005.jpg,https://oleks-netizen.github.io/product-images/L501-042038/006.jpg,https://oleks-netizen.github.io/product-images/L501-042038/007.jpg</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>L87229-1</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87229-1/001.jpg,https://oleks-netizen.github.io/product-images/L87229-1/002.jpg,https://oleks-netizen.github.io/product-images/L87229-1/003.jpg,https://oleks-netizen.github.io/product-images/L87229-1/004.jpg,https://oleks-netizen.github.io/product-images/L87229-1/005.jpg,https://oleks-netizen.github.io/product-images/L87229-1/006.jpg,https://oleks-netizen.github.io/product-images/L87229-1/007.jpg,https://oleks-netizen.github.io/product-images/L87229-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>L88003-32</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L88003-32/001.jpg,https://oleks-netizen.github.io/product-images/L88003-32/003.jpg,https://oleks-netizen.github.io/product-images/L88003-32/004.jpg,https://oleks-netizen.github.io/product-images/L88003-32/005.jpg,https://oleks-netizen.github.io/product-images/L88003-32/006.jpg,https://oleks-netizen.github.io/product-images/L88003-32/007.jpg,https://oleks-netizen.github.io/product-images/L88003-32/008.jpg</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>LC47208K-1</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47208K-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1/003.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1/005.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1/006.jpg</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>LC47208K-1X</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47208K-1X/001.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1X/002.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1X/003.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1X/004.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1X/005.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1X/006.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1X/007.jpg,https://oleks-netizen.github.io/product-images/LC47208K-1X/008.jpg</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>LC47208K-92</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47208K-92/001.jpg,https://oleks-netizen.github.io/product-images/LC47208K-92/002.jpg,https://oleks-netizen.github.io/product-images/LC47208K-92/003.jpg,https://oleks-netizen.github.io/product-images/LC47208K-92/004.jpg,https://oleks-netizen.github.io/product-images/LC47208K-92/005.jpg,https://oleks-netizen.github.io/product-images/LC47208K-92/006.jpg</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>LC47210-1</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47210-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47210-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47210-1/003.jpg,https://oleks-netizen.github.io/product-images/LC47210-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47210-1/005.jpg</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>LC47210-1X</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47210-1X/001.jpg,https://oleks-netizen.github.io/product-images/LC47210-1X/002.jpg,https://oleks-netizen.github.io/product-images/LC47210-1X/003.jpg,https://oleks-netizen.github.io/product-images/LC47210-1X/004.jpg,https://oleks-netizen.github.io/product-images/LC47210-1X/005.jpg,https://oleks-netizen.github.io/product-images/LC47210-1X/006.jpg</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>LC47210-92</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47210-92/001.jpg,https://oleks-netizen.github.io/product-images/LC47210-92/002.jpg,https://oleks-netizen.github.io/product-images/LC47210-92/003.jpg,https://oleks-netizen.github.io/product-images/LC47210-92/004.jpg,https://oleks-netizen.github.io/product-images/LC47210-92/005.jpg,https://oleks-netizen.github.io/product-images/LC47210-92/006.jpg,https://oleks-netizen.github.io/product-images/LC47210-92/007.jpg</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>LC47240W-1</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47240W-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47240W-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47240W-1/003.jpg,https://oleks-netizen.github.io/product-images/LC47240W-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47240W-1/005.jpg,https://oleks-netizen.github.io/product-images/LC47240W-1/006.jpg</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>LC47240W-1X</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47240W-1X/001.jpg,https://oleks-netizen.github.io/product-images/LC47240W-1X/002.jpg,https://oleks-netizen.github.io/product-images/LC47240W-1X/003.jpg,https://oleks-netizen.github.io/product-images/LC47240W-1X/004.jpg,https://oleks-netizen.github.io/product-images/LC47240W-1X/005.jpg,https://oleks-netizen.github.io/product-images/LC47240W-1X/006.jpg</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>LC47240W-92</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47240W-92/001.jpg,https://oleks-netizen.github.io/product-images/LC47240W-92/002.jpg,https://oleks-netizen.github.io/product-images/LC47240W-92/003.jpg,https://oleks-netizen.github.io/product-images/LC47240W-92/004.jpg,https://oleks-netizen.github.io/product-images/LC47240W-92/005.jpg,https://oleks-netizen.github.io/product-images/LC47240W-92/006.jpg,https://oleks-netizen.github.io/product-images/LC47240W-92/007.jpg</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>LC47539-1</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47539-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47539-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47539-1/003.jpg,https://oleks-netizen.github.io/product-images/LC47539-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47539-1/005.jpg</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>LC47539-92</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47539-92/001.jpg,https://oleks-netizen.github.io/product-images/LC47539-92/002.jpg,https://oleks-netizen.github.io/product-images/LC47539-92/003.jpg,https://oleks-netizen.github.io/product-images/LC47539-92/004.jpg,https://oleks-netizen.github.io/product-images/LC47539-92/005.jpg,https://oleks-netizen.github.io/product-images/LC47539-92/006.jpg,https://oleks-netizen.github.io/product-images/LC47539-92/007.jpg</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>LC47632F-1</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47632F-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1/003.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1/006.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>LC47632F-92</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47632F-92/001.jpg,https://oleks-netizen.github.io/product-images/LC47632F-92/002.jpg,https://oleks-netizen.github.io/product-images/LC47632F-92/003.jpg,https://oleks-netizen.github.io/product-images/LC47632F-92/004.jpg,https://oleks-netizen.github.io/product-images/LC47632F-92/005.jpg,https://oleks-netizen.github.io/product-images/LC47632F-92/006.jpg,https://oleks-netizen.github.io/product-images/LC47632F-92/007.jpg</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>LC47695-1</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47695-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47695-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47695-1/003.jpg,https://oleks-netizen.github.io/product-images/LC47695-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47695-1/005.jpg,https://oleks-netizen.github.io/product-images/LC47695-1/006.jpg,https://oleks-netizen.github.io/product-images/LC47695-1/007.jpg,https://oleks-netizen.github.io/product-images/LC47695-1/008.jpg,https://oleks-netizen.github.io/product-images/LC47695-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>LC47832-1</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47832-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47832-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47832-1/003.jpg,https://oleks-netizen.github.io/product-images/LC47832-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47832-1/005.jpg,https://oleks-netizen.github.io/product-images/LC47832-1/006.jpg,https://oleks-netizen.github.io/product-images/LC47832-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>LC47832-92</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47832-92/001.jpg,https://oleks-netizen.github.io/product-images/LC47832-92/002.jpg,https://oleks-netizen.github.io/product-images/LC47832-92/003.jpg,https://oleks-netizen.github.io/product-images/LC47832-92/004.jpg,https://oleks-netizen.github.io/product-images/LC47832-92/005.jpg,https://oleks-netizen.github.io/product-images/LC47832-92/006.jpg,https://oleks-netizen.github.io/product-images/LC47832-92/007.jpg</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>LC47891-1</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47891-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47891-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47891-1/003.jpg,https://oleks-netizen.github.io/product-images/LC47891-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47891-1/005.jpg,https://oleks-netizen.github.io/product-images/LC47891-1/006.jpg</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>LC47891-92</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47891-92/001.jpg,https://oleks-netizen.github.io/product-images/LC47891-92/002.jpg,https://oleks-netizen.github.io/product-images/LC47891-92/003.jpg,https://oleks-netizen.github.io/product-images/LC47891-92/004.jpg,https://oleks-netizen.github.io/product-images/LC47891-92/005.jpg,https://oleks-netizen.github.io/product-images/LC47891-92/006.jpg,https://oleks-netizen.github.io/product-images/LC47891-92/007.jpg</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>LC47991-1A</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47991-1A/001.jpg,https://oleks-netizen.github.io/product-images/LC47991-1A/002.jpg,https://oleks-netizen.github.io/product-images/LC47991-1A/003.jpg,https://oleks-netizen.github.io/product-images/LC47991-1A/004.jpg,https://oleks-netizen.github.io/product-images/LC47991-1A/005.jpg</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>LC47991-92</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC47991-92/001.jpg,https://oleks-netizen.github.io/product-images/LC47991-92/002.jpg,https://oleks-netizen.github.io/product-images/LC47991-92/003.jpg,https://oleks-netizen.github.io/product-images/LC47991-92/004.jpg,https://oleks-netizen.github.io/product-images/LC47991-92/005.jpg,https://oleks-netizen.github.io/product-images/LC47991-92/006.jpg,https://oleks-netizen.github.io/product-images/LC47991-92/007.jpg</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Lim-181GA</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/Lim-181GA/001.jpg,https://oleks-netizen.github.io/product-images/Lim-181GA/002.jpg,https://oleks-netizen.github.io/product-images/Lim-181GA/003.jpg,https://oleks-netizen.github.io/product-images/Lim-181GA/005.jpg,https://oleks-netizen.github.io/product-images/Lim-181GA/006.jpg,https://oleks-netizen.github.io/product-images/Lim-181GA/007.jpg,https://oleks-netizen.github.io/product-images/Lim-181GA/008.jpg</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>lim-22-115</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/lim-22-115/001.jpg,https://oleks-netizen.github.io/product-images/lim-22-115/002.jpg,https://oleks-netizen.github.io/product-images/lim-22-115/003.jpg,https://oleks-netizen.github.io/product-images/lim-22-115/004.jpg</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>lim-28-115</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/lim-28-115/001.jpg,https://oleks-netizen.github.io/product-images/lim-28-115/002.jpg,https://oleks-netizen.github.io/product-images/lim-28-115/003.jpg,https://oleks-netizen.github.io/product-images/lim-28-115/004.jpg</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Lim-372RC</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/Lim-372RC/001.jpg,https://oleks-netizen.github.io/product-images/Lim-372RC/002.jpg,https://oleks-netizen.github.io/product-images/Lim-372RC/003.jpg,https://oleks-netizen.github.io/product-images/Lim-372RC/005.jpg,https://oleks-netizen.github.io/product-images/Lim-372RC/006.jpg,https://oleks-netizen.github.io/product-images/Lim-372RC/007.jpg,https://oleks-netizen.github.io/product-images/Lim-372RC/008.jpg</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>PH601BR</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/PH601BR/001.jpg,https://oleks-netizen.github.io/product-images/PH601BR/002.jpg,https://oleks-netizen.github.io/product-images/PH601BR/003.jpg,https://oleks-netizen.github.io/product-images/PH601BR/004.jpg,https://oleks-netizen.github.io/product-images/PH601BR/005.jpg</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>PH601_BLK</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/PH601_BLK/001.jpg,https://oleks-netizen.github.io/product-images/PH601_BLK/002.jpg,https://oleks-netizen.github.io/product-images/PH601_BLK/003.jpg,https://oleks-netizen.github.io/product-images/PH601_BLK/004.jpg,https://oleks-netizen.github.io/product-images/PH601_BLK/005.jpg,https://oleks-netizen.github.io/product-images/PH601_BLK/006.jpg,https://oleks-netizen.github.io/product-images/PH601_BLK/007.jpg</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>PH602TAN</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/PH602TAN/001.jpg,https://oleks-netizen.github.io/product-images/PH602TAN/002.jpg,https://oleks-netizen.github.io/product-images/PH602TAN/003.jpg,https://oleks-netizen.github.io/product-images/PH602TAN/004.jpg,https://oleks-netizen.github.io/product-images/PH602TAN/005.jpg,https://oleks-netizen.github.io/product-images/PH602TAN/006.jpg,https://oleks-netizen.github.io/product-images/PH602TAN/007.jpg</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>PH602_CROC-PLN_BRN</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/PH602_CROC-PLN_BRN/001.jpg,https://oleks-netizen.github.io/product-images/PH602_CROC-PLN_BRN/002.jpg,https://oleks-netizen.github.io/product-images/PH602_CROC-PLN_BRN/003.jpg,https://oleks-netizen.github.io/product-images/PH602_CROC-PLN_BRN/004.jpg,https://oleks-netizen.github.io/product-images/PH602_CROC-PLN_BRN/005.jpg,https://oleks-netizen.github.io/product-images/PH602_CROC-PLN_BRN/006.jpg</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>PH602_GRN</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/PH602_GRN/001.jpg,https://oleks-netizen.github.io/product-images/PH602_GRN/002.jpg,https://oleks-netizen.github.io/product-images/PH602_GRN/003.jpg,https://oleks-netizen.github.io/product-images/PH602_GRN/004.jpg,https://oleks-netizen.github.io/product-images/PH602_GRN/005.jpg</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>RA-1046-3md</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RA-1046-3md/001.jpg,https://oleks-netizen.github.io/product-images/RA-1046-3md/002.jpg,https://oleks-netizen.github.io/product-images/RA-1046-3md/003.jpg,https://oleks-netizen.github.io/product-images/RA-1046-3md/005.jpg,https://oleks-netizen.github.io/product-images/RA-1046-3md/006.jpg,https://oleks-netizen.github.io/product-images/RA-1046-3md/007.jpg,https://oleks-netizen.github.io/product-images/RA-1046-3md/008.jpg,https://oleks-netizen.github.io/product-images/RA-1046-3md/009.jpg</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>RA-1342-3md</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RA-1342-3md/001.jpg,https://oleks-netizen.github.io/product-images/RA-1342-3md/002.jpg,https://oleks-netizen.github.io/product-images/RA-1342-3md/003.jpg,https://oleks-netizen.github.io/product-images/RA-1342-3md/004.jpg,https://oleks-netizen.github.io/product-images/RA-1342-3md/005.jpg</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>RA-1403-4lx</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RA-1403-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RA-1403-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RA-1403-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RA-1403-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RA-1403-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RA-1403-4lx/006.jpg</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>RA-1501-3md</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RA-1501-3md/001.jpg,https://oleks-netizen.github.io/product-images/RA-1501-3md/002.jpg,https://oleks-netizen.github.io/product-images/RA-1501-3md/003.jpg,https://oleks-netizen.github.io/product-images/RA-1501-3md/004.jpg,https://oleks-netizen.github.io/product-images/RA-1501-3md/005.jpg,https://oleks-netizen.github.io/product-images/RA-1501-3md/006.jpg,https://oleks-netizen.github.io/product-images/RA-1501-3md/007.jpg</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>RA-7122-3md</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RA-7122-3md/001.jpg,https://oleks-netizen.github.io/product-images/RA-7122-3md/002.jpg,https://oleks-netizen.github.io/product-images/RA-7122-3md/003.jpg,https://oleks-netizen.github.io/product-images/RA-7122-3md/004.jpg,https://oleks-netizen.github.io/product-images/RA-7122-3md/005.jpg,https://oleks-netizen.github.io/product-images/RA-7122-3md/006.jpg</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>RAc-6690-4lx</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RAc-6690-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RAc-6690-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RAc-6690-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RAc-6690-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RAc-6690-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RAc-6690-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RAc-6690-4lx/008.jpg</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>RAg-1905-3md</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RAg-1905-3md/001.jpg,https://oleks-netizen.github.io/product-images/RAg-1905-3md/002.jpg,https://oleks-netizen.github.io/product-images/RAg-1905-3md/003.jpg,https://oleks-netizen.github.io/product-images/RAg-1905-3md/004.jpg,https://oleks-netizen.github.io/product-images/RAg-1905-3md/006.jpg,https://oleks-netizen.github.io/product-images/RAg-1905-3md/007.jpg,https://oleks-netizen.github.io/product-images/RAg-1905-3md/008.jpg</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>RB-2200RL-4lx</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RB-2200RL-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RB-2200RL-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RB-2200RL-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RB-2200RL-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RB-2200RL-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RB-2200RL-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RB-2200RL-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RB-2200RL-4lx/008.jpg,https://oleks-netizen.github.io/product-images/RB-2200RL-4lx/009.jpg,https://oleks-netizen.github.io/product-images/RB-2200RL-4lx/010.jpg</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>RB-3960-4lx</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RB-3960-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RB-3960-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RB-3960-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RB-3960-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RB-3960-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RB-3960-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RB-3960-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RB-3960-4lx/008.jpg,https://oleks-netizen.github.io/product-images/RB-3960-4lx/009.jpg</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>RB-7122-3mdL</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RB-7122-3mdL/001.jpg,https://oleks-netizen.github.io/product-images/RB-7122-3mdL/002.jpg,https://oleks-netizen.github.io/product-images/RB-7122-3mdL/003.jpg,https://oleks-netizen.github.io/product-images/RB-7122-3mdL/004.jpg,https://oleks-netizen.github.io/product-images/RB-7122-3mdL/005.jpg,https://oleks-netizen.github.io/product-images/RB-7122-3mdL/006.jpg,https://oleks-netizen.github.io/product-images/RB-7122-3mdL/007.jpg,https://oleks-netizen.github.io/product-images/RB-7122-3mdL/008.jpg,https://oleks-netizen.github.io/product-images/RB-7122-3mdL/009.jpg</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>RB-7340-3md</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RB-7340-3md/001.jpg,https://oleks-netizen.github.io/product-images/RB-7340-3md/002.jpg,https://oleks-netizen.github.io/product-images/RB-7340-3md/003.jpg,https://oleks-netizen.github.io/product-images/RB-7340-3md/004.jpg,https://oleks-netizen.github.io/product-images/RB-7340-3md/006.jpg,https://oleks-netizen.github.io/product-images/RB-7340-3md/007.jpg,https://oleks-netizen.github.io/product-images/RB-7340-3md/008.jpg,https://oleks-netizen.github.io/product-images/RB-7340-3md/009.jpg,https://oleks-netizen.github.io/product-images/RB-7340-3md/010.jpg,https://oleks-netizen.github.io/product-images/RB-7340-3md/011.jpg</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>RC-2200RL-4lx</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RC-2200RL-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RC-2200RL-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RC-2200RL-4lx/003.jpg</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>RC-60121-3md</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RC-60121-3md/001.jpg,https://oleks-netizen.github.io/product-images/RC-60121-3md/002.jpg,https://oleks-netizen.github.io/product-images/RC-60121-3md/003.jpg,https://oleks-netizen.github.io/product-images/RC-60121-3md/004.jpg,https://oleks-netizen.github.io/product-images/RC-60121-3md/005.jpg,https://oleks-netizen.github.io/product-images/RC-60121-3md/006.jpg,https://oleks-netizen.github.io/product-images/RC-60121-3md/007.jpg,https://oleks-netizen.github.io/product-images/RC-60121-3md/008.jpg</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>RC-7122-3mdL</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RC-7122-3mdL/001.jpg,https://oleks-netizen.github.io/product-images/RC-7122-3mdL/003.jpg,https://oleks-netizen.github.io/product-images/RC-7122-3mdL/004.jpg,https://oleks-netizen.github.io/product-images/RC-7122-3mdL/005.jpg,https://oleks-netizen.github.io/product-images/RC-7122-3mdL/006.jpg,https://oleks-netizen.github.io/product-images/RC-7122-3mdL/007.jpg</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>RC-7290-3md</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RC-7290-3md/001.jpg,https://oleks-netizen.github.io/product-images/RC-7290-3md/003.jpg,https://oleks-netizen.github.io/product-images/RC-7290-3md/004.jpg,https://oleks-netizen.github.io/product-images/RC-7290-3md/005.jpg,https://oleks-netizen.github.io/product-images/RC-7290-3md/006.jpg,https://oleks-netizen.github.io/product-images/RC-7290-3md/007.jpg,https://oleks-netizen.github.io/product-images/RC-7290-3md/008.jpg,https://oleks-netizen.github.io/product-images/RC-7290-3md/009.jpg</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>RC-7340-3md</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RC-7340-3md/001.jpg,https://oleks-netizen.github.io/product-images/RC-7340-3md/002.jpg,https://oleks-netizen.github.io/product-images/RC-7340-3md/003.jpg,https://oleks-netizen.github.io/product-images/RC-7340-3md/004.jpg,https://oleks-netizen.github.io/product-images/RC-7340-3md/005.jpg,https://oleks-netizen.github.io/product-images/RC-7340-3md/007.jpg,https://oleks-netizen.github.io/product-images/RC-7340-3md/008.jpg,https://oleks-netizen.github.io/product-images/RC-7340-3md/009.jpg,https://oleks-netizen.github.io/product-images/RC-7340-3md/010.jpg,https://oleks-netizen.github.io/product-images/RC-7340-3md/011.jpg</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>RCc-1905-3md</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RCc-1905-3md/001.jpg,https://oleks-netizen.github.io/product-images/RCc-1905-3md/002.jpg,https://oleks-netizen.github.io/product-images/RCc-1905-3md/004.jpg,https://oleks-netizen.github.io/product-images/RCc-1905-3md/005.jpg,https://oleks-netizen.github.io/product-images/RCc-1905-3md/006.jpg,https://oleks-netizen.github.io/product-images/RCc-1905-3md/007.jpg</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>RCC-3920-3md</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RCC-3920-3md/001.jpg,https://oleks-netizen.github.io/product-images/RCC-3920-3md/002.jpg,https://oleks-netizen.github.io/product-images/RCC-3920-3md/003.jpg,https://oleks-netizen.github.io/product-images/RCC-3920-3md/004.jpg,https://oleks-netizen.github.io/product-images/RCC-3920-3md/005.jpg,https://oleks-netizen.github.io/product-images/RCC-3920-3md/006.jpg,https://oleks-netizen.github.io/product-images/RCC-3920-3md/007.jpg,https://oleks-netizen.github.io/product-images/RCC-3920-3md/008.jpg,https://oleks-netizen.github.io/product-images/RCC-3920-3md/009.jpg</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>RCc-6600-3md</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RCc-6600-3md/001.jpg,https://oleks-netizen.github.io/product-images/RCc-6600-3md/002.jpg,https://oleks-netizen.github.io/product-images/RCc-6600-3md/003.jpg,https://oleks-netizen.github.io/product-images/RCc-6600-3md/004.jpg,https://oleks-netizen.github.io/product-images/RCc-6600-3md/006.jpg,https://oleks-netizen.github.io/product-images/RCc-6600-3md/007.jpg,https://oleks-netizen.github.io/product-images/RCc-6600-3md/008.jpg,https://oleks-netizen.github.io/product-images/RCc-6600-3md/009.jpg</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>RCk-3420-3md</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RCk-3420-3md/001.jpg,https://oleks-netizen.github.io/product-images/RCk-3420-3md/002.jpg,https://oleks-netizen.github.io/product-images/RCk-3420-3md/003.jpg,https://oleks-netizen.github.io/product-images/RCk-3420-3md/004.jpg,https://oleks-netizen.github.io/product-images/RCk-3420-3md/005.jpg,https://oleks-netizen.github.io/product-images/RCk-3420-3md/006.jpg,https://oleks-netizen.github.io/product-images/RCk-3420-3md/007.jpg,https://oleks-netizen.github.io/product-images/RCk-3420-3md/008.jpg</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>RCs-1905-3md</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RCs-1905-3md/001.jpg,https://oleks-netizen.github.io/product-images/RCs-1905-3md/002.jpg,https://oleks-netizen.github.io/product-images/RCs-1905-3md/003.jpg,https://oleks-netizen.github.io/product-images/RCs-1905-3md/004.jpg,https://oleks-netizen.github.io/product-images/RCs-1905-3md/006.jpg,https://oleks-netizen.github.io/product-images/RCs-1905-3md/007.jpg,https://oleks-netizen.github.io/product-images/RCs-1905-3md/008.jpg,https://oleks-netizen.github.io/product-images/RCs-1905-3md/009.jpg</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>RE-1342-3md</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RE-1342-3md/001.jpg,https://oleks-netizen.github.io/product-images/RE-1342-3md/002.jpg,https://oleks-netizen.github.io/product-images/RE-1342-3md/004.jpg,https://oleks-netizen.github.io/product-images/RE-1342-3md/005.jpg,https://oleks-netizen.github.io/product-images/RE-1342-3md/006.jpg</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>RE-30272-3md</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RE-30272-3md/001.jpg,https://oleks-netizen.github.io/product-images/RE-30272-3md/002.jpg,https://oleks-netizen.github.io/product-images/RE-30272-3md/003.jpg,https://oleks-netizen.github.io/product-images/RE-30272-3md/004.jpg,https://oleks-netizen.github.io/product-images/RE-30272-3md/006.jpg,https://oleks-netizen.github.io/product-images/RE-30272-3md/007.jpg,https://oleks-netizen.github.io/product-images/RE-30272-3md/008.jpg,https://oleks-netizen.github.io/product-images/RE-30272-3md/009.jpg,https://oleks-netizen.github.io/product-images/RE-30272-3md/010.jpg</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>RK-1342-3md</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RK-1342-3md/001.jpg,https://oleks-netizen.github.io/product-images/RK-1342-3md/002.jpg,https://oleks-netizen.github.io/product-images/RK-1342-3md/004.jpg,https://oleks-netizen.github.io/product-images/RK-1342-3md/005.jpg,https://oleks-netizen.github.io/product-images/RK-1342-3md/006.jpg</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>RK-7122-3md</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RK-7122-3md/001.jpg,https://oleks-netizen.github.io/product-images/RK-7122-3md/002.jpg,https://oleks-netizen.github.io/product-images/RK-7122-3md/003.jpg,https://oleks-netizen.github.io/product-images/RK-7122-3md/004.jpg,https://oleks-netizen.github.io/product-images/RK-7122-3md/005.jpg,https://oleks-netizen.github.io/product-images/RK-7122-3md/006.jpg</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>RYw-3027-4lx</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RYw-3027-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RYw-3027-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RYw-3027-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RYw-3027-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RYw-3027-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RYw-3027-4lx/006.jpg</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>RА-3990-3md</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RА-3990-3md/001.jpg,https://oleks-netizen.github.io/product-images/RА-3990-3md/002.jpg,https://oleks-netizen.github.io/product-images/RА-3990-3md/004.jpg,https://oleks-netizen.github.io/product-images/RА-3990-3md/005.jpg,https://oleks-netizen.github.io/product-images/RА-3990-3md/006.jpg,https://oleks-netizen.github.io/product-images/RА-3990-3md/007.jpg,https://oleks-netizen.github.io/product-images/RА-3990-3md/008.jpg,https://oleks-netizen.github.io/product-images/RА-3990-3md/009.jpg,https://oleks-netizen.github.io/product-images/RА-3990-3md/010.jpg</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>RС-1342-3md</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RС-1342-3md/001.jpg,https://oleks-netizen.github.io/product-images/RС-1342-3md/002.jpg,https://oleks-netizen.github.io/product-images/RС-1342-3md/003.jpg,https://oleks-netizen.github.io/product-images/RС-1342-3md/004.jpg,https://oleks-netizen.github.io/product-images/RС-1342-3md/005.jpg</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>SB1164BRN</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/SB1164BRN/001.jpg,https://oleks-netizen.github.io/product-images/SB1164BRN/002.jpg,https://oleks-netizen.github.io/product-images/SB1164BRN/004.jpg,https://oleks-netizen.github.io/product-images/SB1164BRN/005.jpg,https://oleks-netizen.github.io/product-images/SB1164BRN/006.jpg,https://oleks-netizen.github.io/product-images/SB1164BRN/007.jpg</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>T0138А</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/T0138А/001.jpg,https://oleks-netizen.github.io/product-images/T0138А/002.jpg,https://oleks-netizen.github.io/product-images/T0138А/004.jpg</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>TA-0042-4lx</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TA-0042-4lx/001.jpg,https://oleks-netizen.github.io/product-images/TA-0042-4lx/002.jpg,https://oleks-netizen.github.io/product-images/TA-0042-4lx/004.jpg,https://oleks-netizen.github.io/product-images/TA-0042-4lx/005.jpg,https://oleks-netizen.github.io/product-images/TA-0042-4lx/006.jpg,https://oleks-netizen.github.io/product-images/TA-0042-4lx/007.jpg,https://oleks-netizen.github.io/product-images/TA-0042-4lx/008.jpg</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>TA-5664-4lx</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TA-5664-4lx/001.jpg,https://oleks-netizen.github.io/product-images/TA-5664-4lx/002.jpg,https://oleks-netizen.github.io/product-images/TA-5664-4lx/003.jpg,https://oleks-netizen.github.io/product-images/TA-5664-4lx/004.jpg,https://oleks-netizen.github.io/product-images/TA-5664-4lx/005.jpg,https://oleks-netizen.github.io/product-images/TA-5664-4lx/006.jpg,https://oleks-netizen.github.io/product-images/TA-5664-4lx/007.jpg,https://oleks-netizen.github.io/product-images/TA-5664-4lx/008.jpg</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>TC4002 MH</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TC4002 MH/001.jpg,https://oleks-netizen.github.io/product-images/TC4002 MH/002.jpg,https://oleks-netizen.github.io/product-images/TC4002 MH/003.jpg,https://oleks-netizen.github.io/product-images/TC4002 MH/004.jpg,https://oleks-netizen.github.io/product-images/TC4002 MH/005.jpg,https://oleks-netizen.github.io/product-images/TC4002 MH/006.jpg,https://oleks-netizen.github.io/product-images/TC4002 MH/008.jpg,https://oleks-netizen.github.io/product-images/TC4002 MH/009.jpg,https://oleks-netizen.github.io/product-images/TC4002 MH/010.jpg</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>TC4003_BU</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TC4003_BU/001.jpg,https://oleks-netizen.github.io/product-images/TC4003_BU/002.jpg,https://oleks-netizen.github.io/product-images/TC4003_BU/003.jpg,https://oleks-netizen.github.io/product-images/TC4003_BU/004.jpg,https://oleks-netizen.github.io/product-images/TC4003_BU/005.jpg,https://oleks-netizen.github.io/product-images/TC4003_BU/006.jpg,https://oleks-netizen.github.io/product-images/TC4003_BU/008.jpg,https://oleks-netizen.github.io/product-images/TC4003_BU/009.jpg</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>TC4004BR</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TC4004BR/001.jpg,https://oleks-netizen.github.io/product-images/TC4004BR/002.jpg,https://oleks-netizen.github.io/product-images/TC4004BR/003.jpg,https://oleks-netizen.github.io/product-images/TC4004BR/004.jpg,https://oleks-netizen.github.io/product-images/TC4004BR/005.jpg,https://oleks-netizen.github.io/product-images/TC4004BR/006.jpg,https://oleks-netizen.github.io/product-images/TC4004BR/007.jpg,https://oleks-netizen.github.io/product-images/TC4004BR/009.jpg</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>TC4004_BLK</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TC4004_BLK/001.jpg,https://oleks-netizen.github.io/product-images/TC4004_BLK/002.jpg,https://oleks-netizen.github.io/product-images/TC4004_BLK/003.jpg,https://oleks-netizen.github.io/product-images/TC4004_BLK/004.jpg,https://oleks-netizen.github.io/product-images/TC4004_BLK/005.jpg,https://oleks-netizen.github.io/product-images/TC4004_BLK/007.jpg,https://oleks-netizen.github.io/product-images/TC4004_BLK/008.jpg,https://oleks-netizen.github.io/product-images/TC4004_BLK/009.jpg</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>TC4004_BU</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TC4004_BU/001.jpg,https://oleks-netizen.github.io/product-images/TC4004_BU/002.jpg,https://oleks-netizen.github.io/product-images/TC4004_BU/003.jpg,https://oleks-netizen.github.io/product-images/TC4004_BU/004.jpg,https://oleks-netizen.github.io/product-images/TC4004_BU/005.jpg,https://oleks-netizen.github.io/product-images/TC4004_BU/006.jpg,https://oleks-netizen.github.io/product-images/TC4004_BU/007.jpg,https://oleks-netizen.github.io/product-images/TC4004_BU/009.jpg</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>tid3027</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/tid3027/001.jpg,https://oleks-netizen.github.io/product-images/tid3027/002.jpg,https://oleks-netizen.github.io/product-images/tid3027/003.jpg,https://oleks-netizen.github.io/product-images/tid3027/004.jpg,https://oleks-netizen.github.io/product-images/tid3027/005.jpg</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>TR34 BLK_RED</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TR34 BLK_RED/001.jpg,https://oleks-netizen.github.io/product-images/TR34 BLK_RED/002.jpg,https://oleks-netizen.github.io/product-images/TR34 BLK_RED/003.jpg,https://oleks-netizen.github.io/product-images/TR34 BLK_RED/005.jpg</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>TW-Bella-black</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Bella-black/001.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-black/002.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-black/003.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-black/004.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-black/005.jpg</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>TW-Bella-dark-brown</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Bella-dark-brown/001.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-dark-brown/003.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-dark-brown/004.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-dark-brown/005.jpg</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>TW-Bella-mokko</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Bella-mokko/001.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-mokko/002.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-mokko/003.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-mokko/005.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-mokko/006.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-mokko/007.jpg</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>TW-Bella-olive</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Bella-olive/001.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-olive/002.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-olive/003.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-olive/004.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-olive/006.jpg</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>TW-Bella-red</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Bella-red/001.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-red/002.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-red/004.jpg,https://oleks-netizen.github.io/product-images/TW-Bella-red/005.jpg</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>TW-Bridget-white</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Bridget-white/001.jpg,https://oleks-netizen.github.io/product-images/TW-Bridget-white/002.jpg,https://oleks-netizen.github.io/product-images/TW-Bridget-white/003.jpg,https://oleks-netizen.github.io/product-images/TW-Bridget-white/004.jpg</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>TW-Business-black</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Business-black/001.jpg,https://oleks-netizen.github.io/product-images/TW-Business-black/002.jpg,https://oleks-netizen.github.io/product-images/TW-Business-black/003.jpg</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>TW-Business-dark-blue</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Business-dark-blue/001.jpg,https://oleks-netizen.github.io/product-images/TW-Business-dark-blue/002.jpg,https://oleks-netizen.github.io/product-images/TW-Business-dark-blue/004.jpg,https://oleks-netizen.github.io/product-images/TW-Business-dark-blue/005.jpg</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>TW-Business-mars</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Business-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-Business-mars/002.jpg,https://oleks-netizen.github.io/product-images/TW-Business-mars/003.jpg,https://oleks-netizen.github.io/product-images/TW-Business-mars/004.jpg,https://oleks-netizen.github.io/product-images/TW-Business-mars/005.jpg</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>TW-CB-8-black</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-CB-8-black/001.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-black/002.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-black/003.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-black/004.jpg</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>TW-CB-8-light-beige</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-CB-8-light-beige/001.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-light-beige/002.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-light-beige/003.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-light-beige/004.jpg</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>TW-CB-8-mars</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-CB-8-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-mars/002.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-mars/003.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-mars/004.jpg</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>TW-CB-8-mokko</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-CB-8-mokko/001.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-mokko/002.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-mokko/003.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-mokko/004.jpg</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>TW-CB-8-pink</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-CB-8-pink/001.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-pink/002.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-pink/003.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-pink/004.jpg</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>TW-CB-8-red</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-CB-8-red/001.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-red/003.jpg,https://oleks-netizen.github.io/product-images/TW-CB-8-red/004.jpg</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>TW-Classic-mokko</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Classic-mokko/001.jpg,https://oleks-netizen.github.io/product-images/TW-Classic-mokko/002.jpg,https://oleks-netizen.github.io/product-images/TW-Classic-mokko/003.jpg,https://oleks-netizen.github.io/product-images/TW-Classic-mokko/005.jpg,https://oleks-netizen.github.io/product-images/TW-Classic-mokko/006.jpg</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>TW-Explorer-S-mars</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Explorer-S-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-Explorer-S-mars/002.jpg</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>TW-Faith-mars</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Faith-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-Faith-mars/002.jpg</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>TW-Futsy-mars</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Futsy-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-Futsy-mars/002.jpg</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>TW-Holly-mars</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Holly-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-Holly-mars/002.jpg,https://oleks-netizen.github.io/product-images/TW-Holly-mars/003.jpg,https://oleks-netizen.github.io/product-images/TW-Holly-mars/004.jpg,https://oleks-netizen.github.io/product-images/TW-Holly-mars/005.jpg,https://oleks-netizen.github.io/product-images/TW-Holly-mars/006.jpg,https://oleks-netizen.github.io/product-images/TW-Holly-mars/007.jpg,https://oleks-netizen.github.io/product-images/TW-Holly-mars/008.jpg</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>TW-Jill-caramel</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Jill-caramel/001.jpg,https://oleks-netizen.github.io/product-images/TW-Jill-caramel/002.jpg,https://oleks-netizen.github.io/product-images/TW-Jill-caramel/003.jpg,https://oleks-netizen.github.io/product-images/TW-Jill-caramel/004.jpg,https://oleks-netizen.github.io/product-images/TW-Jill-caramel/006.jpg</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>TW-Jill-red</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Jill-red/001.jpg,https://oleks-netizen.github.io/product-images/TW-Jill-red/002.jpg</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>TW-KL-5-mars</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-KL-5-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-KL-5-mars/002.jpg,https://oleks-netizen.github.io/product-images/TW-KL-5-mars/003.jpg,https://oleks-netizen.github.io/product-images/TW-KL-5-mars/004.jpg,https://oleks-netizen.github.io/product-images/TW-KL-5-mars/005.jpg</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>TW-Moment-mars</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Moment-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-Moment-mars/002.jpg</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>TW-Nona-2-k</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Nona-2-k/001.jpg,https://oleks-netizen.github.io/product-images/TW-Nona-2-k/002.jpg,https://oleks-netizen.github.io/product-images/TW-Nona-2-k/003.jpg,https://oleks-netizen.github.io/product-images/TW-Nona-2-k/005.jpg</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>TW-Nona-2-kon</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Nona-2-kon/001.jpg,https://oleks-netizen.github.io/product-images/TW-Nona-2-kon/002.jpg,https://oleks-netizen.github.io/product-images/TW-Nona-2-kon/003.jpg,https://oleks-netizen.github.io/product-images/TW-Nona-2-kon/005.jpg</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>TW-Nona-2-pink</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Nona-2-pink/001.jpg,https://oleks-netizen.github.io/product-images/TW-Nona-2-pink/002.jpg,https://oleks-netizen.github.io/product-images/TW-Nona-2-pink/004.jpg</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>TW-OP-1-black</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-OP-1-black/001.jpg,https://oleks-netizen.github.io/product-images/TW-OP-1-black/002.jpg,https://oleks-netizen.github.io/product-images/TW-OP-1-black/003.jpg</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>TW-OP-1-dark-blue</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-OP-1-dark-blue/001.jpg,https://oleks-netizen.github.io/product-images/TW-OP-1-dark-blue/002.jpg,https://oleks-netizen.github.io/product-images/TW-OP-1-dark-blue/003.jpg</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>TW-OP-1-mars</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-OP-1-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-OP-1-mars/002.jpg,https://oleks-netizen.github.io/product-images/TW-OP-1-mars/003.jpg</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>TW-PM-2-mars</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-PM-2-mars/001.jpg</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>TW-PM-Classic-mars</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-PM-Classic-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-PM-Classic-mars/002.jpg,https://oleks-netizen.github.io/product-images/TW-PM-Classic-mars/003.jpg,https://oleks-netizen.github.io/product-images/TW-PM-Classic-mars/004.jpg</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>TW-PM-Classic-red</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-PM-Classic-red/001.jpg,https://oleks-netizen.github.io/product-images/TW-PM-Classic-red/002.jpg,https://oleks-netizen.github.io/product-images/TW-PM-Classic-red/004.jpg,https://oleks-netizen.github.io/product-images/TW-PM-Classic-red/005.jpg</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>TW-Ruby-big-mars</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/002.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/003.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/005.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/006.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/007.jpg</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>TW-Style-black</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Style-black/001.jpg,https://oleks-netizen.github.io/product-images/TW-Style-black/002.jpg,https://oleks-netizen.github.io/product-images/TW-Style-black/003.jpg,https://oleks-netizen.github.io/product-images/TW-Style-black/004.jpg,https://oleks-netizen.github.io/product-images/TW-Style-black/005.jpg</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>TW-Style-kon</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Style-kon/001.jpg,https://oleks-netizen.github.io/product-images/TW-Style-kon/002.jpg,https://oleks-netizen.github.io/product-images/TW-Style-kon/004.jpg,https://oleks-netizen.github.io/product-images/TW-Style-kon/005.jpg</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>TW-Vacation-vin</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Vacation-vin/001.jpg,https://oleks-netizen.github.io/product-images/TW-Vacation-vin/002.jpg</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>vc001A-orange</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/vc001A-orange/001.jpg,https://oleks-netizen.github.io/product-images/vc001A-orange/002.jpg,https://oleks-netizen.github.io/product-images/vc001A-orange/003.jpg,https://oleks-netizen.github.io/product-images/vc001A-orange/004.jpg</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>vc001a-red</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/vc001a-red/001.jpg,https://oleks-netizen.github.io/product-images/vc001a-red/002.jpg,https://oleks-netizen.github.io/product-images/vc001a-red/003.jpg,https://oleks-netizen.github.io/product-images/vc001a-red/004.jpg</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>VC2234black</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/VC2234black/001.jpg,https://oleks-netizen.github.io/product-images/VC2234black/002.jpg,https://oleks-netizen.github.io/product-images/VC2234black/004.jpg,https://oleks-netizen.github.io/product-images/VC2234black/005.jpg</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>20906_1 (1)</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/20906_1 (1)/006.jpg</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-04-03 20:00:54
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C295"/>
+  <dimension ref="A1:C294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,11 +471,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/20906_1/001.jpg,https://oleks-netizen.github.io/product-images/20906_1/003.jpg,https://oleks-netizen.github.io/product-images/20906_1/004.jpg,https://oleks-netizen.github.io/product-images/20906_1/005.jpg,https://oleks-netizen.github.io/product-images/20906_1/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/20906_1/001.jpg,https://oleks-netizen.github.io/product-images/20906_1/003.jpg,https://oleks-netizen.github.io/product-images/20906_1/004.jpg,https://oleks-netizen.github.io/product-images/20906_1/005.jpg,https://oleks-netizen.github.io/product-images/20906_1/006.jpg,https://oleks-netizen.github.io/product-images/20906_1/007.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -4826,21 +4826,6 @@
       </c>
       <c r="C294" t="n">
         <v>4</v>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="inlineStr">
-        <is>
-          <t>20906_1 (1)</t>
-        </is>
-      </c>
-      <c r="B295" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/20906_1 (1)/006.jpg</t>
-        </is>
-      </c>
-      <c r="C295" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-04-13 20:14:26
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,87 +436,87 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11614</t>
+          <t>WELL-10210</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/11614/001.jpg,https://oleks-netizen.github.io/product-images/11614/002.jpg,https://oleks-netizen.github.io/product-images/11614/003.jpg,https://oleks-netizen.github.io/product-images/11614/005.jpg,https://oleks-netizen.github.io/product-images/11614/006.jpg,https://oleks-netizen.github.io/product-images/11614/007.jpg,https://oleks-netizen.github.io/product-images/11614/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10210/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10210/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10210/003.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>11615</t>
+          <t>WELL-10300</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/11615/001.jpg,https://oleks-netizen.github.io/product-images/11615/002.jpg,https://oleks-netizen.github.io/product-images/11615/004.jpg,https://oleks-netizen.github.io/product-images/11615/005.jpg,https://oleks-netizen.github.io/product-images/11615/006.jpg,https://oleks-netizen.github.io/product-images/11615/007.jpg,https://oleks-netizen.github.io/product-images/11615/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10300/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10300/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10300/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10300/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10300/005.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>11616</t>
+          <t>WELL-10301</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/11616/001.jpg,https://oleks-netizen.github.io/product-images/11616/002.jpg,https://oleks-netizen.github.io/product-images/11616/003.jpg,https://oleks-netizen.github.io/product-images/11616/004.jpg,https://oleks-netizen.github.io/product-images/11616/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10301/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10301/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10301/003.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>55000</t>
+          <t>WELL-10304</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/55000/001.jpg,https://oleks-netizen.github.io/product-images/55000/002.jpg,https://oleks-netizen.github.io/product-images/55000/003.jpg,https://oleks-netizen.github.io/product-images/55000/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10304/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10304/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10304/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10304/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10304/005.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>80460410</t>
+          <t>WELL-10305</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80460410/001.jpg,https://oleks-netizen.github.io/product-images/80460410/002.jpg,https://oleks-netizen.github.io/product-images/80460410/003.jpg,https://oleks-netizen.github.io/product-images/80460410/004.jpg,https://oleks-netizen.github.io/product-images/80460410/005.jpg,https://oleks-netizen.github.io/product-images/80460410/006.jpg,https://oleks-netizen.github.io/product-images/80460410/007.jpg,https://oleks-netizen.github.io/product-images/80460410/008.jpg,https://oleks-netizen.github.io/product-images/80460410/010.jpg,https://oleks-netizen.github.io/product-images/80460410/011.jpg,https://oleks-netizen.github.io/product-images/80460410/012.jpg,https://oleks-netizen.github.io/product-images/80460410/013.jpg,https://oleks-netizen.github.io/product-images/80460410/014.jpg,https://oleks-netizen.github.io/product-images/80460410/015.jpg,https://oleks-netizen.github.io/product-images/80460410/016.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10305/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10305/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10305/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10305/004.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BN-BK1-red</t>
+          <t>WELL-10309</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK1-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK1-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-BK1-red/004.jpg,https://oleks-netizen.github.io/product-images/BN-BK1-red/005.jpg,https://oleks-netizen.github.io/product-images/BN-BK1-red/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10309/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10309/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10309/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10309/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10309/005.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -526,72 +526,72 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BN-BK10-malachite</t>
+          <t>WELL-10400</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK10-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK10-malachite/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10400/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10400/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10400/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10400/004.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BN-BK11-g</t>
+          <t>WELL-10404</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK11-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK11-g/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10404/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10404/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10404/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10404/005.jpg,https://oleks-netizen.github.io/product-images/WELL-10404/006.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BN-BK12-o</t>
+          <t>WELL-10405</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK12-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK12-o/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10405/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10405/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10405/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10405/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10405/005.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BN-BK13-beige</t>
+          <t>WELL-10409</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK13-beige/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK13-beige/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10409/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10409/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10409/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10409/005.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BN-BK15-choko</t>
+          <t>WELL-10410</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK15-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-choko/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10410/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10410/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10410/003.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -601,12 +601,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BN-BK15-g</t>
+          <t>WELL-10411</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK15-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-g/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10411/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10411/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10411/004.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -616,57 +616,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BN-BK15-k</t>
+          <t>WELL-10503</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK15-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-k/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10503/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10503/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10503/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10503/004.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BN-BK15-light-beige</t>
+          <t>WELL-10505</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK15-light-beige/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-light-beige/002.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-light-beige/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10505/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10505/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10505/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10505/005.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BN-BK15-malachite</t>
+          <t>WELL-10524</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK15-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-malachite/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10524/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10524/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10524/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10524/004.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BN-BK15-red</t>
+          <t>WELL-10528</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK15-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-red/003.jpg,https://oleks-netizen.github.io/product-images/BN-BK15-red/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10528/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10528/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10528/003.jpg</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -676,132 +676,132 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BN-BK16-choko</t>
+          <t>WELL-10529</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK16-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK16-choko/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10529/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10529/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10529/003.jpg</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BN-BK17-g</t>
+          <t>WELL-10601</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK17-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK17-g/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10601/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10601/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10601/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10601/004.jpg</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BN-BK18-g</t>
+          <t>WELL-10604</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK18-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK18-g/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10604/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10604/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10604/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10604/004.jpg</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BN-BK2</t>
+          <t>WELL-10701</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK2/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK2/002.jpg,https://oleks-netizen.github.io/product-images/BN-BK2/003.jpg,https://oleks-netizen.github.io/product-images/BN-BK2/005.jpg,https://oleks-netizen.github.io/product-images/BN-BK2/006.jpg,https://oleks-netizen.github.io/product-images/BN-BK2/007.jpg,https://oleks-netizen.github.io/product-images/BN-BK2/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10701/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10701/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10701/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10701/004.jpg</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BN-BK2-3-red</t>
+          <t>WELL-10703</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK2-3-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK2-3-red/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10703/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10703/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10703/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10703/005.jpg</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BN-BK2-4-light</t>
+          <t>WELL-10704</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK2-4-light/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK2-4-light/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10704/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10704/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10704/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10704/005.jpg</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BN-BK2-4-pink-peach</t>
+          <t>WELL-10705</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK2-4-pink-peach/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK2-4-pink-peach/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10705/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10705/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10705/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10705/005.jpg</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BN-BK2-4-shadow</t>
+          <t>WELL-10724</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK2-4-shadow/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK2-4-shadow/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10724/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10724/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10724/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10724/005.jpg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BN-BK2-5-tiffany</t>
+          <t>WELL-10728</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK2-5-tiffany/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK2-5-tiffany/002.jpg,https://oleks-netizen.github.io/product-images/BN-BK2-5-tiffany/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10728/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10728/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10728/003.jpg</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -811,102 +811,102 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BN-BK3</t>
+          <t>WELL-10729</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK3/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK3/002.jpg,https://oleks-netizen.github.io/product-images/BN-BK3/004.jpg,https://oleks-netizen.github.io/product-images/BN-BK3/005.jpg,https://oleks-netizen.github.io/product-images/BN-BK3/006.jpg,https://oleks-netizen.github.io/product-images/BN-BK3/007.jpg,https://oleks-netizen.github.io/product-images/BN-BK3/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10729/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10729/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10729/004.jpg,https://oleks-netizen.github.io/product-images/WELL-10729/005.jpg</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BN-BK4-blue-ylw</t>
+          <t>WELL-10801</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK4-blue-ylw/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK4-blue-ylw/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10801/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10801/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10801/003.jpg</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BN-BK4-choko</t>
+          <t>WELL-10804</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK4-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK4-choko/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10804/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10804/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10804/003.jpg</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BN-BK4-k</t>
+          <t>WELL-10805</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK4-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK4-k/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10805/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10805/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10805/003.jpg</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BN-BK4-malachite</t>
+          <t>WELL-10807</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK4-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK4-malachite/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10807/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10807/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10807/003.jpg</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BN-BK4-navy-blue</t>
+          <t>WELL-10822</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK4-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK4-navy-blue/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10822/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10822/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10822/003.jpg</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BN-BK4-vin</t>
+          <t>WELL-10824</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK4-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK4-vin/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10824/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10824/003.jpg</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -916,132 +916,132 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BN-BK5-choko</t>
+          <t>WELL-10825</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK5-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK5-choko/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10825/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10825/002.jpg,https://oleks-netizen.github.io/product-images/WELL-10825/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10825/004.jpg</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BN-BK6-navy-blue</t>
+          <t>WELL-10829</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK6-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK6-navy-blue/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-10829/001.jpg,https://oleks-netizen.github.io/product-images/WELL-10829/003.jpg,https://oleks-netizen.github.io/product-images/WELL-10829/004.jpg</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>BN-BK7-iz</t>
+          <t>WELL-11000</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK7-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK7-iz/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11000/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11000/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11000/003.jpg</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BN-BK8-k</t>
+          <t>WELL-11002</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK8-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK8-k/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11002/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11002/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11002/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11002/005.jpg,https://oleks-netizen.github.io/product-images/WELL-11002/006.jpg</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BN-BK9-coral</t>
+          <t>WELL-11004</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BK9-coral/001.jpg,https://oleks-netizen.github.io/product-images/BN-BK9-coral/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11004/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11004/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11004/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11004/004.jpg</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BN-GC-32-1-g</t>
+          <t>WELL-11006</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-32-1-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-1-g/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11006/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11006/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11006/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11006/005.jpg</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BN-GC-32-1-vin</t>
+          <t>WELL-11009</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-32-1-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-1-vin/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11009/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11009/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11009/003.jpg</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BN-GC-32-choko</t>
+          <t>WELL-11019</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-32-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-choko/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-choko/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11019/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11019/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11019/003.jpg</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BN-GC-32-g</t>
+          <t>WELL-11100</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-32-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-g/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-g/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11100/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11100/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11100/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11100/005.jpg,https://oleks-netizen.github.io/product-images/WELL-11100/006.jpg</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1051,147 +1051,147 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BN-GC-32-k</t>
+          <t>WELL-11102</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-32-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-k/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-k/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11102/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11102/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11102/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11102/005.jpg</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BN-GC-32-malachite</t>
+          <t>WELL-11104</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-32-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-malachite/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-malachite/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11104/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11104/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11104/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11104/005.jpg</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BN-GC-32-navy-blue</t>
+          <t>WELL-11105</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-32-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-navy-blue/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-navy-blue/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11105/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11105/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11105/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11105/005.jpg</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>BN-GC-32-vin</t>
+          <t>WELL-11109</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-32-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-vin/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-vin/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-vin/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-32-vin/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11109/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11109/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11109/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11109/005.jpg</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BN-SB-8-k</t>
+          <t>WELL-11119</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-8-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-k/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11119/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11119/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11119/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11119/005.jpg</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BN-SB-8-navy-blue</t>
+          <t>WELL-11204</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-8-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-navy-blue/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11204/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11204/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11204/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11204/005.jpg</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>BN-SB-8-nn</t>
+          <t>WELL-11205</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-8-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-nn/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-nn/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11205/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11205/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11205/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11205/005.jpg,https://oleks-netizen.github.io/product-images/WELL-11205/006.jpg</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BN-SB-8-o</t>
+          <t>WELL-11303</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-8-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-o/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-o/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11303/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11303/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11303/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11303/005.jpg</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BN-SB-8-red</t>
+          <t>WELL-11304</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-8-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-red/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11304/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11304/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11304/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11304/005.jpg,https://oleks-netizen.github.io/product-images/WELL-11304/006.jpg</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BN-SB-8-vin</t>
+          <t>WELL-11404</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-8-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-vin/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-8-vin/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11404/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11404/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11404/003.jpg</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1201,57 +1201,57 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BN-SB-9-2-A4-choko</t>
+          <t>WELL-11406</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-choko/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11406/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11406/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11406/004.jpg</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BN-SB-9-2-A4-g</t>
+          <t>WELL-11409</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-g/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11409/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11409/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11409/003.jpg</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BN-SB-9-2-A4-iz</t>
+          <t>WELL-11419</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-iz/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-iz/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11419/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11419/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11419/003.jpg</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>BN-SB-9-2-A4-k</t>
+          <t>WELL-11501</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-k/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11501/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11501/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11501/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11501/004.jpg</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1261,27 +1261,27 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BN-SB-9-2-A4-navy-blue</t>
+          <t>WELL-11502</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-navy-blue/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11502/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11502/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11502/004.jpg</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>BN-SB-9-2-A4-vin-kr</t>
+          <t>WELL-11503</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-vin-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-vin-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-vin-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-2-A4-vin-kr/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11503/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11503/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11503/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11503/005.jpg</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -1291,57 +1291,57 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BN-SB-9-3-A5-choko</t>
+          <t>WELL-11504</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-choko/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11504/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11504/002.jpg</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BN-SB-9-3-A5-g</t>
+          <t>WELL-11601</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-g/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11601/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11601/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11601/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11601/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11601/005.jpg</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BN-SB-9-3-A5-iz</t>
+          <t>WELL-11608</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-iz/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-iz/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11608/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11608/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11608/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11608/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11608/005.jpg</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BN-SB-9-3-A5-k</t>
+          <t>WELL-11609</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-k/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11609/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11609/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11609/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11609/004.jpg</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -1351,27 +1351,27 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BN-SB-9-3-A5-navy-blue</t>
+          <t>WELL-11701</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-navy-blue/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11701/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11701/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11701/003.jpg</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BN-SB-9-3-A5-vin-kr</t>
+          <t>WELL-11702</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-vin-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-vin-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-vin-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-3-A5-vin-kr/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11702/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11702/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11702/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11702/004.jpg</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -1381,496 +1381,3241 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BN-SB-9-4-choko</t>
+          <t>WELL-11704</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-4-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-choko/004.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-choko/005.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-choko/006.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-choko/007.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-choko/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11704/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11704/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11704/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11704/004.jpg</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BN-SB-9-4-g</t>
+          <t>WELL-11709</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-4-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-g/004.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-g/005.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-g/006.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-g/007.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-g/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11709/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11709/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11709/003.jpg</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>BN-SB-9-4-k</t>
+          <t>WELL-11800</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-4-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-k/004.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-k/005.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-k/006.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-k/007.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-k/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11800/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11800/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11800/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11800/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11800/005.jpg</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>BN-SB-9-4-light-beige</t>
+          <t>WELL-11804</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-4-light-beige/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-light-beige/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-light-beige/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-light-beige/004.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-light-beige/005.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-light-beige/006.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-light-beige/007.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-light-beige/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11804/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11804/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11804/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11804/004.jpg</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BN-SB-9-4-navy-blue</t>
+          <t>WELL-11902</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-4-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-navy-blue/004.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-navy-blue/005.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-navy-blue/006.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-navy-blue/007.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-navy-blue/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11902/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11902/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11902/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11902/004.jpg</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BN-SB-9-4-red</t>
+          <t>WELL-11904</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-4-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-red/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-red/004.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-red/005.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-red/006.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-red/007.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-4-red/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11904/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11904/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11904/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11904/004.jpg</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BN-SB-9-soft-k-kr</t>
+          <t>WELL-11905</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-soft-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-soft-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-soft-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-soft-k-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-soft-k-kr/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11905/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11905/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11905/003.jpg</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>S32008-1</t>
+          <t>WELL-11909</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32008-1/001.jpg,https://oleks-netizen.github.io/product-images/S32008-1/002.jpg,https://oleks-netizen.github.io/product-images/S32008-1/003.jpg,https://oleks-netizen.github.io/product-images/S32008-1/004.jpg,https://oleks-netizen.github.io/product-images/S32008-1/005.jpg,https://oleks-netizen.github.io/product-images/S32008-1/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11909/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11909/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11909/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11909/004.jpg</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>S32008-2</t>
+          <t>WELL-12000</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32008-2/001.jpg,https://oleks-netizen.github.io/product-images/S32008-2/002.jpg,https://oleks-netizen.github.io/product-images/S32008-2/003.jpg,https://oleks-netizen.github.io/product-images/S32008-2/004.jpg,https://oleks-netizen.github.io/product-images/S32008-2/005.jpg,https://oleks-netizen.github.io/product-images/S32008-2/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12000/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12000/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12000/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12000/004.jpg</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>S32008-4</t>
+          <t>WELL-12004</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32008-4/001.jpg,https://oleks-netizen.github.io/product-images/S32008-4/002.jpg,https://oleks-netizen.github.io/product-images/S32008-4/003.jpg,https://oleks-netizen.github.io/product-images/S32008-4/004.jpg,https://oleks-netizen.github.io/product-images/S32008-4/005.jpg,https://oleks-netizen.github.io/product-images/S32008-4/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12004/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12004/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12004/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12004/004.jpg,https://oleks-netizen.github.io/product-images/WELL-12004/005.jpg</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>S32008-5</t>
+          <t>WELL-12005</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32008-5/001.jpg,https://oleks-netizen.github.io/product-images/S32008-5/002.jpg,https://oleks-netizen.github.io/product-images/S32008-5/003.jpg,https://oleks-netizen.github.io/product-images/S32008-5/004.jpg,https://oleks-netizen.github.io/product-images/S32008-5/005.jpg,https://oleks-netizen.github.io/product-images/S32008-5/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12005/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12005/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12005/003.jpg</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>S32008-6</t>
+          <t>WELL-12009</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32008-6/001.jpg,https://oleks-netizen.github.io/product-images/S32008-6/002.jpg,https://oleks-netizen.github.io/product-images/S32008-6/004.jpg,https://oleks-netizen.github.io/product-images/S32008-6/005.jpg,https://oleks-netizen.github.io/product-images/S32008-6/006.jpg,https://oleks-netizen.github.io/product-images/S32008-6/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12009/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12009/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12009/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12009/004.jpg</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>S32101-1</t>
+          <t>WELL-12124</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32101-1/001.jpg,https://oleks-netizen.github.io/product-images/S32101-1/002.jpg,https://oleks-netizen.github.io/product-images/S32101-1/004.jpg,https://oleks-netizen.github.io/product-images/S32101-1/005.jpg,https://oleks-netizen.github.io/product-images/S32101-1/006.jpg,https://oleks-netizen.github.io/product-images/S32101-1/007.jpg,https://oleks-netizen.github.io/product-images/S32101-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12124/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12124/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12124/003.jpg</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>S32101-5</t>
+          <t>WELL-12128</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32101-5/001.jpg,https://oleks-netizen.github.io/product-images/S32101-5/002.jpg,https://oleks-netizen.github.io/product-images/S32101-5/003.jpg,https://oleks-netizen.github.io/product-images/S32101-5/004.jpg,https://oleks-netizen.github.io/product-images/S32101-5/005.jpg,https://oleks-netizen.github.io/product-images/S32101-5/006.jpg,https://oleks-netizen.github.io/product-images/S32101-5/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12128/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12128/002.jpg</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>S32103-1</t>
+          <t>WELL-12129</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32103-1/001.jpg,https://oleks-netizen.github.io/product-images/S32103-1/002.jpg,https://oleks-netizen.github.io/product-images/S32103-1/003.jpg,https://oleks-netizen.github.io/product-images/S32103-1/004.jpg,https://oleks-netizen.github.io/product-images/S32103-1/005.jpg,https://oleks-netizen.github.io/product-images/S32103-1/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12129/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12129/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12129/003.jpg</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>S32103-2</t>
+          <t>WELL-12205</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32103-2/001.jpg,https://oleks-netizen.github.io/product-images/S32103-2/002.jpg,https://oleks-netizen.github.io/product-images/S32103-2/003.jpg,https://oleks-netizen.github.io/product-images/S32103-2/004.jpg,https://oleks-netizen.github.io/product-images/S32103-2/005.jpg,https://oleks-netizen.github.io/product-images/S32103-2/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12205/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12205/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12205/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12205/004.jpg</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>S32103-4</t>
+          <t>WELL-12208</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32103-4/001.jpg,https://oleks-netizen.github.io/product-images/S32103-4/002.jpg,https://oleks-netizen.github.io/product-images/S32103-4/003.jpg,https://oleks-netizen.github.io/product-images/S32103-4/004.jpg,https://oleks-netizen.github.io/product-images/S32103-4/005.jpg,https://oleks-netizen.github.io/product-images/S32103-4/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12208/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12208/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12208/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12208/004.jpg</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>S32103-5</t>
+          <t>WELL-12209</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32103-5/001.jpg,https://oleks-netizen.github.io/product-images/S32103-5/002.jpg,https://oleks-netizen.github.io/product-images/S32103-5/003.jpg,https://oleks-netizen.github.io/product-images/S32103-5/004.jpg,https://oleks-netizen.github.io/product-images/S32103-5/005.jpg,https://oleks-netizen.github.io/product-images/S32103-5/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12209/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12209/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12209/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12209/004.jpg</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>S32106-1</t>
+          <t>WELL-12304</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32106-1/001.jpg,https://oleks-netizen.github.io/product-images/S32106-1/002.jpg,https://oleks-netizen.github.io/product-images/S32106-1/004.jpg,https://oleks-netizen.github.io/product-images/S32106-1/005.jpg,https://oleks-netizen.github.io/product-images/S32106-1/006.jpg,https://oleks-netizen.github.io/product-images/S32106-1/007.jpg,https://oleks-netizen.github.io/product-images/S32106-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12304/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12304/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12304/003.jpg</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>S32106-2</t>
+          <t>WELL-12305</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32106-2/001.jpg,https://oleks-netizen.github.io/product-images/S32106-2/002.jpg,https://oleks-netizen.github.io/product-images/S32106-2/004.jpg,https://oleks-netizen.github.io/product-images/S32106-2/005.jpg,https://oleks-netizen.github.io/product-images/S32106-2/006.jpg,https://oleks-netizen.github.io/product-images/S32106-2/007.jpg,https://oleks-netizen.github.io/product-images/S32106-2/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12305/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12305/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12305/003.jpg</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>S32106-3</t>
+          <t>WELL-12309</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32106-3/001.jpg,https://oleks-netizen.github.io/product-images/S32106-3/002.jpg,https://oleks-netizen.github.io/product-images/S32106-3/004.jpg,https://oleks-netizen.github.io/product-images/S32106-3/005.jpg,https://oleks-netizen.github.io/product-images/S32106-3/006.jpg,https://oleks-netizen.github.io/product-images/S32106-3/007.jpg,https://oleks-netizen.github.io/product-images/S32106-3/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12309/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12309/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12309/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12309/004.jpg</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>S32106-4</t>
+          <t>WELL-12404</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32106-4/001.jpg,https://oleks-netizen.github.io/product-images/S32106-4/002.jpg,https://oleks-netizen.github.io/product-images/S32106-4/004.jpg,https://oleks-netizen.github.io/product-images/S32106-4/005.jpg,https://oleks-netizen.github.io/product-images/S32106-4/006.jpg,https://oleks-netizen.github.io/product-images/S32106-4/007.jpg,https://oleks-netizen.github.io/product-images/S32106-4/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12404/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12404/002.jpg</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>S32106-5</t>
+          <t>WELL-12405</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32106-5/001.jpg,https://oleks-netizen.github.io/product-images/S32106-5/002.jpg,https://oleks-netizen.github.io/product-images/S32106-5/004.jpg,https://oleks-netizen.github.io/product-images/S32106-5/005.jpg,https://oleks-netizen.github.io/product-images/S32106-5/006.jpg,https://oleks-netizen.github.io/product-images/S32106-5/007.jpg,https://oleks-netizen.github.io/product-images/S32106-5/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12405/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12405/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12405/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12405/004.jpg</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>S32110-1</t>
+          <t>WELL-12409</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32110-1/001.jpg,https://oleks-netizen.github.io/product-images/S32110-1/003.jpg,https://oleks-netizen.github.io/product-images/S32110-1/004.jpg,https://oleks-netizen.github.io/product-images/S32110-1/005.jpg,https://oleks-netizen.github.io/product-images/S32110-1/006.jpg,https://oleks-netizen.github.io/product-images/S32110-1/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12409/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12409/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12409/003.jpg</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>S32110-2</t>
+          <t>WELL-12504</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32110-2/001.jpg,https://oleks-netizen.github.io/product-images/S32110-2/002.jpg,https://oleks-netizen.github.io/product-images/S32110-2/003.jpg,https://oleks-netizen.github.io/product-images/S32110-2/004.jpg,https://oleks-netizen.github.io/product-images/S32110-2/005.jpg,https://oleks-netizen.github.io/product-images/S32110-2/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12504/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12504/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12504/003.jpg</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>S32110-3</t>
+          <t>WELL-12505</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32110-3/001.jpg,https://oleks-netizen.github.io/product-images/S32110-3/002.jpg,https://oleks-netizen.github.io/product-images/S32110-3/003.jpg,https://oleks-netizen.github.io/product-images/S32110-3/004.jpg,https://oleks-netizen.github.io/product-images/S32110-3/005.jpg,https://oleks-netizen.github.io/product-images/S32110-3/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12505/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12505/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12505/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12505/004.jpg</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>S32110-4</t>
+          <t>WELL-12507</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32110-4/001.jpg,https://oleks-netizen.github.io/product-images/S32110-4/002.jpg,https://oleks-netizen.github.io/product-images/S32110-4/003.jpg,https://oleks-netizen.github.io/product-images/S32110-4/004.jpg,https://oleks-netizen.github.io/product-images/S32110-4/005.jpg,https://oleks-netizen.github.io/product-images/S32110-4/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12507/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12507/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12507/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12507/004.jpg</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>S32110-5</t>
+          <t>WELL-12509</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32110-5/001.jpg,https://oleks-netizen.github.io/product-images/S32110-5/002.jpg,https://oleks-netizen.github.io/product-images/S32110-5/003.jpg,https://oleks-netizen.github.io/product-images/S32110-5/004.jpg,https://oleks-netizen.github.io/product-images/S32110-5/005.jpg,https://oleks-netizen.github.io/product-images/S32110-5/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12509/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12509/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12509/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12509/004.jpg</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>S32112-1</t>
+          <t>WELL-12602</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32112-1/001.jpg,https://oleks-netizen.github.io/product-images/S32112-1/002.jpg,https://oleks-netizen.github.io/product-images/S32112-1/004.jpg,https://oleks-netizen.github.io/product-images/S32112-1/005.jpg,https://oleks-netizen.github.io/product-images/S32112-1/006.jpg,https://oleks-netizen.github.io/product-images/S32112-1/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12602/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12602/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12602/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12602/004.jpg</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>S32112-2</t>
+          <t>WELL-12607</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32112-2/001.jpg,https://oleks-netizen.github.io/product-images/S32112-2/002.jpg,https://oleks-netizen.github.io/product-images/S32112-2/004.jpg,https://oleks-netizen.github.io/product-images/S32112-2/005.jpg,https://oleks-netizen.github.io/product-images/S32112-2/006.jpg,https://oleks-netizen.github.io/product-images/S32112-2/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12607/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12607/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12607/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12607/004.jpg,https://oleks-netizen.github.io/product-images/WELL-12607/005.jpg</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>S32112-3</t>
+          <t>WELL-12609</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32112-3/001.jpg,https://oleks-netizen.github.io/product-images/S32112-3/002.jpg,https://oleks-netizen.github.io/product-images/S32112-3/004.jpg,https://oleks-netizen.github.io/product-images/S32112-3/005.jpg,https://oleks-netizen.github.io/product-images/S32112-3/006.jpg,https://oleks-netizen.github.io/product-images/S32112-3/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12609/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12609/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12609/003.jpg</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>S32112-4</t>
+          <t>WELL-12704</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32112-4/001.jpg,https://oleks-netizen.github.io/product-images/S32112-4/002.jpg,https://oleks-netizen.github.io/product-images/S32112-4/004.jpg,https://oleks-netizen.github.io/product-images/S32112-4/005.jpg,https://oleks-netizen.github.io/product-images/S32112-4/006.jpg,https://oleks-netizen.github.io/product-images/S32112-4/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12704/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12704/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12704/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12704/004.jpg</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>S32112-5</t>
+          <t>WELL-12708</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/S32112-5/001.jpg,https://oleks-netizen.github.io/product-images/S32112-5/002.jpg,https://oleks-netizen.github.io/product-images/S32112-5/004.jpg,https://oleks-netizen.github.io/product-images/S32112-5/005.jpg,https://oleks-netizen.github.io/product-images/S32112-5/006.jpg,https://oleks-netizen.github.io/product-images/S32112-5/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12708/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12708/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12708/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12708/004.jpg</t>
         </is>
       </c>
       <c r="C97" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>WELL-12709</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12709/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12709/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12709/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12709/004.jpg</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>WELL-12801</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12801/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12801/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12801/003.jpg</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>WELL-12802</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12802/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12802/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12802/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12802/004.jpg</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>WELL-12804</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12804/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12804/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12804/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12804/004.jpg</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>WELL-12805</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12805/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12805/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12805/003.jpg</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>WELL-12807</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12807/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12807/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12807/003.jpg,https://oleks-netizen.github.io/product-images/WELL-12807/004.jpg</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>WELL-12809</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12809/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12809/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12809/003.jpg</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>WELL-13004</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13004/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13004/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13004/003.jpg,https://oleks-netizen.github.io/product-images/WELL-13004/004.jpg</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>WELL-13102</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13102/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13102/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13102/003.jpg,https://oleks-netizen.github.io/product-images/WELL-13102/004.jpg</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>WELL-13104</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13104/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13104/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13104/003.jpg,https://oleks-netizen.github.io/product-images/WELL-13104/004.jpg</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>WELL-13109</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13109/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13109/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13109/003.jpg</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>WELL-13555</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13555/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13555/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13555/003.jpg,https://oleks-netizen.github.io/product-images/WELL-13555/004.jpg,https://oleks-netizen.github.io/product-images/WELL-13555/005.jpg</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>WELL-13559</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13559/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13559/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13559/003.jpg,https://oleks-netizen.github.io/product-images/WELL-13559/004.jpg</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>WELL-13604</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13604/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13604/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13604/003.jpg</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>WELL-13606</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13606/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13606/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13606/003.jpg</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>WELL-13609</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13609/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13609/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13609/003.jpg</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>WELL-13803</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13803/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13803/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13803/003.jpg</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>WELL-13804</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13804/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13804/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13804/003.jpg</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>WELL-13809</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-13809/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13809/002.jpg,https://oleks-netizen.github.io/product-images/WELL-13809/003.jpg</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>WELL-14003</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-14003/001.jpg,https://oleks-netizen.github.io/product-images/WELL-14003/002.jpg,https://oleks-netizen.github.io/product-images/WELL-14003/003.jpg</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>WELL-14004</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-14004/001.jpg,https://oleks-netizen.github.io/product-images/WELL-14004/002.jpg,https://oleks-netizen.github.io/product-images/WELL-14004/003.jpg</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>WELL-14009</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-14009/001.jpg,https://oleks-netizen.github.io/product-images/WELL-14009/002.jpg</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>WELL-14103</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-14103/001.jpg,https://oleks-netizen.github.io/product-images/WELL-14103/002.jpg,https://oleks-netizen.github.io/product-images/WELL-14103/003.jpg</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>WELL-14104</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-14104/001.jpg,https://oleks-netizen.github.io/product-images/WELL-14104/002.jpg,https://oleks-netizen.github.io/product-images/WELL-14104/003.jpg</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>WELL-14202</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-14202/001.jpg,https://oleks-netizen.github.io/product-images/WELL-14202/002.jpg</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>WELL-14209</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-14209/001.jpg,https://oleks-netizen.github.io/product-images/WELL-14209/002.jpg</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>WELL-14254</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-14254/001.jpg,https://oleks-netizen.github.io/product-images/WELL-14254/002.jpg,https://oleks-netizen.github.io/product-images/WELL-14254/003.jpg,https://oleks-netizen.github.io/product-images/WELL-14254/004.jpg,https://oleks-netizen.github.io/product-images/WELL-14254/005.jpg</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>WELL-14300</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-14300/001.jpg,https://oleks-netizen.github.io/product-images/WELL-14300/002.jpg,https://oleks-netizen.github.io/product-images/WELL-14300/003.jpg</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>WELL-15002</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15002/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15002/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15002/003.jpg</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>WELL-15004</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15004/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15004/002.jpg</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>WELL-15005</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15005/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15005/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15005/003.jpg</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>WELL-15007</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15007/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15007/002.jpg</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>WELL-15009</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15009/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15009/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15009/003.jpg</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>WELL-15154</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15154/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15154/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15154/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15154/004.jpg</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>WELL-15155</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15155/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15155/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15155/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15155/004.jpg</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>WELL-15157</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15157/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15157/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15157/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15157/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15157/005.jpg</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>WELL-15159</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15159/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15159/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15159/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15159/004.jpg</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>WELL-15252</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15252/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15252/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15252/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15252/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15252/005.jpg</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>WELL-15254</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15254/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15254/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15254/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15254/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15254/005.jpg</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>WELL-15255</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15255/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15255/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15255/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15255/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15255/005.jpg</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>WELL-15257</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15257/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15257/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15257/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15257/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15257/005.jpg</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>WELL-15259</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15259/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15259/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15259/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15259/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15259/005.jpg</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>WELL-15304</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15304/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15304/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15304/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15304/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15304/005.jpg</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>WELL-15305</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15305/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15305/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15305/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15305/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15305/005.jpg</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>WELL-15308</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15308/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15308/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15308/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15308/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15308/005.jpg</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>WELL-15309</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15309/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15309/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15309/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15309/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15309/005.jpg</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>WELL-15454</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15454/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15454/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15454/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15454/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15454/005.jpg</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>WELL-15455</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15455/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15455/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15455/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15455/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15455/005.jpg</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>WELL-15504</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15504/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15504/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15504/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15504/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15504/005.jpg</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>WELL-15505</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15505/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15505/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15505/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15505/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15505/005.jpg,https://oleks-netizen.github.io/product-images/WELL-15505/006.jpg</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>WELL-15507</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15507/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15507/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15507/003.jpg</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>WELL-15509</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15509/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15509/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15509/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15509/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15509/005.jpg</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>WELL-15654</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15654/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15654/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15654/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15654/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15654/005.jpg</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>WELL-15655</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15655/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15655/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15655/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15655/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15655/005.jpg</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>WELL-15657</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15657/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15657/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15657/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15657/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15657/005.jpg</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>WELL-15659</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15659/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15659/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15659/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15659/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15659/005.jpg</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>WELL-15702</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15702/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15702/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15702/003.jpg</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>WELL-15704</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15704/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15704/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15704/003.jpg</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>WELL-15705</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15705/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15705/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15705/003.jpg</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>WELL-15707</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15707/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15707/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15707/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15707/004.jpg</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>WELL-15709</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15709/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15709/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15709/003.jpg</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>WELL-15802</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15802/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15802/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15802/003.jpg</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>WELL-15804</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15804/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15804/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15804/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15804/004.jpg</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>WELL-15805</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15805/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15805/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15805/003.jpg</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>WELL-15809</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15809/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15809/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15809/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15809/004.jpg</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>WELL-15955</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-15955/001.jpg,https://oleks-netizen.github.io/product-images/WELL-15955/002.jpg,https://oleks-netizen.github.io/product-images/WELL-15955/003.jpg,https://oleks-netizen.github.io/product-images/WELL-15955/004.jpg,https://oleks-netizen.github.io/product-images/WELL-15955/005.jpg</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>WELL-44201</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44201/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44201/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44201/003.jpg,https://oleks-netizen.github.io/product-images/WELL-44201/004.jpg,https://oleks-netizen.github.io/product-images/WELL-44201/005.jpg</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>WELL-44205</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44205/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44205/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44205/003.jpg,https://oleks-netizen.github.io/product-images/WELL-44205/004.jpg</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>WELL-44206</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44206/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44206/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44206/003.jpg,https://oleks-netizen.github.io/product-images/WELL-44206/004.jpg</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>WELL-44208</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44208/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44208/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44208/003.jpg,https://oleks-netizen.github.io/product-images/WELL-44208/004.jpg</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>WELL-44209</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44209/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44209/002.jpg</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>WELL-44210</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44210/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44210/002.jpg</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>WELL-44213</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44213/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44213/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44213/003.jpg,https://oleks-netizen.github.io/product-images/WELL-44213/004.jpg</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>WELL-44312</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44312/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44312/002.jpg</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>WELL-44415</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44415/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44415/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44415/003.jpg</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>WELL-44419</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44419/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44419/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44419/003.jpg</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>WELL-44425</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44425/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44425/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44425/003.jpg</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>WELL-44429</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44429/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44429/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44429/003.jpg</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>WELL-44444</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44444/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44444/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44444/003.jpg</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>WELL-44601</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44601/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44601/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44601/003.jpg,https://oleks-netizen.github.io/product-images/WELL-44601/004.jpg</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>WELL-44603</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44603/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44603/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44603/003.jpg,https://oleks-netizen.github.io/product-images/WELL-44603/004.jpg</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>WELL-44606</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44606/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44606/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44606/003.jpg,https://oleks-netizen.github.io/product-images/WELL-44606/004.jpg,https://oleks-netizen.github.io/product-images/WELL-44606/005.jpg</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>WELL-44607</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44607/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44607/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44607/003.jpg,https://oleks-netizen.github.io/product-images/WELL-44607/004.jpg,https://oleks-netizen.github.io/product-images/WELL-44607/005.jpg</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>WELL-44608</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-44608/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44608/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44608/003.jpg,https://oleks-netizen.github.io/product-images/WELL-44608/004.jpg</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>WELL-45352</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-45352/001.jpg,https://oleks-netizen.github.io/product-images/WELL-45352/002.jpg,https://oleks-netizen.github.io/product-images/WELL-45352/003.jpg,https://oleks-netizen.github.io/product-images/WELL-45352/004.jpg</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>WELL-45505</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-45505/001.jpg,https://oleks-netizen.github.io/product-images/WELL-45505/002.jpg,https://oleks-netizen.github.io/product-images/WELL-45505/003.jpg,https://oleks-netizen.github.io/product-images/WELL-45505/004.jpg</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>WELL-45508</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-45508/001.jpg,https://oleks-netizen.github.io/product-images/WELL-45508/002.jpg,https://oleks-netizen.github.io/product-images/WELL-45508/003.jpg,https://oleks-netizen.github.io/product-images/WELL-45508/004.jpg</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>WELL-45510</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-45510/001.jpg,https://oleks-netizen.github.io/product-images/WELL-45510/002.jpg,https://oleks-netizen.github.io/product-images/WELL-45510/003.jpg,https://oleks-netizen.github.io/product-images/WELL-45510/004.jpg</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>WELL-45601</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-45601/001.jpg,https://oleks-netizen.github.io/product-images/WELL-45601/002.jpg,https://oleks-netizen.github.io/product-images/WELL-45601/003.jpg,https://oleks-netizen.github.io/product-images/WELL-45601/004.jpg</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>WELL-45602</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-45602/001.jpg,https://oleks-netizen.github.io/product-images/WELL-45602/002.jpg,https://oleks-netizen.github.io/product-images/WELL-45602/003.jpg,https://oleks-netizen.github.io/product-images/WELL-45602/004.jpg</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>WELL-45603</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-45603/001.jpg,https://oleks-netizen.github.io/product-images/WELL-45603/002.jpg,https://oleks-netizen.github.io/product-images/WELL-45603/003.jpg,https://oleks-netizen.github.io/product-images/WELL-45603/004.jpg</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>WELL-46109</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46109/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46109/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46109/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46109/004.jpg</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>WELL-46110</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46110/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46110/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46110/003.jpg</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>WELL-46111</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46111/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46111/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46111/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46111/004.jpg</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>WELL-46113</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46113/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46113/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46113/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46113/004.jpg</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>WELL-46202</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46202/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46202/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46202/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46202/004.jpg</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>WELL-46407</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46407/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46407/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46407/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46407/004.jpg</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>WELL-46427</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46427/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46427/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46427/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46427/004.jpg</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>WELL-46500</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46500/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46500/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46500/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46500/004.jpg</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>WELL-46501</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46501/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46501/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46501/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46501/004.jpg</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>WELL-46504</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46504/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46504/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46504/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46504/004.jpg,https://oleks-netizen.github.io/product-images/WELL-46504/005.jpg</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>WELL-46507</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46507/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46507/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46507/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46507/004.jpg,https://oleks-netizen.github.io/product-images/WELL-46507/005.jpg</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>WELL-46601</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46601/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46601/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46601/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46601/004.jpg</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>WELL-46707</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46707/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46707/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46707/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46707/004.jpg,https://oleks-netizen.github.io/product-images/WELL-46707/005.jpg</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>WELL-46708</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46708/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46708/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46708/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46708/004.jpg,https://oleks-netizen.github.io/product-images/WELL-46708/005.jpg</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>WELL-46711</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46711/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46711/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46711/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46711/004.jpg,https://oleks-netizen.github.io/product-images/WELL-46711/005.jpg</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>WELL-46900</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46900/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46900/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46900/003.jpg</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>WELL-46904</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46904/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46904/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46904/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46904/004.jpg</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>WELL-46908</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46908/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46908/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46908/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46908/004.jpg</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>WELL-46909</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46909/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46909/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46909/003.jpg</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>WELL-47208</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-47208/001.jpg,https://oleks-netizen.github.io/product-images/WELL-47208/002.jpg,https://oleks-netizen.github.io/product-images/WELL-47208/003.jpg,https://oleks-netizen.github.io/product-images/WELL-47208/004.jpg</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>WELL-47400</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-47400/001.jpg,https://oleks-netizen.github.io/product-images/WELL-47400/002.jpg,https://oleks-netizen.github.io/product-images/WELL-47400/003.jpg,https://oleks-netizen.github.io/product-images/WELL-47400/004.jpg</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>WELL-47401</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-47401/001.jpg,https://oleks-netizen.github.io/product-images/WELL-47401/002.jpg,https://oleks-netizen.github.io/product-images/WELL-47401/003.jpg,https://oleks-netizen.github.io/product-images/WELL-47401/004.jpg</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>WELL-47404</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-47404/001.jpg,https://oleks-netizen.github.io/product-images/WELL-47404/002.jpg,https://oleks-netizen.github.io/product-images/WELL-47404/003.jpg,https://oleks-netizen.github.io/product-images/WELL-47404/004.jpg,https://oleks-netizen.github.io/product-images/WELL-47404/005.jpg</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>WELL-47409</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-47409/001.jpg,https://oleks-netizen.github.io/product-images/WELL-47409/002.jpg,https://oleks-netizen.github.io/product-images/WELL-47409/003.jpg,https://oleks-netizen.github.io/product-images/WELL-47409/004.jpg</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>WELL-55354</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-55354/001.jpg,https://oleks-netizen.github.io/product-images/WELL-55354/002.jpg,https://oleks-netizen.github.io/product-images/WELL-55354/003.jpg,https://oleks-netizen.github.io/product-images/WELL-55354/004.jpg</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>WELL-56300</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56300/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56300/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56300/003.jpg,https://oleks-netizen.github.io/product-images/WELL-56300/004.jpg</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>WELL-56304</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56304/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56304/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56304/003.jpg,https://oleks-netizen.github.io/product-images/WELL-56304/004.jpg,https://oleks-netizen.github.io/product-images/WELL-56304/005.jpg</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>WELL-56310</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56310/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56310/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56310/003.jpg</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>WELL-56500</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56500/001.jpg</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>WELL-56600</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56600/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56600/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56600/003.jpg,https://oleks-netizen.github.io/product-images/WELL-56600/004.jpg,https://oleks-netizen.github.io/product-images/WELL-56600/005.jpg</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>WELL-56604</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56604/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56604/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56604/003.jpg,https://oleks-netizen.github.io/product-images/WELL-56604/004.jpg,https://oleks-netizen.github.io/product-images/WELL-56604/005.jpg</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>WELL-56605</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56605/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56605/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56605/003.jpg,https://oleks-netizen.github.io/product-images/WELL-56605/004.jpg,https://oleks-netizen.github.io/product-images/WELL-56605/005.jpg</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>WELL-56609</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56609/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56609/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56609/003.jpg,https://oleks-netizen.github.io/product-images/WELL-56609/004.jpg,https://oleks-netizen.github.io/product-images/WELL-56609/005.jpg</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>WELL-56630</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56630/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56630/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56630/003.jpg,https://oleks-netizen.github.io/product-images/WELL-56630/004.jpg</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>WELL-56631</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56631/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56631/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56631/003.jpg,https://oleks-netizen.github.io/product-images/WELL-56631/004.jpg</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>WELL-56902</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56902/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56902/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56902/003.jpg,https://oleks-netizen.github.io/product-images/WELL-56902/004.jpg</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>WELL-56907</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-56907/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56907/002.jpg</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>WELL-57806</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-57806/001.jpg,https://oleks-netizen.github.io/product-images/WELL-57806/002.jpg,https://oleks-netizen.github.io/product-images/WELL-57806/003.jpg,https://oleks-netizen.github.io/product-images/WELL-57806/004.jpg</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>WELL-57808</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-57808/001.jpg,https://oleks-netizen.github.io/product-images/WELL-57808/002.jpg,https://oleks-netizen.github.io/product-images/WELL-57808/003.jpg,https://oleks-netizen.github.io/product-images/WELL-57808/004.jpg</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>WELL-57809</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-57809/001.jpg,https://oleks-netizen.github.io/product-images/WELL-57809/002.jpg,https://oleks-netizen.github.io/product-images/WELL-57809/003.jpg,https://oleks-netizen.github.io/product-images/WELL-57809/004.jpg</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>WELL-58001</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-58001/001.jpg,https://oleks-netizen.github.io/product-images/WELL-58001/002.jpg,https://oleks-netizen.github.io/product-images/WELL-58001/003.jpg,https://oleks-netizen.github.io/product-images/WELL-58001/004.jpg</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>WELL-58004</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-58004/001.jpg,https://oleks-netizen.github.io/product-images/WELL-58004/002.jpg,https://oleks-netizen.github.io/product-images/WELL-58004/003.jpg,https://oleks-netizen.github.io/product-images/WELL-58004/004.jpg</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>WELL-58010</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-58010/001.jpg,https://oleks-netizen.github.io/product-images/WELL-58010/002.jpg,https://oleks-netizen.github.io/product-images/WELL-58010/003.jpg,https://oleks-netizen.github.io/product-images/WELL-58010/004.jpg</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>WELL-58013</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-58013/001.jpg,https://oleks-netizen.github.io/product-images/WELL-58013/002.jpg,https://oleks-netizen.github.io/product-images/WELL-58013/003.jpg,https://oleks-netizen.github.io/product-images/WELL-58013/004.jpg</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>WELL-58411</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-58411/001.jpg,https://oleks-netizen.github.io/product-images/WELL-58411/002.jpg,https://oleks-netizen.github.io/product-images/WELL-58411/003.jpg,https://oleks-netizen.github.io/product-images/WELL-58411/004.jpg,https://oleks-netizen.github.io/product-images/WELL-58411/005.jpg</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>WELL-58412</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-58412/001.jpg,https://oleks-netizen.github.io/product-images/WELL-58412/002.jpg,https://oleks-netizen.github.io/product-images/WELL-58412/003.jpg,https://oleks-netizen.github.io/product-images/WELL-58412/004.jpg</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>WELL-58501</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-58501/001.jpg,https://oleks-netizen.github.io/product-images/WELL-58501/002.jpg,https://oleks-netizen.github.io/product-images/WELL-58501/003.jpg,https://oleks-netizen.github.io/product-images/WELL-58501/004.jpg</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>WELL-60003</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60003/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60003/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60003/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60003/004.jpg</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>WELL-60004</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60004/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60004/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60004/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60004/004.jpg</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>WELL-60009</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60009/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60009/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60009/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60009/004.jpg</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>WELL-60303</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60303/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60303/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60303/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60303/004.jpg,https://oleks-netizen.github.io/product-images/WELL-60303/005.jpg</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>WELL-60305</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60305/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60305/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60305/003.jpg</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>WELL-60403</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60403/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60403/002.jpg</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>WELL-60408</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60408/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60408/002.jpg</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>WELL-60411</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60411/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60411/002.jpg</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>WELL-60413</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60413/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60413/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60413/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60413/004.jpg</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>WELL-60500</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60500/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60500/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60500/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60500/004.jpg</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>WELL-60501</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60501/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60501/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60501/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60501/004.jpg</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>WELL-60509</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60509/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60509/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60509/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60509/004.jpg</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>WELL-60510</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60510/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60510/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60510/003.jpg</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>WELL-60604</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60604/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60604/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60604/003.jpg</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>WELL-60609</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60609/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60609/002.jpg</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>WELL-60610</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60610/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60610/002.jpg</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>WELL-60654</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60654/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60654/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60654/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60654/004.jpg</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>WELL-60711</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60711/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60711/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60711/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60711/004.jpg</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>WELL-60805</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60805/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60805/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60805/003.jpg</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>WELL-60806</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60806/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60806/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60806/003.jpg</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>WELL-60814</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60814/001.jpg</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>WELL-60824</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60824/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60824/002.jpg</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>WELL-60902</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60902/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60902/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60902/003.jpg</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>WELL-60903</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60903/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60903/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60903/003.jpg</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>WELL-60905</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60905/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60905/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60905/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60905/004.jpg</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>WELL-60907</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60907/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60907/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60907/003.jpg</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>WELL-61001</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61001/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61001/002.jpg</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>WELL-61004</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61004/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61004/002.jpg</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>WELL-61006</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61006/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61006/002.jpg</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>WELL-61007</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61007/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61007/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61007/003.jpg,https://oleks-netizen.github.io/product-images/WELL-61007/004.jpg,https://oleks-netizen.github.io/product-images/WELL-61007/005.jpg</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>WELL-61010</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61010/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61010/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61010/003.jpg</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>WELL-61024</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61024/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61024/002.jpg</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>WELL-61030</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61030/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61030/002.jpg</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>WELL-61035</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61035/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61035/002.jpg</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>WELL-61036</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61036/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61036/002.jpg</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>WELL-61301</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61301/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61301/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61301/003.jpg</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>WELL-61302</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61302/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61302/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61302/003.jpg</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>WELL-61303</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61303/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61303/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61303/003.jpg</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>WELL-61400</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61400/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61400/002.jpg</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>WELL-61503</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61503/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61503/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61503/003.jpg,https://oleks-netizen.github.io/product-images/WELL-61503/004.jpg</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>WELL-61602</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61602/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61602/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61602/003.jpg,https://oleks-netizen.github.io/product-images/WELL-61602/004.jpg,https://oleks-netizen.github.io/product-images/WELL-61602/005.jpg</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>WELL-61610</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61610/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61610/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61610/003.jpg,https://oleks-netizen.github.io/product-images/WELL-61610/004.jpg</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>WELL-61614</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61614/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61614/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61614/003.jpg</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>WELL-61804</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61804/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61804/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61804/003.jpg</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>WELL-62200</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-62200/001.jpg,https://oleks-netizen.github.io/product-images/WELL-62200/002.jpg,https://oleks-netizen.github.io/product-images/WELL-62200/003.jpg,https://oleks-netizen.github.io/product-images/WELL-62200/004.jpg</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-05-03 18:11:24
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,27 +436,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>125V1FX92-BLACK</t>
+          <t>1065618885</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/125V1FX92-BLACK/001.jpg,https://oleks-netizen.github.io/product-images/125V1FX92-BLACK/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/1065618885/001.jpg,https://oleks-netizen.github.io/product-images/1065618885/002.jpg,https://oleks-netizen.github.io/product-images/1065618885/003.jpg,https://oleks-netizen.github.io/product-images/1065618885/004.jpg,https://oleks-netizen.github.io/product-images/1065618885/006.jpg,https://oleks-netizen.github.io/product-images/1065618885/007.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>125V1GENAV37-BLACK</t>
+          <t>30311066</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/125V1GENAV37-BLACK/001.jpg,https://oleks-netizen.github.io/product-images/125V1GENAV37-BLACK/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/30311066/001.jpg,https://oleks-netizen.github.io/product-images/30311066/002.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -466,12 +466,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>150V1GENAV36-BLACK</t>
+          <t>30311067</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/150V1GENAV36-BLACK/001.jpg,https://oleks-netizen.github.io/product-images/150V1GENAV36-BLACK/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/30311067/001.jpg,https://oleks-netizen.github.io/product-images/30311067/002.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -481,12 +481,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>150VFX85-BLACK</t>
+          <t>30311068</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/150VFX85-BLACK/001.jpg,https://oleks-netizen.github.io/product-images/150VFX85-BLACK/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/30311068/001.jpg,https://oleks-netizen.github.io/product-images/30311068/002.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -496,27 +496,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18010</t>
+          <t>31111120</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/18010/001.jpg,https://oleks-netizen.github.io/product-images/18010/002.jpg,https://oleks-netizen.github.io/product-images/18010/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/31111120/001.jpg,https://oleks-netizen.github.io/product-images/31111120/003.jpg,https://oleks-netizen.github.io/product-images/31111120/004.jpg,https://oleks-netizen.github.io/product-images/31111120/005.jpg,https://oleks-netizen.github.io/product-images/31111120/006.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18240</t>
+          <t>31211120</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/18240/001.jpg,https://oleks-netizen.github.io/product-images/18240/002.jpg,https://oleks-netizen.github.io/product-images/18240/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/31211120/001.jpg,https://oleks-netizen.github.io/product-images/31211120/002.jpg,https://oleks-netizen.github.io/product-images/31211120/003.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -526,166 +526,391 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BN-BELT-3-RAVEN</t>
+          <t>50223060</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BELT-3-RAVEN/001.jpg,https://oleks-netizen.github.io/product-images/BN-BELT-3-RAVEN/002.jpg,https://oleks-netizen.github.io/product-images/BN-BELT-3-RAVEN/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/50223060/001.jpg,https://oleks-netizen.github.io/product-images/50223060/002.jpg,https://oleks-netizen.github.io/product-images/50223060/003.jpg,https://oleks-netizen.github.io/product-images/50223060/004.jpg,https://oleks-netizen.github.io/product-images/50223060/005.jpg,https://oleks-netizen.github.io/product-images/50223060/007.jpg,https://oleks-netizen.github.io/product-images/50223060/008.jpg,https://oleks-netizen.github.io/product-images/50223060/009.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BN-BELT-8-RAVEN</t>
+          <t>50223161</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BELT-8-RAVEN/001.jpg,https://oleks-netizen.github.io/product-images/BN-BELT-8-RAVEN/002.jpg,https://oleks-netizen.github.io/product-images/BN-BELT-8-RAVEN/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/50223161/001.jpg,https://oleks-netizen.github.io/product-images/50223161/002.jpg,https://oleks-netizen.github.io/product-images/50223161/003.jpg,https://oleks-netizen.github.io/product-images/50223161/005.jpg,https://oleks-netizen.github.io/product-images/50223161/006.jpg,https://oleks-netizen.github.io/product-images/50223161/007.jpg,https://oleks-netizen.github.io/product-images/50223161/008.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BS70106-01</t>
+          <t>50223401</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BS70106-01/001.jpg,https://oleks-netizen.github.io/product-images/BS70106-01/002.jpg,https://oleks-netizen.github.io/product-images/BS70106-01/003.jpg,https://oleks-netizen.github.io/product-images/BS70106-01/004.jpg,https://oleks-netizen.github.io/product-images/BS70106-01/005.jpg,https://oleks-netizen.github.io/product-images/BS70106-01/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/50223401/001.jpg,https://oleks-netizen.github.io/product-images/50223401/002.jpg,https://oleks-netizen.github.io/product-images/50223401/003.jpg,https://oleks-netizen.github.io/product-images/50223401/004.jpg,https://oleks-netizen.github.io/product-images/50223401/005.jpg,https://oleks-netizen.github.io/product-images/50223401/007.jpg,https://oleks-netizen.github.io/product-images/50223401/008.jpg,https://oleks-netizen.github.io/product-images/50223401/009.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NEW-ALN-010</t>
+          <t>50223406</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/NEW-ALN-010/001.jpg,https://oleks-netizen.github.io/product-images/NEW-ALN-010/002.jpg,https://oleks-netizen.github.io/product-images/NEW-ALN-010/003.jpg,https://oleks-netizen.github.io/product-images/NEW-ALN-010/004.jpg,https://oleks-netizen.github.io/product-images/NEW-ALN-010/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/50223406/001.jpg,https://oleks-netizen.github.io/product-images/50223406/003.jpg,https://oleks-netizen.github.io/product-images/50223406/004.jpg,https://oleks-netizen.github.io/product-images/50223406/005.jpg,https://oleks-netizen.github.io/product-images/50223406/006.jpg,https://oleks-netizen.github.io/product-images/50223406/007.jpg,https://oleks-netizen.github.io/product-images/50223406/008.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NW-TUR-35K-0014</t>
+          <t>51411101</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/NW-TUR-35K-0014/001.jpg,https://oleks-netizen.github.io/product-images/NW-TUR-35K-0014/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411101/001.jpg,https://oleks-netizen.github.io/product-images/51411101/002.jpg,https://oleks-netizen.github.io/product-images/51411101/003.jpg,https://oleks-netizen.github.io/product-images/51411101/004.jpg,https://oleks-netizen.github.io/product-images/51411101/006.jpg,https://oleks-netizen.github.io/product-images/51411101/007.jpg,https://oleks-netizen.github.io/product-images/51411101/008.jpg,https://oleks-netizen.github.io/product-images/51411101/009.jpg,https://oleks-netizen.github.io/product-images/51411101/010.jpg,https://oleks-netizen.github.io/product-images/51411101/011.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NW-TUR-35K-0016</t>
+          <t>53400066</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/NW-TUR-35K-0016/001.jpg,https://oleks-netizen.github.io/product-images/NW-TUR-35K-0016/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400066/001.jpg,https://oleks-netizen.github.io/product-images/53400066/002.jpg,https://oleks-netizen.github.io/product-images/53400066/004.jpg,https://oleks-netizen.github.io/product-images/53400066/005.jpg,https://oleks-netizen.github.io/product-images/53400066/006.jpg,https://oleks-netizen.github.io/product-images/53400066/007.jpg,https://oleks-netizen.github.io/product-images/53400066/008.jpg,https://oleks-netizen.github.io/product-images/53400066/009.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NWKZ-38MM-KIT-006</t>
+          <t>53400067</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/NWKZ-38MM-KIT-006/001.jpg,https://oleks-netizen.github.io/product-images/NWKZ-38MM-KIT-006/002.jpg,https://oleks-netizen.github.io/product-images/NWKZ-38MM-KIT-006/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400067/001.jpg,https://oleks-netizen.github.io/product-images/53400067/002.jpg,https://oleks-netizen.github.io/product-images/53400067/003.jpg,https://oleks-netizen.github.io/product-images/53400067/004.jpg,https://oleks-netizen.github.io/product-images/53400067/005.jpg,https://oleks-netizen.github.io/product-images/53400067/007.jpg,https://oleks-netizen.github.io/product-images/53400067/008.jpg,https://oleks-netizen.github.io/product-images/53400067/009.jpg,https://oleks-netizen.github.io/product-images/53400067/010.jpg,https://oleks-netizen.github.io/product-images/53400067/011.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>V1125FX01-BLACK</t>
+          <t>54650001</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/V1125FX01-BLACK/001.jpg,https://oleks-netizen.github.io/product-images/V1125FX01-BLACK/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/54650001/001.jpg,https://oleks-netizen.github.io/product-images/54650001/002.jpg,https://oleks-netizen.github.io/product-images/54650001/003.jpg,https://oleks-netizen.github.io/product-images/54650001/004.jpg,https://oleks-netizen.github.io/product-images/54650001/005.jpg,https://oleks-netizen.github.io/product-images/54650001/006.jpg,https://oleks-netizen.github.io/product-images/54650001/007.jpg,https://oleks-netizen.github.io/product-images/54650001/008.jpg,https://oleks-netizen.github.io/product-images/54650001/010.jpg,https://oleks-netizen.github.io/product-images/54650001/011.jpg,https://oleks-netizen.github.io/product-images/54650001/012.jpg,https://oleks-netizen.github.io/product-images/54650001/013.jpg,https://oleks-netizen.github.io/product-images/54650001/014.jpg,https://oleks-netizen.github.io/product-images/54650001/015.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>V1N-GEN4R-125X2</t>
+          <t>80460406</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/V1N-GEN4R-125X2/001.jpg,https://oleks-netizen.github.io/product-images/V1N-GEN4R-125X2/002.jpg,https://oleks-netizen.github.io/product-images/V1N-GEN4R-125X2/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/80460406/001.jpg,https://oleks-netizen.github.io/product-images/80460406/002.jpg,https://oleks-netizen.github.io/product-images/80460406/003.jpg,https://oleks-netizen.github.io/product-images/80460406/004.jpg,https://oleks-netizen.github.io/product-images/80460406/005.jpg,https://oleks-netizen.github.io/product-images/80460406/006.jpg,https://oleks-netizen.github.io/product-images/80460406/007.jpg,https://oleks-netizen.github.io/product-images/80460406/008.jpg,https://oleks-netizen.github.io/product-images/80460406/010.jpg,https://oleks-netizen.github.io/product-images/80460406/011.jpg,https://oleks-netizen.github.io/product-images/80460406/012.jpg,https://oleks-netizen.github.io/product-images/80460406/013.jpg,https://oleks-netizen.github.io/product-images/80460406/014.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>V1N-GEN4R-125X3</t>
+          <t>80460419</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/V1N-GEN4R-125X3/001.jpg,https://oleks-netizen.github.io/product-images/V1N-GEN4R-125X3/002.jpg,https://oleks-netizen.github.io/product-images/V1N-GEN4R-125X3/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/80460419/001.jpg,https://oleks-netizen.github.io/product-images/80460419/002.jpg,https://oleks-netizen.github.io/product-images/80460419/003.jpg,https://oleks-netizen.github.io/product-images/80460419/004.jpg,https://oleks-netizen.github.io/product-images/80460419/005.jpg,https://oleks-netizen.github.io/product-images/80460419/006.jpg,https://oleks-netizen.github.io/product-images/80460419/007.jpg,https://oleks-netizen.github.io/product-images/80460419/008.jpg,https://oleks-netizen.github.io/product-images/80460419/009.jpg,https://oleks-netizen.github.io/product-images/80460419/010.jpg,https://oleks-netizen.github.io/product-images/80460419/011.jpg,https://oleks-netizen.github.io/product-images/80460419/012.jpg,https://oleks-netizen.github.io/product-images/80460419/014.jpg</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BN-BELT-3-FLINT</t>
+          <t>BN-PM-12-light-beige</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BELT-3-FLINT/002.jpg,https://oleks-netizen.github.io/product-images/BN-BELT-3-FLINT/003.jpg,https://oleks-netizen.github.io/product-images/BN-BELT-3-FLINT/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-PM-12-light-beige/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-light-beige/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-light-beige/004.jpg</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BN-PM-12-navy-blue</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-PM-12-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-navy-blue/003.jpg</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BN-PM-12-red</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-PM-12-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-red/003.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-red/004.jpg</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DRS17009-1</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRS17009-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DRS17012-1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRS17012-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/003.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DRS17015-1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRS17015-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DRS17038-1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRS17038-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DRS17082-1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRS17082-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DRS17083-1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRS17083-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/003.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DRS17203-1-26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRS17203-1-26/001.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/002.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/003.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/005.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/006.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/007.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/008.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/009.jpg</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DRS17306-1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRS17306-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/003.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DRS17708-1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRS17708-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/003.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DRS17927-1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/DRS17927-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/003.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/008.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>L340-037744</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L340-037744/001.jpg,https://oleks-netizen.github.io/product-images/L340-037744/003.jpg,https://oleks-netizen.github.io/product-images/L340-037744/004.jpg,https://oleks-netizen.github.io/product-images/L340-037744/005.jpg,https://oleks-netizen.github.io/product-images/L340-037744/006.jpg,https://oleks-netizen.github.io/product-images/L340-037744/007.jpg,https://oleks-netizen.github.io/product-images/L340-037744/008.jpg,https://oleks-netizen.github.io/product-images/L340-037744/009.jpg,https://oleks-netizen.github.io/product-images/L340-037744/010.jpg</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ua-33mkr-0014-1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/ua-33mkr-0014-1/001.jpg</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>WELL-11705</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/WELL-11705/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11705/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11705/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11705/005.jpg</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-05-04 17:12:53
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,57 +436,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1065618885</t>
+          <t>1102060033-96492</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1065618885/001.jpg,https://oleks-netizen.github.io/product-images/1065618885/002.jpg,https://oleks-netizen.github.io/product-images/1065618885/003.jpg,https://oleks-netizen.github.io/product-images/1065618885/004.jpg,https://oleks-netizen.github.io/product-images/1065618885/006.jpg,https://oleks-netizen.github.io/product-images/1065618885/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/1102060033-96492/001.jpg,https://oleks-netizen.github.io/product-images/1102060033-96492/002.jpg,https://oleks-netizen.github.io/product-images/1102060033-96492/004.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>30311066</t>
+          <t>463110</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/30311066/001.jpg,https://oleks-netizen.github.io/product-images/30311066/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/463110/001.jpg,https://oleks-netizen.github.io/product-images/463110/002.jpg,https://oleks-netizen.github.io/product-images/463110/003.jpg,https://oleks-netizen.github.io/product-images/463110/004.jpg,https://oleks-netizen.github.io/product-images/463110/005.jpg,https://oleks-netizen.github.io/product-images/463110/007.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>30311067</t>
+          <t>463120</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/30311067/001.jpg,https://oleks-netizen.github.io/product-images/30311067/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/463120/001.jpg,https://oleks-netizen.github.io/product-images/463120/002.jpg,https://oleks-netizen.github.io/product-images/463120/004.jpg,https://oleks-netizen.github.io/product-images/463120/005.jpg,https://oleks-netizen.github.io/product-images/463120/006.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>30311068</t>
+          <t>463610</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/30311068/001.jpg,https://oleks-netizen.github.io/product-images/30311068/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/463610/001.jpg,https://oleks-netizen.github.io/product-images/463610/002.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -496,57 +496,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>31111120</t>
+          <t>5241701</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/31111120/001.jpg,https://oleks-netizen.github.io/product-images/31111120/003.jpg,https://oleks-netizen.github.io/product-images/31111120/004.jpg,https://oleks-netizen.github.io/product-images/31111120/005.jpg,https://oleks-netizen.github.io/product-images/31111120/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5241701/001.jpg,https://oleks-netizen.github.io/product-images/5241701/002.jpg,https://oleks-netizen.github.io/product-images/5241701/004.jpg,https://oleks-netizen.github.io/product-images/5241701/005.jpg,https://oleks-netizen.github.io/product-images/5241701/006.jpg,https://oleks-netizen.github.io/product-images/5241701/007.jpg,https://oleks-netizen.github.io/product-images/5241701/008.jpg,https://oleks-netizen.github.io/product-images/5241701/009.jpg,https://oleks-netizen.github.io/product-images/5241701/010.jpg,https://oleks-netizen.github.io/product-images/5241701/011.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>31211120</t>
+          <t>5241801</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/31211120/001.jpg,https://oleks-netizen.github.io/product-images/31211120/002.jpg,https://oleks-netizen.github.io/product-images/31211120/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5241801/001.jpg,https://oleks-netizen.github.io/product-images/5241801/003.jpg,https://oleks-netizen.github.io/product-images/5241801/004.jpg,https://oleks-netizen.github.io/product-images/5241801/005.jpg,https://oleks-netizen.github.io/product-images/5241801/006.jpg,https://oleks-netizen.github.io/product-images/5241801/007.jpg,https://oleks-netizen.github.io/product-images/5241801/008.jpg,https://oleks-netizen.github.io/product-images/5241801/009.jpg,https://oleks-netizen.github.io/product-images/5241801/010.jpg,https://oleks-netizen.github.io/product-images/5241801/011.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>50223060</t>
+          <t>5246801W</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/50223060/001.jpg,https://oleks-netizen.github.io/product-images/50223060/002.jpg,https://oleks-netizen.github.io/product-images/50223060/003.jpg,https://oleks-netizen.github.io/product-images/50223060/004.jpg,https://oleks-netizen.github.io/product-images/50223060/005.jpg,https://oleks-netizen.github.io/product-images/50223060/007.jpg,https://oleks-netizen.github.io/product-images/50223060/008.jpg,https://oleks-netizen.github.io/product-images/50223060/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/5246801W/001.jpg,https://oleks-netizen.github.io/product-images/5246801W/002.jpg,https://oleks-netizen.github.io/product-images/5246801W/003.jpg,https://oleks-netizen.github.io/product-images/5246801W/004.jpg,https://oleks-netizen.github.io/product-images/5246801W/006.jpg,https://oleks-netizen.github.io/product-images/5246801W/007.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>50223161</t>
+          <t>bx3101</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/50223161/001.jpg,https://oleks-netizen.github.io/product-images/50223161/002.jpg,https://oleks-netizen.github.io/product-images/50223161/003.jpg,https://oleks-netizen.github.io/product-images/50223161/005.jpg,https://oleks-netizen.github.io/product-images/50223161/006.jpg,https://oleks-netizen.github.io/product-images/50223161/007.jpg,https://oleks-netizen.github.io/product-images/50223161/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/bx3101/001.jpg,https://oleks-netizen.github.io/product-images/bx3101/002.jpg,https://oleks-netizen.github.io/product-images/bx3101/003.jpg,https://oleks-netizen.github.io/product-images/bx3101/004.jpg,https://oleks-netizen.github.io/product-images/bx3101/005.jpg,https://oleks-netizen.github.io/product-images/bx3101/007.jpg,https://oleks-netizen.github.io/product-images/bx3101/008.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -556,222 +556,222 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>50223401</t>
+          <t>bx3101br</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/50223401/001.jpg,https://oleks-netizen.github.io/product-images/50223401/002.jpg,https://oleks-netizen.github.io/product-images/50223401/003.jpg,https://oleks-netizen.github.io/product-images/50223401/004.jpg,https://oleks-netizen.github.io/product-images/50223401/005.jpg,https://oleks-netizen.github.io/product-images/50223401/007.jpg,https://oleks-netizen.github.io/product-images/50223401/008.jpg,https://oleks-netizen.github.io/product-images/50223401/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/bx3101br/001.jpg,https://oleks-netizen.github.io/product-images/bx3101br/002.jpg,https://oleks-netizen.github.io/product-images/bx3101br/003.jpg,https://oleks-netizen.github.io/product-images/bx3101br/004.jpg,https://oleks-netizen.github.io/product-images/bx3101br/006.jpg,https://oleks-netizen.github.io/product-images/bx3101br/007.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>50223406</t>
+          <t>FA-0910-4lx</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/50223406/001.jpg,https://oleks-netizen.github.io/product-images/50223406/003.jpg,https://oleks-netizen.github.io/product-images/50223406/004.jpg,https://oleks-netizen.github.io/product-images/50223406/005.jpg,https://oleks-netizen.github.io/product-images/50223406/006.jpg,https://oleks-netizen.github.io/product-images/50223406/007.jpg,https://oleks-netizen.github.io/product-images/50223406/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/FA-0910-4lx/001.jpg,https://oleks-netizen.github.io/product-images/FA-0910-4lx/002.jpg,https://oleks-netizen.github.io/product-images/FA-0910-4lx/004.jpg,https://oleks-netizen.github.io/product-images/FA-0910-4lx/005.jpg,https://oleks-netizen.github.io/product-images/FA-0910-4lx/006.jpg,https://oleks-netizen.github.io/product-images/FA-0910-4lx/007.jpg,https://oleks-netizen.github.io/product-images/FA-0910-4lx/008.jpg,https://oleks-netizen.github.io/product-images/FA-0910-4lx/009.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>51411101</t>
+          <t>FA-5402-4lx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/51411101/001.jpg,https://oleks-netizen.github.io/product-images/51411101/002.jpg,https://oleks-netizen.github.io/product-images/51411101/003.jpg,https://oleks-netizen.github.io/product-images/51411101/004.jpg,https://oleks-netizen.github.io/product-images/51411101/006.jpg,https://oleks-netizen.github.io/product-images/51411101/007.jpg,https://oleks-netizen.github.io/product-images/51411101/008.jpg,https://oleks-netizen.github.io/product-images/51411101/009.jpg,https://oleks-netizen.github.io/product-images/51411101/010.jpg,https://oleks-netizen.github.io/product-images/51411101/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/FA-5402-4lx/001.jpg,https://oleks-netizen.github.io/product-images/FA-5402-4lx/002.jpg,https://oleks-netizen.github.io/product-images/FA-5402-4lx/003.jpg,https://oleks-netizen.github.io/product-images/FA-5402-4lx/004.jpg,https://oleks-netizen.github.io/product-images/FA-5402-4lx/005.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>53400066</t>
+          <t>FC-5402-4lx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53400066/001.jpg,https://oleks-netizen.github.io/product-images/53400066/002.jpg,https://oleks-netizen.github.io/product-images/53400066/004.jpg,https://oleks-netizen.github.io/product-images/53400066/005.jpg,https://oleks-netizen.github.io/product-images/53400066/006.jpg,https://oleks-netizen.github.io/product-images/53400066/007.jpg,https://oleks-netizen.github.io/product-images/53400066/008.jpg,https://oleks-netizen.github.io/product-images/53400066/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/FC-5402-4lx/001.jpg,https://oleks-netizen.github.io/product-images/FC-5402-4lx/002.jpg,https://oleks-netizen.github.io/product-images/FC-5402-4lx/004.jpg,https://oleks-netizen.github.io/product-images/FC-5402-4lx/005.jpg,https://oleks-netizen.github.io/product-images/FC-5402-4lx/006.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>53400067</t>
+          <t>fz375235_taup</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53400067/001.jpg,https://oleks-netizen.github.io/product-images/53400067/002.jpg,https://oleks-netizen.github.io/product-images/53400067/003.jpg,https://oleks-netizen.github.io/product-images/53400067/004.jpg,https://oleks-netizen.github.io/product-images/53400067/005.jpg,https://oleks-netizen.github.io/product-images/53400067/007.jpg,https://oleks-netizen.github.io/product-images/53400067/008.jpg,https://oleks-netizen.github.io/product-images/53400067/009.jpg,https://oleks-netizen.github.io/product-images/53400067/010.jpg,https://oleks-netizen.github.io/product-images/53400067/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/fz375235_taup/001.jpg,https://oleks-netizen.github.io/product-images/fz375235_taup/002.jpg,https://oleks-netizen.github.io/product-images/fz375235_taup/003.jpg,https://oleks-netizen.github.io/product-images/fz375235_taup/004.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>54650001</t>
+          <t>fz376023_chok</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/54650001/001.jpg,https://oleks-netizen.github.io/product-images/54650001/002.jpg,https://oleks-netizen.github.io/product-images/54650001/003.jpg,https://oleks-netizen.github.io/product-images/54650001/004.jpg,https://oleks-netizen.github.io/product-images/54650001/005.jpg,https://oleks-netizen.github.io/product-images/54650001/006.jpg,https://oleks-netizen.github.io/product-images/54650001/007.jpg,https://oleks-netizen.github.io/product-images/54650001/008.jpg,https://oleks-netizen.github.io/product-images/54650001/010.jpg,https://oleks-netizen.github.io/product-images/54650001/011.jpg,https://oleks-netizen.github.io/product-images/54650001/012.jpg,https://oleks-netizen.github.io/product-images/54650001/013.jpg,https://oleks-netizen.github.io/product-images/54650001/014.jpg,https://oleks-netizen.github.io/product-images/54650001/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/fz376023_chok/001.jpg,https://oleks-netizen.github.io/product-images/fz376023_chok/002.jpg,https://oleks-netizen.github.io/product-images/fz376023_chok/004.jpg,https://oleks-netizen.github.io/product-images/fz376023_chok/005.jpg,https://oleks-netizen.github.io/product-images/fz376023_chok/006.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>80460406</t>
+          <t>fz378839_chok</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80460406/001.jpg,https://oleks-netizen.github.io/product-images/80460406/002.jpg,https://oleks-netizen.github.io/product-images/80460406/003.jpg,https://oleks-netizen.github.io/product-images/80460406/004.jpg,https://oleks-netizen.github.io/product-images/80460406/005.jpg,https://oleks-netizen.github.io/product-images/80460406/006.jpg,https://oleks-netizen.github.io/product-images/80460406/007.jpg,https://oleks-netizen.github.io/product-images/80460406/008.jpg,https://oleks-netizen.github.io/product-images/80460406/010.jpg,https://oleks-netizen.github.io/product-images/80460406/011.jpg,https://oleks-netizen.github.io/product-images/80460406/012.jpg,https://oleks-netizen.github.io/product-images/80460406/013.jpg,https://oleks-netizen.github.io/product-images/80460406/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/fz378839_chok/001.jpg,https://oleks-netizen.github.io/product-images/fz378839_chok/002.jpg,https://oleks-netizen.github.io/product-images/fz378839_chok/004.jpg,https://oleks-netizen.github.io/product-images/fz378839_chok/005.jpg,https://oleks-netizen.github.io/product-images/fz378839_chok/006.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>80460419</t>
+          <t>fz379037_dtaup</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80460419/001.jpg,https://oleks-netizen.github.io/product-images/80460419/002.jpg,https://oleks-netizen.github.io/product-images/80460419/003.jpg,https://oleks-netizen.github.io/product-images/80460419/004.jpg,https://oleks-netizen.github.io/product-images/80460419/005.jpg,https://oleks-netizen.github.io/product-images/80460419/006.jpg,https://oleks-netizen.github.io/product-images/80460419/007.jpg,https://oleks-netizen.github.io/product-images/80460419/008.jpg,https://oleks-netizen.github.io/product-images/80460419/009.jpg,https://oleks-netizen.github.io/product-images/80460419/010.jpg,https://oleks-netizen.github.io/product-images/80460419/011.jpg,https://oleks-netizen.github.io/product-images/80460419/012.jpg,https://oleks-netizen.github.io/product-images/80460419/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/fz379037_dtaup/001.jpg,https://oleks-netizen.github.io/product-images/fz379037_dtaup/002.jpg,https://oleks-netizen.github.io/product-images/fz379037_dtaup/003.jpg,https://oleks-netizen.github.io/product-images/fz379037_dtaup/005.jpg,https://oleks-netizen.github.io/product-images/fz379037_dtaup/006.jpg</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BN-PM-12-light-beige</t>
+          <t>GA-5402-4lx</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-PM-12-light-beige/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-light-beige/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-light-beige/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/GA-5402-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GA-5402-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GA-5402-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GA-5402-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GA-5402-4lx/006.jpg</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BN-PM-12-navy-blue</t>
+          <t>GA-7310-4lx</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-PM-12-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-navy-blue/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/GA-7310-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GA-7310-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GA-7310-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GA-7310-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GA-7310-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GA-7310-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GA-7310-4lx/008.jpg,https://oleks-netizen.github.io/product-images/GA-7310-4lx/009.jpg,https://oleks-netizen.github.io/product-images/GA-7310-4lx/010.jpg</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BN-PM-12-red</t>
+          <t>GA-9552-4lx</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-PM-12-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-red/003.jpg,https://oleks-netizen.github.io/product-images/BN-PM-12-red/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/GA-9552-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GA-9552-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GA-9552-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GA-9552-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GA-9552-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GA-9552-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GA-9552-4lx/008.jpg,https://oleks-netizen.github.io/product-images/GA-9552-4lx/009.jpg,https://oleks-netizen.github.io/product-images/GA-9552-4lx/010.jpg,https://oleks-netizen.github.io/product-images/GA-9552-4lx/011.jpg</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DRS17009-1</t>
+          <t>GC-5402-4lx</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/DRS17009-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17009-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/GC-5402-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GC-5402-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GC-5402-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GC-5402-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GC-5402-4lx/006.jpg</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DRS17012-1</t>
+          <t>GC-9552-4lx</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/DRS17012-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/003.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17012-1/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/GC-9552-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GC-9552-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GC-9552-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GC-9552-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GC-9552-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GC-9552-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GC-9552-4lx/008.jpg,https://oleks-netizen.github.io/product-images/GC-9552-4lx/009.jpg,https://oleks-netizen.github.io/product-images/GC-9552-4lx/010.jpg</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DRS17015-1</t>
+          <t>GSE-5565-4lx</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/DRS17015-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17015-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/GSE-5565-4lx/001.jpg,https://oleks-netizen.github.io/product-images/GSE-5565-4lx/002.jpg,https://oleks-netizen.github.io/product-images/GSE-5565-4lx/003.jpg,https://oleks-netizen.github.io/product-images/GSE-5565-4lx/004.jpg,https://oleks-netizen.github.io/product-images/GSE-5565-4lx/005.jpg,https://oleks-netizen.github.io/product-images/GSE-5565-4lx/006.jpg,https://oleks-netizen.github.io/product-images/GSE-5565-4lx/007.jpg,https://oleks-netizen.github.io/product-images/GSE-5565-4lx/008.jpg</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DRS17038-1</t>
+          <t>GX-7280-3md</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/DRS17038-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17038-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/GX-7280-3md/001.jpg,https://oleks-netizen.github.io/product-images/GX-7280-3md/002.jpg,https://oleks-netizen.github.io/product-images/GX-7280-3md/003.jpg,https://oleks-netizen.github.io/product-images/GX-7280-3md/004.jpg,https://oleks-netizen.github.io/product-images/GX-7280-3md/005.jpg,https://oleks-netizen.github.io/product-images/GX-7280-3md/006.jpg,https://oleks-netizen.github.io/product-images/GX-7280-3md/007.jpg</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -781,136 +781,811 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DRS17082-1</t>
+          <t>HB03334Beige</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/DRS17082-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17082-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/HB03334Beige/001.jpg,https://oleks-netizen.github.io/product-images/HB03334Beige/002.jpg,https://oleks-netizen.github.io/product-images/HB03334Beige/003.jpg,https://oleks-netizen.github.io/product-images/HB03334Beige/004.jpg,https://oleks-netizen.github.io/product-images/HB03334Beige/006.jpg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DRS17083-1</t>
+          <t>HB15295B</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/DRS17083-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/002.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/003.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17083-1/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/HB15295B/001.jpg,https://oleks-netizen.github.io/product-images/HB15295B/002.jpg,https://oleks-netizen.github.io/product-images/HB15295B/003.jpg,https://oleks-netizen.github.io/product-images/HB15295B/004.jpg,https://oleks-netizen.github.io/product-images/HB15295B/005.jpg,https://oleks-netizen.github.io/product-images/HB15295B/007.jpg</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DRS17203-1-26</t>
+          <t>ht-st1-ga1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/DRS17203-1-26/001.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/002.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/003.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/005.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/006.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/007.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/008.jpg,https://oleks-netizen.github.io/product-images/DRS17203-1-26/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ht-st1-ga1/001.jpg,https://oleks-netizen.github.io/product-images/ht-st1-ga1/002.jpg,https://oleks-netizen.github.io/product-images/ht-st1-ga1/003.jpg,https://oleks-netizen.github.io/product-images/ht-st1-ga1/004.jpg,https://oleks-netizen.github.io/product-images/ht-st1-ga1/005.jpg,https://oleks-netizen.github.io/product-images/ht-st1-ga1/006.jpg</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DRS17306-1</t>
+          <t>ht-st1-ga2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/DRS17306-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/003.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17306-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ht-st1-ga2/001.jpg,https://oleks-netizen.github.io/product-images/ht-st1-ga2/002.jpg,https://oleks-netizen.github.io/product-images/ht-st1-ga2/003.jpg,https://oleks-netizen.github.io/product-images/ht-st1-ga2/004.jpg,https://oleks-netizen.github.io/product-images/ht-st1-ga2/005.jpg</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DRS17708-1</t>
+          <t>ht-st1-rb1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/DRS17708-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/003.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17708-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ht-st1-rb1/001.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb1/002.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb1/003.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb1/004.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb1/005.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb1/006.jpg</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DRS17927-1</t>
+          <t>ht-st1-rb2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/DRS17927-1/001.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/003.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/004.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/005.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/006.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/007.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/008.jpg,https://oleks-netizen.github.io/product-images/DRS17927-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ht-st1-rb2/001.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb2/002.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb2/003.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb2/004.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb2/005.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb2/006.jpg</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>L340-037744</t>
+          <t>ht-st1-rb3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L340-037744/001.jpg,https://oleks-netizen.github.io/product-images/L340-037744/003.jpg,https://oleks-netizen.github.io/product-images/L340-037744/004.jpg,https://oleks-netizen.github.io/product-images/L340-037744/005.jpg,https://oleks-netizen.github.io/product-images/L340-037744/006.jpg,https://oleks-netizen.github.io/product-images/L340-037744/007.jpg,https://oleks-netizen.github.io/product-images/L340-037744/008.jpg,https://oleks-netizen.github.io/product-images/L340-037744/009.jpg,https://oleks-netizen.github.io/product-images/L340-037744/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ht-st1-rb3/001.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb3/002.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb3/003.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb3/004.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb3/005.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb3/006.jpg</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ua-33mkr-0014-1</t>
+          <t>ht-st1-rb4</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-33mkr-0014-1/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ht-st1-rb4/001.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb4/002.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb4/003.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb4/004.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb4/005.jpg,https://oleks-netizen.github.io/product-images/ht-st1-rb4/006.jpg</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>WELL-11705</t>
+          <t>ht-st2-ga1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-11705/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11705/003.jpg,https://oleks-netizen.github.io/product-images/WELL-11705/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11705/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ht-st2-ga1/001.jpg,https://oleks-netizen.github.io/product-images/ht-st2-ga1/002.jpg,https://oleks-netizen.github.io/product-images/ht-st2-ga1/003.jpg,https://oleks-netizen.github.io/product-images/ht-st2-ga1/004.jpg,https://oleks-netizen.github.io/product-images/ht-st2-ga1/005.jpg</t>
         </is>
       </c>
       <c r="C33" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ht-st2-rb1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/ht-st2-rb1/001.jpg,https://oleks-netizen.github.io/product-images/ht-st2-rb1/002.jpg,https://oleks-netizen.github.io/product-images/ht-st2-rb1/003.jpg,https://oleks-netizen.github.io/product-images/ht-st2-rb1/004.jpg,https://oleks-netizen.github.io/product-images/ht-st2-rb1/005.jpg,https://oleks-netizen.github.io/product-images/ht-st2-rb1/006.jpg</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ht-st2-rb2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/ht-st2-rb2/001.jpg,https://oleks-netizen.github.io/product-images/ht-st2-rb2/002.jpg,https://oleks-netizen.github.io/product-images/ht-st2-rb2/003.jpg,https://oleks-netizen.github.io/product-images/ht-st2-rb2/004.jpg,https://oleks-netizen.github.io/product-images/ht-st2-rb2/005.jpg,https://oleks-netizen.github.io/product-images/ht-st2-rb2/006.jpg</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ht-st3-rb1</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/ht-st3-rb1/001.jpg,https://oleks-netizen.github.io/product-images/ht-st3-rb1/002.jpg,https://oleks-netizen.github.io/product-images/ht-st3-rb1/003.jpg,https://oleks-netizen.github.io/product-images/ht-st3-rb1/004.jpg,https://oleks-netizen.github.io/product-images/ht-st3-rb1/005.jpg</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>JD4024B</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/JD4024B/001.jpg,https://oleks-netizen.github.io/product-images/JD4024B/003.jpg,https://oleks-netizen.github.io/product-images/JD4024B/004.jpg,https://oleks-netizen.github.io/product-images/JD4024B/005.jpg,https://oleks-netizen.github.io/product-images/JD4024B/006.jpg,https://oleks-netizen.github.io/product-images/JD4024B/007.jpg,https://oleks-netizen.github.io/product-images/JD4024B/008.jpg,https://oleks-netizen.github.io/product-images/JD4024B/009.jpg,https://oleks-netizen.github.io/product-images/JD4024B/010.jpg,https://oleks-netizen.github.io/product-images/JD4024B/011.jpg</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Lim-760FA</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/Lim-760FA/001.jpg,https://oleks-netizen.github.io/product-images/Lim-760FA/002.jpg,https://oleks-netizen.github.io/product-images/Lim-760FA/003.jpg,https://oleks-netizen.github.io/product-images/Lim-760FA/004.jpg,https://oleks-netizen.github.io/product-images/Lim-760FA/006.jpg,https://oleks-netizen.github.io/product-images/Lim-760FA/007.jpg</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Lim-760FC</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/Lim-760FC/001.jpg,https://oleks-netizen.github.io/product-images/Lim-760FC/002.jpg,https://oleks-netizen.github.io/product-images/Lim-760FC/003.jpg,https://oleks-netizen.github.io/product-images/Lim-760FC/005.jpg,https://oleks-netizen.github.io/product-images/Lim-760FC/006.jpg</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Lim-760RE</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/Lim-760RE/001.jpg,https://oleks-netizen.github.io/product-images/Lim-760RE/002.jpg,https://oleks-netizen.github.io/product-images/Lim-760RE/003.jpg,https://oleks-netizen.github.io/product-images/Lim-760RE/004.jpg,https://oleks-netizen.github.io/product-images/Lim-760RE/006.jpg,https://oleks-netizen.github.io/product-images/Lim-760RE/007.jpg,https://oleks-netizen.github.io/product-images/Lim-760RE/008.jpg</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>RA-1304-4lx</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RA-1304-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RA-1304-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RA-1304-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RA-1304-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RA-1304-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RA-1304-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RA-1304-4lx/008.jpg</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>RA-5402-4lx</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RA-5402-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RA-5402-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RA-5402-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RA-5402-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RA-5402-4lx/006.jpg</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>RB-1501-3md</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RB-1501-3md/001.jpg,https://oleks-netizen.github.io/product-images/RB-1501-3md/002.jpg,https://oleks-netizen.github.io/product-images/RB-1501-3md/004.jpg,https://oleks-netizen.github.io/product-images/RB-1501-3md/005.jpg,https://oleks-netizen.github.io/product-images/RB-1501-3md/006.jpg,https://oleks-netizen.github.io/product-images/RB-1501-3md/007.jpg</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>RB-7287-3md</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RB-7287-3md/001.jpg,https://oleks-netizen.github.io/product-images/RB-7287-3md/002.jpg,https://oleks-netizen.github.io/product-images/RB-7287-3md/003.jpg,https://oleks-netizen.github.io/product-images/RB-7287-3md/005.jpg,https://oleks-netizen.github.io/product-images/RB-7287-3md/006.jpg,https://oleks-netizen.github.io/product-images/RB-7287-3md/007.jpg,https://oleks-netizen.github.io/product-images/RB-7287-3md/008.jpg,https://oleks-netizen.github.io/product-images/RB-7287-3md/009.jpg,https://oleks-netizen.github.io/product-images/RB-7287-3md/010.jpg,https://oleks-netizen.github.io/product-images/RB-7287-3md/011.jpg</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>RBw-4027-3md</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RBw-4027-3md/001.jpg,https://oleks-netizen.github.io/product-images/RBw-4027-3md/002.jpg,https://oleks-netizen.github.io/product-images/RBw-4027-3md/003.jpg,https://oleks-netizen.github.io/product-images/RBw-4027-3md/004.jpg,https://oleks-netizen.github.io/product-images/RBw-4027-3md/005.jpg,https://oleks-netizen.github.io/product-images/RBw-4027-3md/006.jpg</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>RC-1819-3md</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RC-1819-3md/001.jpg,https://oleks-netizen.github.io/product-images/RC-1819-3md/002.jpg,https://oleks-netizen.github.io/product-images/RC-1819-3md/004.jpg,https://oleks-netizen.github.io/product-images/RC-1819-3md/005.jpg,https://oleks-netizen.github.io/product-images/RC-1819-3md/006.jpg,https://oleks-netizen.github.io/product-images/RC-1819-3md/007.jpg</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>RC-3724-4lx</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RC-3724-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RC-3724-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RC-3724-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RC-3724-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RC-3724-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RC-3724-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RC-3724-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RC-3724-4lx/009.jpg</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>RC-5402-4lx</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RC-5402-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RC-5402-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RC-5402-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RC-5402-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RC-5402-4lx/006.jpg</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>RC-wall-005</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RC-wall-005/001.jpg,https://oleks-netizen.github.io/product-images/RC-wall-005/002.jpg,https://oleks-netizen.github.io/product-images/RC-wall-005/003.jpg,https://oleks-netizen.github.io/product-images/RC-wall-005/004.jpg,https://oleks-netizen.github.io/product-images/RC-wall-005/006.jpg</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>RCw-4027-3md</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RCw-4027-3md/001.jpg,https://oleks-netizen.github.io/product-images/RCw-4027-3md/002.jpg,https://oleks-netizen.github.io/product-images/RCw-4027-3md/003.jpg,https://oleks-netizen.github.io/product-images/RCw-4027-3md/005.jpg,https://oleks-netizen.github.io/product-images/RCw-4027-3md/006.jpg,https://oleks-netizen.github.io/product-images/RCw-4027-3md/007.jpg,https://oleks-netizen.github.io/product-images/RCw-4027-3md/008.jpg</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>RE-1304-4lx</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RE-1304-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RE-1304-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RE-1304-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RE-1304-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RE-1304-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RE-1304-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RE-1304-4lx/008.jpg,https://oleks-netizen.github.io/product-images/RE-1304-4lx/009.jpg</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>RE-1501-3md</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RE-1501-3md/001.jpg,https://oleks-netizen.github.io/product-images/RE-1501-3md/002.jpg,https://oleks-netizen.github.io/product-images/RE-1501-3md/004.jpg,https://oleks-netizen.github.io/product-images/RE-1501-3md/005.jpg,https://oleks-netizen.github.io/product-images/RE-1501-3md/006.jpg,https://oleks-netizen.github.io/product-images/RE-1501-3md/007.jpg</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>RE-7084-3md</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RE-7084-3md/001.jpg,https://oleks-netizen.github.io/product-images/RE-7084-3md/003.jpg,https://oleks-netizen.github.io/product-images/RE-7084-3md/004.jpg,https://oleks-netizen.github.io/product-images/RE-7084-3md/005.jpg,https://oleks-netizen.github.io/product-images/RE-7084-3md/006.jpg,https://oleks-netizen.github.io/product-images/RE-7084-3md/007.jpg,https://oleks-netizen.github.io/product-images/RE-7084-3md/008.jpg,https://oleks-netizen.github.io/product-images/RE-7084-3md/009.jpg,https://oleks-netizen.github.io/product-images/RE-7084-3md/010.jpg,https://oleks-netizen.github.io/product-images/RE-7084-3md/011.jpg</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>REE-6402-3md</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/REE-6402-3md/001.jpg,https://oleks-netizen.github.io/product-images/REE-6402-3md/002.jpg,https://oleks-netizen.github.io/product-images/REE-6402-3md/004.jpg,https://oleks-netizen.github.io/product-images/REE-6402-3md/005.jpg,https://oleks-netizen.github.io/product-images/REE-6402-3md/006.jpg,https://oleks-netizen.github.io/product-images/REE-6402-3md/007.jpg,https://oleks-netizen.github.io/product-images/REE-6402-3md/008.jpg</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>RepA-3027-4lx</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RepA-3027-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RepA-3027-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RepA-3027-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RepA-3027-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RepA-3027-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RepA-3027-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RepA-3027-4lx/008.jpg</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>REv-1819-4lx</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/REv-1819-4lx/001.jpg,https://oleks-netizen.github.io/product-images/REv-1819-4lx/002.jpg,https://oleks-netizen.github.io/product-images/REv-1819-4lx/003.jpg,https://oleks-netizen.github.io/product-images/REv-1819-4lx/005.jpg</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>RJ-4027-3md</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RJ-4027-3md/001.jpg,https://oleks-netizen.github.io/product-images/RJ-4027-3md/002.jpg,https://oleks-netizen.github.io/product-images/RJ-4027-3md/003.jpg,https://oleks-netizen.github.io/product-images/RJ-4027-3md/005.jpg,https://oleks-netizen.github.io/product-images/RJ-4027-3md/006.jpg,https://oleks-netizen.github.io/product-images/RJ-4027-3md/007.jpg,https://oleks-netizen.github.io/product-images/RJ-4027-3md/008.jpg,https://oleks-netizen.github.io/product-images/RJ-4027-3md/009.jpg</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>RJv-1819-4lx</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RJv-1819-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RJv-1819-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RJv-1819-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RJv-1819-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RJv-1819-4lx/006.jpg</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>RJv-5402-4lx</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RJv-5402-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RJv-5402-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RJv-5402-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RJv-5402-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RJv-5402-4lx/006.jpg</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>RJv-8033-4lx</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RJv-8033-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RJv-8033-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RJv-8033-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RJv-8033-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RJv-8033-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RJv-8033-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RJv-8033-4lx/008.jpg</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>RK-2801-3md</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RK-2801-3md/001.jpg,https://oleks-netizen.github.io/product-images/RK-2801-3md/002.jpg,https://oleks-netizen.github.io/product-images/RK-2801-3md/003.jpg,https://oleks-netizen.github.io/product-images/RK-2801-3md/004.jpg,https://oleks-netizen.github.io/product-images/RK-2801-3md/005.jpg,https://oleks-netizen.github.io/product-images/RK-2801-3md/006.jpg,https://oleks-netizen.github.io/product-images/RK-2801-3md/007.jpg,https://oleks-netizen.github.io/product-images/RK-2801-3md/008.jpg,https://oleks-netizen.github.io/product-images/RK-2801-3md/010.jpg</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>RKj-7880-4lx</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RKj-7880-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RKj-7880-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RKj-7880-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RKj-7880-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RKj-7880-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RKj-7880-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RKj-7880-4lx/008.jpg,https://oleks-netizen.github.io/product-images/RKj-7880-4lx/009.jpg,https://oleks-netizen.github.io/product-images/RKj-7880-4lx/010.jpg</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>RY-4027-3md</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RY-4027-3md/001.jpg,https://oleks-netizen.github.io/product-images/RY-4027-3md/002.jpg,https://oleks-netizen.github.io/product-images/RY-4027-3md/003.jpg,https://oleks-netizen.github.io/product-images/RY-4027-3md/004.jpg,https://oleks-netizen.github.io/product-images/RY-4027-3md/006.jpg,https://oleks-netizen.github.io/product-images/RY-4027-3md/007.jpg</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>RYv-1819-4lx</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RYv-1819-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RYv-1819-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RYv-1819-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RYv-1819-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RYv-1819-4lx/006.jpg</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>RYv-5402-4lx</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RYv-5402-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RYv-5402-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RYv-5402-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RYv-5402-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RYv-5402-4lx/006.jpg</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>RYv-8033-4lx</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RYv-8033-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RYv-8033-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RYv-8033-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RYv-8033-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RYv-8033-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RYv-8033-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RYv-8033-4lx/008.jpg</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>RЕ-1818-3md</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RЕ-1818-3md/001.jpg,https://oleks-netizen.github.io/product-images/RЕ-1818-3md/002.jpg,https://oleks-netizen.github.io/product-images/RЕ-1818-3md/003.jpg,https://oleks-netizen.github.io/product-images/RЕ-1818-3md/004.jpg,https://oleks-netizen.github.io/product-images/RЕ-1818-3md/005.jpg,https://oleks-netizen.github.io/product-images/RЕ-1818-3md/006.jpg,https://oleks-netizen.github.io/product-images/RЕ-1818-3md/008.jpg,https://oleks-netizen.github.io/product-images/RЕ-1818-3md/009.jpg</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>RС-1818-3md</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RС-1818-3md/001.jpg,https://oleks-netizen.github.io/product-images/RС-1818-3md/002.jpg,https://oleks-netizen.github.io/product-images/RС-1818-3md/003.jpg,https://oleks-netizen.github.io/product-images/RС-1818-3md/004.jpg,https://oleks-netizen.github.io/product-images/RС-1818-3md/006.jpg,https://oleks-netizen.github.io/product-images/RС-1818-3md/007.jpg,https://oleks-netizen.github.io/product-images/RС-1818-3md/008.jpg,https://oleks-netizen.github.io/product-images/RС-1818-3md/009.jpg</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>sk350115-1</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/sk350115-1/001.jpg,https://oleks-netizen.github.io/product-images/sk350115-1/003.jpg,https://oleks-netizen.github.io/product-images/sk350115-1/004.jpg</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>sk400330A</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/sk400330A/001.jpg,https://oleks-netizen.github.io/product-images/sk400330A/002.jpg,https://oleks-netizen.github.io/product-images/sk400330A/003.jpg,https://oleks-netizen.github.io/product-images/sk400330A/004.jpg,https://oleks-netizen.github.io/product-images/sk400330A/006.jpg</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>st04454</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/st04454/001.jpg,https://oleks-netizen.github.io/product-images/st04454/002.jpg,https://oleks-netizen.github.io/product-images/st04454/004.jpg,https://oleks-netizen.github.io/product-images/st04454/005.jpg</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>TA-1819-3md</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TA-1819-3md/001.jpg,https://oleks-netizen.github.io/product-images/TA-1819-3md/002.jpg,https://oleks-netizen.github.io/product-images/TA-1819-3md/004.jpg,https://oleks-netizen.github.io/product-images/TA-1819-3md/005.jpg,https://oleks-netizen.github.io/product-images/TA-1819-3md/006.jpg</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>tid9666LA</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/tid9666LA/001.jpg,https://oleks-netizen.github.io/product-images/tid9666LA/002.jpg,https://oleks-netizen.github.io/product-images/tid9666LA/003.jpg,https://oleks-netizen.github.io/product-images/tid9666LA/004.jpg,https://oleks-netizen.github.io/product-images/tid9666LA/005.jpg,https://oleks-netizen.github.io/product-images/tid9666LA/007.jpg,https://oleks-netizen.github.io/product-images/tid9666LA/008.jpg</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>TW033A</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW033A/001.jpg,https://oleks-netizen.github.io/product-images/TW033A/002.jpg,https://oleks-netizen.github.io/product-images/TW033A/004.jpg,https://oleks-netizen.github.io/product-images/TW033A/005.jpg,https://oleks-netizen.github.io/product-images/TW033A/006.jpg</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>TW033AV</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW033AV/001.jpg,https://oleks-netizen.github.io/product-images/TW033AV/002.jpg,https://oleks-netizen.github.io/product-images/TW033AV/004.jpg,https://oleks-netizen.github.io/product-images/TW033AV/005.jpg,https://oleks-netizen.github.io/product-images/TW033AV/006.jpg</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>TW033BV</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW033BV/001.jpg,https://oleks-netizen.github.io/product-images/TW033BV/002.jpg,https://oleks-netizen.github.io/product-images/TW033BV/004.jpg,https://oleks-netizen.github.io/product-images/TW033BV/005.jpg,https://oleks-netizen.github.io/product-images/TW033BV/006.jpg</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>TW033C</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW033C/001.jpg,https://oleks-netizen.github.io/product-images/TW033C/002.jpg,https://oleks-netizen.github.io/product-images/TW033C/003.jpg,https://oleks-netizen.github.io/product-images/TW033C/004.jpg,https://oleks-netizen.github.io/product-images/TW033C/006.jpg</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ZAw-7084-3md</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/ZAw-7084-3md/001.jpg,https://oleks-netizen.github.io/product-images/ZAw-7084-3md/002.jpg,https://oleks-netizen.github.io/product-images/ZAw-7084-3md/004.jpg,https://oleks-netizen.github.io/product-images/ZAw-7084-3md/005.jpg,https://oleks-netizen.github.io/product-images/ZAw-7084-3md/006.jpg,https://oleks-netizen.github.io/product-images/ZAw-7084-3md/007.jpg,https://oleks-netizen.github.io/product-images/ZAw-7084-3md/008.jpg</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-05-09 07:29:15
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -501,11 +501,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3148-1/001.jpg,https://oleks-netizen.github.io/product-images/3148-1/002.jpg,https://oleks-netizen.github.io/product-images/3148-1/003.jpg,https://oleks-netizen.github.io/product-images/3148-1/004.jpg,https://oleks-netizen.github.io/product-images/3148-1/005.jpg,https://oleks-netizen.github.io/product-images/3148-1/006.jpg,https://oleks-netizen.github.io/product-images/3148-1/007.jpg,https://oleks-netizen.github.io/product-images/3148-1/008.jpg,https://oleks-netizen.github.io/product-images/3148-1/009.jpg,https://oleks-netizen.github.io/product-images/3148-1/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3148-1/001.jpg,https://oleks-netizen.github.io/product-images/3148-1/002.jpg,https://oleks-netizen.github.io/product-images/3148-1/003.jpg,https://oleks-netizen.github.io/product-images/3148-1/005.jpg,https://oleks-netizen.github.io/product-images/3148-1/006.jpg,https://oleks-netizen.github.io/product-images/3148-1/007.jpg,https://oleks-netizen.github.io/product-images/3148-1/008.jpg,https://oleks-netizen.github.io/product-images/3148-1/009.jpg,https://oleks-netizen.github.io/product-images/3148-1/010.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -516,11 +516,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3149 Paris/001.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/002.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/003.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/004.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/005.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/006.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/007.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/008.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3149 Paris/001.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/002.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/003.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/005.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/006.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/007.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/008.jpg,https://oleks-netizen.github.io/product-images/3149 Paris/009.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -531,11 +531,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/001.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/002.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/003.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/004.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/005.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/006.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/007.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/001.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/002.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/003.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/005.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/006.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/007.jpg,https://oleks-netizen.github.io/product-images/3149 Ейфелева Вежа/008.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -546,11 +546,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3149 Кіт/001.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/002.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/003.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/004.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/005.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/006.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/007.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/008.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3149 Кіт/001.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/002.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/003.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/005.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/006.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/007.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/008.jpg,https://oleks-netizen.github.io/product-images/3149 Кіт/009.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -561,11 +561,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/001.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/002.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/003.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/004.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/005.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/006.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/007.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/008.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/001.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/002.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/003.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/005.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/006.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/007.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/008.jpg,https://oleks-netizen.github.io/product-images/3149 Кава в Парижі/009.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -576,11 +576,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3149 Слід/001.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/002.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/003.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/004.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/005.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/006.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/007.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3149 Слід/001.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/002.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/003.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/005.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/006.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/007.jpg,https://oleks-netizen.github.io/product-images/3149 Слід/008.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -606,11 +606,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3150 France/001.jpg,https://oleks-netizen.github.io/product-images/3150 France/002.jpg,https://oleks-netizen.github.io/product-images/3150 France/003.jpg,https://oleks-netizen.github.io/product-images/3150 France/004.jpg,https://oleks-netizen.github.io/product-images/3150 France/005.jpg,https://oleks-netizen.github.io/product-images/3150 France/006.jpg,https://oleks-netizen.github.io/product-images/3150 France/007.jpg,https://oleks-netizen.github.io/product-images/3150 France/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3150 France/001.jpg,https://oleks-netizen.github.io/product-images/3150 France/002.jpg,https://oleks-netizen.github.io/product-images/3150 France/003.jpg,https://oleks-netizen.github.io/product-images/3150 France/004.jpg,https://oleks-netizen.github.io/product-images/3150 France/006.jpg,https://oleks-netizen.github.io/product-images/3150 France/007.jpg,https://oleks-netizen.github.io/product-images/3150 France/008.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -621,11 +621,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3150 Paris/001.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/002.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/003.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/004.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/005.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/006.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/007.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/008.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3150 Paris/001.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/002.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/003.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/006.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/007.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/008.jpg,https://oleks-netizen.github.io/product-images/3150 Paris/009.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -636,11 +636,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/001.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/002.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/003.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/004.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/005.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/006.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/007.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/008.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/001.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/002.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/003.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/004.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/006.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/007.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/008.jpg,https://oleks-netizen.github.io/product-images/3150 Прогулянка в Парижі/009.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -651,11 +651,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3150 Сліди/001.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/002.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/003.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/004.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/005.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/006.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/007.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/008.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3150 Сліди/001.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/002.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/003.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/005.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/006.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/007.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/008.jpg,https://oleks-netizen.github.io/product-images/3150 Сліди/009.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
@@ -681,11 +681,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3225 Біла/001.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/002.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/003.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/004.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/005.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/006.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/007.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/008.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3225 Біла/001.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/002.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/003.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/004.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/006.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/007.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/008.jpg,https://oleks-netizen.github.io/product-images/3225 Біла/009.jpg</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
@@ -711,11 +711,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3225 Кремова/001.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/002.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/003.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/004.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/005.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/006.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/007.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/008.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3225 Кремова/001.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/002.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/003.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/004.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/006.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/007.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/008.jpg,https://oleks-netizen.github.io/product-images/3225 Кремова/009.jpg</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21">
@@ -741,11 +741,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3225 Синя/001.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/002.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/003.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/004.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/005.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/006.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/007.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/008.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3225 Синя/001.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/002.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/003.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/005.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/006.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/007.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/008.jpg,https://oleks-netizen.github.io/product-images/3225 Синя/009.jpg</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
@@ -756,11 +756,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3225 Фіолетова/001.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/002.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/003.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/004.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/005.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/006.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/007.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/008.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3225 Фіолетова/001.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/002.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/003.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/005.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/006.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/007.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/008.jpg,https://oleks-netizen.github.io/product-images/3225 Фіолетова/009.jpg</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24">
@@ -786,11 +786,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3226 Зірки/001.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/002.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/003.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/004.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/005.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/006.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/007.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/008.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3226 Зірки/001.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/002.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/003.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/005.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/006.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/007.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/008.jpg,https://oleks-netizen.github.io/product-images/3226 Зірки/009.jpg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26">
@@ -801,11 +801,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3226 Кіт/001.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/002.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/003.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/004.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/005.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/006.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/007.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3226 Кіт/001.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/002.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/003.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/005.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/006.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/007.jpg,https://oleks-netizen.github.io/product-images/3226 Кіт/008.jpg</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27">
@@ -816,11 +816,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3226 Місто/001.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/002.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/003.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/004.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/005.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/006.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/007.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/008.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3226 Місто/001.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/002.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/003.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/005.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/006.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/007.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/008.jpg,https://oleks-netizen.github.io/product-images/3226 Місто/009.jpg</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -846,11 +846,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/3226 Сяйво/001.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/002.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/003.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/004.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/005.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/006.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/007.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/008.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/3226 Сяйво/001.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/002.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/003.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/005.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/006.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/007.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/008.jpg,https://oleks-netizen.github.io/product-images/3226 Сяйво/009.jpg</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30">
@@ -1191,11 +1191,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L20002-22/001.jpg,https://oleks-netizen.github.io/product-images/L20002-22/002.jpg,https://oleks-netizen.github.io/product-images/L20002-22/004.jpg,https://oleks-netizen.github.io/product-images/L20002-22/005.jpg,https://oleks-netizen.github.io/product-images/L20002-22/006.jpg,https://oleks-netizen.github.io/product-images/L20002-22/007.jpg,https://oleks-netizen.github.io/product-images/L20002-22/008.jpg,https://oleks-netizen.github.io/product-images/L20002-22/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L20002-22/001.jpg,https://oleks-netizen.github.io/product-images/L20002-22/002.jpg,https://oleks-netizen.github.io/product-images/L20002-22/004.jpg,https://oleks-netizen.github.io/product-images/L20002-22/005.jpg,https://oleks-netizen.github.io/product-images/L20002-22/006.jpg,https://oleks-netizen.github.io/product-images/L20002-22/007.jpg,https://oleks-netizen.github.io/product-images/L20002-22/009.jpg</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -1206,11 +1206,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L20020-1/001.jpg,https://oleks-netizen.github.io/product-images/L20020-1/002.jpg,https://oleks-netizen.github.io/product-images/L20020-1/003.jpg,https://oleks-netizen.github.io/product-images/L20020-1/004.jpg,https://oleks-netizen.github.io/product-images/L20020-1/005.jpg,https://oleks-netizen.github.io/product-images/L20020-1/006.jpg,https://oleks-netizen.github.io/product-images/L20020-1/007.jpg,https://oleks-netizen.github.io/product-images/L20020-1/008.jpg,https://oleks-netizen.github.io/product-images/L20020-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L20020-1/001.jpg,https://oleks-netizen.github.io/product-images/L20020-1/002.jpg,https://oleks-netizen.github.io/product-images/L20020-1/003.jpg,https://oleks-netizen.github.io/product-images/L20020-1/004.jpg,https://oleks-netizen.github.io/product-images/L20020-1/005.jpg,https://oleks-netizen.github.io/product-images/L20020-1/006.jpg,https://oleks-netizen.github.io/product-images/L20020-1/007.jpg,https://oleks-netizen.github.io/product-images/L20020-1/008.jpg</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54">
@@ -1221,11 +1221,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L20026-1/001.jpg,https://oleks-netizen.github.io/product-images/L20026-1/002.jpg,https://oleks-netizen.github.io/product-images/L20026-1/004.jpg,https://oleks-netizen.github.io/product-images/L20026-1/005.jpg,https://oleks-netizen.github.io/product-images/L20026-1/006.jpg,https://oleks-netizen.github.io/product-images/L20026-1/007.jpg,https://oleks-netizen.github.io/product-images/L20026-1/008.jpg,https://oleks-netizen.github.io/product-images/L20026-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L20026-1/001.jpg,https://oleks-netizen.github.io/product-images/L20026-1/002.jpg,https://oleks-netizen.github.io/product-images/L20026-1/004.jpg,https://oleks-netizen.github.io/product-images/L20026-1/005.jpg,https://oleks-netizen.github.io/product-images/L20026-1/006.jpg,https://oleks-netizen.github.io/product-images/L20026-1/007.jpg,https://oleks-netizen.github.io/product-images/L20026-1/009.jpg</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55">
@@ -1236,11 +1236,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L20633-15/001.jpg,https://oleks-netizen.github.io/product-images/L20633-15/002.jpg,https://oleks-netizen.github.io/product-images/L20633-15/004.jpg,https://oleks-netizen.github.io/product-images/L20633-15/005.jpg,https://oleks-netizen.github.io/product-images/L20633-15/006.jpg,https://oleks-netizen.github.io/product-images/L20633-15/007.jpg,https://oleks-netizen.github.io/product-images/L20633-15/008.jpg,https://oleks-netizen.github.io/product-images/L20633-15/009.jpg,https://oleks-netizen.github.io/product-images/L20633-15/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L20633-15/001.jpg,https://oleks-netizen.github.io/product-images/L20633-15/002.jpg,https://oleks-netizen.github.io/product-images/L20633-15/004.jpg,https://oleks-netizen.github.io/product-images/L20633-15/005.jpg,https://oleks-netizen.github.io/product-images/L20633-15/006.jpg,https://oleks-netizen.github.io/product-images/L20633-15/007.jpg,https://oleks-netizen.github.io/product-images/L20633-15/008.jpg,https://oleks-netizen.github.io/product-images/L20633-15/010.jpg</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="56">
@@ -1251,11 +1251,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L20633-82/001.jpg,https://oleks-netizen.github.io/product-images/L20633-82/002.jpg,https://oleks-netizen.github.io/product-images/L20633-82/004.jpg,https://oleks-netizen.github.io/product-images/L20633-82/005.jpg,https://oleks-netizen.github.io/product-images/L20633-82/006.jpg,https://oleks-netizen.github.io/product-images/L20633-82/007.jpg,https://oleks-netizen.github.io/product-images/L20633-82/008.jpg,https://oleks-netizen.github.io/product-images/L20633-82/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L20633-82/001.jpg,https://oleks-netizen.github.io/product-images/L20633-82/002.jpg,https://oleks-netizen.github.io/product-images/L20633-82/004.jpg,https://oleks-netizen.github.io/product-images/L20633-82/005.jpg,https://oleks-netizen.github.io/product-images/L20633-82/006.jpg,https://oleks-netizen.github.io/product-images/L20633-82/007.jpg,https://oleks-netizen.github.io/product-images/L20633-82/009.jpg</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="57">
@@ -1266,11 +1266,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L20666-1/001.jpg,https://oleks-netizen.github.io/product-images/L20666-1/002.jpg,https://oleks-netizen.github.io/product-images/L20666-1/003.jpg,https://oleks-netizen.github.io/product-images/L20666-1/004.jpg,https://oleks-netizen.github.io/product-images/L20666-1/005.jpg,https://oleks-netizen.github.io/product-images/L20666-1/006.jpg,https://oleks-netizen.github.io/product-images/L20666-1/007.jpg,https://oleks-netizen.github.io/product-images/L20666-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L20666-1/001.jpg,https://oleks-netizen.github.io/product-images/L20666-1/002.jpg,https://oleks-netizen.github.io/product-images/L20666-1/003.jpg,https://oleks-netizen.github.io/product-images/L20666-1/004.jpg,https://oleks-netizen.github.io/product-images/L20666-1/005.jpg,https://oleks-netizen.github.io/product-images/L20666-1/006.jpg,https://oleks-netizen.github.io/product-images/L20666-1/007.jpg</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="58">
@@ -1311,11 +1311,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21035-1/001.jpg,https://oleks-netizen.github.io/product-images/L21035-1/002.jpg,https://oleks-netizen.github.io/product-images/L21035-1/003.jpg,https://oleks-netizen.github.io/product-images/L21035-1/004.jpg,https://oleks-netizen.github.io/product-images/L21035-1/005.jpg,https://oleks-netizen.github.io/product-images/L21035-1/006.jpg,https://oleks-netizen.github.io/product-images/L21035-1/007.jpg,https://oleks-netizen.github.io/product-images/L21035-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L21035-1/001.jpg,https://oleks-netizen.github.io/product-images/L21035-1/002.jpg,https://oleks-netizen.github.io/product-images/L21035-1/003.jpg,https://oleks-netizen.github.io/product-images/L21035-1/004.jpg,https://oleks-netizen.github.io/product-images/L21035-1/005.jpg,https://oleks-netizen.github.io/product-images/L21035-1/006.jpg,https://oleks-netizen.github.io/product-images/L21035-1/007.jpg</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="61">
@@ -1326,11 +1326,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21533-130/001.jpg,https://oleks-netizen.github.io/product-images/L21533-130/002.jpg,https://oleks-netizen.github.io/product-images/L21533-130/004.jpg,https://oleks-netizen.github.io/product-images/L21533-130/005.jpg,https://oleks-netizen.github.io/product-images/L21533-130/006.jpg,https://oleks-netizen.github.io/product-images/L21533-130/007.jpg,https://oleks-netizen.github.io/product-images/L21533-130/008.jpg,https://oleks-netizen.github.io/product-images/L21533-130/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L21533-130/001.jpg,https://oleks-netizen.github.io/product-images/L21533-130/002.jpg,https://oleks-netizen.github.io/product-images/L21533-130/004.jpg,https://oleks-netizen.github.io/product-images/L21533-130/005.jpg,https://oleks-netizen.github.io/product-images/L21533-130/006.jpg,https://oleks-netizen.github.io/product-images/L21533-130/007.jpg,https://oleks-netizen.github.io/product-images/L21533-130/009.jpg</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="62">
@@ -1341,11 +1341,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L21547-79/001.jpg,https://oleks-netizen.github.io/product-images/L21547-79/002.jpg,https://oleks-netizen.github.io/product-images/L21547-79/003.jpg,https://oleks-netizen.github.io/product-images/L21547-79/004.jpg,https://oleks-netizen.github.io/product-images/L21547-79/005.jpg,https://oleks-netizen.github.io/product-images/L21547-79/006.jpg,https://oleks-netizen.github.io/product-images/L21547-79/007.jpg,https://oleks-netizen.github.io/product-images/L21547-79/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L21547-79/001.jpg,https://oleks-netizen.github.io/product-images/L21547-79/002.jpg,https://oleks-netizen.github.io/product-images/L21547-79/003.jpg,https://oleks-netizen.github.io/product-images/L21547-79/004.jpg,https://oleks-netizen.github.io/product-images/L21547-79/005.jpg,https://oleks-netizen.github.io/product-images/L21547-79/006.jpg,https://oleks-netizen.github.io/product-images/L21547-79/007.jpg</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63">
@@ -1386,11 +1386,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L22098-8/001.jpg,https://oleks-netizen.github.io/product-images/L22098-8/002.jpg,https://oleks-netizen.github.io/product-images/L22098-8/004.jpg,https://oleks-netizen.github.io/product-images/L22098-8/005.jpg,https://oleks-netizen.github.io/product-images/L22098-8/006.jpg,https://oleks-netizen.github.io/product-images/L22098-8/007.jpg,https://oleks-netizen.github.io/product-images/L22098-8/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L22098-8/001.jpg,https://oleks-netizen.github.io/product-images/L22098-8/002.jpg,https://oleks-netizen.github.io/product-images/L22098-8/004.jpg,https://oleks-netizen.github.io/product-images/L22098-8/005.jpg,https://oleks-netizen.github.io/product-images/L22098-8/006.jpg,https://oleks-netizen.github.io/product-images/L22098-8/008.jpg</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66">
@@ -1401,11 +1401,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L22537-1/001.jpg,https://oleks-netizen.github.io/product-images/L22537-1/002.jpg,https://oleks-netizen.github.io/product-images/L22537-1/004.jpg,https://oleks-netizen.github.io/product-images/L22537-1/005.jpg,https://oleks-netizen.github.io/product-images/L22537-1/006.jpg,https://oleks-netizen.github.io/product-images/L22537-1/007.jpg,https://oleks-netizen.github.io/product-images/L22537-1/008.jpg,https://oleks-netizen.github.io/product-images/L22537-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L22537-1/001.jpg,https://oleks-netizen.github.io/product-images/L22537-1/002.jpg,https://oleks-netizen.github.io/product-images/L22537-1/004.jpg,https://oleks-netizen.github.io/product-images/L22537-1/005.jpg,https://oleks-netizen.github.io/product-images/L22537-1/006.jpg,https://oleks-netizen.github.io/product-images/L22537-1/007.jpg,https://oleks-netizen.github.io/product-images/L22537-1/009.jpg</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="67">
@@ -1416,11 +1416,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L22613-1S/001.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/002.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/003.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/004.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/005.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/006.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/007.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L22613-1S/001.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/002.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/003.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/004.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/005.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/006.jpg,https://oleks-netizen.github.io/product-images/L22613-1S/007.jpg</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="68">
@@ -1431,11 +1431,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L22813-01S/001.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/002.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/004.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/005.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/006.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/007.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/008.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/009.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L22813-01S/001.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/002.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/004.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/005.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/006.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/007.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/008.jpg,https://oleks-netizen.github.io/product-images/L22813-01S/010.jpg</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="69">
@@ -1461,11 +1461,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L26827-1/001.jpg,https://oleks-netizen.github.io/product-images/L26827-1/002.jpg,https://oleks-netizen.github.io/product-images/L26827-1/004.jpg,https://oleks-netizen.github.io/product-images/L26827-1/005.jpg,https://oleks-netizen.github.io/product-images/L26827-1/006.jpg,https://oleks-netizen.github.io/product-images/L26827-1/007.jpg,https://oleks-netizen.github.io/product-images/L26827-1/008.jpg,https://oleks-netizen.github.io/product-images/L26827-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L26827-1/001.jpg,https://oleks-netizen.github.io/product-images/L26827-1/002.jpg,https://oleks-netizen.github.io/product-images/L26827-1/004.jpg,https://oleks-netizen.github.io/product-images/L26827-1/005.jpg,https://oleks-netizen.github.io/product-images/L26827-1/006.jpg,https://oleks-netizen.github.io/product-images/L26827-1/007.jpg,https://oleks-netizen.github.io/product-images/L26827-1/009.jpg</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="71">
@@ -1491,11 +1491,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L29056-05/001.jpg,https://oleks-netizen.github.io/product-images/L29056-05/002.jpg,https://oleks-netizen.github.io/product-images/L29056-05/004.jpg,https://oleks-netizen.github.io/product-images/L29056-05/005.jpg,https://oleks-netizen.github.io/product-images/L29056-05/006.jpg,https://oleks-netizen.github.io/product-images/L29056-05/007.jpg,https://oleks-netizen.github.io/product-images/L29056-05/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L29056-05/001.jpg,https://oleks-netizen.github.io/product-images/L29056-05/002.jpg,https://oleks-netizen.github.io/product-images/L29056-05/004.jpg,https://oleks-netizen.github.io/product-images/L29056-05/005.jpg,https://oleks-netizen.github.io/product-images/L29056-05/006.jpg,https://oleks-netizen.github.io/product-images/L29056-05/008.jpg</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="73">
@@ -1566,11 +1566,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L85351-1/001.jpg,https://oleks-netizen.github.io/product-images/L85351-1/002.jpg,https://oleks-netizen.github.io/product-images/L85351-1/004.jpg,https://oleks-netizen.github.io/product-images/L85351-1/005.jpg,https://oleks-netizen.github.io/product-images/L85351-1/006.jpg,https://oleks-netizen.github.io/product-images/L85351-1/007.jpg,https://oleks-netizen.github.io/product-images/L85351-1/008.jpg,https://oleks-netizen.github.io/product-images/L85351-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L85351-1/001.jpg,https://oleks-netizen.github.io/product-images/L85351-1/002.jpg,https://oleks-netizen.github.io/product-images/L85351-1/004.jpg,https://oleks-netizen.github.io/product-images/L85351-1/005.jpg,https://oleks-netizen.github.io/product-images/L85351-1/006.jpg,https://oleks-netizen.github.io/product-images/L85351-1/007.jpg,https://oleks-netizen.github.io/product-images/L85351-1/009.jpg</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="78">
@@ -1611,11 +1611,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87027-1W/001.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/002.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/004.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/005.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/006.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/007.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/008.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/009.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L87027-1W/001.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/002.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/004.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/005.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/006.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/007.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/008.jpg,https://oleks-netizen.github.io/product-images/L87027-1W/010.jpg</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="81">
@@ -1641,11 +1641,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87159-1/001.jpg,https://oleks-netizen.github.io/product-images/L87159-1/002.jpg,https://oleks-netizen.github.io/product-images/L87159-1/004.jpg,https://oleks-netizen.github.io/product-images/L87159-1/005.jpg,https://oleks-netizen.github.io/product-images/L87159-1/006.jpg,https://oleks-netizen.github.io/product-images/L87159-1/007.jpg,https://oleks-netizen.github.io/product-images/L87159-1/008.jpg,https://oleks-netizen.github.io/product-images/L87159-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L87159-1/001.jpg,https://oleks-netizen.github.io/product-images/L87159-1/002.jpg,https://oleks-netizen.github.io/product-images/L87159-1/004.jpg,https://oleks-netizen.github.io/product-images/L87159-1/005.jpg,https://oleks-netizen.github.io/product-images/L87159-1/006.jpg,https://oleks-netizen.github.io/product-images/L87159-1/007.jpg,https://oleks-netizen.github.io/product-images/L87159-1/009.jpg</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="83">
@@ -1701,11 +1701,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87438-61/001.jpg,https://oleks-netizen.github.io/product-images/L87438-61/002.jpg,https://oleks-netizen.github.io/product-images/L87438-61/004.jpg,https://oleks-netizen.github.io/product-images/L87438-61/005.jpg,https://oleks-netizen.github.io/product-images/L87438-61/006.jpg,https://oleks-netizen.github.io/product-images/L87438-61/007.jpg,https://oleks-netizen.github.io/product-images/L87438-61/008.jpg,https://oleks-netizen.github.io/product-images/L87438-61/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L87438-61/001.jpg,https://oleks-netizen.github.io/product-images/L87438-61/002.jpg,https://oleks-netizen.github.io/product-images/L87438-61/004.jpg,https://oleks-netizen.github.io/product-images/L87438-61/005.jpg,https://oleks-netizen.github.io/product-images/L87438-61/006.jpg,https://oleks-netizen.github.io/product-images/L87438-61/007.jpg,https://oleks-netizen.github.io/product-images/L87438-61/009.jpg</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="87">
@@ -1716,11 +1716,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/L87480-1W/001.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/002.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/004.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/005.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/006.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/007.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/008.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/009.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/L87480-1W/001.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/002.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/004.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/005.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/006.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/007.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/008.jpg,https://oleks-netizen.github.io/product-images/L87480-1W/010.jpg</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88">
@@ -1776,11 +1776,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LS22696-108/001.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/002.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/004.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/005.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/006.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/007.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/008.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/LS22696-108/001.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/002.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/004.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/005.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/006.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/007.jpg,https://oleks-netizen.github.io/product-images/LS22696-108/009.jpg</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="92">

</xml_diff>

<commit_message>
Auto update 2026-05-21 18:01:38
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,12 +436,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1060418530</t>
+          <t>BN-BAG-10-k</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1060418530/001.jpg,https://oleks-netizen.github.io/product-images/1060418530/002.jpg,https://oleks-netizen.github.io/product-images/1060418530/003.jpg,https://oleks-netizen.github.io/product-images/1060418530/004.jpg,https://oleks-netizen.github.io/product-images/1060418530/005.jpg,https://oleks-netizen.github.io/product-images/1060418530/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-10-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-k/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-k/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-k/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-k/007.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -451,102 +451,102 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1079119520</t>
+          <t>BN-BAG-10-nn</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1079119520/001.jpg,https://oleks-netizen.github.io/product-images/1079119520/002.jpg,https://oleks-netizen.github.io/product-images/1079119520/004.jpg,https://oleks-netizen.github.io/product-images/1079119520/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-10-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-nn/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-nn/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-nn/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-nn/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-nn/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-nn/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-nn/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-10-nn/010.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1079121110</t>
+          <t>BN-BAG-12-iz</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1079121110/001.jpg,https://oleks-netizen.github.io/product-images/1079121110/002.jpg,https://oleks-netizen.github.io/product-images/1079121110/004.jpg,https://oleks-netizen.github.io/product-images/1079121110/005.jpg,https://oleks-netizen.github.io/product-images/1079121110/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-12-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-iz/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-iz/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-iz/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-iz/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-iz/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-iz/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-iz/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-iz/010.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1113320510</t>
+          <t>BN-BAG-12-o</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1113320510/001.jpg,https://oleks-netizen.github.io/product-images/1113320510/002.jpg,https://oleks-netizen.github.io/product-images/1113320510/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-12-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-o/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-o/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-o/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-o/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-o/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-o/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-o/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-o/010.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1121720890</t>
+          <t>BN-BAG-12-vin</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1121720890/001.jpg,https://oleks-netizen.github.io/product-images/1121720890/002.jpg,https://oleks-netizen.github.io/product-images/1121720890/003.jpg,https://oleks-netizen.github.io/product-images/1121720890/004.jpg,https://oleks-netizen.github.io/product-images/1121720890/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-12-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-vin/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-vin/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-vin/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-vin/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-vin/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-vin/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-12-vin/010.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1121920900</t>
+          <t>BN-BAG-13-g</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1121920900/001.jpg,https://oleks-netizen.github.io/product-images/1121920900/002.jpg,https://oleks-netizen.github.io/product-images/1121920900/003.jpg,https://oleks-netizen.github.io/product-images/1121920900/004.jpg,https://oleks-netizen.github.io/product-images/1121920900/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-13-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-13-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-13-g/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-13-g/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-13-g/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-13-g/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-13-g/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-13-g/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-13-g/010.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1140321760</t>
+          <t>BN-BAG-15-white</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1140321760/001.jpg,https://oleks-netizen.github.io/product-images/1140321760/002.jpg,https://oleks-netizen.github.io/product-images/1140321760/003.jpg,https://oleks-netizen.github.io/product-images/1140321760/004.jpg,https://oleks-netizen.github.io/product-images/1140321760/005.jpg,https://oleks-netizen.github.io/product-images/1140321760/006.jpg,https://oleks-netizen.github.io/product-images/1140321760/007.jpg,https://oleks-netizen.github.io/product-images/1140321760/009.jpg,https://oleks-netizen.github.io/product-images/1140321760/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-15-white/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-15-white/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-15-white/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-15-white/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-15-white/006.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1143021830</t>
+          <t>BN-BAG-16-rubin</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1143021830/001.jpg,https://oleks-netizen.github.io/product-images/1143021830/002.jpg,https://oleks-netizen.github.io/product-images/1143021830/003.jpg,https://oleks-netizen.github.io/product-images/1143021830/004.jpg,https://oleks-netizen.github.io/product-images/1143021830/005.jpg,https://oleks-netizen.github.io/product-images/1143021830/006.jpg,https://oleks-netizen.github.io/product-images/1143021830/007.jpg,https://oleks-netizen.github.io/product-images/1143021830/008.jpg,https://oleks-netizen.github.io/product-images/1143021830/009.jpg,https://oleks-netizen.github.io/product-images/1143021830/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-16-rubin/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-16-rubin/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-16-rubin/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-16-rubin/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-16-rubin/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-16-rubin/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-16-rubin/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-16-rubin/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-16-rubin/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-16-rubin/010.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -556,207 +556,207 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1143421840</t>
+          <t>BN-BAG-18-navy-blue</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1143421840/001.jpg,https://oleks-netizen.github.io/product-images/1143421840/003.jpg,https://oleks-netizen.github.io/product-images/1143421840/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-18-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-18-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-18-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-18-navy-blue/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-18-navy-blue/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-18-navy-blue/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-18-navy-blue/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-18-navy-blue/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-18-navy-blue/010.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-18-navy-blue/011.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1202123518</t>
+          <t>BN-BAG-22-navy-blue</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202123518/001.jpg,https://oleks-netizen.github.io/product-images/1202123518/003.jpg,https://oleks-netizen.github.io/product-images/1202123518/004.jpg,https://oleks-netizen.github.io/product-images/1202123518/005.jpg,https://oleks-netizen.github.io/product-images/1202123518/006.jpg,https://oleks-netizen.github.io/product-images/1202123518/007.jpg,https://oleks-netizen.github.io/product-images/1202123518/008.jpg,https://oleks-netizen.github.io/product-images/1202123518/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-22-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-22-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-22-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-22-navy-blue/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-22-navy-blue/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-22-navy-blue/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-22-navy-blue/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-22-navy-blue/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-22-navy-blue/010.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1202123519</t>
+          <t>BN-BAG-24-malachite</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202123519/001.jpg,https://oleks-netizen.github.io/product-images/1202123519/003.jpg,https://oleks-netizen.github.io/product-images/1202123519/004.jpg,https://oleks-netizen.github.io/product-images/1202123519/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-24-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-malachite/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-malachite/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-malachite/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-malachite/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-malachite/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-malachite/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-malachite/010.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1202123805</t>
+          <t>BN-BAG-3-k-kr</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202123805/001.jpg,https://oleks-netizen.github.io/product-images/1202123805/003.jpg,https://oleks-netizen.github.io/product-images/1202123805/004.jpg,https://oleks-netizen.github.io/product-images/1202123805/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-3-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-k-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-k-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-k-kr/006.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1202123806</t>
+          <t>BN-BAG-3-malachite</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202123806/001.jpg,https://oleks-netizen.github.io/product-images/1202123806/003.jpg,https://oleks-netizen.github.io/product-images/1202123806/004.jpg,https://oleks-netizen.github.io/product-images/1202123806/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-3-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-malachite/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-malachite/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-malachite/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-malachite/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-malachite/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-malachite/010.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-3-malachite/011.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1202223520</t>
+          <t>BN-BAG-30-light</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202223520/001.jpg,https://oleks-netizen.github.io/product-images/1202223520/003.jpg,https://oleks-netizen.github.io/product-images/1202223520/004.jpg,https://oleks-netizen.github.io/product-images/1202223520/005.jpg,https://oleks-netizen.github.io/product-images/1202223520/006.jpg,https://oleks-netizen.github.io/product-images/1202223520/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-30-light/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-30-light/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-30-light/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-30-light/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-30-light/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-30-light/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-30-light/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-30-light/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-30-light/010.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-30-light/011.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1202223521</t>
+          <t>BN-BAG-31-g</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202223521/001.jpg,https://oleks-netizen.github.io/product-images/1202223521/003.jpg,https://oleks-netizen.github.io/product-images/1202223521/004.jpg,https://oleks-netizen.github.io/product-images/1202223521/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-31-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-31-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-31-g/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-31-g/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-31-g/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-31-g/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-31-g/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-31-g/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-31-g/010.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1202223522</t>
+          <t>BN-BAG-33-nn</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202223522/001.jpg,https://oleks-netizen.github.io/product-images/1202223522/003.jpg,https://oleks-netizen.github.io/product-images/1202223522/004.jpg,https://oleks-netizen.github.io/product-images/1202223522/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-33-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-33-nn/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-33-nn/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-33-nn/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-33-nn/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-33-nn/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-33-nn/009.jpg</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1202223804</t>
+          <t>BN-BAG-41-mystic</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202223804/001.jpg,https://oleks-netizen.github.io/product-images/1202223804/003.jpg,https://oleks-netizen.github.io/product-images/1202223804/004.jpg,https://oleks-netizen.github.io/product-images/1202223804/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-41-mystic/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-41-mystic/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-41-mystic/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-41-mystic/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-41-mystic/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-41-mystic/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-41-mystic/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-41-mystic/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-41-mystic/010.jpg</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1202323523</t>
+          <t>BN-BAG-6-choko</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202323523/001.jpg,https://oleks-netizen.github.io/product-images/1202323523/003.jpg,https://oleks-netizen.github.io/product-images/1202323523/004.jpg,https://oleks-netizen.github.io/product-images/1202323523/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-6-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-choko/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-choko/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-choko/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-choko/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-choko/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-choko/010.jpg</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1202423525</t>
+          <t>BN-BAG-6-malachite</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202423525/001.jpg,https://oleks-netizen.github.io/product-images/1202423525/002.jpg,https://oleks-netizen.github.io/product-images/1202423525/003.jpg,https://oleks-netizen.github.io/product-images/1202423525/004.jpg,https://oleks-netizen.github.io/product-images/1202423525/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-6-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-malachite/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-malachite/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-malachite/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-malachite/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-malachite/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-malachite/010.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-6-malachite/011.jpg</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1202423526</t>
+          <t>BN-BAG-7-nn</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202423526/001.jpg,https://oleks-netizen.github.io/product-images/1202423526/003.jpg,https://oleks-netizen.github.io/product-images/1202423526/004.jpg,https://oleks-netizen.github.io/product-images/1202423526/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-7-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-nn/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-nn/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-nn/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-nn/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-nn/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-nn/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-nn/009.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-nn/010.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-nn/011.jpg</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1202423527</t>
+          <t>BN-BAG-7-vin-kr</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202423527/001.jpg,https://oleks-netizen.github.io/product-images/1202423527/003.jpg,https://oleks-netizen.github.io/product-images/1202423527/004.jpg,https://oleks-netizen.github.io/product-images/1202423527/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-7-vin-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-vin-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-vin-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-vin-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-vin-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-vin-kr/006.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-vin-kr/007.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-vin-kr/008.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-7-vin-kr/009.jpg</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1202423807</t>
+          <t>BN-CB-1-onyx</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1202423807/001.jpg,https://oleks-netizen.github.io/product-images/1202423807/003.jpg,https://oleks-netizen.github.io/product-images/1202423807/004.jpg,https://oleks-netizen.github.io/product-images/1202423807/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-1-onyx/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-1-onyx/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-1-onyx/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-1-onyx/006.jpg</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -766,12 +766,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1205123604</t>
+          <t>BN-CB-2-vin</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1205123604/001.jpg,https://oleks-netizen.github.io/product-images/1205123604/003.jpg,https://oleks-netizen.github.io/product-images/1205123604/004.jpg,https://oleks-netizen.github.io/product-images/1205123604/005.jpg,https://oleks-netizen.github.io/product-images/1205123604/006.jpg,https://oleks-netizen.github.io/product-images/1205123604/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-2-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-2-vin/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-2-vin/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-2-vin/005.jpg,https://oleks-netizen.github.io/product-images/BN-CB-2-vin/006.jpg,https://oleks-netizen.github.io/product-images/BN-CB-2-vin/008.jpg</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -781,117 +781,117 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1205123605</t>
+          <t>BN-CB-3-red</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1205123605/001.jpg,https://oleks-netizen.github.io/product-images/1205123605/003.jpg,https://oleks-netizen.github.io/product-images/1205123605/004.jpg,https://oleks-netizen.github.io/product-images/1205123605/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CB-3-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-CB-3-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-CB-3-red/003.jpg,https://oleks-netizen.github.io/product-images/BN-CB-3-red/004.jpg,https://oleks-netizen.github.io/product-images/BN-CB-3-red/005.jpg,https://oleks-netizen.github.io/product-images/BN-CB-3-red/006.jpg,https://oleks-netizen.github.io/product-images/BN-CB-3-red/009.jpg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1205123606</t>
+          <t>BN-CW-1-red</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1205123606/001.jpg,https://oleks-netizen.github.io/product-images/1205123606/003.jpg,https://oleks-netizen.github.io/product-images/1205123606/004.jpg,https://oleks-netizen.github.io/product-images/1205123606/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CW-1-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-CW-1-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-CW-1-red/003.jpg,https://oleks-netizen.github.io/product-images/BN-CW-1-red/004.jpg,https://oleks-netizen.github.io/product-images/BN-CW-1-red/005.jpg</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1205223607</t>
+          <t>BN-CW-1-vin</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1205223607/001.jpg,https://oleks-netizen.github.io/product-images/1205223607/003.jpg,https://oleks-netizen.github.io/product-images/1205223607/004.jpg,https://oleks-netizen.github.io/product-images/1205223607/005.jpg,https://oleks-netizen.github.io/product-images/1205223607/006.jpg,https://oleks-netizen.github.io/product-images/1205223607/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-CW-1-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-CW-1-vin/002.jpg,https://oleks-netizen.github.io/product-images/BN-CW-1-vin/003.jpg,https://oleks-netizen.github.io/product-images/BN-CW-1-vin/004.jpg,https://oleks-netizen.github.io/product-images/BN-CW-1-vin/005.jpg</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1205223608</t>
+          <t>BN-DC-3-choko</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1205223608/001.jpg,https://oleks-netizen.github.io/product-images/1205223608/003.jpg,https://oleks-netizen.github.io/product-images/1205223608/004.jpg,https://oleks-netizen.github.io/product-images/1205223608/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-DC-3-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-DC-3-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-DC-3-choko/003.jpg</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1205223803</t>
+          <t>BN-DC-3-navy-blue</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1205223803/001.jpg,https://oleks-netizen.github.io/product-images/1205223803/003.jpg,https://oleks-netizen.github.io/product-images/1205223803/004.jpg,https://oleks-netizen.github.io/product-images/1205223803/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-DC-3-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-DC-3-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-DC-3-navy-blue/003.jpg</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1205323609</t>
+          <t>BN-GC-12-1-navy-blue</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1205323609/001.jpg,https://oleks-netizen.github.io/product-images/1205323609/003.jpg,https://oleks-netizen.github.io/product-images/1205323609/004.jpg,https://oleks-netizen.github.io/product-images/1205323609/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-12-1-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-12-1-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-12-1-navy-blue/004.jpg</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1205323611</t>
+          <t>BN-GC-12-1-nn</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1205323611/001.jpg,https://oleks-netizen.github.io/product-images/1205323611/003.jpg,https://oleks-netizen.github.io/product-images/1205323611/004.jpg,https://oleks-netizen.github.io/product-images/1205323611/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-12-1-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-12-1-nn/003.jpg</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1205323802</t>
+          <t>BN-GC-13-1-iz-felt-d</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1205323802/001.jpg,https://oleks-netizen.github.io/product-images/1205323802/003.jpg,https://oleks-netizen.github.io/product-images/1205323802/004.jpg,https://oleks-netizen.github.io/product-images/1205323802/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-13-1-iz-felt-d/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-13-1-iz-felt-d/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-13-1-iz-felt-d/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-13-1-iz-felt-d/005.jpg</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -901,42 +901,42 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1214223808</t>
+          <t>BN-GC-31-maxi-caramel</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1214223808/001.jpg,https://oleks-netizen.github.io/product-images/1214223808/003.jpg,https://oleks-netizen.github.io/product-images/1214223808/004.jpg,https://oleks-netizen.github.io/product-images/1214223808/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-31-maxi-caramel/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-31-maxi-caramel/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-31-maxi-caramel/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-31-maxi-caramel/005.jpg,https://oleks-netizen.github.io/product-images/BN-GC-31-maxi-caramel/006.jpg,https://oleks-netizen.github.io/product-images/BN-GC-31-maxi-caramel/007.jpg</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1214223809</t>
+          <t>BN-GC-7-k</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1214223809/001.jpg,https://oleks-netizen.github.io/product-images/1214223809/003.jpg,https://oleks-netizen.github.io/product-images/1214223809/004.jpg,https://oleks-netizen.github.io/product-images/1214223809/005.jpg,https://oleks-netizen.github.io/product-images/1214223809/006.jpg,https://oleks-netizen.github.io/product-images/1214223809/007.jpg,https://oleks-netizen.github.io/product-images/1214223809/008.jpg,https://oleks-netizen.github.io/product-images/1214223809/009.jpg,https://oleks-netizen.github.io/product-images/1214223809/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-k/002.jpg</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1214323811</t>
+          <t>BN-KK-7-1-iz-pero</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1214323811/001.jpg,https://oleks-netizen.github.io/product-images/1214323811/002.jpg,https://oleks-netizen.github.io/product-images/1214323811/003.jpg,https://oleks-netizen.github.io/product-images/1214323811/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-KK-7-1-iz-pero/001.jpg,https://oleks-netizen.github.io/product-images/BN-KK-7-1-iz-pero/002.jpg,https://oleks-netizen.github.io/product-images/BN-KK-7-1-iz-pero/003.jpg,https://oleks-netizen.github.io/product-images/BN-KK-7-1-iz-pero/004.jpg</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -946,87 +946,87 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1214423812</t>
+          <t>BN-KK-7-1-nn-pero</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1214423812/001.jpg,https://oleks-netizen.github.io/product-images/1214423812/003.jpg,https://oleks-netizen.github.io/product-images/1214423812/004.jpg,https://oleks-netizen.github.io/product-images/1214423812/005.jpg,https://oleks-netizen.github.io/product-images/1214423812/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-KK-7-1-nn-pero/001.jpg,https://oleks-netizen.github.io/product-images/BN-KK-7-1-nn-pero/002.jpg,https://oleks-netizen.github.io/product-images/BN-KK-7-1-nn-pero/003.jpg</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>22991</t>
+          <t>BN-KLATCH-5-red</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/22991/001.jpg,https://oleks-netizen.github.io/product-images/22991/002.jpg,https://oleks-netizen.github.io/product-images/22991/003.jpg,https://oleks-netizen.github.io/product-images/22991/004.jpg,https://oleks-netizen.github.io/product-images/22991/005.jpg,https://oleks-netizen.github.io/product-images/22991/006.jpg,https://oleks-netizen.github.io/product-images/22991/007.jpg,https://oleks-netizen.github.io/product-images/22991/008.jpg,https://oleks-netizen.github.io/product-images/22991/009.jpg,https://oleks-netizen.github.io/product-images/22991/010.jpg,https://oleks-netizen.github.io/product-images/22991/011.jpg,https://oleks-netizen.github.io/product-images/22991/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-KLATCH-5-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-KLATCH-5-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-KLATCH-5-red/003.jpg,https://oleks-netizen.github.io/product-images/BN-KLATCH-5-red/004.jpg,https://oleks-netizen.github.io/product-images/BN-KLATCH-5-red/005.jpg,https://oleks-netizen.github.io/product-images/BN-KLATCH-5-red/006.jpg,https://oleks-netizen.github.io/product-images/BN-KLATCH-5-red/007.jpg</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>54500020</t>
+          <t>BN-OP-7-4-k</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/54500020/001.jpg,https://oleks-netizen.github.io/product-images/54500020/002.jpg,https://oleks-netizen.github.io/product-images/54500020/003.jpg,https://oleks-netizen.github.io/product-images/54500020/005.jpg,https://oleks-netizen.github.io/product-images/54500020/006.jpg,https://oleks-netizen.github.io/product-images/54500020/007.jpg,https://oleks-netizen.github.io/product-images/54500020/008.jpg,https://oleks-netizen.github.io/product-images/54500020/009.jpg,https://oleks-netizen.github.io/product-images/54500020/010.jpg,https://oleks-netizen.github.io/product-images/54500020/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-7-4-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-7-4-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-7-4-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-7-4-k/004.jpg</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>54650030</t>
+          <t>BN-PM-13-g</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/54650030/001.jpg,https://oleks-netizen.github.io/product-images/54650030/002.jpg,https://oleks-netizen.github.io/product-images/54650030/003.jpg,https://oleks-netizen.github.io/product-images/54650030/004.jpg,https://oleks-netizen.github.io/product-images/54650030/005.jpg,https://oleks-netizen.github.io/product-images/54650030/006.jpg,https://oleks-netizen.github.io/product-images/54650030/007.jpg,https://oleks-netizen.github.io/product-images/54650030/009.jpg,https://oleks-netizen.github.io/product-images/54650030/010.jpg,https://oleks-netizen.github.io/product-images/54650030/011.jpg,https://oleks-netizen.github.io/product-images/54650030/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-PM-13-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-13-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-13-g/004.jpg,https://oleks-netizen.github.io/product-images/BN-PM-13-g/005.jpg</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>648911780</t>
+          <t>BN-PM-13-iz</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/648911780/001.jpg,https://oleks-netizen.github.io/product-images/648911780/002.jpg,https://oleks-netizen.github.io/product-images/648911780/003.jpg,https://oleks-netizen.github.io/product-images/648911780/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-PM-13-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-13-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-13-iz/003.jpg,https://oleks-netizen.github.io/product-images/BN-PM-13-iz/004.jpg,https://oleks-netizen.github.io/product-images/BN-PM-13-iz/005.jpg,https://oleks-netizen.github.io/product-images/BN-PM-13-iz/006.jpg,https://oleks-netizen.github.io/product-images/BN-PM-13-iz/007.jpg,https://oleks-netizen.github.io/product-images/BN-PM-13-iz/008.jpg</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>648911790</t>
+          <t>BN-PM-4-2-k</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/648911790/001.jpg,https://oleks-netizen.github.io/product-images/648911790/002.jpg,https://oleks-netizen.github.io/product-images/648911790/003.jpg,https://oleks-netizen.github.io/product-images/648911790/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-PM-4-2-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-4-2-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-4-2-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-PM-4-2-k/006.jpg</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1036,12 +1036,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>662211610</t>
+          <t>BN-PM-7-nn</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/662211610/001.jpg,https://oleks-netizen.github.io/product-images/662211610/002.jpg,https://oleks-netizen.github.io/product-images/662211610/003.jpg,https://oleks-netizen.github.io/product-images/662211610/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-PM-7-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-7-nn/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-7-nn/003.jpg,https://oleks-netizen.github.io/product-images/BN-PM-7-nn/004.jpg</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1051,297 +1051,297 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>662214550</t>
+          <t>BN-PM-8-k</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/662214550/001.jpg,https://oleks-netizen.github.io/product-images/662214550/002.jpg,https://oleks-netizen.github.io/product-images/662214550/003.jpg,https://oleks-netizen.github.io/product-images/662214550/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-PM-8-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-8-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-8-k/004.jpg</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>80460102</t>
+          <t>BN-PM-9-1-k</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80460102/001.jpg,https://oleks-netizen.github.io/product-images/80460102/003.jpg,https://oleks-netizen.github.io/product-images/80460102/004.jpg,https://oleks-netizen.github.io/product-images/80460102/005.jpg,https://oleks-netizen.github.io/product-images/80460102/006.jpg,https://oleks-netizen.github.io/product-images/80460102/007.jpg,https://oleks-netizen.github.io/product-images/80460102/008.jpg,https://oleks-netizen.github.io/product-images/80460102/009.jpg,https://oleks-netizen.github.io/product-images/80460102/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-PM-9-1-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-PM-9-1-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-PM-9-1-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-PM-9-1-k/004.jpg,https://oleks-netizen.github.io/product-images/BN-PM-9-1-k/005.jpg,https://oleks-netizen.github.io/product-images/BN-PM-9-1-k/006.jpg</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>935614100</t>
+          <t>BN-SB-1-st-choko</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/935614100/001.jpg,https://oleks-netizen.github.io/product-images/935614100/002.jpg,https://oleks-netizen.github.io/product-images/935614100/003.jpg,https://oleks-netizen.github.io/product-images/935614100/004.jpg,https://oleks-netizen.github.io/product-images/935614100/005.jpg,https://oleks-netizen.github.io/product-images/935614100/006.jpg,https://oleks-netizen.github.io/product-images/935614100/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-SB-1-st-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-1-st-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-1-st-choko/004.jpg</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>951119160</t>
+          <t>BN-SB-3-mi-g-kr</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/951119160/001.jpg,https://oleks-netizen.github.io/product-images/951119160/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-SB-3-mi-g-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-3-mi-g-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-3-mi-g-kr/003.jpg</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>96193002</t>
+          <t>BN-SB-5-1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/96193002/001.jpg,https://oleks-netizen.github.io/product-images/96193002/002.jpg,https://oleks-netizen.github.io/product-images/96193002/003.jpg,https://oleks-netizen.github.io/product-images/96193002/005.jpg,https://oleks-netizen.github.io/product-images/96193002/006.jpg,https://oleks-netizen.github.io/product-images/96193002/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-SB-5-1/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-5-1/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-5-1/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-5-1/004.jpg,https://oleks-netizen.github.io/product-images/BN-SB-5-1/005.jpg</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>96193072</t>
+          <t>BN-SB-7-k</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/96193072/001.jpg,https://oleks-netizen.github.io/product-images/96193072/002.jpg,https://oleks-netizen.github.io/product-images/96193072/003.jpg,https://oleks-netizen.github.io/product-images/96193072/004.jpg,https://oleks-netizen.github.io/product-images/96193072/006.jpg,https://oleks-netizen.github.io/product-images/96193072/007.jpg,https://oleks-netizen.github.io/product-images/96193072/008.jpg,https://oleks-netizen.github.io/product-images/96193072/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-SB-7-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-7-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-7-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-7-k/004.jpg</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>BN-BAG-24-llight-beige-ksr</t>
+          <t>BN-SB-9-1-g-kr</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-BAG-24-llight-beige-ksr/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-llight-beige-ksr/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-llight-beige-ksr/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-24-llight-beige-ksr/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-1-g-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-1-g-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-1-g-kr/003.jpg</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BN-OP-37-beige</t>
+          <t>BN-SB-9-A4-soft-iz</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-37-beige/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-beige/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-beige/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-beige/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-beige/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-beige/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-A4-soft-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-A4-soft-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-A4-soft-iz/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-A4-soft-iz/004.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-A4-soft-iz/005.jpg</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BN-OP-37-g</t>
+          <t>BN-SB-9-hard-navy-blue</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-37-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-g/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-g/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-g/006.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-g/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-hard-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-hard-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-hard-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-hard-navy-blue/004.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-hard-navy-blue/005.jpg</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BN-OP-37-haki-kr</t>
+          <t>BN-SB-9-hard-tiffany</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-37-haki-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-haki-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-haki-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-haki-kr/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-haki-kr/006.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-haki-kr/007.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-haki-kr/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-SB-9-hard-tiffany/001.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-hard-tiffany/002.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-hard-tiffany/003.jpg,https://oleks-netizen.github.io/product-images/BN-SB-9-hard-tiffany/004.jpg</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BN-OP-37-iz</t>
+          <t>BN-TK-1-navy-blue</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-37-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-iz/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-iz/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-iz/006.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-iz/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-TK-1-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-TK-1-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-TK-1-navy-blue/003.jpg</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BN-OP-37-navy-blue</t>
+          <t>BN-TK-1-shadow-pink</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-37-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-navy-blue/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-navy-blue/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-navy-blue/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-TK-1-shadow-pink/001.jpg,https://oleks-netizen.github.io/product-images/BN-TK-1-shadow-pink/002.jpg,https://oleks-netizen.github.io/product-images/BN-TK-1-shadow-pink/003.jpg</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BN-OP-37-red</t>
+          <t>BN-TK-2-1-red</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-37-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-red/004.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-red/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-red/006.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-red/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-TK-2-1-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-TK-2-1-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-TK-2-1-red/004.jpg</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>BN-OP-37-vin</t>
+          <t>BN-TK-5-g</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-OP-37-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-vin/002.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-vin/003.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-vin/005.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-vin/006.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-vin/007.jpg,https://oleks-netizen.github.io/product-images/BN-OP-37-vin/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-TK-5-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-TK-5-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-TK-5-g/003.jpg,https://oleks-netizen.github.io/product-images/BN-TK-5-g/004.jpg,https://oleks-netizen.github.io/product-images/BN-TK-5-g/005.jpg</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>FA-3106-3lx</t>
+          <t>BN-W-2-1-shadow</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/FA-3106-3lx/001.jpg,https://oleks-netizen.github.io/product-images/FA-3106-3lx/002.jpg,https://oleks-netizen.github.io/product-images/FA-3106-3lx/003.jpg,https://oleks-netizen.github.io/product-images/FA-3106-3lx/004.jpg,https://oleks-netizen.github.io/product-images/FA-3106-3lx/005.jpg,https://oleks-netizen.github.io/product-images/FA-3106-3lx/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-W-2-1-shadow/001.jpg,https://oleks-netizen.github.io/product-images/BN-W-2-1-shadow/002.jpg,https://oleks-netizen.github.io/product-images/BN-W-2-1-shadow/003.jpg,https://oleks-netizen.github.io/product-images/BN-W-2-1-shadow/004.jpg</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>lim-354RY</t>
+          <t>BN-W-2-1-vin-kr</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/lim-354RY/001.jpg,https://oleks-netizen.github.io/product-images/lim-354RY/002.jpg,https://oleks-netizen.github.io/product-images/lim-354RY/004.jpg,https://oleks-netizen.github.io/product-images/lim-354RY/005.jpg,https://oleks-netizen.github.io/product-images/lim-354RY/006.jpg,https://oleks-netizen.github.io/product-images/lim-354RY/007.jpg,https://oleks-netizen.github.io/product-images/lim-354RY/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-W-2-1-vin-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-W-2-1-vin-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-W-2-1-vin-kr/004.jpg,https://oleks-netizen.github.io/product-images/BN-W-2-1-vin-kr/005.jpg</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>RAw-4027-3md</t>
+          <t>TW-Explorer-S-black</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RAw-4027-3md/001.jpg,https://oleks-netizen.github.io/product-images/RAw-4027-3md/002.jpg,https://oleks-netizen.github.io/product-images/RAw-4027-3md/003.jpg,https://oleks-netizen.github.io/product-images/RAw-4027-3md/004.jpg,https://oleks-netizen.github.io/product-images/RAw-4027-3md/006.jpg,https://oleks-netizen.github.io/product-images/RAw-4027-3md/007.jpg,https://oleks-netizen.github.io/product-images/RAw-4027-3md/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/TW-Explorer-S-black/001.jpg,https://oleks-netizen.github.io/product-images/TW-Explorer-S-black/002.jpg,https://oleks-netizen.github.io/product-images/TW-Explorer-S-black/003.jpg,https://oleks-netizen.github.io/product-images/TW-Explorer-S-black/004.jpg,https://oleks-netizen.github.io/product-images/TW-Explorer-S-black/005.jpg</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>RB-2203R-2202L</t>
+          <t>TW-Explorer-S-brown</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RB-2203R-2202L/001.jpg,https://oleks-netizen.github.io/product-images/RB-2203R-2202L/002.jpg,https://oleks-netizen.github.io/product-images/RB-2203R-2202L/003.jpg,https://oleks-netizen.github.io/product-images/RB-2203R-2202L/004.jpg,https://oleks-netizen.github.io/product-images/RB-2203R-2202L/005.jpg,https://oleks-netizen.github.io/product-images/RB-2203R-2202L/007.jpg,https://oleks-netizen.github.io/product-images/RB-2203R-2202L/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/TW-Explorer-S-brown/001.jpg,https://oleks-netizen.github.io/product-images/TW-Explorer-S-brown/002.jpg,https://oleks-netizen.github.io/product-images/TW-Explorer-S-brown/003.jpg,https://oleks-netizen.github.io/product-images/TW-Explorer-S-brown/004.jpg</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>RC-7266-3md</t>
+          <t>TW-Groove-S-dark-beige-flo</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RC-7266-3md/001.jpg,https://oleks-netizen.github.io/product-images/RC-7266-3md/002.jpg,https://oleks-netizen.github.io/product-images/RC-7266-3md/003.jpg,https://oleks-netizen.github.io/product-images/RC-7266-3md/004.jpg,https://oleks-netizen.github.io/product-images/RC-7266-3md/005.jpg,https://oleks-netizen.github.io/product-images/RC-7266-3md/006.jpg,https://oleks-netizen.github.io/product-images/RC-7266-3md/008.jpg,https://oleks-netizen.github.io/product-images/RC-7266-3md/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/TW-Groove-S-dark-beige-flo/001.jpg,https://oleks-netizen.github.io/product-images/TW-Groove-S-dark-beige-flo/002.jpg,https://oleks-netizen.github.io/product-images/TW-Groove-S-dark-beige-flo/003.jpg,https://oleks-netizen.github.io/product-images/TW-Groove-S-dark-beige-flo/005.jpg,https://oleks-netizen.github.io/product-images/TW-Groove-S-dark-beige-flo/006.jpg,https://oleks-netizen.github.io/product-images/TW-Groove-S-dark-beige-flo/007.jpg</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Rcam-3027-4lx</t>
+          <t>TW-Kelly-black</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/Rcam-3027-4lx/001.jpg,https://oleks-netizen.github.io/product-images/Rcam-3027-4lx/002.jpg,https://oleks-netizen.github.io/product-images/Rcam-3027-4lx/003.jpg,https://oleks-netizen.github.io/product-images/Rcam-3027-4lx/005.jpg,https://oleks-netizen.github.io/product-images/Rcam-3027-4lx/006.jpg,https://oleks-netizen.github.io/product-images/Rcam-3027-4lx/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/TW-Kelly-black/001.jpg,https://oleks-netizen.github.io/product-images/TW-Kelly-black/002.jpg,https://oleks-netizen.github.io/product-images/TW-Kelly-black/003.jpg,https://oleks-netizen.github.io/product-images/TW-Kelly-black/004.jpg,https://oleks-netizen.github.io/product-images/TW-Kelly-black/005.jpg,https://oleks-netizen.github.io/product-images/TW-Kelly-black/007.jpg</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -1351,16 +1351,271 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>RW-30271-3md</t>
+          <t>TW-Molly-green</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RW-30271-3md/001.jpg,https://oleks-netizen.github.io/product-images/RW-30271-3md/002.jpg,https://oleks-netizen.github.io/product-images/RW-30271-3md/004.jpg,https://oleks-netizen.github.io/product-images/RW-30271-3md/005.jpg,https://oleks-netizen.github.io/product-images/RW-30271-3md/006.jpg,https://oleks-netizen.github.io/product-images/RW-30271-3md/007.jpg,https://oleks-netizen.github.io/product-images/RW-30271-3md/008.jpg,https://oleks-netizen.github.io/product-images/RW-30271-3md/009.jpg,https://oleks-netizen.github.io/product-images/RW-30271-3md/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/TW-Molly-green/001.jpg,https://oleks-netizen.github.io/product-images/TW-Molly-green/002.jpg,https://oleks-netizen.github.io/product-images/TW-Molly-green/003.jpg,https://oleks-netizen.github.io/product-images/TW-Molly-green/004.jpg,https://oleks-netizen.github.io/product-images/TW-Molly-green/005.jpg</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>9</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>TW-Rubby-small-light-blue</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Rubby-small-light-blue/001.jpg,https://oleks-netizen.github.io/product-images/TW-Rubby-small-light-blue/003.jpg</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>TW-Ruby-big-beige</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Ruby-big-beige/001.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-beige/003.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-beige/004.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-beige/005.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-beige/006.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-beige/007.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-beige/008.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-beige/009.jpg</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>TW-Ruby-big-mars</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/001.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/002.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/003.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/004.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/005.jpg,https://oleks-netizen.github.io/product-images/TW-Ruby-big-mars/006.jpg</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>TW-Stella-dark-blue</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Stella-dark-blue/001.jpg,https://oleks-netizen.github.io/product-images/TW-Stella-dark-blue/002.jpg,https://oleks-netizen.github.io/product-images/TW-Stella-dark-blue/003.jpg,https://oleks-netizen.github.io/product-images/TW-Stella-dark-blue/004.jpg,https://oleks-netizen.github.io/product-images/TW-Stella-dark-blue/005.jpg,https://oleks-netizen.github.io/product-images/TW-Stella-dark-blue/006.jpg</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>TW-Tammy-light</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Tammy-light/001.jpg,https://oleks-netizen.github.io/product-images/TW-Tammy-light/002.jpg,https://oleks-netizen.github.io/product-images/TW-Tammy-light/003.jpg,https://oleks-netizen.github.io/product-images/TW-Tammy-light/004.jpg,https://oleks-netizen.github.io/product-images/TW-Tammy-light/005.jpg,https://oleks-netizen.github.io/product-images/TW-Tammy-light/006.jpg,https://oleks-netizen.github.io/product-images/TW-Tammy-light/007.jpg,https://oleks-netizen.github.io/product-images/TW-Tammy-light/009.jpg</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>TW-Yoko-olive</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Yoko-olive/001.jpg,https://oleks-netizen.github.io/product-images/TW-Yoko-olive/002.jpg,https://oleks-netizen.github.io/product-images/TW-Yoko-olive/003.jpg,https://oleks-netizen.github.io/product-images/TW-Yoko-olive/004.jpg,https://oleks-netizen.github.io/product-images/TW-Yoko-olive/005.jpg</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>BN-GC-11-1-g</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-11-1-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-11-1-g/004.jpg</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>BN-GC-29-malachite</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-29-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-29-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-29-malachite/004.jpg,https://oleks-netizen.github.io/product-images/BN-GC-29-malachite/006.jpg</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>BN-GC-9-navy-blue</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-9-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-9-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-9-navy-blue/005.jpg</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>BN-GC-9-tiffany</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-9-tiffany/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-9-tiffany/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-9-tiffany/005.jpg</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>BN-KK-5-malachite</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-KK-5-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-KK-5-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-KK-5-malachite/005.jpg</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>BN-KK-5-nn</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-KK-5-nn/002.jpg,https://oleks-netizen.github.io/product-images/BN-KK-5-nn/003.jpg,https://oleks-netizen.github.io/product-images/BN-KK-5-nn/004.jpg,https://oleks-netizen.github.io/product-images/BN-KK-5-nn/005.jpg,https://oleks-netizen.github.io/product-images/BN-KK-5-nn/007.jpg</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>BN-KL-1-navy-blue</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-KL-1-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-KL-1-navy-blue/003.jpg,https://oleks-netizen.github.io/product-images/BN-KL-1-navy-blue/004.jpg,https://oleks-netizen.github.io/product-images/BN-KL-1-navy-blue/005.jpg,https://oleks-netizen.github.io/product-images/BN-KL-1-navy-blue/007.jpg</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>BN-KL-3-1-crem-brule</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-KL-3-1-crem-brule/002.jpg,https://oleks-netizen.github.io/product-images/BN-KL-3-1-crem-brule/003.jpg,https://oleks-netizen.github.io/product-images/BN-KL-3-1-crem-brule/005.jpg</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>BN-KL-5-choko</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-KL-5-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-choko/003.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-choko/004.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-choko/005.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-choko/006.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-choko/007.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-choko/009.jpg</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>BN-KL-5-k</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-KL-5-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-k/004.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-k/005.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-k/006.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-k/007.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-k/009.jpg</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>BN-KL-5-malachite</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-KL-5-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-malachite/004.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-malachite/005.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-malachite/006.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-malachite/007.jpg,https://oleks-netizen.github.io/product-images/BN-KL-5-malachite/009.jpg</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-07-22 12:26:26
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,12 +436,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WELL-11108</t>
+          <t>WELL-12402</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-11108/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11108/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11108/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12402/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12402/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12402/003.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -451,102 +451,102 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WELL-11901</t>
+          <t>WELL-12508</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-11901/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11901/002.jpg,https://oleks-netizen.github.io/product-images/WELL-11901/004.jpg,https://oleks-netizen.github.io/product-images/WELL-11901/005.jpg,https://oleks-netizen.github.io/product-images/WELL-11901/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-12508/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12508/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12508/004.jpg,https://oleks-netizen.github.io/product-images/WELL-12508/005.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>WELL-13002</t>
+          <t>WELL-46514</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-13002/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13002/003.jpg,https://oleks-netizen.github.io/product-images/WELL-13002/004.jpg,https://oleks-netizen.github.io/product-images/WELL-13002/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-46514/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46514/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46514/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46514/005.jpg,https://oleks-netizen.github.io/product-images/WELL-46514/006.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WELL-13009</t>
+          <t>WELL-47304</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-13009/001.jpg,https://oleks-netizen.github.io/product-images/WELL-13009/003.jpg,https://oleks-netizen.github.io/product-images/WELL-13009/004.jpg,https://oleks-netizen.github.io/product-images/WELL-13009/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-47304/001.jpg,https://oleks-netizen.github.io/product-images/WELL-47304/002.jpg,https://oleks-netizen.github.io/product-images/WELL-47304/004.jpg,https://oleks-netizen.github.io/product-images/WELL-47304/005.jpg,https://oleks-netizen.github.io/product-images/WELL-47304/006.jpg,https://oleks-netizen.github.io/product-images/WELL-47304/007.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WELL-44455</t>
+          <t>WELL-60206</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-44455/001.jpg,https://oleks-netizen.github.io/product-images/WELL-44455/002.jpg,https://oleks-netizen.github.io/product-images/WELL-44455/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-60206/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60206/002.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WELL-45107</t>
+          <t>WELL-61404</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-45107/001.jpg,https://oleks-netizen.github.io/product-images/WELL-45107/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61404/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61404/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61404/003.jpg,https://oleks-netizen.github.io/product-images/WELL-61404/004.jpg,https://oleks-netizen.github.io/product-images/WELL-61404/005.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WELL-46401</t>
+          <t>WELL-61409</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-46401/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46401/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46401/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46401/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61409/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61409/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61409/003.jpg,https://oleks-netizen.github.io/product-images/WELL-61409/004.jpg,https://oleks-netizen.github.io/product-images/WELL-61409/005.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>WELL-47309</t>
+          <t>WELL-61600</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-47309/001.jpg,https://oleks-netizen.github.io/product-images/WELL-47309/003.jpg,https://oleks-netizen.github.io/product-images/WELL-47309/004.jpg,https://oleks-netizen.github.io/product-images/WELL-47309/005.jpg,https://oleks-netizen.github.io/product-images/WELL-47309/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-61600/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61600/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61600/003.jpg,https://oleks-netizen.github.io/product-images/WELL-61600/004.jpg,https://oleks-netizen.github.io/product-images/WELL-61600/005.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -556,27 +556,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>WELL-56311</t>
+          <t>WELL-66802</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-56311/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56311/002.jpg,https://oleks-netizen.github.io/product-images/WELL-56311/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-66802/001.jpg,https://oleks-netizen.github.io/product-images/WELL-66802/002.jpg,https://oleks-netizen.github.io/product-images/WELL-66802/003.jpg,https://oleks-netizen.github.io/product-images/WELL-66802/004.jpg,https://oleks-netizen.github.io/product-images/WELL-66802/005.jpg,https://oleks-netizen.github.io/product-images/WELL-66802/006.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>WELL-56510</t>
+          <t>WELL-67209</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-56510/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56510/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-67209/001.jpg,https://oleks-netizen.github.io/product-images/WELL-67209/002.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -586,135 +586,60 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WELL-56511</t>
+          <t>WELL-68404</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-56511/001.jpg,https://oleks-netizen.github.io/product-images/WELL-56511/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-68404/001.jpg,https://oleks-netizen.github.io/product-images/WELL-68404/003.jpg,https://oleks-netizen.github.io/product-images/WELL-68404/004.jpg,https://oleks-netizen.github.io/product-images/WELL-68404/005.jpg,https://oleks-netizen.github.io/product-images/WELL-68404/006.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>WELL-60127</t>
+          <t>WELL-69505</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-60127/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60127/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60127/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-69505/001.jpg,https://oleks-netizen.github.io/product-images/WELL-69505/003.jpg,https://oleks-netizen.github.io/product-images/WELL-69505/004.jpg,https://oleks-netizen.github.io/product-images/WELL-69505/005.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WELL-60504</t>
+          <t>WELL-69604</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-60504/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60504/002.jpg,https://oleks-netizen.github.io/product-images/WELL-60504/003.jpg,https://oleks-netizen.github.io/product-images/WELL-60504/004.jpg,https://oleks-netizen.github.io/product-images/WELL-60504/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-69604/001.jpg,https://oleks-netizen.github.io/product-images/WELL-69604/003.jpg,https://oleks-netizen.github.io/product-images/WELL-69604/004.jpg,https://oleks-netizen.github.io/product-images/WELL-69604/005.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>WELL-61013</t>
+          <t>WELL-90201</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-61013/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61013/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/WELL-90201/001.jpg,https://oleks-netizen.github.io/product-images/WELL-90201/002.jpg,https://oleks-netizen.github.io/product-images/WELL-90201/003.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>WELL-62404</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-62404/001.jpg,https://oleks-netizen.github.io/product-images/WELL-62404/003.jpg,https://oleks-netizen.github.io/product-images/WELL-62404/004.jpg,https://oleks-netizen.github.io/product-images/WELL-62404/005.jpg,https://oleks-netizen.github.io/product-images/WELL-62404/006.jpg</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>WELL-63204</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-63204/001.jpg,https://oleks-netizen.github.io/product-images/WELL-63204/003.jpg,https://oleks-netizen.github.io/product-images/WELL-63204/004.jpg,https://oleks-netizen.github.io/product-images/WELL-63204/005.jpg,https://oleks-netizen.github.io/product-images/WELL-63204/006.jpg</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>WELL-65621</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-65621/001.jpg,https://oleks-netizen.github.io/product-images/WELL-65621/002.jpg,https://oleks-netizen.github.io/product-images/WELL-65621/003.jpg,https://oleks-netizen.github.io/product-images/WELL-65621/004.jpg</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>WELL-70101</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-70101/001.jpg,https://oleks-netizen.github.io/product-images/WELL-70101/002.jpg,https://oleks-netizen.github.io/product-images/WELL-70101/003.jpg</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>WELL-70104</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-70104/001.jpg,https://oleks-netizen.github.io/product-images/WELL-70104/002.jpg,https://oleks-netizen.github.io/product-images/WELL-70104/003.jpg</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update 2026-07-23 08:37:00
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,57 +436,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WELL-12402</t>
+          <t>90002</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-12402/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12402/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12402/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90002/001.jpg,https://oleks-netizen.github.io/product-images/90002/002.jpg,https://oleks-netizen.github.io/product-images/90002/004.jpg,https://oleks-netizen.github.io/product-images/90002/005.jpg,https://oleks-netizen.github.io/product-images/90002/006.jpg,https://oleks-netizen.github.io/product-images/90002/007.jpg,https://oleks-netizen.github.io/product-images/90002/008.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WELL-12508</t>
+          <t>90021</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-12508/001.jpg,https://oleks-netizen.github.io/product-images/WELL-12508/002.jpg,https://oleks-netizen.github.io/product-images/WELL-12508/004.jpg,https://oleks-netizen.github.io/product-images/WELL-12508/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90021/001.jpg,https://oleks-netizen.github.io/product-images/90021/003.jpg,https://oleks-netizen.github.io/product-images/90021/004.jpg,https://oleks-netizen.github.io/product-images/90021/005.jpg,https://oleks-netizen.github.io/product-images/90021/006.jpg,https://oleks-netizen.github.io/product-images/90021/007.jpg,https://oleks-netizen.github.io/product-images/90021/008.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>WELL-46514</t>
+          <t>90022</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-46514/001.jpg,https://oleks-netizen.github.io/product-images/WELL-46514/002.jpg,https://oleks-netizen.github.io/product-images/WELL-46514/003.jpg,https://oleks-netizen.github.io/product-images/WELL-46514/005.jpg,https://oleks-netizen.github.io/product-images/WELL-46514/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90022/001.jpg,https://oleks-netizen.github.io/product-images/90022/003.jpg,https://oleks-netizen.github.io/product-images/90022/004.jpg,https://oleks-netizen.github.io/product-images/90022/005.jpg,https://oleks-netizen.github.io/product-images/90022/006.jpg,https://oleks-netizen.github.io/product-images/90022/007.jpg,https://oleks-netizen.github.io/product-images/90022/008.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WELL-47304</t>
+          <t>90027</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-47304/001.jpg,https://oleks-netizen.github.io/product-images/WELL-47304/002.jpg,https://oleks-netizen.github.io/product-images/WELL-47304/004.jpg,https://oleks-netizen.github.io/product-images/WELL-47304/005.jpg,https://oleks-netizen.github.io/product-images/WELL-47304/006.jpg,https://oleks-netizen.github.io/product-images/WELL-47304/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90027/001.jpg,https://oleks-netizen.github.io/product-images/90027/002.jpg,https://oleks-netizen.github.io/product-images/90027/003.jpg,https://oleks-netizen.github.io/product-images/90027/004.jpg,https://oleks-netizen.github.io/product-images/90027/005.jpg,https://oleks-netizen.github.io/product-images/90027/006.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -496,151 +496,1141 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WELL-60206</t>
+          <t>90028</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-60206/001.jpg,https://oleks-netizen.github.io/product-images/WELL-60206/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90028/001.jpg,https://oleks-netizen.github.io/product-images/90028/002.jpg,https://oleks-netizen.github.io/product-images/90028/004.jpg,https://oleks-netizen.github.io/product-images/90028/005.jpg,https://oleks-netizen.github.io/product-images/90028/006.jpg,https://oleks-netizen.github.io/product-images/90028/007.jpg,https://oleks-netizen.github.io/product-images/90028/008.jpg,https://oleks-netizen.github.io/product-images/90028/009.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WELL-61404</t>
+          <t>90029</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-61404/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61404/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61404/003.jpg,https://oleks-netizen.github.io/product-images/WELL-61404/004.jpg,https://oleks-netizen.github.io/product-images/WELL-61404/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90029/001.jpg,https://oleks-netizen.github.io/product-images/90029/002.jpg,https://oleks-netizen.github.io/product-images/90029/004.jpg,https://oleks-netizen.github.io/product-images/90029/005.jpg,https://oleks-netizen.github.io/product-images/90029/006.jpg,https://oleks-netizen.github.io/product-images/90029/007.jpg,https://oleks-netizen.github.io/product-images/90029/008.jpg,https://oleks-netizen.github.io/product-images/90029/009.jpg,https://oleks-netizen.github.io/product-images/90029/010.jpg,https://oleks-netizen.github.io/product-images/90029/011.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WELL-61409</t>
+          <t>90065</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-61409/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61409/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61409/003.jpg,https://oleks-netizen.github.io/product-images/WELL-61409/004.jpg,https://oleks-netizen.github.io/product-images/WELL-61409/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90065/001.jpg,https://oleks-netizen.github.io/product-images/90065/002.jpg,https://oleks-netizen.github.io/product-images/90065/004.jpg,https://oleks-netizen.github.io/product-images/90065/005.jpg,https://oleks-netizen.github.io/product-images/90065/006.jpg,https://oleks-netizen.github.io/product-images/90065/007.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>WELL-61600</t>
+          <t>90087</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-61600/001.jpg,https://oleks-netizen.github.io/product-images/WELL-61600/002.jpg,https://oleks-netizen.github.io/product-images/WELL-61600/003.jpg,https://oleks-netizen.github.io/product-images/WELL-61600/004.jpg,https://oleks-netizen.github.io/product-images/WELL-61600/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90087/001.jpg,https://oleks-netizen.github.io/product-images/90087/002.jpg,https://oleks-netizen.github.io/product-images/90087/004.jpg,https://oleks-netizen.github.io/product-images/90087/005.jpg,https://oleks-netizen.github.io/product-images/90087/006.jpg,https://oleks-netizen.github.io/product-images/90087/007.jpg,https://oleks-netizen.github.io/product-images/90087/008.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>WELL-66802</t>
+          <t>90152</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-66802/001.jpg,https://oleks-netizen.github.io/product-images/WELL-66802/002.jpg,https://oleks-netizen.github.io/product-images/WELL-66802/003.jpg,https://oleks-netizen.github.io/product-images/WELL-66802/004.jpg,https://oleks-netizen.github.io/product-images/WELL-66802/005.jpg,https://oleks-netizen.github.io/product-images/WELL-66802/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90152/001.jpg,https://oleks-netizen.github.io/product-images/90152/002.jpg,https://oleks-netizen.github.io/product-images/90152/003.jpg,https://oleks-netizen.github.io/product-images/90152/004.jpg,https://oleks-netizen.github.io/product-images/90152/005.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>WELL-67209</t>
+          <t>90153</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-67209/001.jpg,https://oleks-netizen.github.io/product-images/WELL-67209/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90153/001.jpg,https://oleks-netizen.github.io/product-images/90153/002.jpg,https://oleks-netizen.github.io/product-images/90153/003.jpg,https://oleks-netizen.github.io/product-images/90153/004.jpg,https://oleks-netizen.github.io/product-images/90153/005.jpg,https://oleks-netizen.github.io/product-images/90153/006.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WELL-68404</t>
+          <t>90154</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-68404/001.jpg,https://oleks-netizen.github.io/product-images/WELL-68404/003.jpg,https://oleks-netizen.github.io/product-images/WELL-68404/004.jpg,https://oleks-netizen.github.io/product-images/WELL-68404/005.jpg,https://oleks-netizen.github.io/product-images/WELL-68404/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90154/001.jpg,https://oleks-netizen.github.io/product-images/90154/002.jpg,https://oleks-netizen.github.io/product-images/90154/003.jpg,https://oleks-netizen.github.io/product-images/90154/004.jpg,https://oleks-netizen.github.io/product-images/90154/005.jpg,https://oleks-netizen.github.io/product-images/90154/006.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>WELL-69505</t>
+          <t>90155</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-69505/001.jpg,https://oleks-netizen.github.io/product-images/WELL-69505/003.jpg,https://oleks-netizen.github.io/product-images/WELL-69505/004.jpg,https://oleks-netizen.github.io/product-images/WELL-69505/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90155/001.jpg,https://oleks-netizen.github.io/product-images/90155/002.jpg,https://oleks-netizen.github.io/product-images/90155/003.jpg,https://oleks-netizen.github.io/product-images/90155/004.jpg,https://oleks-netizen.github.io/product-images/90155/005.jpg,https://oleks-netizen.github.io/product-images/90155/006.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WELL-69604</t>
+          <t>90156</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-69604/001.jpg,https://oleks-netizen.github.io/product-images/WELL-69604/003.jpg,https://oleks-netizen.github.io/product-images/WELL-69604/004.jpg,https://oleks-netizen.github.io/product-images/WELL-69604/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90156/001.jpg,https://oleks-netizen.github.io/product-images/90156/002.jpg,https://oleks-netizen.github.io/product-images/90156/003.jpg,https://oleks-netizen.github.io/product-images/90156/004.jpg,https://oleks-netizen.github.io/product-images/90156/005.jpg,https://oleks-netizen.github.io/product-images/90156/006.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>WELL-90201</t>
+          <t>90157</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-90201/001.jpg,https://oleks-netizen.github.io/product-images/WELL-90201/002.jpg,https://oleks-netizen.github.io/product-images/WELL-90201/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90157/001.jpg,https://oleks-netizen.github.io/product-images/90157/002.jpg,https://oleks-netizen.github.io/product-images/90157/003.jpg,https://oleks-netizen.github.io/product-images/90157/004.jpg,https://oleks-netizen.github.io/product-images/90157/005.jpg,https://oleks-netizen.github.io/product-images/90157/006.jpg,https://oleks-netizen.github.io/product-images/90157/007.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>90158</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90158/001.jpg,https://oleks-netizen.github.io/product-images/90158/002.jpg,https://oleks-netizen.github.io/product-images/90158/003.jpg,https://oleks-netizen.github.io/product-images/90158/004.jpg,https://oleks-netizen.github.io/product-images/90158/005.jpg,https://oleks-netizen.github.io/product-images/90158/006.jpg,https://oleks-netizen.github.io/product-images/90158/007.jpg</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>90159</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90159/001.jpg,https://oleks-netizen.github.io/product-images/90159/002.jpg,https://oleks-netizen.github.io/product-images/90159/003.jpg,https://oleks-netizen.github.io/product-images/90159/004.jpg,https://oleks-netizen.github.io/product-images/90159/005.jpg,https://oleks-netizen.github.io/product-images/90159/006.jpg,https://oleks-netizen.github.io/product-images/90159/007.jpg</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>90160</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90160/001.jpg,https://oleks-netizen.github.io/product-images/90160/002.jpg,https://oleks-netizen.github.io/product-images/90160/003.jpg,https://oleks-netizen.github.io/product-images/90160/004.jpg,https://oleks-netizen.github.io/product-images/90160/005.jpg,https://oleks-netizen.github.io/product-images/90160/006.jpg,https://oleks-netizen.github.io/product-images/90160/007.jpg</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>90161</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90161/001.jpg,https://oleks-netizen.github.io/product-images/90161/002.jpg,https://oleks-netizen.github.io/product-images/90161/003.jpg,https://oleks-netizen.github.io/product-images/90161/004.jpg,https://oleks-netizen.github.io/product-images/90161/005.jpg</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>90162</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90162/001.jpg,https://oleks-netizen.github.io/product-images/90162/002.jpg,https://oleks-netizen.github.io/product-images/90162/003.jpg,https://oleks-netizen.github.io/product-images/90162/004.jpg,https://oleks-netizen.github.io/product-images/90162/005.jpg,https://oleks-netizen.github.io/product-images/90162/006.jpg,https://oleks-netizen.github.io/product-images/90162/007.jpg</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>90163</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90163/001.jpg,https://oleks-netizen.github.io/product-images/90163/002.jpg,https://oleks-netizen.github.io/product-images/90163/003.jpg,https://oleks-netizen.github.io/product-images/90163/004.jpg,https://oleks-netizen.github.io/product-images/90163/005.jpg,https://oleks-netizen.github.io/product-images/90163/006.jpg,https://oleks-netizen.github.io/product-images/90163/007.jpg</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>90164</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90164/001.jpg,https://oleks-netizen.github.io/product-images/90164/002.jpg,https://oleks-netizen.github.io/product-images/90164/003.jpg,https://oleks-netizen.github.io/product-images/90164/004.jpg,https://oleks-netizen.github.io/product-images/90164/005.jpg,https://oleks-netizen.github.io/product-images/90164/006.jpg,https://oleks-netizen.github.io/product-images/90164/007.jpg</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>90166</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90166/001.jpg,https://oleks-netizen.github.io/product-images/90166/002.jpg,https://oleks-netizen.github.io/product-images/90166/003.jpg,https://oleks-netizen.github.io/product-images/90166/004.jpg,https://oleks-netizen.github.io/product-images/90166/005.jpg,https://oleks-netizen.github.io/product-images/90166/006.jpg</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>90168</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90168/001.jpg,https://oleks-netizen.github.io/product-images/90168/002.jpg,https://oleks-netizen.github.io/product-images/90168/003.jpg,https://oleks-netizen.github.io/product-images/90168/004.jpg,https://oleks-netizen.github.io/product-images/90168/005.jpg,https://oleks-netizen.github.io/product-images/90168/006.jpg,https://oleks-netizen.github.io/product-images/90168/007.jpg,https://oleks-netizen.github.io/product-images/90168/008.jpg,https://oleks-netizen.github.io/product-images/90168/009.jpg</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>90169</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90169/001.jpg,https://oleks-netizen.github.io/product-images/90169/002.jpg,https://oleks-netizen.github.io/product-images/90169/003.jpg,https://oleks-netizen.github.io/product-images/90169/004.jpg,https://oleks-netizen.github.io/product-images/90169/005.jpg,https://oleks-netizen.github.io/product-images/90169/006.jpg</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>90170</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90170/001.jpg,https://oleks-netizen.github.io/product-images/90170/002.jpg,https://oleks-netizen.github.io/product-images/90170/003.jpg,https://oleks-netizen.github.io/product-images/90170/004.jpg,https://oleks-netizen.github.io/product-images/90170/005.jpg,https://oleks-netizen.github.io/product-images/90170/006.jpg</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>90171</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90171/001.jpg,https://oleks-netizen.github.io/product-images/90171/002.jpg,https://oleks-netizen.github.io/product-images/90171/003.jpg,https://oleks-netizen.github.io/product-images/90171/004.jpg,https://oleks-netizen.github.io/product-images/90171/005.jpg,https://oleks-netizen.github.io/product-images/90171/006.jpg</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>90172</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90172/001.jpg,https://oleks-netizen.github.io/product-images/90172/002.jpg,https://oleks-netizen.github.io/product-images/90172/004.jpg,https://oleks-netizen.github.io/product-images/90172/005.jpg,https://oleks-netizen.github.io/product-images/90172/006.jpg,https://oleks-netizen.github.io/product-images/90172/007.jpg,https://oleks-netizen.github.io/product-images/90172/008.jpg</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>90173</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90173/001.jpg,https://oleks-netizen.github.io/product-images/90173/002.jpg,https://oleks-netizen.github.io/product-images/90173/004.jpg,https://oleks-netizen.github.io/product-images/90173/005.jpg,https://oleks-netizen.github.io/product-images/90173/006.jpg,https://oleks-netizen.github.io/product-images/90173/007.jpg,https://oleks-netizen.github.io/product-images/90173/008.jpg</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>90174</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90174/001.jpg,https://oleks-netizen.github.io/product-images/90174/002.jpg,https://oleks-netizen.github.io/product-images/90174/003.jpg,https://oleks-netizen.github.io/product-images/90174/004.jpg,https://oleks-netizen.github.io/product-images/90174/005.jpg,https://oleks-netizen.github.io/product-images/90174/006.jpg</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>90297</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90297/001.jpg,https://oleks-netizen.github.io/product-images/90297/002.jpg,https://oleks-netizen.github.io/product-images/90297/004.jpg,https://oleks-netizen.github.io/product-images/90297/005.jpg,https://oleks-netizen.github.io/product-images/90297/006.jpg,https://oleks-netizen.github.io/product-images/90297/007.jpg</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>90298</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90298/001.jpg,https://oleks-netizen.github.io/product-images/90298/002.jpg,https://oleks-netizen.github.io/product-images/90298/003.jpg,https://oleks-netizen.github.io/product-images/90298/004.jpg,https://oleks-netizen.github.io/product-images/90298/005.jpg,https://oleks-netizen.github.io/product-images/90298/006.jpg</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>90299</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90299/001.jpg,https://oleks-netizen.github.io/product-images/90299/002.jpg,https://oleks-netizen.github.io/product-images/90299/004.jpg,https://oleks-netizen.github.io/product-images/90299/005.jpg,https://oleks-netizen.github.io/product-images/90299/006.jpg,https://oleks-netizen.github.io/product-images/90299/007.jpg,https://oleks-netizen.github.io/product-images/90299/008.jpg</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>90300</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90300/001.jpg,https://oleks-netizen.github.io/product-images/90300/002.jpg,https://oleks-netizen.github.io/product-images/90300/004.jpg,https://oleks-netizen.github.io/product-images/90300/005.jpg,https://oleks-netizen.github.io/product-images/90300/006.jpg,https://oleks-netizen.github.io/product-images/90300/007.jpg</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>90301</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90301/001.jpg,https://oleks-netizen.github.io/product-images/90301/003.jpg,https://oleks-netizen.github.io/product-images/90301/004.jpg,https://oleks-netizen.github.io/product-images/90301/005.jpg,https://oleks-netizen.github.io/product-images/90301/006.jpg,https://oleks-netizen.github.io/product-images/90301/007.jpg,https://oleks-netizen.github.io/product-images/90301/008.jpg</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>90331</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90331/001.jpg,https://oleks-netizen.github.io/product-images/90331/002.jpg,https://oleks-netizen.github.io/product-images/90331/003.jpg,https://oleks-netizen.github.io/product-images/90331/004.jpg,https://oleks-netizen.github.io/product-images/90331/005.jpg</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>90347</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90347/001.jpg,https://oleks-netizen.github.io/product-images/90347/002.jpg,https://oleks-netizen.github.io/product-images/90347/003.jpg,https://oleks-netizen.github.io/product-images/90347/005.jpg,https://oleks-netizen.github.io/product-images/90347/006.jpg,https://oleks-netizen.github.io/product-images/90347/007.jpg,https://oleks-netizen.github.io/product-images/90347/008.jpg</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>90386</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90386/001.jpg,https://oleks-netizen.github.io/product-images/90386/002.jpg,https://oleks-netizen.github.io/product-images/90386/003.jpg,https://oleks-netizen.github.io/product-images/90386/004.jpg,https://oleks-netizen.github.io/product-images/90386/005.jpg</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>90387</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90387/001.jpg,https://oleks-netizen.github.io/product-images/90387/002.jpg,https://oleks-netizen.github.io/product-images/90387/004.jpg,https://oleks-netizen.github.io/product-images/90387/005.jpg,https://oleks-netizen.github.io/product-images/90387/006.jpg</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>90491</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90491/001.jpg,https://oleks-netizen.github.io/product-images/90491/002.jpg,https://oleks-netizen.github.io/product-images/90491/003.jpg,https://oleks-netizen.github.io/product-images/90491/004.jpg,https://oleks-netizen.github.io/product-images/90491/005.jpg,https://oleks-netizen.github.io/product-images/90491/006.jpg,https://oleks-netizen.github.io/product-images/90491/007.jpg,https://oleks-netizen.github.io/product-images/90491/008.jpg,https://oleks-netizen.github.io/product-images/90491/009.jpg,https://oleks-netizen.github.io/product-images/90491/010.jpg</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>90492</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90492/001.jpg,https://oleks-netizen.github.io/product-images/90492/002.jpg,https://oleks-netizen.github.io/product-images/90492/003.jpg,https://oleks-netizen.github.io/product-images/90492/004.jpg,https://oleks-netizen.github.io/product-images/90492/005.jpg,https://oleks-netizen.github.io/product-images/90492/006.jpg,https://oleks-netizen.github.io/product-images/90492/007.jpg,https://oleks-netizen.github.io/product-images/90492/009.jpg,https://oleks-netizen.github.io/product-images/90492/010.jpg,https://oleks-netizen.github.io/product-images/90492/011.jpg</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>90493</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90493/001.jpg,https://oleks-netizen.github.io/product-images/90493/002.jpg,https://oleks-netizen.github.io/product-images/90493/003.jpg,https://oleks-netizen.github.io/product-images/90493/004.jpg,https://oleks-netizen.github.io/product-images/90493/005.jpg,https://oleks-netizen.github.io/product-images/90493/006.jpg,https://oleks-netizen.github.io/product-images/90493/007.jpg,https://oleks-netizen.github.io/product-images/90493/008.jpg</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>90494</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90494/001.jpg,https://oleks-netizen.github.io/product-images/90494/002.jpg,https://oleks-netizen.github.io/product-images/90494/003.jpg,https://oleks-netizen.github.io/product-images/90494/004.jpg,https://oleks-netizen.github.io/product-images/90494/006.jpg,https://oleks-netizen.github.io/product-images/90494/007.jpg,https://oleks-netizen.github.io/product-images/90494/008.jpg,https://oleks-netizen.github.io/product-images/90494/009.jpg,https://oleks-netizen.github.io/product-images/90494/010.jpg,https://oleks-netizen.github.io/product-images/90494/011.jpg</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>90495</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90495/001.jpg,https://oleks-netizen.github.io/product-images/90495/002.jpg,https://oleks-netizen.github.io/product-images/90495/003.jpg,https://oleks-netizen.github.io/product-images/90495/004.jpg,https://oleks-netizen.github.io/product-images/90495/005.jpg,https://oleks-netizen.github.io/product-images/90495/006.jpg,https://oleks-netizen.github.io/product-images/90495/007.jpg</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>90496</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90496/001.jpg,https://oleks-netizen.github.io/product-images/90496/002.jpg,https://oleks-netizen.github.io/product-images/90496/003.jpg,https://oleks-netizen.github.io/product-images/90496/004.jpg,https://oleks-netizen.github.io/product-images/90496/005.jpg,https://oleks-netizen.github.io/product-images/90496/006.jpg,https://oleks-netizen.github.io/product-images/90496/007.jpg,https://oleks-netizen.github.io/product-images/90496/008.jpg,https://oleks-netizen.github.io/product-images/90496/009.jpg</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>90498</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90498/001.jpg,https://oleks-netizen.github.io/product-images/90498/002.jpg,https://oleks-netizen.github.io/product-images/90498/003.jpg,https://oleks-netizen.github.io/product-images/90498/004.jpg,https://oleks-netizen.github.io/product-images/90498/005.jpg,https://oleks-netizen.github.io/product-images/90498/006.jpg,https://oleks-netizen.github.io/product-images/90498/007.jpg</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>90499</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90499/001.jpg,https://oleks-netizen.github.io/product-images/90499/002.jpg,https://oleks-netizen.github.io/product-images/90499/004.jpg,https://oleks-netizen.github.io/product-images/90499/005.jpg,https://oleks-netizen.github.io/product-images/90499/006.jpg,https://oleks-netizen.github.io/product-images/90499/007.jpg</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>90500</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90500/001.jpg,https://oleks-netizen.github.io/product-images/90500/002.jpg,https://oleks-netizen.github.io/product-images/90500/003.jpg,https://oleks-netizen.github.io/product-images/90500/004.jpg,https://oleks-netizen.github.io/product-images/90500/006.jpg,https://oleks-netizen.github.io/product-images/90500/007.jpg</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>90509</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90509/001.jpg,https://oleks-netizen.github.io/product-images/90509/002.jpg,https://oleks-netizen.github.io/product-images/90509/004.jpg,https://oleks-netizen.github.io/product-images/90509/005.jpg,https://oleks-netizen.github.io/product-images/90509/006.jpg,https://oleks-netizen.github.io/product-images/90509/007.jpg</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>90510</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90510/001.jpg,https://oleks-netizen.github.io/product-images/90510/002.jpg,https://oleks-netizen.github.io/product-images/90510/003.jpg,https://oleks-netizen.github.io/product-images/90510/004.jpg,https://oleks-netizen.github.io/product-images/90510/006.jpg,https://oleks-netizen.github.io/product-images/90510/007.jpg,https://oleks-netizen.github.io/product-images/90510/008.jpg</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>90511</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90511/001.jpg,https://oleks-netizen.github.io/product-images/90511/002.jpg,https://oleks-netizen.github.io/product-images/90511/003.jpg,https://oleks-netizen.github.io/product-images/90511/005.jpg,https://oleks-netizen.github.io/product-images/90511/006.jpg,https://oleks-netizen.github.io/product-images/90511/007.jpg</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>90512</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90512/001.jpg,https://oleks-netizen.github.io/product-images/90512/002.jpg,https://oleks-netizen.github.io/product-images/90512/003.jpg,https://oleks-netizen.github.io/product-images/90512/005.jpg,https://oleks-netizen.github.io/product-images/90512/006.jpg,https://oleks-netizen.github.io/product-images/90512/007.jpg</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>90513</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90513/001.jpg,https://oleks-netizen.github.io/product-images/90513/002.jpg,https://oleks-netizen.github.io/product-images/90513/003.jpg,https://oleks-netizen.github.io/product-images/90513/004.jpg,https://oleks-netizen.github.io/product-images/90513/005.jpg</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>90514</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90514/001.jpg,https://oleks-netizen.github.io/product-images/90514/002.jpg,https://oleks-netizen.github.io/product-images/90514/003.jpg,https://oleks-netizen.github.io/product-images/90514/004.jpg,https://oleks-netizen.github.io/product-images/90514/005.jpg</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>90515</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90515/001.jpg,https://oleks-netizen.github.io/product-images/90515/002.jpg,https://oleks-netizen.github.io/product-images/90515/003.jpg,https://oleks-netizen.github.io/product-images/90515/004.jpg,https://oleks-netizen.github.io/product-images/90515/005.jpg</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>90516</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90516/001.jpg,https://oleks-netizen.github.io/product-images/90516/002.jpg,https://oleks-netizen.github.io/product-images/90516/003.jpg,https://oleks-netizen.github.io/product-images/90516/004.jpg,https://oleks-netizen.github.io/product-images/90516/005.jpg</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>90517</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90517/001.jpg,https://oleks-netizen.github.io/product-images/90517/002.jpg,https://oleks-netizen.github.io/product-images/90517/004.jpg,https://oleks-netizen.github.io/product-images/90517/005.jpg,https://oleks-netizen.github.io/product-images/90517/006.jpg</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>90525</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90525/001.jpg,https://oleks-netizen.github.io/product-images/90525/002.jpg,https://oleks-netizen.github.io/product-images/90525/003.jpg,https://oleks-netizen.github.io/product-images/90525/004.jpg,https://oleks-netizen.github.io/product-images/90525/005.jpg,https://oleks-netizen.github.io/product-images/90525/006.jpg,https://oleks-netizen.github.io/product-images/90525/007.jpg</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>90526</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90526/001.jpg,https://oleks-netizen.github.io/product-images/90526/002.jpg,https://oleks-netizen.github.io/product-images/90526/003.jpg,https://oleks-netizen.github.io/product-images/90526/004.jpg,https://oleks-netizen.github.io/product-images/90526/006.jpg,https://oleks-netizen.github.io/product-images/90526/007.jpg,https://oleks-netizen.github.io/product-images/90526/008.jpg</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>90527</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90527/001.jpg,https://oleks-netizen.github.io/product-images/90527/002.jpg,https://oleks-netizen.github.io/product-images/90527/004.jpg,https://oleks-netizen.github.io/product-images/90527/005.jpg,https://oleks-netizen.github.io/product-images/90527/006.jpg,https://oleks-netizen.github.io/product-images/90527/007.jpg,https://oleks-netizen.github.io/product-images/90527/008.jpg,https://oleks-netizen.github.io/product-images/90527/009.jpg</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>90528</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90528/001.jpg,https://oleks-netizen.github.io/product-images/90528/002.jpg,https://oleks-netizen.github.io/product-images/90528/003.jpg,https://oleks-netizen.github.io/product-images/90528/004.jpg,https://oleks-netizen.github.io/product-images/90528/005.jpg,https://oleks-netizen.github.io/product-images/90528/006.jpg,https://oleks-netizen.github.io/product-images/90528/008.jpg,https://oleks-netizen.github.io/product-images/90528/009.jpg</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>90530</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90530/001.jpg,https://oleks-netizen.github.io/product-images/90530/002.jpg,https://oleks-netizen.github.io/product-images/90530/003.jpg,https://oleks-netizen.github.io/product-images/90530/005.jpg,https://oleks-netizen.github.io/product-images/90530/006.jpg,https://oleks-netizen.github.io/product-images/90530/007.jpg,https://oleks-netizen.github.io/product-images/90530/008.jpg</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>90531</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90531/001.jpg,https://oleks-netizen.github.io/product-images/90531/002.jpg,https://oleks-netizen.github.io/product-images/90531/004.jpg,https://oleks-netizen.github.io/product-images/90531/005.jpg,https://oleks-netizen.github.io/product-images/90531/006.jpg,https://oleks-netizen.github.io/product-images/90531/007.jpg,https://oleks-netizen.github.io/product-images/90531/008.jpg,https://oleks-netizen.github.io/product-images/90531/009.jpg</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>90532</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90532/001.jpg,https://oleks-netizen.github.io/product-images/90532/002.jpg,https://oleks-netizen.github.io/product-images/90532/004.jpg,https://oleks-netizen.github.io/product-images/90532/005.jpg,https://oleks-netizen.github.io/product-images/90532/006.jpg</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>90533</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90533/001.jpg,https://oleks-netizen.github.io/product-images/90533/002.jpg,https://oleks-netizen.github.io/product-images/90533/004.jpg,https://oleks-netizen.github.io/product-images/90533/005.jpg,https://oleks-netizen.github.io/product-images/90533/006.jpg</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>90534</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90534/001.jpg,https://oleks-netizen.github.io/product-images/90534/002.jpg,https://oleks-netizen.github.io/product-images/90534/004.jpg,https://oleks-netizen.github.io/product-images/90534/005.jpg,https://oleks-netizen.github.io/product-images/90534/006.jpg</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>90557</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90557/001.jpg,https://oleks-netizen.github.io/product-images/90557/002.jpg,https://oleks-netizen.github.io/product-images/90557/004.jpg,https://oleks-netizen.github.io/product-images/90557/005.jpg,https://oleks-netizen.github.io/product-images/90557/006.jpg,https://oleks-netizen.github.io/product-images/90557/007.jpg</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>90558</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90558/001.jpg,https://oleks-netizen.github.io/product-images/90558/002.jpg,https://oleks-netizen.github.io/product-images/90558/004.jpg,https://oleks-netizen.github.io/product-images/90558/005.jpg,https://oleks-netizen.github.io/product-images/90558/006.jpg,https://oleks-netizen.github.io/product-images/90558/007.jpg</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>90559</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90559/001.jpg,https://oleks-netizen.github.io/product-images/90559/002.jpg,https://oleks-netizen.github.io/product-images/90559/004.jpg,https://oleks-netizen.github.io/product-images/90559/005.jpg,https://oleks-netizen.github.io/product-images/90559/006.jpg</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>90599</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90599/001.jpg,https://oleks-netizen.github.io/product-images/90599/002.jpg,https://oleks-netizen.github.io/product-images/90599/003.jpg,https://oleks-netizen.github.io/product-images/90599/004.jpg,https://oleks-netizen.github.io/product-images/90599/005.jpg,https://oleks-netizen.github.io/product-images/90599/006.jpg,https://oleks-netizen.github.io/product-images/90599/007.jpg,https://oleks-netizen.github.io/product-images/90599/008.jpg,https://oleks-netizen.github.io/product-images/90599/009.jpg,https://oleks-netizen.github.io/product-images/90599/011.jpg,https://oleks-netizen.github.io/product-images/90599/012.jpg,https://oleks-netizen.github.io/product-images/90599/013.jpg</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>90600</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90600/001.jpg,https://oleks-netizen.github.io/product-images/90600/002.jpg,https://oleks-netizen.github.io/product-images/90600/003.jpg,https://oleks-netizen.github.io/product-images/90600/004.jpg,https://oleks-netizen.github.io/product-images/90600/005.jpg,https://oleks-netizen.github.io/product-images/90600/006.jpg,https://oleks-netizen.github.io/product-images/90600/007.jpg,https://oleks-netizen.github.io/product-images/90600/008.jpg,https://oleks-netizen.github.io/product-images/90600/010.jpg,https://oleks-netizen.github.io/product-images/90600/011.jpg,https://oleks-netizen.github.io/product-images/90600/012.jpg</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>90601</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90601/001.jpg,https://oleks-netizen.github.io/product-images/90601/002.jpg,https://oleks-netizen.github.io/product-images/90601/003.jpg,https://oleks-netizen.github.io/product-images/90601/004.jpg,https://oleks-netizen.github.io/product-images/90601/005.jpg,https://oleks-netizen.github.io/product-images/90601/006.jpg,https://oleks-netizen.github.io/product-images/90601/007.jpg,https://oleks-netizen.github.io/product-images/90601/008.jpg,https://oleks-netizen.github.io/product-images/90601/009.jpg,https://oleks-netizen.github.io/product-images/90601/011.jpg,https://oleks-netizen.github.io/product-images/90601/012.jpg</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>90602</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90602/001.jpg,https://oleks-netizen.github.io/product-images/90602/002.jpg,https://oleks-netizen.github.io/product-images/90602/004.jpg,https://oleks-netizen.github.io/product-images/90602/005.jpg,https://oleks-netizen.github.io/product-images/90602/006.jpg,https://oleks-netizen.github.io/product-images/90602/007.jpg,https://oleks-netizen.github.io/product-images/90602/008.jpg,https://oleks-netizen.github.io/product-images/90602/009.jpg,https://oleks-netizen.github.io/product-images/90602/010.jpg,https://oleks-netizen.github.io/product-images/90602/011.jpg</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>90603</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90603/001.jpg,https://oleks-netizen.github.io/product-images/90603/002.jpg,https://oleks-netizen.github.io/product-images/90603/004.jpg,https://oleks-netizen.github.io/product-images/90603/005.jpg,https://oleks-netizen.github.io/product-images/90603/006.jpg,https://oleks-netizen.github.io/product-images/90603/007.jpg,https://oleks-netizen.github.io/product-images/90603/008.jpg,https://oleks-netizen.github.io/product-images/90603/009.jpg,https://oleks-netizen.github.io/product-images/90603/010.jpg,https://oleks-netizen.github.io/product-images/90603/011.jpg,https://oleks-netizen.github.io/product-images/90603/012.jpg</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>90661</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90661/001.jpg,https://oleks-netizen.github.io/product-images/90661/002.jpg,https://oleks-netizen.github.io/product-images/90661/004.jpg,https://oleks-netizen.github.io/product-images/90661/005.jpg,https://oleks-netizen.github.io/product-images/90661/006.jpg,https://oleks-netizen.github.io/product-images/90661/007.jpg</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>90662</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90662/001.jpg,https://oleks-netizen.github.io/product-images/90662/002.jpg,https://oleks-netizen.github.io/product-images/90662/003.jpg</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>90663</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90663/001.jpg,https://oleks-netizen.github.io/product-images/90663/002.jpg,https://oleks-netizen.github.io/product-images/90663/003.jpg,https://oleks-netizen.github.io/product-images/90663/004.jpg,https://oleks-netizen.github.io/product-images/90663/005.jpg,https://oleks-netizen.github.io/product-images/90663/006.jpg,https://oleks-netizen.github.io/product-images/90663/007.jpg,https://oleks-netizen.github.io/product-images/90663/009.jpg,https://oleks-netizen.github.io/product-images/90663/010.jpg,https://oleks-netizen.github.io/product-images/90663/011.jpg,https://oleks-netizen.github.io/product-images/90663/012.jpg</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>90671</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90671/001.jpg,https://oleks-netizen.github.io/product-images/90671/002.jpg,https://oleks-netizen.github.io/product-images/90671/003.jpg,https://oleks-netizen.github.io/product-images/90671/004.jpg,https://oleks-netizen.github.io/product-images/90671/006.jpg</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>90672</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90672/001.jpg,https://oleks-netizen.github.io/product-images/90672/002.jpg,https://oleks-netizen.github.io/product-images/90672/003.jpg,https://oleks-netizen.github.io/product-images/90672/004.jpg,https://oleks-netizen.github.io/product-images/90672/005.jpg,https://oleks-netizen.github.io/product-images/90672/006.jpg,https://oleks-netizen.github.io/product-images/90672/007.jpg</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>90673</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90673/001.jpg,https://oleks-netizen.github.io/product-images/90673/002.jpg,https://oleks-netizen.github.io/product-images/90673/003.jpg,https://oleks-netizen.github.io/product-images/90673/004.jpg,https://oleks-netizen.github.io/product-images/90673/005.jpg,https://oleks-netizen.github.io/product-images/90673/007.jpg,https://oleks-netizen.github.io/product-images/90673/008.jpg</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>90674</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/90674/001.jpg,https://oleks-netizen.github.io/product-images/90674/002.jpg,https://oleks-netizen.github.io/product-images/90674/004.jpg,https://oleks-netizen.github.io/product-images/90674/005.jpg,https://oleks-netizen.github.io/product-images/90674/006.jpg,https://oleks-netizen.github.io/product-images/90674/007.jpg,https://oleks-netizen.github.io/product-images/90674/008.jpg</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-07-24 21:14:40
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,57 +436,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>90002</t>
+          <t>0026-2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90002/001.jpg,https://oleks-netizen.github.io/product-images/90002/002.jpg,https://oleks-netizen.github.io/product-images/90002/004.jpg,https://oleks-netizen.github.io/product-images/90002/005.jpg,https://oleks-netizen.github.io/product-images/90002/006.jpg,https://oleks-netizen.github.io/product-images/90002/007.jpg,https://oleks-netizen.github.io/product-images/90002/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/0026-2/001.jpg,https://oleks-netizen.github.io/product-images/0026-2/002.jpg,https://oleks-netizen.github.io/product-images/0026-2/004.jpg,https://oleks-netizen.github.io/product-images/0026-2/005.jpg,https://oleks-netizen.github.io/product-images/0026-2/006.jpg,https://oleks-netizen.github.io/product-images/0026-2/007.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>90021</t>
+          <t>0026-3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90021/001.jpg,https://oleks-netizen.github.io/product-images/90021/003.jpg,https://oleks-netizen.github.io/product-images/90021/004.jpg,https://oleks-netizen.github.io/product-images/90021/005.jpg,https://oleks-netizen.github.io/product-images/90021/006.jpg,https://oleks-netizen.github.io/product-images/90021/007.jpg,https://oleks-netizen.github.io/product-images/90021/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/0026-3/001.jpg,https://oleks-netizen.github.io/product-images/0026-3/002.jpg,https://oleks-netizen.github.io/product-images/0026-3/003.jpg,https://oleks-netizen.github.io/product-images/0026-3/004.jpg,https://oleks-netizen.github.io/product-images/0026-3/005.jpg,https://oleks-netizen.github.io/product-images/0026-3/006.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>90022</t>
+          <t>0026-5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90022/001.jpg,https://oleks-netizen.github.io/product-images/90022/003.jpg,https://oleks-netizen.github.io/product-images/90022/004.jpg,https://oleks-netizen.github.io/product-images/90022/005.jpg,https://oleks-netizen.github.io/product-images/90022/006.jpg,https://oleks-netizen.github.io/product-images/90022/007.jpg,https://oleks-netizen.github.io/product-images/90022/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/0026-5/001.jpg,https://oleks-netizen.github.io/product-images/0026-5/002.jpg,https://oleks-netizen.github.io/product-images/0026-5/003.jpg,https://oleks-netizen.github.io/product-images/0026-5/004.jpg,https://oleks-netizen.github.io/product-images/0026-5/005.jpg,https://oleks-netizen.github.io/product-images/0026-5/006.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>90027</t>
+          <t>0026-7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90027/001.jpg,https://oleks-netizen.github.io/product-images/90027/002.jpg,https://oleks-netizen.github.io/product-images/90027/003.jpg,https://oleks-netizen.github.io/product-images/90027/004.jpg,https://oleks-netizen.github.io/product-images/90027/005.jpg,https://oleks-netizen.github.io/product-images/90027/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/0026-7/001.jpg,https://oleks-netizen.github.io/product-images/0026-7/002.jpg,https://oleks-netizen.github.io/product-images/0026-7/003.jpg,https://oleks-netizen.github.io/product-images/0026-7/004.jpg,https://oleks-netizen.github.io/product-images/0026-7/005.jpg,https://oleks-netizen.github.io/product-images/0026-7/006.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -496,687 +496,687 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>90028</t>
+          <t>009-4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90028/001.jpg,https://oleks-netizen.github.io/product-images/90028/002.jpg,https://oleks-netizen.github.io/product-images/90028/004.jpg,https://oleks-netizen.github.io/product-images/90028/005.jpg,https://oleks-netizen.github.io/product-images/90028/006.jpg,https://oleks-netizen.github.io/product-images/90028/007.jpg,https://oleks-netizen.github.io/product-images/90028/008.jpg,https://oleks-netizen.github.io/product-images/90028/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/009-4/001.jpg,https://oleks-netizen.github.io/product-images/009-4/002.jpg,https://oleks-netizen.github.io/product-images/009-4/003.jpg,https://oleks-netizen.github.io/product-images/009-4/004.jpg,https://oleks-netizen.github.io/product-images/009-4/005.jpg,https://oleks-netizen.github.io/product-images/009-4/006.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>90029</t>
+          <t>1140321760</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90029/001.jpg,https://oleks-netizen.github.io/product-images/90029/002.jpg,https://oleks-netizen.github.io/product-images/90029/004.jpg,https://oleks-netizen.github.io/product-images/90029/005.jpg,https://oleks-netizen.github.io/product-images/90029/006.jpg,https://oleks-netizen.github.io/product-images/90029/007.jpg,https://oleks-netizen.github.io/product-images/90029/008.jpg,https://oleks-netizen.github.io/product-images/90029/009.jpg,https://oleks-netizen.github.io/product-images/90029/010.jpg,https://oleks-netizen.github.io/product-images/90029/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/1140321760/001.jpg,https://oleks-netizen.github.io/product-images/1140321760/002.jpg,https://oleks-netizen.github.io/product-images/1140321760/003.jpg,https://oleks-netizen.github.io/product-images/1140321760/004.jpg,https://oleks-netizen.github.io/product-images/1140321760/005.jpg,https://oleks-netizen.github.io/product-images/1140321760/006.jpg,https://oleks-netizen.github.io/product-images/1140321760/007.jpg,https://oleks-netizen.github.io/product-images/1140321760/008.jpg,https://oleks-netizen.github.io/product-images/1140321760/009.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>90065</t>
+          <t>16348</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90065/001.jpg,https://oleks-netizen.github.io/product-images/90065/002.jpg,https://oleks-netizen.github.io/product-images/90065/004.jpg,https://oleks-netizen.github.io/product-images/90065/005.jpg,https://oleks-netizen.github.io/product-images/90065/006.jpg,https://oleks-netizen.github.io/product-images/90065/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/16348/001.jpg,https://oleks-netizen.github.io/product-images/16348/002.jpg,https://oleks-netizen.github.io/product-images/16348/003.jpg,https://oleks-netizen.github.io/product-images/16348/004.jpg,https://oleks-netizen.github.io/product-images/16348/005.jpg,https://oleks-netizen.github.io/product-images/16348/006.jpg,https://oleks-netizen.github.io/product-images/16348/007.jpg,https://oleks-netizen.github.io/product-images/16348/008.jpg,https://oleks-netizen.github.io/product-images/16348/009.jpg,https://oleks-netizen.github.io/product-images/16348/010.jpg,https://oleks-netizen.github.io/product-images/16348/011.jpg,https://oleks-netizen.github.io/product-images/16348/012.jpg,https://oleks-netizen.github.io/product-images/16348/013.jpg,https://oleks-netizen.github.io/product-images/16348/014.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>90087</t>
+          <t>16351</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90087/001.jpg,https://oleks-netizen.github.io/product-images/90087/002.jpg,https://oleks-netizen.github.io/product-images/90087/004.jpg,https://oleks-netizen.github.io/product-images/90087/005.jpg,https://oleks-netizen.github.io/product-images/90087/006.jpg,https://oleks-netizen.github.io/product-images/90087/007.jpg,https://oleks-netizen.github.io/product-images/90087/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/16351/001.jpg,https://oleks-netizen.github.io/product-images/16351/003.jpg,https://oleks-netizen.github.io/product-images/16351/004.jpg,https://oleks-netizen.github.io/product-images/16351/005.jpg,https://oleks-netizen.github.io/product-images/16351/006.jpg,https://oleks-netizen.github.io/product-images/16351/007.jpg,https://oleks-netizen.github.io/product-images/16351/008.jpg,https://oleks-netizen.github.io/product-images/16351/009.jpg,https://oleks-netizen.github.io/product-images/16351/010.jpg,https://oleks-netizen.github.io/product-images/16351/011.jpg,https://oleks-netizen.github.io/product-images/16351/012.jpg,https://oleks-netizen.github.io/product-images/16351/013.jpg,https://oleks-netizen.github.io/product-images/16351/014.jpg,https://oleks-netizen.github.io/product-images/16351/015.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>90152</t>
+          <t>20407</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90152/001.jpg,https://oleks-netizen.github.io/product-images/90152/002.jpg,https://oleks-netizen.github.io/product-images/90152/003.jpg,https://oleks-netizen.github.io/product-images/90152/004.jpg,https://oleks-netizen.github.io/product-images/90152/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/20407/001.jpg,https://oleks-netizen.github.io/product-images/20407/003.jpg,https://oleks-netizen.github.io/product-images/20407/004.jpg,https://oleks-netizen.github.io/product-images/20407/005.jpg,https://oleks-netizen.github.io/product-images/20407/006.jpg,https://oleks-netizen.github.io/product-images/20407/007.jpg,https://oleks-netizen.github.io/product-images/20407/008.jpg,https://oleks-netizen.github.io/product-images/20407/009.jpg,https://oleks-netizen.github.io/product-images/20407/010.jpg,https://oleks-netizen.github.io/product-images/20407/011.jpg,https://oleks-netizen.github.io/product-images/20407/012.jpg,https://oleks-netizen.github.io/product-images/20407/013.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>90153</t>
+          <t>20685</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90153/001.jpg,https://oleks-netizen.github.io/product-images/90153/002.jpg,https://oleks-netizen.github.io/product-images/90153/003.jpg,https://oleks-netizen.github.io/product-images/90153/004.jpg,https://oleks-netizen.github.io/product-images/90153/005.jpg,https://oleks-netizen.github.io/product-images/90153/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/20685/001.jpg,https://oleks-netizen.github.io/product-images/20685/003.jpg,https://oleks-netizen.github.io/product-images/20685/004.jpg,https://oleks-netizen.github.io/product-images/20685/005.jpg,https://oleks-netizen.github.io/product-images/20685/006.jpg,https://oleks-netizen.github.io/product-images/20685/007.jpg,https://oleks-netizen.github.io/product-images/20685/008.jpg,https://oleks-netizen.github.io/product-images/20685/009.jpg,https://oleks-netizen.github.io/product-images/20685/010.jpg,https://oleks-netizen.github.io/product-images/20685/011.jpg,https://oleks-netizen.github.io/product-images/20685/012.jpg,https://oleks-netizen.github.io/product-images/20685/013.jpg,https://oleks-netizen.github.io/product-images/20685/014.jpg,https://oleks-netizen.github.io/product-images/20685/015.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>90154</t>
+          <t>22327</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90154/001.jpg,https://oleks-netizen.github.io/product-images/90154/002.jpg,https://oleks-netizen.github.io/product-images/90154/003.jpg,https://oleks-netizen.github.io/product-images/90154/004.jpg,https://oleks-netizen.github.io/product-images/90154/005.jpg,https://oleks-netizen.github.io/product-images/90154/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22327/001.jpg,https://oleks-netizen.github.io/product-images/22327/003.jpg,https://oleks-netizen.github.io/product-images/22327/004.jpg,https://oleks-netizen.github.io/product-images/22327/005.jpg,https://oleks-netizen.github.io/product-images/22327/006.jpg,https://oleks-netizen.github.io/product-images/22327/007.jpg,https://oleks-netizen.github.io/product-images/22327/008.jpg,https://oleks-netizen.github.io/product-images/22327/009.jpg,https://oleks-netizen.github.io/product-images/22327/010.jpg,https://oleks-netizen.github.io/product-images/22327/011.jpg,https://oleks-netizen.github.io/product-images/22327/012.jpg,https://oleks-netizen.github.io/product-images/22327/013.jpg,https://oleks-netizen.github.io/product-images/22327/014.jpg,https://oleks-netizen.github.io/product-images/22327/015.jpg,https://oleks-netizen.github.io/product-images/22327/016.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>90155</t>
+          <t>22783</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90155/001.jpg,https://oleks-netizen.github.io/product-images/90155/002.jpg,https://oleks-netizen.github.io/product-images/90155/003.jpg,https://oleks-netizen.github.io/product-images/90155/004.jpg,https://oleks-netizen.github.io/product-images/90155/005.jpg,https://oleks-netizen.github.io/product-images/90155/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22783/001.jpg,https://oleks-netizen.github.io/product-images/22783/003.jpg,https://oleks-netizen.github.io/product-images/22783/004.jpg,https://oleks-netizen.github.io/product-images/22783/005.jpg,https://oleks-netizen.github.io/product-images/22783/006.jpg,https://oleks-netizen.github.io/product-images/22783/007.jpg,https://oleks-netizen.github.io/product-images/22783/008.jpg,https://oleks-netizen.github.io/product-images/22783/009.jpg,https://oleks-netizen.github.io/product-images/22783/010.jpg,https://oleks-netizen.github.io/product-images/22783/011.jpg,https://oleks-netizen.github.io/product-images/22783/012.jpg,https://oleks-netizen.github.io/product-images/22783/013.jpg,https://oleks-netizen.github.io/product-images/22783/014.jpg,https://oleks-netizen.github.io/product-images/22783/015.jpg,https://oleks-netizen.github.io/product-images/22783/016.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>90156</t>
+          <t>22802</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90156/001.jpg,https://oleks-netizen.github.io/product-images/90156/002.jpg,https://oleks-netizen.github.io/product-images/90156/003.jpg,https://oleks-netizen.github.io/product-images/90156/004.jpg,https://oleks-netizen.github.io/product-images/90156/005.jpg,https://oleks-netizen.github.io/product-images/90156/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22802/001.jpg,https://oleks-netizen.github.io/product-images/22802/003.jpg,https://oleks-netizen.github.io/product-images/22802/004.jpg,https://oleks-netizen.github.io/product-images/22802/005.jpg,https://oleks-netizen.github.io/product-images/22802/006.jpg,https://oleks-netizen.github.io/product-images/22802/007.jpg,https://oleks-netizen.github.io/product-images/22802/008.jpg,https://oleks-netizen.github.io/product-images/22802/009.jpg,https://oleks-netizen.github.io/product-images/22802/010.jpg,https://oleks-netizen.github.io/product-images/22802/011.jpg,https://oleks-netizen.github.io/product-images/22802/012.jpg,https://oleks-netizen.github.io/product-images/22802/013.jpg,https://oleks-netizen.github.io/product-images/22802/014.jpg,https://oleks-netizen.github.io/product-images/22802/015.jpg,https://oleks-netizen.github.io/product-images/22802/016.jpg,https://oleks-netizen.github.io/product-images/22802/017.jpg,https://oleks-netizen.github.io/product-images/22802/018.jpg,https://oleks-netizen.github.io/product-images/22802/019.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>90157</t>
+          <t>22809</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90157/001.jpg,https://oleks-netizen.github.io/product-images/90157/002.jpg,https://oleks-netizen.github.io/product-images/90157/003.jpg,https://oleks-netizen.github.io/product-images/90157/004.jpg,https://oleks-netizen.github.io/product-images/90157/005.jpg,https://oleks-netizen.github.io/product-images/90157/006.jpg,https://oleks-netizen.github.io/product-images/90157/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22809/001.jpg,https://oleks-netizen.github.io/product-images/22809/003.jpg,https://oleks-netizen.github.io/product-images/22809/004.jpg,https://oleks-netizen.github.io/product-images/22809/005.jpg,https://oleks-netizen.github.io/product-images/22809/006.jpg,https://oleks-netizen.github.io/product-images/22809/007.jpg,https://oleks-netizen.github.io/product-images/22809/008.jpg,https://oleks-netizen.github.io/product-images/22809/009.jpg,https://oleks-netizen.github.io/product-images/22809/010.jpg,https://oleks-netizen.github.io/product-images/22809/011.jpg,https://oleks-netizen.github.io/product-images/22809/012.jpg,https://oleks-netizen.github.io/product-images/22809/013.jpg,https://oleks-netizen.github.io/product-images/22809/014.jpg,https://oleks-netizen.github.io/product-images/22809/015.jpg,https://oleks-netizen.github.io/product-images/22809/016.jpg,https://oleks-netizen.github.io/product-images/22809/017.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>90158</t>
+          <t>22810</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90158/001.jpg,https://oleks-netizen.github.io/product-images/90158/002.jpg,https://oleks-netizen.github.io/product-images/90158/003.jpg,https://oleks-netizen.github.io/product-images/90158/004.jpg,https://oleks-netizen.github.io/product-images/90158/005.jpg,https://oleks-netizen.github.io/product-images/90158/006.jpg,https://oleks-netizen.github.io/product-images/90158/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22810/001.jpg,https://oleks-netizen.github.io/product-images/22810/003.jpg,https://oleks-netizen.github.io/product-images/22810/004.jpg,https://oleks-netizen.github.io/product-images/22810/005.jpg,https://oleks-netizen.github.io/product-images/22810/006.jpg,https://oleks-netizen.github.io/product-images/22810/007.jpg,https://oleks-netizen.github.io/product-images/22810/008.jpg,https://oleks-netizen.github.io/product-images/22810/009.jpg,https://oleks-netizen.github.io/product-images/22810/010.jpg,https://oleks-netizen.github.io/product-images/22810/011.jpg,https://oleks-netizen.github.io/product-images/22810/012.jpg,https://oleks-netizen.github.io/product-images/22810/013.jpg,https://oleks-netizen.github.io/product-images/22810/014.jpg,https://oleks-netizen.github.io/product-images/22810/015.jpg,https://oleks-netizen.github.io/product-images/22810/016.jpg,https://oleks-netizen.github.io/product-images/22810/017.jpg,https://oleks-netizen.github.io/product-images/22810/018.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>90159</t>
+          <t>22835</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90159/001.jpg,https://oleks-netizen.github.io/product-images/90159/002.jpg,https://oleks-netizen.github.io/product-images/90159/003.jpg,https://oleks-netizen.github.io/product-images/90159/004.jpg,https://oleks-netizen.github.io/product-images/90159/005.jpg,https://oleks-netizen.github.io/product-images/90159/006.jpg,https://oleks-netizen.github.io/product-images/90159/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22835/001.jpg,https://oleks-netizen.github.io/product-images/22835/003.jpg,https://oleks-netizen.github.io/product-images/22835/004.jpg,https://oleks-netizen.github.io/product-images/22835/005.jpg,https://oleks-netizen.github.io/product-images/22835/006.jpg,https://oleks-netizen.github.io/product-images/22835/007.jpg,https://oleks-netizen.github.io/product-images/22835/008.jpg,https://oleks-netizen.github.io/product-images/22835/009.jpg,https://oleks-netizen.github.io/product-images/22835/010.jpg,https://oleks-netizen.github.io/product-images/22835/011.jpg,https://oleks-netizen.github.io/product-images/22835/012.jpg,https://oleks-netizen.github.io/product-images/22835/013.jpg,https://oleks-netizen.github.io/product-images/22835/014.jpg,https://oleks-netizen.github.io/product-images/22835/015.jpg,https://oleks-netizen.github.io/product-images/22835/016.jpg</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>90160</t>
+          <t>22841</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90160/001.jpg,https://oleks-netizen.github.io/product-images/90160/002.jpg,https://oleks-netizen.github.io/product-images/90160/003.jpg,https://oleks-netizen.github.io/product-images/90160/004.jpg,https://oleks-netizen.github.io/product-images/90160/005.jpg,https://oleks-netizen.github.io/product-images/90160/006.jpg,https://oleks-netizen.github.io/product-images/90160/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22841/001.jpg,https://oleks-netizen.github.io/product-images/22841/003.jpg,https://oleks-netizen.github.io/product-images/22841/004.jpg,https://oleks-netizen.github.io/product-images/22841/005.jpg,https://oleks-netizen.github.io/product-images/22841/006.jpg,https://oleks-netizen.github.io/product-images/22841/007.jpg,https://oleks-netizen.github.io/product-images/22841/008.jpg,https://oleks-netizen.github.io/product-images/22841/009.jpg,https://oleks-netizen.github.io/product-images/22841/010.jpg,https://oleks-netizen.github.io/product-images/22841/011.jpg,https://oleks-netizen.github.io/product-images/22841/012.jpg,https://oleks-netizen.github.io/product-images/22841/013.jpg,https://oleks-netizen.github.io/product-images/22841/014.jpg,https://oleks-netizen.github.io/product-images/22841/015.jpg,https://oleks-netizen.github.io/product-images/22841/016.jpg</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>90161</t>
+          <t>22845</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90161/001.jpg,https://oleks-netizen.github.io/product-images/90161/002.jpg,https://oleks-netizen.github.io/product-images/90161/003.jpg,https://oleks-netizen.github.io/product-images/90161/004.jpg,https://oleks-netizen.github.io/product-images/90161/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22845/001.jpg,https://oleks-netizen.github.io/product-images/22845/003.jpg,https://oleks-netizen.github.io/product-images/22845/004.jpg,https://oleks-netizen.github.io/product-images/22845/005.jpg,https://oleks-netizen.github.io/product-images/22845/006.jpg,https://oleks-netizen.github.io/product-images/22845/007.jpg,https://oleks-netizen.github.io/product-images/22845/008.jpg,https://oleks-netizen.github.io/product-images/22845/009.jpg,https://oleks-netizen.github.io/product-images/22845/010.jpg,https://oleks-netizen.github.io/product-images/22845/011.jpg,https://oleks-netizen.github.io/product-images/22845/012.jpg,https://oleks-netizen.github.io/product-images/22845/013.jpg,https://oleks-netizen.github.io/product-images/22845/014.jpg,https://oleks-netizen.github.io/product-images/22845/015.jpg,https://oleks-netizen.github.io/product-images/22845/016.jpg,https://oleks-netizen.github.io/product-images/22845/017.jpg</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>90162</t>
+          <t>22909</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90162/001.jpg,https://oleks-netizen.github.io/product-images/90162/002.jpg,https://oleks-netizen.github.io/product-images/90162/003.jpg,https://oleks-netizen.github.io/product-images/90162/004.jpg,https://oleks-netizen.github.io/product-images/90162/005.jpg,https://oleks-netizen.github.io/product-images/90162/006.jpg,https://oleks-netizen.github.io/product-images/90162/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22909/001.jpg,https://oleks-netizen.github.io/product-images/22909/003.jpg,https://oleks-netizen.github.io/product-images/22909/004.jpg,https://oleks-netizen.github.io/product-images/22909/005.jpg,https://oleks-netizen.github.io/product-images/22909/006.jpg,https://oleks-netizen.github.io/product-images/22909/007.jpg,https://oleks-netizen.github.io/product-images/22909/008.jpg,https://oleks-netizen.github.io/product-images/22909/009.jpg,https://oleks-netizen.github.io/product-images/22909/010.jpg,https://oleks-netizen.github.io/product-images/22909/011.jpg,https://oleks-netizen.github.io/product-images/22909/012.jpg</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>90163</t>
+          <t>22972</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90163/001.jpg,https://oleks-netizen.github.io/product-images/90163/002.jpg,https://oleks-netizen.github.io/product-images/90163/003.jpg,https://oleks-netizen.github.io/product-images/90163/004.jpg,https://oleks-netizen.github.io/product-images/90163/005.jpg,https://oleks-netizen.github.io/product-images/90163/006.jpg,https://oleks-netizen.github.io/product-images/90163/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22972/001.jpg,https://oleks-netizen.github.io/product-images/22972/002.jpg,https://oleks-netizen.github.io/product-images/22972/004.jpg,https://oleks-netizen.github.io/product-images/22972/005.jpg,https://oleks-netizen.github.io/product-images/22972/006.jpg,https://oleks-netizen.github.io/product-images/22972/007.jpg,https://oleks-netizen.github.io/product-images/22972/008.jpg,https://oleks-netizen.github.io/product-images/22972/009.jpg,https://oleks-netizen.github.io/product-images/22972/010.jpg,https://oleks-netizen.github.io/product-images/22972/011.jpg,https://oleks-netizen.github.io/product-images/22972/012.jpg,https://oleks-netizen.github.io/product-images/22972/013.jpg,https://oleks-netizen.github.io/product-images/22972/014.jpg,https://oleks-netizen.github.io/product-images/22972/015.jpg,https://oleks-netizen.github.io/product-images/22972/016.jpg</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>90164</t>
+          <t>22973</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90164/001.jpg,https://oleks-netizen.github.io/product-images/90164/002.jpg,https://oleks-netizen.github.io/product-images/90164/003.jpg,https://oleks-netizen.github.io/product-images/90164/004.jpg,https://oleks-netizen.github.io/product-images/90164/005.jpg,https://oleks-netizen.github.io/product-images/90164/006.jpg,https://oleks-netizen.github.io/product-images/90164/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/22973/001.jpg,https://oleks-netizen.github.io/product-images/22973/003.jpg,https://oleks-netizen.github.io/product-images/22973/004.jpg,https://oleks-netizen.github.io/product-images/22973/005.jpg,https://oleks-netizen.github.io/product-images/22973/006.jpg,https://oleks-netizen.github.io/product-images/22973/007.jpg,https://oleks-netizen.github.io/product-images/22973/008.jpg,https://oleks-netizen.github.io/product-images/22973/009.jpg,https://oleks-netizen.github.io/product-images/22973/010.jpg,https://oleks-netizen.github.io/product-images/22973/011.jpg,https://oleks-netizen.github.io/product-images/22973/012.jpg,https://oleks-netizen.github.io/product-images/22973/013.jpg,https://oleks-netizen.github.io/product-images/22973/014.jpg,https://oleks-netizen.github.io/product-images/22973/015.jpg,https://oleks-netizen.github.io/product-images/22973/016.jpg,https://oleks-netizen.github.io/product-images/22973/017.jpg</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>90166</t>
+          <t>23003</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90166/001.jpg,https://oleks-netizen.github.io/product-images/90166/002.jpg,https://oleks-netizen.github.io/product-images/90166/003.jpg,https://oleks-netizen.github.io/product-images/90166/004.jpg,https://oleks-netizen.github.io/product-images/90166/005.jpg,https://oleks-netizen.github.io/product-images/90166/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/23003/001.jpg,https://oleks-netizen.github.io/product-images/23003/003.jpg,https://oleks-netizen.github.io/product-images/23003/004.jpg,https://oleks-netizen.github.io/product-images/23003/005.jpg,https://oleks-netizen.github.io/product-images/23003/006.jpg,https://oleks-netizen.github.io/product-images/23003/007.jpg,https://oleks-netizen.github.io/product-images/23003/008.jpg,https://oleks-netizen.github.io/product-images/23003/009.jpg,https://oleks-netizen.github.io/product-images/23003/010.jpg,https://oleks-netizen.github.io/product-images/23003/011.jpg,https://oleks-netizen.github.io/product-images/23003/012.jpg,https://oleks-netizen.github.io/product-images/23003/013.jpg,https://oleks-netizen.github.io/product-images/23003/014.jpg,https://oleks-netizen.github.io/product-images/23003/015.jpg,https://oleks-netizen.github.io/product-images/23003/016.jpg</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>90168</t>
+          <t>23016</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90168/001.jpg,https://oleks-netizen.github.io/product-images/90168/002.jpg,https://oleks-netizen.github.io/product-images/90168/003.jpg,https://oleks-netizen.github.io/product-images/90168/004.jpg,https://oleks-netizen.github.io/product-images/90168/005.jpg,https://oleks-netizen.github.io/product-images/90168/006.jpg,https://oleks-netizen.github.io/product-images/90168/007.jpg,https://oleks-netizen.github.io/product-images/90168/008.jpg,https://oleks-netizen.github.io/product-images/90168/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/23016/001.jpg,https://oleks-netizen.github.io/product-images/23016/003.jpg,https://oleks-netizen.github.io/product-images/23016/004.jpg,https://oleks-netizen.github.io/product-images/23016/005.jpg,https://oleks-netizen.github.io/product-images/23016/006.jpg,https://oleks-netizen.github.io/product-images/23016/007.jpg,https://oleks-netizen.github.io/product-images/23016/008.jpg,https://oleks-netizen.github.io/product-images/23016/009.jpg,https://oleks-netizen.github.io/product-images/23016/010.jpg,https://oleks-netizen.github.io/product-images/23016/011.jpg,https://oleks-netizen.github.io/product-images/23016/012.jpg,https://oleks-netizen.github.io/product-images/23016/013.jpg,https://oleks-netizen.github.io/product-images/23016/014.jpg,https://oleks-netizen.github.io/product-images/23016/015.jpg,https://oleks-netizen.github.io/product-images/23016/016.jpg,https://oleks-netizen.github.io/product-images/23016/017.jpg</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>90169</t>
+          <t>23054</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90169/001.jpg,https://oleks-netizen.github.io/product-images/90169/002.jpg,https://oleks-netizen.github.io/product-images/90169/003.jpg,https://oleks-netizen.github.io/product-images/90169/004.jpg,https://oleks-netizen.github.io/product-images/90169/005.jpg,https://oleks-netizen.github.io/product-images/90169/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/23054/001.jpg,https://oleks-netizen.github.io/product-images/23054/003.jpg,https://oleks-netizen.github.io/product-images/23054/004.jpg,https://oleks-netizen.github.io/product-images/23054/005.jpg,https://oleks-netizen.github.io/product-images/23054/006.jpg,https://oleks-netizen.github.io/product-images/23054/007.jpg,https://oleks-netizen.github.io/product-images/23054/008.jpg,https://oleks-netizen.github.io/product-images/23054/009.jpg,https://oleks-netizen.github.io/product-images/23054/010.jpg,https://oleks-netizen.github.io/product-images/23054/011.jpg,https://oleks-netizen.github.io/product-images/23054/012.jpg,https://oleks-netizen.github.io/product-images/23054/013.jpg,https://oleks-netizen.github.io/product-images/23054/014.jpg,https://oleks-netizen.github.io/product-images/23054/015.jpg,https://oleks-netizen.github.io/product-images/23054/016.jpg,https://oleks-netizen.github.io/product-images/23054/017.jpg,https://oleks-netizen.github.io/product-images/23054/018.jpg,https://oleks-netizen.github.io/product-images/23054/019.jpg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>90170</t>
+          <t>51311506</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90170/001.jpg,https://oleks-netizen.github.io/product-images/90170/002.jpg,https://oleks-netizen.github.io/product-images/90170/003.jpg,https://oleks-netizen.github.io/product-images/90170/004.jpg,https://oleks-netizen.github.io/product-images/90170/005.jpg,https://oleks-netizen.github.io/product-images/90170/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51311506/001.jpg,https://oleks-netizen.github.io/product-images/51311506/003.jpg,https://oleks-netizen.github.io/product-images/51311506/004.jpg,https://oleks-netizen.github.io/product-images/51311506/005.jpg,https://oleks-netizen.github.io/product-images/51311506/006.jpg,https://oleks-netizen.github.io/product-images/51311506/007.jpg,https://oleks-netizen.github.io/product-images/51311506/008.jpg,https://oleks-netizen.github.io/product-images/51311506/009.jpg,https://oleks-netizen.github.io/product-images/51311506/010.jpg,https://oleks-netizen.github.io/product-images/51311506/011.jpg,https://oleks-netizen.github.io/product-images/51311506/012.jpg,https://oleks-netizen.github.io/product-images/51311506/013.jpg,https://oleks-netizen.github.io/product-images/51311506/014.jpg</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>90171</t>
+          <t>53100013</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90171/001.jpg,https://oleks-netizen.github.io/product-images/90171/002.jpg,https://oleks-netizen.github.io/product-images/90171/003.jpg,https://oleks-netizen.github.io/product-images/90171/004.jpg,https://oleks-netizen.github.io/product-images/90171/005.jpg,https://oleks-netizen.github.io/product-images/90171/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53100013/001.jpg,https://oleks-netizen.github.io/product-images/53100013/002.jpg,https://oleks-netizen.github.io/product-images/53100013/003.jpg,https://oleks-netizen.github.io/product-images/53100013/004.jpg,https://oleks-netizen.github.io/product-images/53100013/006.jpg,https://oleks-netizen.github.io/product-images/53100013/007.jpg,https://oleks-netizen.github.io/product-images/53100013/008.jpg,https://oleks-netizen.github.io/product-images/53100013/009.jpg,https://oleks-netizen.github.io/product-images/53100013/010.jpg,https://oleks-netizen.github.io/product-images/53100013/011.jpg,https://oleks-netizen.github.io/product-images/53100013/012.jpg</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>90172</t>
+          <t>53100066</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90172/001.jpg,https://oleks-netizen.github.io/product-images/90172/002.jpg,https://oleks-netizen.github.io/product-images/90172/004.jpg,https://oleks-netizen.github.io/product-images/90172/005.jpg,https://oleks-netizen.github.io/product-images/90172/006.jpg,https://oleks-netizen.github.io/product-images/90172/007.jpg,https://oleks-netizen.github.io/product-images/90172/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53100066/001.jpg,https://oleks-netizen.github.io/product-images/53100066/002.jpg,https://oleks-netizen.github.io/product-images/53100066/003.jpg,https://oleks-netizen.github.io/product-images/53100066/004.jpg,https://oleks-netizen.github.io/product-images/53100066/005.jpg,https://oleks-netizen.github.io/product-images/53100066/006.jpg,https://oleks-netizen.github.io/product-images/53100066/007.jpg,https://oleks-netizen.github.io/product-images/53100066/009.jpg,https://oleks-netizen.github.io/product-images/53100066/010.jpg,https://oleks-netizen.github.io/product-images/53100066/011.jpg,https://oleks-netizen.github.io/product-images/53100066/012.jpg,https://oleks-netizen.github.io/product-images/53100066/013.jpg,https://oleks-netizen.github.io/product-images/53100066/014.jpg,https://oleks-netizen.github.io/product-images/53100066/015.jpg</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>90173</t>
+          <t>53100106</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90173/001.jpg,https://oleks-netizen.github.io/product-images/90173/002.jpg,https://oleks-netizen.github.io/product-images/90173/004.jpg,https://oleks-netizen.github.io/product-images/90173/005.jpg,https://oleks-netizen.github.io/product-images/90173/006.jpg,https://oleks-netizen.github.io/product-images/90173/007.jpg,https://oleks-netizen.github.io/product-images/90173/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53100106/001.jpg,https://oleks-netizen.github.io/product-images/53100106/002.jpg,https://oleks-netizen.github.io/product-images/53100106/003.jpg,https://oleks-netizen.github.io/product-images/53100106/004.jpg,https://oleks-netizen.github.io/product-images/53100106/005.jpg,https://oleks-netizen.github.io/product-images/53100106/006.jpg,https://oleks-netizen.github.io/product-images/53100106/007.jpg,https://oleks-netizen.github.io/product-images/53100106/008.jpg,https://oleks-netizen.github.io/product-images/53100106/009.jpg,https://oleks-netizen.github.io/product-images/53100106/011.jpg,https://oleks-netizen.github.io/product-images/53100106/012.jpg,https://oleks-netizen.github.io/product-images/53100106/013.jpg,https://oleks-netizen.github.io/product-images/53100106/014.jpg,https://oleks-netizen.github.io/product-images/53100106/015.jpg</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>90174</t>
+          <t>53200003</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90174/001.jpg,https://oleks-netizen.github.io/product-images/90174/002.jpg,https://oleks-netizen.github.io/product-images/90174/003.jpg,https://oleks-netizen.github.io/product-images/90174/004.jpg,https://oleks-netizen.github.io/product-images/90174/005.jpg,https://oleks-netizen.github.io/product-images/90174/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53200003/001.jpg,https://oleks-netizen.github.io/product-images/53200003/002.jpg,https://oleks-netizen.github.io/product-images/53200003/003.jpg,https://oleks-netizen.github.io/product-images/53200003/004.jpg,https://oleks-netizen.github.io/product-images/53200003/005.jpg,https://oleks-netizen.github.io/product-images/53200003/006.jpg,https://oleks-netizen.github.io/product-images/53200003/008.jpg,https://oleks-netizen.github.io/product-images/53200003/009.jpg,https://oleks-netizen.github.io/product-images/53200003/010.jpg,https://oleks-netizen.github.io/product-images/53200003/011.jpg,https://oleks-netizen.github.io/product-images/53200003/012.jpg,https://oleks-netizen.github.io/product-images/53200003/013.jpg,https://oleks-netizen.github.io/product-images/53200003/014.jpg</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>90297</t>
+          <t>53200021</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90297/001.jpg,https://oleks-netizen.github.io/product-images/90297/002.jpg,https://oleks-netizen.github.io/product-images/90297/004.jpg,https://oleks-netizen.github.io/product-images/90297/005.jpg,https://oleks-netizen.github.io/product-images/90297/006.jpg,https://oleks-netizen.github.io/product-images/90297/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53200021/001.jpg,https://oleks-netizen.github.io/product-images/53200021/002.jpg,https://oleks-netizen.github.io/product-images/53200021/003.jpg,https://oleks-netizen.github.io/product-images/53200021/004.jpg,https://oleks-netizen.github.io/product-images/53200021/006.jpg,https://oleks-netizen.github.io/product-images/53200021/007.jpg,https://oleks-netizen.github.io/product-images/53200021/008.jpg,https://oleks-netizen.github.io/product-images/53200021/009.jpg,https://oleks-netizen.github.io/product-images/53200021/010.jpg,https://oleks-netizen.github.io/product-images/53200021/011.jpg,https://oleks-netizen.github.io/product-images/53200021/012.jpg,https://oleks-netizen.github.io/product-images/53200021/013.jpg</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>90298</t>
+          <t>53300003</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90298/001.jpg,https://oleks-netizen.github.io/product-images/90298/002.jpg,https://oleks-netizen.github.io/product-images/90298/003.jpg,https://oleks-netizen.github.io/product-images/90298/004.jpg,https://oleks-netizen.github.io/product-images/90298/005.jpg,https://oleks-netizen.github.io/product-images/90298/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53300003/001.jpg,https://oleks-netizen.github.io/product-images/53300003/002.jpg,https://oleks-netizen.github.io/product-images/53300003/003.jpg,https://oleks-netizen.github.io/product-images/53300003/004.jpg,https://oleks-netizen.github.io/product-images/53300003/005.jpg,https://oleks-netizen.github.io/product-images/53300003/006.jpg,https://oleks-netizen.github.io/product-images/53300003/007.jpg,https://oleks-netizen.github.io/product-images/53300003/009.jpg,https://oleks-netizen.github.io/product-images/53300003/010.jpg,https://oleks-netizen.github.io/product-images/53300003/011.jpg,https://oleks-netizen.github.io/product-images/53300003/012.jpg</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>90299</t>
+          <t>53300008</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90299/001.jpg,https://oleks-netizen.github.io/product-images/90299/002.jpg,https://oleks-netizen.github.io/product-images/90299/004.jpg,https://oleks-netizen.github.io/product-images/90299/005.jpg,https://oleks-netizen.github.io/product-images/90299/006.jpg,https://oleks-netizen.github.io/product-images/90299/007.jpg,https://oleks-netizen.github.io/product-images/90299/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53300008/001.jpg,https://oleks-netizen.github.io/product-images/53300008/002.jpg,https://oleks-netizen.github.io/product-images/53300008/003.jpg,https://oleks-netizen.github.io/product-images/53300008/005.jpg,https://oleks-netizen.github.io/product-images/53300008/006.jpg,https://oleks-netizen.github.io/product-images/53300008/007.jpg,https://oleks-netizen.github.io/product-images/53300008/008.jpg,https://oleks-netizen.github.io/product-images/53300008/009.jpg,https://oleks-netizen.github.io/product-images/53300008/010.jpg,https://oleks-netizen.github.io/product-images/53300008/011.jpg,https://oleks-netizen.github.io/product-images/53300008/012.jpg</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>90300</t>
+          <t>53300013</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90300/001.jpg,https://oleks-netizen.github.io/product-images/90300/002.jpg,https://oleks-netizen.github.io/product-images/90300/004.jpg,https://oleks-netizen.github.io/product-images/90300/005.jpg,https://oleks-netizen.github.io/product-images/90300/006.jpg,https://oleks-netizen.github.io/product-images/90300/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53300013/001.jpg,https://oleks-netizen.github.io/product-images/53300013/002.jpg,https://oleks-netizen.github.io/product-images/53300013/003.jpg,https://oleks-netizen.github.io/product-images/53300013/005.jpg,https://oleks-netizen.github.io/product-images/53300013/006.jpg,https://oleks-netizen.github.io/product-images/53300013/007.jpg,https://oleks-netizen.github.io/product-images/53300013/008.jpg,https://oleks-netizen.github.io/product-images/53300013/009.jpg,https://oleks-netizen.github.io/product-images/53300013/010.jpg,https://oleks-netizen.github.io/product-images/53300013/011.jpg,https://oleks-netizen.github.io/product-images/53300013/012.jpg,https://oleks-netizen.github.io/product-images/53300013/013.jpg,https://oleks-netizen.github.io/product-images/53300013/014.jpg</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>90301</t>
+          <t>53300021</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90301/001.jpg,https://oleks-netizen.github.io/product-images/90301/003.jpg,https://oleks-netizen.github.io/product-images/90301/004.jpg,https://oleks-netizen.github.io/product-images/90301/005.jpg,https://oleks-netizen.github.io/product-images/90301/006.jpg,https://oleks-netizen.github.io/product-images/90301/007.jpg,https://oleks-netizen.github.io/product-images/90301/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53300021/001.jpg,https://oleks-netizen.github.io/product-images/53300021/002.jpg,https://oleks-netizen.github.io/product-images/53300021/003.jpg,https://oleks-netizen.github.io/product-images/53300021/004.jpg,https://oleks-netizen.github.io/product-images/53300021/005.jpg,https://oleks-netizen.github.io/product-images/53300021/006.jpg,https://oleks-netizen.github.io/product-images/53300021/007.jpg,https://oleks-netizen.github.io/product-images/53300021/009.jpg,https://oleks-netizen.github.io/product-images/53300021/010.jpg,https://oleks-netizen.github.io/product-images/53300021/011.jpg,https://oleks-netizen.github.io/product-images/53300021/012.jpg,https://oleks-netizen.github.io/product-images/53300021/013.jpg</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>90331</t>
+          <t>53300066</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90331/001.jpg,https://oleks-netizen.github.io/product-images/90331/002.jpg,https://oleks-netizen.github.io/product-images/90331/003.jpg,https://oleks-netizen.github.io/product-images/90331/004.jpg,https://oleks-netizen.github.io/product-images/90331/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53300066/001.jpg,https://oleks-netizen.github.io/product-images/53300066/002.jpg,https://oleks-netizen.github.io/product-images/53300066/003.jpg,https://oleks-netizen.github.io/product-images/53300066/004.jpg,https://oleks-netizen.github.io/product-images/53300066/005.jpg,https://oleks-netizen.github.io/product-images/53300066/007.jpg,https://oleks-netizen.github.io/product-images/53300066/008.jpg,https://oleks-netizen.github.io/product-images/53300066/009.jpg,https://oleks-netizen.github.io/product-images/53300066/010.jpg,https://oleks-netizen.github.io/product-images/53300066/011.jpg,https://oleks-netizen.github.io/product-images/53300066/012.jpg,https://oleks-netizen.github.io/product-images/53300066/013.jpg</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>90347</t>
+          <t>53400020</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90347/001.jpg,https://oleks-netizen.github.io/product-images/90347/002.jpg,https://oleks-netizen.github.io/product-images/90347/003.jpg,https://oleks-netizen.github.io/product-images/90347/005.jpg,https://oleks-netizen.github.io/product-images/90347/006.jpg,https://oleks-netizen.github.io/product-images/90347/007.jpg,https://oleks-netizen.github.io/product-images/90347/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400020/001.jpg,https://oleks-netizen.github.io/product-images/53400020/002.jpg,https://oleks-netizen.github.io/product-images/53400020/004.jpg,https://oleks-netizen.github.io/product-images/53400020/005.jpg,https://oleks-netizen.github.io/product-images/53400020/006.jpg,https://oleks-netizen.github.io/product-images/53400020/007.jpg,https://oleks-netizen.github.io/product-images/53400020/008.jpg,https://oleks-netizen.github.io/product-images/53400020/009.jpg,https://oleks-netizen.github.io/product-images/53400020/010.jpg,https://oleks-netizen.github.io/product-images/53400020/011.jpg,https://oleks-netizen.github.io/product-images/53400020/012.jpg,https://oleks-netizen.github.io/product-images/53400020/013.jpg,https://oleks-netizen.github.io/product-images/53400020/014.jpg</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>90386</t>
+          <t>53400064</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90386/001.jpg,https://oleks-netizen.github.io/product-images/90386/002.jpg,https://oleks-netizen.github.io/product-images/90386/003.jpg,https://oleks-netizen.github.io/product-images/90386/004.jpg,https://oleks-netizen.github.io/product-images/90386/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400064/001.jpg,https://oleks-netizen.github.io/product-images/53400064/002.jpg,https://oleks-netizen.github.io/product-images/53400064/003.jpg,https://oleks-netizen.github.io/product-images/53400064/004.jpg,https://oleks-netizen.github.io/product-images/53400064/005.jpg,https://oleks-netizen.github.io/product-images/53400064/006.jpg,https://oleks-netizen.github.io/product-images/53400064/008.jpg,https://oleks-netizen.github.io/product-images/53400064/009.jpg,https://oleks-netizen.github.io/product-images/53400064/010.jpg,https://oleks-netizen.github.io/product-images/53400064/011.jpg</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>90387</t>
+          <t>53400064m</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90387/001.jpg,https://oleks-netizen.github.io/product-images/90387/002.jpg,https://oleks-netizen.github.io/product-images/90387/004.jpg,https://oleks-netizen.github.io/product-images/90387/005.jpg,https://oleks-netizen.github.io/product-images/90387/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400064m/001.jpg,https://oleks-netizen.github.io/product-images/53400064m/002.jpg,https://oleks-netizen.github.io/product-images/53400064m/003.jpg,https://oleks-netizen.github.io/product-images/53400064m/004.jpg,https://oleks-netizen.github.io/product-images/53400064m/005.jpg,https://oleks-netizen.github.io/product-images/53400064m/006.jpg,https://oleks-netizen.github.io/product-images/53400064m/007.jpg,https://oleks-netizen.github.io/product-images/53400064m/008.jpg,https://oleks-netizen.github.io/product-images/53400064m/009.jpg,https://oleks-netizen.github.io/product-images/53400064m/010.jpg,https://oleks-netizen.github.io/product-images/53400064m/011.jpg</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>90491</t>
+          <t>53400707</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90491/001.jpg,https://oleks-netizen.github.io/product-images/90491/002.jpg,https://oleks-netizen.github.io/product-images/90491/003.jpg,https://oleks-netizen.github.io/product-images/90491/004.jpg,https://oleks-netizen.github.io/product-images/90491/005.jpg,https://oleks-netizen.github.io/product-images/90491/006.jpg,https://oleks-netizen.github.io/product-images/90491/007.jpg,https://oleks-netizen.github.io/product-images/90491/008.jpg,https://oleks-netizen.github.io/product-images/90491/009.jpg,https://oleks-netizen.github.io/product-images/90491/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400707/001.jpg,https://oleks-netizen.github.io/product-images/53400707/002.jpg,https://oleks-netizen.github.io/product-images/53400707/003.jpg,https://oleks-netizen.github.io/product-images/53400707/004.jpg,https://oleks-netizen.github.io/product-images/53400707/005.jpg,https://oleks-netizen.github.io/product-images/53400707/006.jpg,https://oleks-netizen.github.io/product-images/53400707/007.jpg,https://oleks-netizen.github.io/product-images/53400707/008.jpg,https://oleks-netizen.github.io/product-images/53400707/009.jpg,https://oleks-netizen.github.io/product-images/53400707/010.jpg,https://oleks-netizen.github.io/product-images/53400707/011.jpg,https://oleks-netizen.github.io/product-images/53400707/012.jpg</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>90492</t>
+          <t>53400720</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90492/001.jpg,https://oleks-netizen.github.io/product-images/90492/002.jpg,https://oleks-netizen.github.io/product-images/90492/003.jpg,https://oleks-netizen.github.io/product-images/90492/004.jpg,https://oleks-netizen.github.io/product-images/90492/005.jpg,https://oleks-netizen.github.io/product-images/90492/006.jpg,https://oleks-netizen.github.io/product-images/90492/007.jpg,https://oleks-netizen.github.io/product-images/90492/009.jpg,https://oleks-netizen.github.io/product-images/90492/010.jpg,https://oleks-netizen.github.io/product-images/90492/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400720/001.jpg,https://oleks-netizen.github.io/product-images/53400720/002.jpg,https://oleks-netizen.github.io/product-images/53400720/003.jpg,https://oleks-netizen.github.io/product-images/53400720/004.jpg,https://oleks-netizen.github.io/product-images/53400720/005.jpg,https://oleks-netizen.github.io/product-images/53400720/006.jpg,https://oleks-netizen.github.io/product-images/53400720/007.jpg,https://oleks-netizen.github.io/product-images/53400720/008.jpg,https://oleks-netizen.github.io/product-images/53400720/009.jpg,https://oleks-netizen.github.io/product-images/53400720/010.jpg,https://oleks-netizen.github.io/product-images/53400720/011.jpg,https://oleks-netizen.github.io/product-images/53400720/012.jpg</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>90493</t>
+          <t>53400800</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90493/001.jpg,https://oleks-netizen.github.io/product-images/90493/002.jpg,https://oleks-netizen.github.io/product-images/90493/003.jpg,https://oleks-netizen.github.io/product-images/90493/004.jpg,https://oleks-netizen.github.io/product-images/90493/005.jpg,https://oleks-netizen.github.io/product-images/90493/006.jpg,https://oleks-netizen.github.io/product-images/90493/007.jpg,https://oleks-netizen.github.io/product-images/90493/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53400800/001.jpg,https://oleks-netizen.github.io/product-images/53400800/002.jpg,https://oleks-netizen.github.io/product-images/53400800/003.jpg,https://oleks-netizen.github.io/product-images/53400800/004.jpg,https://oleks-netizen.github.io/product-images/53400800/005.jpg,https://oleks-netizen.github.io/product-images/53400800/006.jpg,https://oleks-netizen.github.io/product-images/53400800/007.jpg,https://oleks-netizen.github.io/product-images/53400800/008.jpg,https://oleks-netizen.github.io/product-images/53400800/009.jpg,https://oleks-netizen.github.io/product-images/53400800/010.jpg</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>90494</t>
+          <t>70566001</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90494/001.jpg,https://oleks-netizen.github.io/product-images/90494/002.jpg,https://oleks-netizen.github.io/product-images/90494/003.jpg,https://oleks-netizen.github.io/product-images/90494/004.jpg,https://oleks-netizen.github.io/product-images/90494/006.jpg,https://oleks-netizen.github.io/product-images/90494/007.jpg,https://oleks-netizen.github.io/product-images/90494/008.jpg,https://oleks-netizen.github.io/product-images/90494/009.jpg,https://oleks-netizen.github.io/product-images/90494/010.jpg,https://oleks-netizen.github.io/product-images/90494/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/70566001/001.jpg,https://oleks-netizen.github.io/product-images/70566001/002.jpg,https://oleks-netizen.github.io/product-images/70566001/003.jpg,https://oleks-netizen.github.io/product-images/70566001/004.jpg,https://oleks-netizen.github.io/product-images/70566001/005.jpg,https://oleks-netizen.github.io/product-images/70566001/006.jpg,https://oleks-netizen.github.io/product-images/70566001/007.jpg,https://oleks-netizen.github.io/product-images/70566001/008.jpg</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>90495</t>
+          <t>80460401</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90495/001.jpg,https://oleks-netizen.github.io/product-images/90495/002.jpg,https://oleks-netizen.github.io/product-images/90495/003.jpg,https://oleks-netizen.github.io/product-images/90495/004.jpg,https://oleks-netizen.github.io/product-images/90495/005.jpg,https://oleks-netizen.github.io/product-images/90495/006.jpg,https://oleks-netizen.github.io/product-images/90495/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/80460401/001.jpg,https://oleks-netizen.github.io/product-images/80460401/002.jpg,https://oleks-netizen.github.io/product-images/80460401/003.jpg,https://oleks-netizen.github.io/product-images/80460401/004.jpg,https://oleks-netizen.github.io/product-images/80460401/005.jpg,https://oleks-netizen.github.io/product-images/80460401/006.jpg,https://oleks-netizen.github.io/product-images/80460401/007.jpg,https://oleks-netizen.github.io/product-images/80460401/008.jpg,https://oleks-netizen.github.io/product-images/80460401/009.jpg,https://oleks-netizen.github.io/product-images/80460401/010.jpg,https://oleks-netizen.github.io/product-images/80460401/011.jpg,https://oleks-netizen.github.io/product-images/80460401/012.jpg,https://oleks-netizen.github.io/product-images/80460401/013.jpg,https://oleks-netizen.github.io/product-images/80460401/014.jpg,https://oleks-netizen.github.io/product-images/80460401/015.jpg</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>90496</t>
+          <t>80460410</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90496/001.jpg,https://oleks-netizen.github.io/product-images/90496/002.jpg,https://oleks-netizen.github.io/product-images/90496/003.jpg,https://oleks-netizen.github.io/product-images/90496/004.jpg,https://oleks-netizen.github.io/product-images/90496/005.jpg,https://oleks-netizen.github.io/product-images/90496/006.jpg,https://oleks-netizen.github.io/product-images/90496/007.jpg,https://oleks-netizen.github.io/product-images/90496/008.jpg,https://oleks-netizen.github.io/product-images/90496/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/80460410/001.jpg,https://oleks-netizen.github.io/product-images/80460410/003.jpg,https://oleks-netizen.github.io/product-images/80460410/004.jpg,https://oleks-netizen.github.io/product-images/80460410/005.jpg,https://oleks-netizen.github.io/product-images/80460410/006.jpg,https://oleks-netizen.github.io/product-images/80460410/007.jpg,https://oleks-netizen.github.io/product-images/80460410/008.jpg,https://oleks-netizen.github.io/product-images/80460410/009.jpg,https://oleks-netizen.github.io/product-images/80460410/010.jpg,https://oleks-netizen.github.io/product-images/80460410/011.jpg,https://oleks-netizen.github.io/product-images/80460410/012.jpg,https://oleks-netizen.github.io/product-images/80460410/013.jpg,https://oleks-netizen.github.io/product-images/80460410/014.jpg,https://oleks-netizen.github.io/product-images/80460410/015.jpg,https://oleks-netizen.github.io/product-images/80460410/016.jpg</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>90498</t>
+          <t>81341101</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90498/001.jpg,https://oleks-netizen.github.io/product-images/90498/002.jpg,https://oleks-netizen.github.io/product-images/90498/003.jpg,https://oleks-netizen.github.io/product-images/90498/004.jpg,https://oleks-netizen.github.io/product-images/90498/005.jpg,https://oleks-netizen.github.io/product-images/90498/006.jpg,https://oleks-netizen.github.io/product-images/90498/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/81341101/001.jpg,https://oleks-netizen.github.io/product-images/81341101/002.jpg,https://oleks-netizen.github.io/product-images/81341101/003.jpg,https://oleks-netizen.github.io/product-images/81341101/004.jpg,https://oleks-netizen.github.io/product-images/81341101/005.jpg,https://oleks-netizen.github.io/product-images/81341101/007.jpg,https://oleks-netizen.github.io/product-images/81341101/008.jpg,https://oleks-netizen.github.io/product-images/81341101/009.jpg,https://oleks-netizen.github.io/product-images/81341101/010.jpg</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>90499</t>
+          <t>85351030</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90499/001.jpg,https://oleks-netizen.github.io/product-images/90499/002.jpg,https://oleks-netizen.github.io/product-images/90499/004.jpg,https://oleks-netizen.github.io/product-images/90499/005.jpg,https://oleks-netizen.github.io/product-images/90499/006.jpg,https://oleks-netizen.github.io/product-images/90499/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/85351030/001.jpg,https://oleks-netizen.github.io/product-images/85351030/003.jpg,https://oleks-netizen.github.io/product-images/85351030/004.jpg,https://oleks-netizen.github.io/product-images/85351030/005.jpg,https://oleks-netizen.github.io/product-images/85351030/006.jpg,https://oleks-netizen.github.io/product-images/85351030/007.jpg,https://oleks-netizen.github.io/product-images/85351030/008.jpg,https://oleks-netizen.github.io/product-images/85351030/009.jpg,https://oleks-netizen.github.io/product-images/85351030/010.jpg,https://oleks-netizen.github.io/product-images/85351030/011.jpg,https://oleks-netizen.github.io/product-images/85351030/012.jpg</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>90500</t>
+          <t>96193001</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90500/001.jpg,https://oleks-netizen.github.io/product-images/90500/002.jpg,https://oleks-netizen.github.io/product-images/90500/003.jpg,https://oleks-netizen.github.io/product-images/90500/004.jpg,https://oleks-netizen.github.io/product-images/90500/006.jpg,https://oleks-netizen.github.io/product-images/90500/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/96193001/001.jpg,https://oleks-netizen.github.io/product-images/96193001/002.jpg,https://oleks-netizen.github.io/product-images/96193001/003.jpg,https://oleks-netizen.github.io/product-images/96193001/004.jpg,https://oleks-netizen.github.io/product-images/96193001/005.jpg,https://oleks-netizen.github.io/product-images/96193001/006.jpg,https://oleks-netizen.github.io/product-images/96193001/007.jpg,https://oleks-netizen.github.io/product-images/96193001/009.jpg,https://oleks-netizen.github.io/product-images/96193001/010.jpg,https://oleks-netizen.github.io/product-images/96193001/011.jpg,https://oleks-netizen.github.io/product-images/96193001/012.jpg,https://oleks-netizen.github.io/product-images/96193001/013.jpg,https://oleks-netizen.github.io/product-images/96193001/014.jpg</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>90509</t>
+          <t>96193072</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90509/001.jpg,https://oleks-netizen.github.io/product-images/90509/002.jpg,https://oleks-netizen.github.io/product-images/90509/004.jpg,https://oleks-netizen.github.io/product-images/90509/005.jpg,https://oleks-netizen.github.io/product-images/90509/006.jpg,https://oleks-netizen.github.io/product-images/90509/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/96193072/001.jpg,https://oleks-netizen.github.io/product-images/96193072/002.jpg,https://oleks-netizen.github.io/product-images/96193072/003.jpg,https://oleks-netizen.github.io/product-images/96193072/004.jpg,https://oleks-netizen.github.io/product-images/96193072/006.jpg,https://oleks-netizen.github.io/product-images/96193072/007.jpg,https://oleks-netizen.github.io/product-images/96193072/008.jpg,https://oleks-netizen.github.io/product-images/96193072/009.jpg</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>90510</t>
+          <t>96199170</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90510/001.jpg,https://oleks-netizen.github.io/product-images/90510/002.jpg,https://oleks-netizen.github.io/product-images/90510/003.jpg,https://oleks-netizen.github.io/product-images/90510/004.jpg,https://oleks-netizen.github.io/product-images/90510/006.jpg,https://oleks-netizen.github.io/product-images/90510/007.jpg,https://oleks-netizen.github.io/product-images/90510/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/96199170/001.jpg,https://oleks-netizen.github.io/product-images/96199170/002.jpg,https://oleks-netizen.github.io/product-images/96199170/003.jpg,https://oleks-netizen.github.io/product-images/96199170/004.jpg,https://oleks-netizen.github.io/product-images/96199170/005.jpg,https://oleks-netizen.github.io/product-images/96199170/007.jpg,https://oleks-netizen.github.io/product-images/96199170/008.jpg,https://oleks-netizen.github.io/product-images/96199170/009.jpg,https://oleks-netizen.github.io/product-images/96199170/010.jpg,https://oleks-netizen.github.io/product-images/96199170/011.jpg,https://oleks-netizen.github.io/product-images/96199170/012.jpg,https://oleks-netizen.github.io/product-images/96199170/013.jpg</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>90511</t>
+          <t>BV38826-240</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90511/001.jpg,https://oleks-netizen.github.io/product-images/90511/002.jpg,https://oleks-netizen.github.io/product-images/90511/003.jpg,https://oleks-netizen.github.io/product-images/90511/005.jpg,https://oleks-netizen.github.io/product-images/90511/006.jpg,https://oleks-netizen.github.io/product-images/90511/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV38826-240/001.jpg,https://oleks-netizen.github.io/product-images/BV38826-240/003.jpg,https://oleks-netizen.github.io/product-images/BV38826-240/004.jpg,https://oleks-netizen.github.io/product-images/BV38826-240/005.jpg,https://oleks-netizen.github.io/product-images/BV38826-240/006.jpg,https://oleks-netizen.github.io/product-images/BV38826-240/007.jpg</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1186,57 +1186,57 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>90512</t>
+          <t>BV38896-69</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90512/001.jpg,https://oleks-netizen.github.io/product-images/90512/002.jpg,https://oleks-netizen.github.io/product-images/90512/003.jpg,https://oleks-netizen.github.io/product-images/90512/005.jpg,https://oleks-netizen.github.io/product-images/90512/006.jpg,https://oleks-netizen.github.io/product-images/90512/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV38896-69/001.jpg,https://oleks-netizen.github.io/product-images/BV38896-69/003.jpg,https://oleks-netizen.github.io/product-images/BV38896-69/004.jpg,https://oleks-netizen.github.io/product-images/BV38896-69/005.jpg,https://oleks-netizen.github.io/product-images/BV38896-69/006.jpg,https://oleks-netizen.github.io/product-images/BV38896-69/007.jpg,https://oleks-netizen.github.io/product-images/BV38896-69/008.jpg</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>90513</t>
+          <t>BV38915-1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90513/001.jpg,https://oleks-netizen.github.io/product-images/90513/002.jpg,https://oleks-netizen.github.io/product-images/90513/003.jpg,https://oleks-netizen.github.io/product-images/90513/004.jpg,https://oleks-netizen.github.io/product-images/90513/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV38915-1/001.jpg,https://oleks-netizen.github.io/product-images/BV38915-1/003.jpg,https://oleks-netizen.github.io/product-images/BV38915-1/004.jpg,https://oleks-netizen.github.io/product-images/BV38915-1/005.jpg,https://oleks-netizen.github.io/product-images/BV38915-1/006.jpg,https://oleks-netizen.github.io/product-images/BV38915-1/007.jpg,https://oleks-netizen.github.io/product-images/BV38915-1/008.jpg</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>90514</t>
+          <t>BV38915-205</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90514/001.jpg,https://oleks-netizen.github.io/product-images/90514/002.jpg,https://oleks-netizen.github.io/product-images/90514/003.jpg,https://oleks-netizen.github.io/product-images/90514/004.jpg,https://oleks-netizen.github.io/product-images/90514/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BV38915-205/001.jpg,https://oleks-netizen.github.io/product-images/BV38915-205/003.jpg,https://oleks-netizen.github.io/product-images/BV38915-205/004.jpg,https://oleks-netizen.github.io/product-images/BV38915-205/005.jpg,https://oleks-netizen.github.io/product-images/BV38915-205/006.jpg,https://oleks-netizen.github.io/product-images/BV38915-205/007.jpg,https://oleks-netizen.github.io/product-images/BV38915-205/008.jpg</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>90515</t>
+          <t>C12312bl-black</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90515/001.jpg,https://oleks-netizen.github.io/product-images/90515/002.jpg,https://oleks-netizen.github.io/product-images/90515/003.jpg,https://oleks-netizen.github.io/product-images/90515/004.jpg,https://oleks-netizen.github.io/product-images/90515/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/C12312bl-black/001.jpg,https://oleks-netizen.github.io/product-images/C12312bl-black/002.jpg,https://oleks-netizen.github.io/product-images/C12312bl-black/003.jpg,https://oleks-netizen.github.io/product-images/C12312bl-black/004.jpg,https://oleks-netizen.github.io/product-images/C12312bl-black/005.jpg</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -1246,12 +1246,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>90516</t>
+          <t>C12312br-brown</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90516/001.jpg,https://oleks-netizen.github.io/product-images/90516/002.jpg,https://oleks-netizen.github.io/product-images/90516/003.jpg,https://oleks-netizen.github.io/product-images/90516/004.jpg,https://oleks-netizen.github.io/product-images/90516/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/C12312br-brown/001.jpg,https://oleks-netizen.github.io/product-images/C12312br-brown/002.jpg,https://oleks-netizen.github.io/product-images/C12312br-brown/003.jpg,https://oleks-netizen.github.io/product-images/C12312br-brown/004.jpg,https://oleks-netizen.github.io/product-images/C12312br-brown/005.jpg</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1261,87 +1261,87 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>90517</t>
+          <t>C1HSSA0536v-violet</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90517/001.jpg,https://oleks-netizen.github.io/product-images/90517/002.jpg,https://oleks-netizen.github.io/product-images/90517/004.jpg,https://oleks-netizen.github.io/product-images/90517/005.jpg,https://oleks-netizen.github.io/product-images/90517/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/C1HSSA0536v-violet/001.jpg,https://oleks-netizen.github.io/product-images/C1HSSA0536v-violet/002.jpg,https://oleks-netizen.github.io/product-images/C1HSSA0536v-violet/003.jpg,https://oleks-netizen.github.io/product-images/C1HSSA0536v-violet/004.jpg</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>90525</t>
+          <t>C1HSSAX2247bl-black</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90525/001.jpg,https://oleks-netizen.github.io/product-images/90525/002.jpg,https://oleks-netizen.github.io/product-images/90525/003.jpg,https://oleks-netizen.github.io/product-images/90525/004.jpg,https://oleks-netizen.github.io/product-images/90525/005.jpg,https://oleks-netizen.github.io/product-images/90525/006.jpg,https://oleks-netizen.github.io/product-images/90525/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/C1HSSAX2247bl-black/001.jpg,https://oleks-netizen.github.io/product-images/C1HSSAX2247bl-black/002.jpg,https://oleks-netizen.github.io/product-images/C1HSSAX2247bl-black/003.jpg,https://oleks-netizen.github.io/product-images/C1HSSAX2247bl-black/004.jpg,https://oleks-netizen.github.io/product-images/C1HSSAX2247bl-black/005.jpg</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>90526</t>
+          <t>C1HSSAX2247n-navy</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90526/001.jpg,https://oleks-netizen.github.io/product-images/90526/002.jpg,https://oleks-netizen.github.io/product-images/90526/003.jpg,https://oleks-netizen.github.io/product-images/90526/004.jpg,https://oleks-netizen.github.io/product-images/90526/006.jpg,https://oleks-netizen.github.io/product-images/90526/007.jpg,https://oleks-netizen.github.io/product-images/90526/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/C1HSSAX2247n-navy/001.jpg,https://oleks-netizen.github.io/product-images/C1HSSAX2247n-navy/002.jpg,https://oleks-netizen.github.io/product-images/C1HSSAX2247n-navy/003.jpg,https://oleks-netizen.github.io/product-images/C1HSSAX2247n-navy/004.jpg,https://oleks-netizen.github.io/product-images/C1HSSAX2247n-navy/005.jpg</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>90527</t>
+          <t>C34618-3008</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90527/001.jpg,https://oleks-netizen.github.io/product-images/90527/002.jpg,https://oleks-netizen.github.io/product-images/90527/004.jpg,https://oleks-netizen.github.io/product-images/90527/005.jpg,https://oleks-netizen.github.io/product-images/90527/006.jpg,https://oleks-netizen.github.io/product-images/90527/007.jpg,https://oleks-netizen.github.io/product-images/90527/008.jpg,https://oleks-netizen.github.io/product-images/90527/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/C34618-3008/001.jpg,https://oleks-netizen.github.io/product-images/C34618-3008/003.jpg,https://oleks-netizen.github.io/product-images/C34618-3008/004.jpg,https://oleks-netizen.github.io/product-images/C34618-3008/005.jpg,https://oleks-netizen.github.io/product-images/C34618-3008/006.jpg,https://oleks-netizen.github.io/product-images/C34618-3008/007.jpg,https://oleks-netizen.github.io/product-images/C34618-3008/008.jpg</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>90528</t>
+          <t>C34618-4024</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90528/001.jpg,https://oleks-netizen.github.io/product-images/90528/002.jpg,https://oleks-netizen.github.io/product-images/90528/003.jpg,https://oleks-netizen.github.io/product-images/90528/004.jpg,https://oleks-netizen.github.io/product-images/90528/005.jpg,https://oleks-netizen.github.io/product-images/90528/006.jpg,https://oleks-netizen.github.io/product-images/90528/008.jpg,https://oleks-netizen.github.io/product-images/90528/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/C34618-4024/001.jpg,https://oleks-netizen.github.io/product-images/C34618-4024/003.jpg,https://oleks-netizen.github.io/product-images/C34618-4024/004.jpg,https://oleks-netizen.github.io/product-images/C34618-4024/005.jpg,https://oleks-netizen.github.io/product-images/C34618-4024/006.jpg,https://oleks-netizen.github.io/product-images/C34618-4024/007.jpg,https://oleks-netizen.github.io/product-images/C34618-4024/008.jpg</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>90530</t>
+          <t>C34815-1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90530/001.jpg,https://oleks-netizen.github.io/product-images/90530/002.jpg,https://oleks-netizen.github.io/product-images/90530/003.jpg,https://oleks-netizen.github.io/product-images/90530/005.jpg,https://oleks-netizen.github.io/product-images/90530/006.jpg,https://oleks-netizen.github.io/product-images/90530/007.jpg,https://oleks-netizen.github.io/product-images/90530/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/C34815-1/001.jpg,https://oleks-netizen.github.io/product-images/C34815-1/003.jpg,https://oleks-netizen.github.io/product-images/C34815-1/004.jpg,https://oleks-netizen.github.io/product-images/C34815-1/005.jpg,https://oleks-netizen.github.io/product-images/C34815-1/006.jpg,https://oleks-netizen.github.io/product-images/C34815-1/007.jpg,https://oleks-netizen.github.io/product-images/C34815-1/008.jpg</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -1351,12 +1351,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>90531</t>
+          <t>DS30002-162</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90531/001.jpg,https://oleks-netizen.github.io/product-images/90531/002.jpg,https://oleks-netizen.github.io/product-images/90531/004.jpg,https://oleks-netizen.github.io/product-images/90531/005.jpg,https://oleks-netizen.github.io/product-images/90531/006.jpg,https://oleks-netizen.github.io/product-images/90531/007.jpg,https://oleks-netizen.github.io/product-images/90531/008.jpg,https://oleks-netizen.github.io/product-images/90531/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/DS30002-162/001.jpg,https://oleks-netizen.github.io/product-images/DS30002-162/003.jpg,https://oleks-netizen.github.io/product-images/DS30002-162/004.jpg,https://oleks-netizen.github.io/product-images/DS30002-162/005.jpg,https://oleks-netizen.github.io/product-images/DS30002-162/006.jpg,https://oleks-netizen.github.io/product-images/DS30002-162/007.jpg,https://oleks-netizen.github.io/product-images/DS30002-162/008.jpg,https://oleks-netizen.github.io/product-images/DS30002-162/009.jpg</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -1366,87 +1366,87 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>90532</t>
+          <t>DS30002-287</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90532/001.jpg,https://oleks-netizen.github.io/product-images/90532/002.jpg,https://oleks-netizen.github.io/product-images/90532/004.jpg,https://oleks-netizen.github.io/product-images/90532/005.jpg,https://oleks-netizen.github.io/product-images/90532/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/DS30002-287/001.jpg,https://oleks-netizen.github.io/product-images/DS30002-287/003.jpg,https://oleks-netizen.github.io/product-images/DS30002-287/004.jpg,https://oleks-netizen.github.io/product-images/DS30002-287/005.jpg,https://oleks-netizen.github.io/product-images/DS30002-287/006.jpg,https://oleks-netizen.github.io/product-images/DS30002-287/007.jpg,https://oleks-netizen.github.io/product-images/DS30002-287/008.jpg,https://oleks-netizen.github.io/product-images/DS30002-287/009.jpg</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>90533</t>
+          <t>DS30002-288</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90533/001.jpg,https://oleks-netizen.github.io/product-images/90533/002.jpg,https://oleks-netizen.github.io/product-images/90533/004.jpg,https://oleks-netizen.github.io/product-images/90533/005.jpg,https://oleks-netizen.github.io/product-images/90533/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/DS30002-288/001.jpg,https://oleks-netizen.github.io/product-images/DS30002-288/003.jpg,https://oleks-netizen.github.io/product-images/DS30002-288/004.jpg,https://oleks-netizen.github.io/product-images/DS30002-288/005.jpg,https://oleks-netizen.github.io/product-images/DS30002-288/006.jpg,https://oleks-netizen.github.io/product-images/DS30002-288/007.jpg,https://oleks-netizen.github.io/product-images/DS30002-288/008.jpg,https://oleks-netizen.github.io/product-images/DS30002-288/009.jpg</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>90534</t>
+          <t>fz3752_bordo</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90534/001.jpg,https://oleks-netizen.github.io/product-images/90534/002.jpg,https://oleks-netizen.github.io/product-images/90534/004.jpg,https://oleks-netizen.github.io/product-images/90534/005.jpg,https://oleks-netizen.github.io/product-images/90534/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/fz3752_bordo/001.jpg,https://oleks-netizen.github.io/product-images/fz3752_bordo/003.jpg,https://oleks-netizen.github.io/product-images/fz3752_bordo/004.jpg,https://oleks-netizen.github.io/product-images/fz3752_bordo/005.jpg,https://oleks-netizen.github.io/product-images/fz3752_bordo/006.jpg,https://oleks-netizen.github.io/product-images/fz3752_bordo/007.jpg,https://oleks-netizen.github.io/product-images/fz3752_bordo/008.jpg</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>90557</t>
+          <t>K10018bl-black</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90557/001.jpg,https://oleks-netizen.github.io/product-images/90557/002.jpg,https://oleks-netizen.github.io/product-images/90557/004.jpg,https://oleks-netizen.github.io/product-images/90557/005.jpg,https://oleks-netizen.github.io/product-images/90557/006.jpg,https://oleks-netizen.github.io/product-images/90557/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K10018bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K10018bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K10018bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K10018bl-black/005.jpg,https://oleks-netizen.github.io/product-images/K10018bl-black/006.jpg</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>90558</t>
+          <t>k1105-blue</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90558/001.jpg,https://oleks-netizen.github.io/product-images/90558/002.jpg,https://oleks-netizen.github.io/product-images/90558/004.jpg,https://oleks-netizen.github.io/product-images/90558/005.jpg,https://oleks-netizen.github.io/product-images/90558/006.jpg,https://oleks-netizen.github.io/product-images/90558/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/k1105-blue/001.jpg,https://oleks-netizen.github.io/product-images/k1105-blue/003.jpg,https://oleks-netizen.github.io/product-images/k1105-blue/004.jpg,https://oleks-netizen.github.io/product-images/k1105-blue/005.jpg,https://oleks-netizen.github.io/product-images/k1105-blue/006.jpg</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>90559</t>
+          <t>K11512be-beige</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90559/001.jpg,https://oleks-netizen.github.io/product-images/90559/002.jpg,https://oleks-netizen.github.io/product-images/90559/004.jpg,https://oleks-netizen.github.io/product-images/90559/005.jpg,https://oleks-netizen.github.io/product-images/90559/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K11512be-beige/001.jpg,https://oleks-netizen.github.io/product-images/K11512be-beige/002.jpg,https://oleks-netizen.github.io/product-images/K11512be-beige/003.jpg,https://oleks-netizen.github.io/product-images/K11512be-beige/004.jpg,https://oleks-netizen.github.io/product-images/K11512be-beige/005.jpg</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -1456,132 +1456,132 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>90599</t>
+          <t>K11512bl-black</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90599/001.jpg,https://oleks-netizen.github.io/product-images/90599/002.jpg,https://oleks-netizen.github.io/product-images/90599/003.jpg,https://oleks-netizen.github.io/product-images/90599/004.jpg,https://oleks-netizen.github.io/product-images/90599/005.jpg,https://oleks-netizen.github.io/product-images/90599/006.jpg,https://oleks-netizen.github.io/product-images/90599/007.jpg,https://oleks-netizen.github.io/product-images/90599/008.jpg,https://oleks-netizen.github.io/product-images/90599/009.jpg,https://oleks-netizen.github.io/product-images/90599/011.jpg,https://oleks-netizen.github.io/product-images/90599/012.jpg,https://oleks-netizen.github.io/product-images/90599/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K11512bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K11512bl-black/002.jpg,https://oleks-netizen.github.io/product-images/K11512bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K11512bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K11512bl-black/005.jpg</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>90600</t>
+          <t>K11512w-white</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90600/001.jpg,https://oleks-netizen.github.io/product-images/90600/002.jpg,https://oleks-netizen.github.io/product-images/90600/003.jpg,https://oleks-netizen.github.io/product-images/90600/004.jpg,https://oleks-netizen.github.io/product-images/90600/005.jpg,https://oleks-netizen.github.io/product-images/90600/006.jpg,https://oleks-netizen.github.io/product-images/90600/007.jpg,https://oleks-netizen.github.io/product-images/90600/008.jpg,https://oleks-netizen.github.io/product-images/90600/010.jpg,https://oleks-netizen.github.io/product-images/90600/011.jpg,https://oleks-netizen.github.io/product-images/90600/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K11512w-white/001.jpg,https://oleks-netizen.github.io/product-images/K11512w-white/002.jpg,https://oleks-netizen.github.io/product-images/K11512w-white/003.jpg,https://oleks-netizen.github.io/product-images/K11512w-white/004.jpg,https://oleks-netizen.github.io/product-images/K11512w-white/005.jpg</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>90601</t>
+          <t>K11512z-green</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90601/001.jpg,https://oleks-netizen.github.io/product-images/90601/002.jpg,https://oleks-netizen.github.io/product-images/90601/003.jpg,https://oleks-netizen.github.io/product-images/90601/004.jpg,https://oleks-netizen.github.io/product-images/90601/005.jpg,https://oleks-netizen.github.io/product-images/90601/006.jpg,https://oleks-netizen.github.io/product-images/90601/007.jpg,https://oleks-netizen.github.io/product-images/90601/008.jpg,https://oleks-netizen.github.io/product-images/90601/009.jpg,https://oleks-netizen.github.io/product-images/90601/011.jpg,https://oleks-netizen.github.io/product-images/90601/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K11512z-green/001.jpg,https://oleks-netizen.github.io/product-images/K11512z-green/002.jpg,https://oleks-netizen.github.io/product-images/K11512z-green/003.jpg,https://oleks-netizen.github.io/product-images/K11512z-green/004.jpg,https://oleks-netizen.github.io/product-images/K11512z-green/005.jpg</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>90602</t>
+          <t>K11668or-ginger</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90602/001.jpg,https://oleks-netizen.github.io/product-images/90602/002.jpg,https://oleks-netizen.github.io/product-images/90602/004.jpg,https://oleks-netizen.github.io/product-images/90602/005.jpg,https://oleks-netizen.github.io/product-images/90602/006.jpg,https://oleks-netizen.github.io/product-images/90602/007.jpg,https://oleks-netizen.github.io/product-images/90602/008.jpg,https://oleks-netizen.github.io/product-images/90602/009.jpg,https://oleks-netizen.github.io/product-images/90602/010.jpg,https://oleks-netizen.github.io/product-images/90602/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K11668or-ginger/001.jpg,https://oleks-netizen.github.io/product-images/K11668or-ginger/003.jpg,https://oleks-netizen.github.io/product-images/K11668or-ginger/004.jpg,https://oleks-netizen.github.io/product-images/K11668or-ginger/005.jpg,https://oleks-netizen.github.io/product-images/K11668or-ginger/006.jpg</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>90603</t>
+          <t>K11668v-violet</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90603/001.jpg,https://oleks-netizen.github.io/product-images/90603/002.jpg,https://oleks-netizen.github.io/product-images/90603/004.jpg,https://oleks-netizen.github.io/product-images/90603/005.jpg,https://oleks-netizen.github.io/product-images/90603/006.jpg,https://oleks-netizen.github.io/product-images/90603/007.jpg,https://oleks-netizen.github.io/product-images/90603/008.jpg,https://oleks-netizen.github.io/product-images/90603/009.jpg,https://oleks-netizen.github.io/product-images/90603/010.jpg,https://oleks-netizen.github.io/product-images/90603/011.jpg,https://oleks-netizen.github.io/product-images/90603/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K11668v-violet/001.jpg,https://oleks-netizen.github.io/product-images/K11668v-violet/003.jpg,https://oleks-netizen.github.io/product-images/K11668v-violet/004.jpg,https://oleks-netizen.github.io/product-images/K11668v-violet/005.jpg,https://oleks-netizen.github.io/product-images/K11668v-violet/006.jpg</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>90661</t>
+          <t>K11670gi-ginger</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90661/001.jpg,https://oleks-netizen.github.io/product-images/90661/002.jpg,https://oleks-netizen.github.io/product-images/90661/004.jpg,https://oleks-netizen.github.io/product-images/90661/005.jpg,https://oleks-netizen.github.io/product-images/90661/006.jpg,https://oleks-netizen.github.io/product-images/90661/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K11670gi-ginger/001.jpg,https://oleks-netizen.github.io/product-images/K11670gi-ginger/003.jpg,https://oleks-netizen.github.io/product-images/K11670gi-ginger/004.jpg,https://oleks-netizen.github.io/product-images/K11670gi-ginger/005.jpg,https://oleks-netizen.github.io/product-images/K11670gi-ginger/006.jpg</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>90662</t>
+          <t>K1211-black</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90662/001.jpg,https://oleks-netizen.github.io/product-images/90662/002.jpg,https://oleks-netizen.github.io/product-images/90662/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K1211-black/001.jpg,https://oleks-netizen.github.io/product-images/K1211-black/002.jpg,https://oleks-netizen.github.io/product-images/K1211-black/003.jpg,https://oleks-netizen.github.io/product-images/K1211-black/004.jpg,https://oleks-netizen.github.io/product-images/K1211-black/005.jpg</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>90663</t>
+          <t>K12202bl-black</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90663/001.jpg,https://oleks-netizen.github.io/product-images/90663/002.jpg,https://oleks-netizen.github.io/product-images/90663/003.jpg,https://oleks-netizen.github.io/product-images/90663/004.jpg,https://oleks-netizen.github.io/product-images/90663/005.jpg,https://oleks-netizen.github.io/product-images/90663/006.jpg,https://oleks-netizen.github.io/product-images/90663/007.jpg,https://oleks-netizen.github.io/product-images/90663/009.jpg,https://oleks-netizen.github.io/product-images/90663/010.jpg,https://oleks-netizen.github.io/product-images/90663/011.jpg,https://oleks-netizen.github.io/product-images/90663/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K12202bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K12202bl-black/002.jpg,https://oleks-netizen.github.io/product-images/K12202bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K12202bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K12202bl-black/005.jpg</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>90671</t>
+          <t>K12228bl-black</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90671/001.jpg,https://oleks-netizen.github.io/product-images/90671/002.jpg,https://oleks-netizen.github.io/product-images/90671/003.jpg,https://oleks-netizen.github.io/product-images/90671/004.jpg,https://oleks-netizen.github.io/product-images/90671/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K12228bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K12228bl-black/002.jpg,https://oleks-netizen.github.io/product-images/K12228bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K12228bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K12228bl-black/005.jpg</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -1591,46 +1591,1756 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>90672</t>
+          <t>K12504bl-black</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90672/001.jpg,https://oleks-netizen.github.io/product-images/90672/002.jpg,https://oleks-netizen.github.io/product-images/90672/003.jpg,https://oleks-netizen.github.io/product-images/90672/004.jpg,https://oleks-netizen.github.io/product-images/90672/005.jpg,https://oleks-netizen.github.io/product-images/90672/006.jpg,https://oleks-netizen.github.io/product-images/90672/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K12504bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K12504bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K12504bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K12504bl-black/005.jpg,https://oleks-netizen.github.io/product-images/K12504bl-black/006.jpg</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>90673</t>
+          <t>K12507bl-black</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90673/001.jpg,https://oleks-netizen.github.io/product-images/90673/002.jpg,https://oleks-netizen.github.io/product-images/90673/003.jpg,https://oleks-netizen.github.io/product-images/90673/004.jpg,https://oleks-netizen.github.io/product-images/90673/005.jpg,https://oleks-netizen.github.io/product-images/90673/007.jpg,https://oleks-netizen.github.io/product-images/90673/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/K12507bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K12507bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K12507bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K12507bl-black/005.jpg,https://oleks-netizen.github.io/product-images/K12507bl-black/006.jpg</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>90674</t>
+          <t>k12511bl-black</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90674/001.jpg,https://oleks-netizen.github.io/product-images/90674/002.jpg,https://oleks-netizen.github.io/product-images/90674/004.jpg,https://oleks-netizen.github.io/product-images/90674/005.jpg,https://oleks-netizen.github.io/product-images/90674/006.jpg,https://oleks-netizen.github.io/product-images/90674/007.jpg,https://oleks-netizen.github.io/product-images/90674/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/k12511bl-black/001.jpg,https://oleks-netizen.github.io/product-images/k12511bl-black/002.jpg,https://oleks-netizen.github.io/product-images/k12511bl-black/003.jpg,https://oleks-netizen.github.io/product-images/k12511bl-black/004.jpg,https://oleks-netizen.github.io/product-images/k12511bl-black/005.jpg,https://oleks-netizen.github.io/product-images/k12511bl-black/006.jpg</t>
         </is>
       </c>
       <c r="C81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>K15-5813be-beige</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K15-5813be-beige/001.jpg,https://oleks-netizen.github.io/product-images/K15-5813be-beige/002.jpg,https://oleks-netizen.github.io/product-images/K15-5813be-beige/003.jpg,https://oleks-netizen.github.io/product-images/K15-5813be-beige/004.jpg</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>K15-5813bl-black</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K15-5813bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K15-5813bl-black/002.jpg,https://oleks-netizen.github.io/product-images/K15-5813bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K15-5813bl-black/004.jpg</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>K15-5813gi-ginger</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K15-5813gi-ginger/001.jpg,https://oleks-netizen.github.io/product-images/K15-5813gi-ginger/002.jpg,https://oleks-netizen.github.io/product-images/K15-5813gi-ginger/003.jpg,https://oleks-netizen.github.io/product-images/K15-5813gi-ginger/004.jpg</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>K15-5813w-white</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K15-5813w-white/001.jpg,https://oleks-netizen.github.io/product-images/K15-5813w-white/002.jpg,https://oleks-netizen.github.io/product-images/K15-5813w-white/003.jpg,https://oleks-netizen.github.io/product-images/K15-5813w-white/004.jpg</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>K15-5818gr-green</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K15-5818gr-green/001.jpg,https://oleks-netizen.github.io/product-images/K15-5818gr-green/002.jpg,https://oleks-netizen.github.io/product-images/K15-5818gr-green/003.jpg,https://oleks-netizen.github.io/product-images/K15-5818gr-green/004.jpg,https://oleks-netizen.github.io/product-images/K15-5818gr-green/005.jpg</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>K15-605gi-ginger</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K15-605gi-ginger/001.jpg,https://oleks-netizen.github.io/product-images/K15-605gi-ginger/002.jpg,https://oleks-netizen.github.io/product-images/K15-605gi-ginger/003.jpg,https://oleks-netizen.github.io/product-images/K15-605gi-ginger/004.jpg,https://oleks-netizen.github.io/product-images/K15-605gi-ginger/005.jpg</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>K16008bl-black</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K16008bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K16008bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K16008bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K16008bl-black/005.jpg,https://oleks-netizen.github.io/product-images/K16008bl-black/006.jpg,https://oleks-netizen.github.io/product-images/K16008bl-black/007.jpg</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>K1607bl-black</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K1607bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K1607bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K1607bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K1607bl-black/005.jpg,https://oleks-netizen.github.io/product-images/K1607bl-black/006.jpg</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>K1608bl-black</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K1608bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K1608bl-black/002.jpg,https://oleks-netizen.github.io/product-images/K1608bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K1608bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K1608bl-black/005.jpg</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>K16101bl-black</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K16101bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K16101bl-black/002.jpg,https://oleks-netizen.github.io/product-images/K16101bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K16101bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K16101bl-black/005.jpg,https://oleks-netizen.github.io/product-images/K16101bl-black/006.jpg</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>K16602light</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K16602light/001.jpg,https://oleks-netizen.github.io/product-images/K16602light/002.jpg,https://oleks-netizen.github.io/product-images/K16602light/003.jpg,https://oleks-netizen.github.io/product-images/K16602light/004.jpg,https://oleks-netizen.github.io/product-images/K16602light/005.jpg</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>K1669bl-black</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K1669bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K1669bl-black/002.jpg,https://oleks-netizen.github.io/product-images/K1669bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K1669bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K1669bl-black/005.jpg</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>K17107bl-black</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K17107bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K17107bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K17107bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K17107bl-black/005.jpg,https://oleks-netizen.github.io/product-images/K17107bl-black/006.jpg</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>K17107w-white</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K17107w-white/001.jpg,https://oleks-netizen.github.io/product-images/K17107w-white/003.jpg,https://oleks-netizen.github.io/product-images/K17107w-white/004.jpg,https://oleks-netizen.github.io/product-images/K17107w-white/005.jpg,https://oleks-netizen.github.io/product-images/K17107w-white/006.jpg</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>K17108bl-black</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K17108bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K17108bl-black/002.jpg,https://oleks-netizen.github.io/product-images/K17108bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K17108bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K17108bl-black/005.jpg</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>K17109bl-black</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K17109bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K17109bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K17109bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K17109bl-black/005.jpg,https://oleks-netizen.github.io/product-images/K17109bl-black/006.jpg</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>K18005bl-black</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K18005bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K18005bl-black/002.jpg,https://oleks-netizen.github.io/product-images/K18005bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K18005bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K18005bl-black/005.jpg</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>k1840-blue</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/k1840-blue/001.jpg,https://oleks-netizen.github.io/product-images/k1840-blue/003.jpg,https://oleks-netizen.github.io/product-images/k1840-blue/004.jpg,https://oleks-netizen.github.io/product-images/k1840-blue/005.jpg,https://oleks-netizen.github.io/product-images/k1840-blue/006.jpg</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>K188084bl-black</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K188084bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K188084bl-black/002.jpg,https://oleks-netizen.github.io/product-images/K188084bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K188084bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K188084bl-black/005.jpg</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>K188084gr-gray</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K188084gr-gray/001.jpg,https://oleks-netizen.github.io/product-images/K188084gr-gray/002.jpg,https://oleks-netizen.github.io/product-images/K188084gr-gray/003.jpg,https://oleks-netizen.github.io/product-images/K188084gr-gray/004.jpg,https://oleks-netizen.github.io/product-images/K188084gr-gray/005.jpg</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>K19922bl-black</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/K19922bl-black/001.jpg,https://oleks-netizen.github.io/product-images/K19922bl-black/003.jpg,https://oleks-netizen.github.io/product-images/K19922bl-black/004.jpg,https://oleks-netizen.github.io/product-images/K19922bl-black/005.jpg,https://oleks-netizen.github.io/product-images/K19922bl-black/006.jpg</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>L20001-22</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20001-22/001.jpg,https://oleks-netizen.github.io/product-images/L20001-22/003.jpg,https://oleks-netizen.github.io/product-images/L20001-22/004.jpg,https://oleks-netizen.github.io/product-images/L20001-22/005.jpg,https://oleks-netizen.github.io/product-images/L20001-22/006.jpg,https://oleks-netizen.github.io/product-images/L20001-22/007.jpg,https://oleks-netizen.github.io/product-images/L20001-22/008.jpg,https://oleks-netizen.github.io/product-images/L20001-22/009.jpg</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>L20011-1</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20011-1/001.jpg,https://oleks-netizen.github.io/product-images/L20011-1/003.jpg,https://oleks-netizen.github.io/product-images/L20011-1/004.jpg,https://oleks-netizen.github.io/product-images/L20011-1/005.jpg,https://oleks-netizen.github.io/product-images/L20011-1/006.jpg,https://oleks-netizen.github.io/product-images/L20011-1/007.jpg,https://oleks-netizen.github.io/product-images/L20011-1/008.jpg,https://oleks-netizen.github.io/product-images/L20011-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>L20011-22</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20011-22/001.jpg,https://oleks-netizen.github.io/product-images/L20011-22/003.jpg,https://oleks-netizen.github.io/product-images/L20011-22/004.jpg,https://oleks-netizen.github.io/product-images/L20011-22/005.jpg,https://oleks-netizen.github.io/product-images/L20011-22/006.jpg,https://oleks-netizen.github.io/product-images/L20011-22/007.jpg,https://oleks-netizen.github.io/product-images/L20011-22/008.jpg,https://oleks-netizen.github.io/product-images/L20011-22/009.jpg</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>L20011-56</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20011-56/001.jpg,https://oleks-netizen.github.io/product-images/L20011-56/003.jpg,https://oleks-netizen.github.io/product-images/L20011-56/004.jpg,https://oleks-netizen.github.io/product-images/L20011-56/005.jpg,https://oleks-netizen.github.io/product-images/L20011-56/006.jpg,https://oleks-netizen.github.io/product-images/L20011-56/007.jpg,https://oleks-netizen.github.io/product-images/L20011-56/008.jpg,https://oleks-netizen.github.io/product-images/L20011-56/009.jpg</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>L20036-8</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20036-8/001.jpg,https://oleks-netizen.github.io/product-images/L20036-8/003.jpg,https://oleks-netizen.github.io/product-images/L20036-8/004.jpg,https://oleks-netizen.github.io/product-images/L20036-8/005.jpg,https://oleks-netizen.github.io/product-images/L20036-8/006.jpg,https://oleks-netizen.github.io/product-images/L20036-8/007.jpg,https://oleks-netizen.github.io/product-images/L20036-8/008.jpg,https://oleks-netizen.github.io/product-images/L20036-8/009.jpg,https://oleks-netizen.github.io/product-images/L20036-8/010.jpg</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>L20713-8</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20713-8/001.jpg,https://oleks-netizen.github.io/product-images/L20713-8/003.jpg,https://oleks-netizen.github.io/product-images/L20713-8/004.jpg,https://oleks-netizen.github.io/product-images/L20713-8/005.jpg,https://oleks-netizen.github.io/product-images/L20713-8/006.jpg,https://oleks-netizen.github.io/product-images/L20713-8/007.jpg,https://oleks-netizen.github.io/product-images/L20713-8/008.jpg,https://oleks-netizen.github.io/product-images/L20713-8/009.jpg,https://oleks-netizen.github.io/product-images/L20713-8/010.jpg</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>L20812-1</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20812-1/001.jpg,https://oleks-netizen.github.io/product-images/L20812-1/003.jpg,https://oleks-netizen.github.io/product-images/L20812-1/004.jpg,https://oleks-netizen.github.io/product-images/L20812-1/005.jpg,https://oleks-netizen.github.io/product-images/L20812-1/006.jpg,https://oleks-netizen.github.io/product-images/L20812-1/007.jpg,https://oleks-netizen.github.io/product-images/L20812-1/008.jpg,https://oleks-netizen.github.io/product-images/L20812-1/009.jpg,https://oleks-netizen.github.io/product-images/L20812-1/010.jpg</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>L20812-56</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20812-56/001.jpg,https://oleks-netizen.github.io/product-images/L20812-56/003.jpg,https://oleks-netizen.github.io/product-images/L20812-56/004.jpg,https://oleks-netizen.github.io/product-images/L20812-56/005.jpg,https://oleks-netizen.github.io/product-images/L20812-56/006.jpg,https://oleks-netizen.github.io/product-images/L20812-56/007.jpg,https://oleks-netizen.github.io/product-images/L20812-56/008.jpg,https://oleks-netizen.github.io/product-images/L20812-56/009.jpg,https://oleks-netizen.github.io/product-images/L20812-56/010.jpg</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>L20853-1</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20853-1/001.jpg,https://oleks-netizen.github.io/product-images/L20853-1/002.jpg,https://oleks-netizen.github.io/product-images/L20853-1/004.jpg,https://oleks-netizen.github.io/product-images/L20853-1/005.jpg,https://oleks-netizen.github.io/product-images/L20853-1/006.jpg,https://oleks-netizen.github.io/product-images/L20853-1/007.jpg,https://oleks-netizen.github.io/product-images/L20853-1/008.jpg,https://oleks-netizen.github.io/product-images/L20853-1/009.jpg,https://oleks-netizen.github.io/product-images/L20853-1/010.jpg</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>L21019-1</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21019-1/001.jpg,https://oleks-netizen.github.io/product-images/L21019-1/003.jpg,https://oleks-netizen.github.io/product-images/L21019-1/004.jpg,https://oleks-netizen.github.io/product-images/L21019-1/005.jpg,https://oleks-netizen.github.io/product-images/L21019-1/006.jpg,https://oleks-netizen.github.io/product-images/L21019-1/007.jpg,https://oleks-netizen.github.io/product-images/L21019-1/008.jpg,https://oleks-netizen.github.io/product-images/L21019-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>L21209-1</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21209-1/001.jpg,https://oleks-netizen.github.io/product-images/L21209-1/003.jpg,https://oleks-netizen.github.io/product-images/L21209-1/004.jpg,https://oleks-netizen.github.io/product-images/L21209-1/005.jpg,https://oleks-netizen.github.io/product-images/L21209-1/006.jpg,https://oleks-netizen.github.io/product-images/L21209-1/007.jpg,https://oleks-netizen.github.io/product-images/L21209-1/008.jpg,https://oleks-netizen.github.io/product-images/L21209-1/009.jpg,https://oleks-netizen.github.io/product-images/L21209-1/010.jpg</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>L21586-010</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21586-010/001.jpg,https://oleks-netizen.github.io/product-images/L21586-010/003.jpg,https://oleks-netizen.github.io/product-images/L21586-010/004.jpg,https://oleks-netizen.github.io/product-images/L21586-010/005.jpg,https://oleks-netizen.github.io/product-images/L21586-010/006.jpg,https://oleks-netizen.github.io/product-images/L21586-010/007.jpg,https://oleks-netizen.github.io/product-images/L21586-010/008.jpg,https://oleks-netizen.github.io/product-images/L21586-010/009.jpg</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>L21586-025</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21586-025/001.jpg,https://oleks-netizen.github.io/product-images/L21586-025/003.jpg,https://oleks-netizen.github.io/product-images/L21586-025/004.jpg,https://oleks-netizen.github.io/product-images/L21586-025/005.jpg,https://oleks-netizen.github.io/product-images/L21586-025/006.jpg,https://oleks-netizen.github.io/product-images/L21586-025/007.jpg,https://oleks-netizen.github.io/product-images/L21586-025/008.jpg,https://oleks-netizen.github.io/product-images/L21586-025/009.jpg</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>L21586-097</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L21586-097/001.jpg,https://oleks-netizen.github.io/product-images/L21586-097/003.jpg,https://oleks-netizen.github.io/product-images/L21586-097/004.jpg,https://oleks-netizen.github.io/product-images/L21586-097/005.jpg,https://oleks-netizen.github.io/product-images/L21586-097/006.jpg,https://oleks-netizen.github.io/product-images/L21586-097/007.jpg,https://oleks-netizen.github.io/product-images/L21586-097/008.jpg,https://oleks-netizen.github.io/product-images/L21586-097/009.jpg</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>L22007-3K</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22007-3K/001.jpg,https://oleks-netizen.github.io/product-images/L22007-3K/003.jpg,https://oleks-netizen.github.io/product-images/L22007-3K/004.jpg,https://oleks-netizen.github.io/product-images/L22007-3K/005.jpg,https://oleks-netizen.github.io/product-images/L22007-3K/006.jpg,https://oleks-netizen.github.io/product-images/L22007-3K/007.jpg,https://oleks-netizen.github.io/product-images/L22007-3K/008.jpg,https://oleks-netizen.github.io/product-images/L22007-3K/009.jpg</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>L22008-12</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22008-12/001.jpg,https://oleks-netizen.github.io/product-images/L22008-12/003.jpg,https://oleks-netizen.github.io/product-images/L22008-12/004.jpg,https://oleks-netizen.github.io/product-images/L22008-12/005.jpg,https://oleks-netizen.github.io/product-images/L22008-12/006.jpg,https://oleks-netizen.github.io/product-images/L22008-12/007.jpg,https://oleks-netizen.github.io/product-images/L22008-12/008.jpg,https://oleks-netizen.github.io/product-images/L22008-12/009.jpg</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>L22008-8</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22008-8/001.jpg,https://oleks-netizen.github.io/product-images/L22008-8/003.jpg,https://oleks-netizen.github.io/product-images/L22008-8/004.jpg,https://oleks-netizen.github.io/product-images/L22008-8/005.jpg,https://oleks-netizen.github.io/product-images/L22008-8/006.jpg,https://oleks-netizen.github.io/product-images/L22008-8/007.jpg,https://oleks-netizen.github.io/product-images/L22008-8/008.jpg,https://oleks-netizen.github.io/product-images/L22008-8/009.jpg,https://oleks-netizen.github.io/product-images/L22008-8/010.jpg</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>L22187-1X</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22187-1X/001.jpg,https://oleks-netizen.github.io/product-images/L22187-1X/002.jpg,https://oleks-netizen.github.io/product-images/L22187-1X/004.jpg,https://oleks-netizen.github.io/product-images/L22187-1X/005.jpg,https://oleks-netizen.github.io/product-images/L22187-1X/006.jpg,https://oleks-netizen.github.io/product-images/L22187-1X/007.jpg,https://oleks-netizen.github.io/product-images/L22187-1X/008.jpg,https://oleks-netizen.github.io/product-images/L22187-1X/009.jpg,https://oleks-netizen.github.io/product-images/L22187-1X/010.jpg</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>L22322-01</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22322-01/001.jpg,https://oleks-netizen.github.io/product-images/L22322-01/003.jpg,https://oleks-netizen.github.io/product-images/L22322-01/004.jpg,https://oleks-netizen.github.io/product-images/L22322-01/005.jpg,https://oleks-netizen.github.io/product-images/L22322-01/006.jpg,https://oleks-netizen.github.io/product-images/L22322-01/007.jpg,https://oleks-netizen.github.io/product-images/L22322-01/008.jpg,https://oleks-netizen.github.io/product-images/L22322-01/009.jpg,https://oleks-netizen.github.io/product-images/L22322-01/010.jpg</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>L22322-1</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22322-1/001.jpg,https://oleks-netizen.github.io/product-images/L22322-1/002.jpg,https://oleks-netizen.github.io/product-images/L22322-1/004.jpg,https://oleks-netizen.github.io/product-images/L22322-1/005.jpg,https://oleks-netizen.github.io/product-images/L22322-1/006.jpg,https://oleks-netizen.github.io/product-images/L22322-1/007.jpg,https://oleks-netizen.github.io/product-images/L22322-1/008.jpg,https://oleks-netizen.github.io/product-images/L22322-1/009.jpg,https://oleks-netizen.github.io/product-images/L22322-1/010.jpg</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>L22532-03</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22532-03/001.jpg,https://oleks-netizen.github.io/product-images/L22532-03/003.jpg,https://oleks-netizen.github.io/product-images/L22532-03/004.jpg,https://oleks-netizen.github.io/product-images/L22532-03/005.jpg,https://oleks-netizen.github.io/product-images/L22532-03/006.jpg,https://oleks-netizen.github.io/product-images/L22532-03/007.jpg,https://oleks-netizen.github.io/product-images/L22532-03/008.jpg,https://oleks-netizen.github.io/product-images/L22532-03/009.jpg</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>L22613-1</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22613-1/001.jpg,https://oleks-netizen.github.io/product-images/L22613-1/003.jpg,https://oleks-netizen.github.io/product-images/L22613-1/004.jpg,https://oleks-netizen.github.io/product-images/L22613-1/005.jpg,https://oleks-netizen.github.io/product-images/L22613-1/006.jpg,https://oleks-netizen.github.io/product-images/L22613-1/007.jpg,https://oleks-netizen.github.io/product-images/L22613-1/008.jpg,https://oleks-netizen.github.io/product-images/L22613-1/009.jpg,https://oleks-netizen.github.io/product-images/L22613-1/010.jpg</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>L22808-1</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22808-1/001.jpg,https://oleks-netizen.github.io/product-images/L22808-1/002.jpg,https://oleks-netizen.github.io/product-images/L22808-1/004.jpg,https://oleks-netizen.github.io/product-images/L22808-1/005.jpg,https://oleks-netizen.github.io/product-images/L22808-1/006.jpg,https://oleks-netizen.github.io/product-images/L22808-1/007.jpg,https://oleks-netizen.github.io/product-images/L22808-1/008.jpg,https://oleks-netizen.github.io/product-images/L22808-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>L22808-1W</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22808-1W/001.jpg,https://oleks-netizen.github.io/product-images/L22808-1W/002.jpg,https://oleks-netizen.github.io/product-images/L22808-1W/004.jpg,https://oleks-netizen.github.io/product-images/L22808-1W/005.jpg,https://oleks-netizen.github.io/product-images/L22808-1W/006.jpg,https://oleks-netizen.github.io/product-images/L22808-1W/007.jpg,https://oleks-netizen.github.io/product-images/L22808-1W/008.jpg,https://oleks-netizen.github.io/product-images/L22808-1W/009.jpg</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>L22813-04S</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L22813-04S/001.jpg,https://oleks-netizen.github.io/product-images/L22813-04S/003.jpg,https://oleks-netizen.github.io/product-images/L22813-04S/004.jpg,https://oleks-netizen.github.io/product-images/L22813-04S/005.jpg,https://oleks-netizen.github.io/product-images/L22813-04S/006.jpg,https://oleks-netizen.github.io/product-images/L22813-04S/007.jpg,https://oleks-netizen.github.io/product-images/L22813-04S/008.jpg,https://oleks-netizen.github.io/product-images/L22813-04S/009.jpg,https://oleks-netizen.github.io/product-images/L22813-04S/010.jpg</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>L26029-017</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L26029-017/001.jpg,https://oleks-netizen.github.io/product-images/L26029-017/002.jpg,https://oleks-netizen.github.io/product-images/L26029-017/004.jpg,https://oleks-netizen.github.io/product-images/L26029-017/005.jpg,https://oleks-netizen.github.io/product-images/L26029-017/006.jpg,https://oleks-netizen.github.io/product-images/L26029-017/007.jpg,https://oleks-netizen.github.io/product-images/L26029-017/008.jpg</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
         <v>7</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>L26290-005</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L26290-005/001.jpg,https://oleks-netizen.github.io/product-images/L26290-005/002.jpg,https://oleks-netizen.github.io/product-images/L26290-005/004.jpg,https://oleks-netizen.github.io/product-images/L26290-005/005.jpg,https://oleks-netizen.github.io/product-images/L26290-005/006.jpg,https://oleks-netizen.github.io/product-images/L26290-005/007.jpg,https://oleks-netizen.github.io/product-images/L26290-005/008.jpg</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>L26835-51</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L26835-51/001.jpg,https://oleks-netizen.github.io/product-images/L26835-51/003.jpg,https://oleks-netizen.github.io/product-images/L26835-51/004.jpg,https://oleks-netizen.github.io/product-images/L26835-51/005.jpg,https://oleks-netizen.github.io/product-images/L26835-51/006.jpg,https://oleks-netizen.github.io/product-images/L26835-51/007.jpg,https://oleks-netizen.github.io/product-images/L26835-51/008.jpg,https://oleks-netizen.github.io/product-images/L26835-51/009.jpg,https://oleks-netizen.github.io/product-images/L26835-51/010.jpg</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>L26836-1</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L26836-1/001.jpg,https://oleks-netizen.github.io/product-images/L26836-1/003.jpg,https://oleks-netizen.github.io/product-images/L26836-1/004.jpg,https://oleks-netizen.github.io/product-images/L26836-1/005.jpg,https://oleks-netizen.github.io/product-images/L26836-1/006.jpg,https://oleks-netizen.github.io/product-images/L26836-1/007.jpg,https://oleks-netizen.github.io/product-images/L26836-1/008.jpg,https://oleks-netizen.github.io/product-images/L26836-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>L26836-25</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L26836-25/001.jpg,https://oleks-netizen.github.io/product-images/L26836-25/003.jpg,https://oleks-netizen.github.io/product-images/L26836-25/004.jpg,https://oleks-netizen.github.io/product-images/L26836-25/005.jpg,https://oleks-netizen.github.io/product-images/L26836-25/006.jpg,https://oleks-netizen.github.io/product-images/L26836-25/007.jpg,https://oleks-netizen.github.io/product-images/L26836-25/008.jpg,https://oleks-netizen.github.io/product-images/L26836-25/009.jpg</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>L26897-025</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L26897-025/001.jpg,https://oleks-netizen.github.io/product-images/L26897-025/002.jpg,https://oleks-netizen.github.io/product-images/L26897-025/004.jpg,https://oleks-netizen.github.io/product-images/L26897-025/005.jpg,https://oleks-netizen.github.io/product-images/L26897-025/006.jpg,https://oleks-netizen.github.io/product-images/L26897-025/007.jpg</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>L27002-3</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L27002-3/001.jpg,https://oleks-netizen.github.io/product-images/L27002-3/002.jpg,https://oleks-netizen.github.io/product-images/L27002-3/004.jpg,https://oleks-netizen.github.io/product-images/L27002-3/005.jpg,https://oleks-netizen.github.io/product-images/L27002-3/006.jpg,https://oleks-netizen.github.io/product-images/L27002-3/007.jpg,https://oleks-netizen.github.io/product-images/L27002-3/008.jpg,https://oleks-netizen.github.io/product-images/L27002-3/009.jpg</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>L28001-4</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28001-4/001.jpg,https://oleks-netizen.github.io/product-images/L28001-4/003.jpg,https://oleks-netizen.github.io/product-images/L28001-4/004.jpg,https://oleks-netizen.github.io/product-images/L28001-4/005.jpg,https://oleks-netizen.github.io/product-images/L28001-4/006.jpg,https://oleks-netizen.github.io/product-images/L28001-4/007.jpg,https://oleks-netizen.github.io/product-images/L28001-4/008.jpg</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>L28028-2</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28028-2/001.jpg,https://oleks-netizen.github.io/product-images/L28028-2/003.jpg,https://oleks-netizen.github.io/product-images/L28028-2/004.jpg,https://oleks-netizen.github.io/product-images/L28028-2/005.jpg,https://oleks-netizen.github.io/product-images/L28028-2/006.jpg,https://oleks-netizen.github.io/product-images/L28028-2/007.jpg,https://oleks-netizen.github.io/product-images/L28028-2/008.jpg,https://oleks-netizen.github.io/product-images/L28028-2/009.jpg</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>L28028-3</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28028-3/001.jpg,https://oleks-netizen.github.io/product-images/L28028-3/003.jpg,https://oleks-netizen.github.io/product-images/L28028-3/004.jpg,https://oleks-netizen.github.io/product-images/L28028-3/005.jpg,https://oleks-netizen.github.io/product-images/L28028-3/006.jpg,https://oleks-netizen.github.io/product-images/L28028-3/007.jpg,https://oleks-netizen.github.io/product-images/L28028-3/008.jpg,https://oleks-netizen.github.io/product-images/L28028-3/009.jpg</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>L28029-2</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L28029-2/001.jpg,https://oleks-netizen.github.io/product-images/L28029-2/003.jpg,https://oleks-netizen.github.io/product-images/L28029-2/004.jpg,https://oleks-netizen.github.io/product-images/L28029-2/005.jpg,https://oleks-netizen.github.io/product-images/L28029-2/006.jpg,https://oleks-netizen.github.io/product-images/L28029-2/007.jpg,https://oleks-netizen.github.io/product-images/L28029-2/008.jpg,https://oleks-netizen.github.io/product-images/L28029-2/009.jpg</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>L29048-02</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L29048-02/001.jpg,https://oleks-netizen.github.io/product-images/L29048-02/003.jpg,https://oleks-netizen.github.io/product-images/L29048-02/004.jpg,https://oleks-netizen.github.io/product-images/L29048-02/005.jpg,https://oleks-netizen.github.io/product-images/L29048-02/006.jpg,https://oleks-netizen.github.io/product-images/L29048-02/007.jpg,https://oleks-netizen.github.io/product-images/L29048-02/008.jpg</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>L29205-27</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L29205-27/001.jpg,https://oleks-netizen.github.io/product-images/L29205-27/003.jpg,https://oleks-netizen.github.io/product-images/L29205-27/004.jpg,https://oleks-netizen.github.io/product-images/L29205-27/005.jpg,https://oleks-netizen.github.io/product-images/L29205-27/006.jpg,https://oleks-netizen.github.io/product-images/L29205-27/007.jpg,https://oleks-netizen.github.io/product-images/L29205-27/008.jpg</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>L85162-1</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L85162-1/001.jpg,https://oleks-netizen.github.io/product-images/L85162-1/003.jpg,https://oleks-netizen.github.io/product-images/L85162-1/004.jpg,https://oleks-netizen.github.io/product-images/L85162-1/005.jpg,https://oleks-netizen.github.io/product-images/L85162-1/006.jpg,https://oleks-netizen.github.io/product-images/L85162-1/007.jpg,https://oleks-netizen.github.io/product-images/L85162-1/008.jpg,https://oleks-netizen.github.io/product-images/L85162-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>L86913-1</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L86913-1/001.jpg,https://oleks-netizen.github.io/product-images/L86913-1/003.jpg,https://oleks-netizen.github.io/product-images/L86913-1/004.jpg,https://oleks-netizen.github.io/product-images/L86913-1/005.jpg,https://oleks-netizen.github.io/product-images/L86913-1/006.jpg,https://oleks-netizen.github.io/product-images/L86913-1/007.jpg,https://oleks-netizen.github.io/product-images/L86913-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>L87006-1</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87006-1/001.jpg,https://oleks-netizen.github.io/product-images/L87006-1/003.jpg,https://oleks-netizen.github.io/product-images/L87006-1/004.jpg,https://oleks-netizen.github.io/product-images/L87006-1/005.jpg,https://oleks-netizen.github.io/product-images/L87006-1/006.jpg,https://oleks-netizen.github.io/product-images/L87006-1/007.jpg,https://oleks-netizen.github.io/product-images/L87006-1/008.jpg,https://oleks-netizen.github.io/product-images/L87006-1/009.jpg,https://oleks-netizen.github.io/product-images/L87006-1/010.jpg</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>L87006-25</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87006-25/001.jpg,https://oleks-netizen.github.io/product-images/L87006-25/003.jpg,https://oleks-netizen.github.io/product-images/L87006-25/004.jpg,https://oleks-netizen.github.io/product-images/L87006-25/005.jpg,https://oleks-netizen.github.io/product-images/L87006-25/006.jpg,https://oleks-netizen.github.io/product-images/L87006-25/007.jpg,https://oleks-netizen.github.io/product-images/L87006-25/008.jpg,https://oleks-netizen.github.io/product-images/L87006-25/009.jpg,https://oleks-netizen.github.io/product-images/L87006-25/010.jpg</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>L87006-51</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87006-51/001.jpg,https://oleks-netizen.github.io/product-images/L87006-51/003.jpg,https://oleks-netizen.github.io/product-images/L87006-51/004.jpg,https://oleks-netizen.github.io/product-images/L87006-51/005.jpg,https://oleks-netizen.github.io/product-images/L87006-51/006.jpg,https://oleks-netizen.github.io/product-images/L87006-51/007.jpg,https://oleks-netizen.github.io/product-images/L87006-51/008.jpg,https://oleks-netizen.github.io/product-images/L87006-51/009.jpg,https://oleks-netizen.github.io/product-images/L87006-51/010.jpg</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>L87024-1</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87024-1/001.jpg,https://oleks-netizen.github.io/product-images/L87024-1/003.jpg,https://oleks-netizen.github.io/product-images/L87024-1/004.jpg,https://oleks-netizen.github.io/product-images/L87024-1/005.jpg,https://oleks-netizen.github.io/product-images/L87024-1/006.jpg,https://oleks-netizen.github.io/product-images/L87024-1/007.jpg,https://oleks-netizen.github.io/product-images/L87024-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>L87169-1W</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87169-1W/001.jpg,https://oleks-netizen.github.io/product-images/L87169-1W/002.jpg,https://oleks-netizen.github.io/product-images/L87169-1W/004.jpg,https://oleks-netizen.github.io/product-images/L87169-1W/005.jpg,https://oleks-netizen.github.io/product-images/L87169-1W/006.jpg,https://oleks-netizen.github.io/product-images/L87169-1W/007.jpg,https://oleks-netizen.github.io/product-images/L87169-1W/008.jpg,https://oleks-netizen.github.io/product-images/L87169-1W/009.jpg</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>L87190-Q38</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87190-Q38/001.jpg,https://oleks-netizen.github.io/product-images/L87190-Q38/003.jpg,https://oleks-netizen.github.io/product-images/L87190-Q38/004.jpg,https://oleks-netizen.github.io/product-images/L87190-Q38/005.jpg,https://oleks-netizen.github.io/product-images/L87190-Q38/006.jpg,https://oleks-netizen.github.io/product-images/L87190-Q38/007.jpg,https://oleks-netizen.github.io/product-images/L87190-Q38/008.jpg,https://oleks-netizen.github.io/product-images/L87190-Q38/009.jpg</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>L87196-1</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87196-1/001.jpg,https://oleks-netizen.github.io/product-images/L87196-1/003.jpg,https://oleks-netizen.github.io/product-images/L87196-1/004.jpg,https://oleks-netizen.github.io/product-images/L87196-1/005.jpg,https://oleks-netizen.github.io/product-images/L87196-1/006.jpg,https://oleks-netizen.github.io/product-images/L87196-1/007.jpg,https://oleks-netizen.github.io/product-images/L87196-1/008.jpg,https://oleks-netizen.github.io/product-images/L87196-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>L87202-F3</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87202-F3/001.jpg,https://oleks-netizen.github.io/product-images/L87202-F3/003.jpg,https://oleks-netizen.github.io/product-images/L87202-F3/004.jpg,https://oleks-netizen.github.io/product-images/L87202-F3/005.jpg,https://oleks-netizen.github.io/product-images/L87202-F3/006.jpg,https://oleks-netizen.github.io/product-images/L87202-F3/007.jpg,https://oleks-netizen.github.io/product-images/L87202-F3/008.jpg,https://oleks-netizen.github.io/product-images/L87202-F3/009.jpg,https://oleks-netizen.github.io/product-images/L87202-F3/010.jpg</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>L87220-1W</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87220-1W/001.jpg,https://oleks-netizen.github.io/product-images/L87220-1W/002.jpg,https://oleks-netizen.github.io/product-images/L87220-1W/004.jpg,https://oleks-netizen.github.io/product-images/L87220-1W/005.jpg,https://oleks-netizen.github.io/product-images/L87220-1W/006.jpg,https://oleks-netizen.github.io/product-images/L87220-1W/007.jpg,https://oleks-netizen.github.io/product-images/L87220-1W/008.jpg</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>L87220-H10</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87220-H10/001.jpg,https://oleks-netizen.github.io/product-images/L87220-H10/003.jpg,https://oleks-netizen.github.io/product-images/L87220-H10/004.jpg,https://oleks-netizen.github.io/product-images/L87220-H10/005.jpg,https://oleks-netizen.github.io/product-images/L87220-H10/006.jpg,https://oleks-netizen.github.io/product-images/L87220-H10/007.jpg,https://oleks-netizen.github.io/product-images/L87220-H10/008.jpg,https://oleks-netizen.github.io/product-images/L87220-H10/009.jpg,https://oleks-netizen.github.io/product-images/L87220-H10/010.jpg</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>L87229-137</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87229-137/001.jpg,https://oleks-netizen.github.io/product-images/L87229-137/003.jpg,https://oleks-netizen.github.io/product-images/L87229-137/004.jpg,https://oleks-netizen.github.io/product-images/L87229-137/005.jpg,https://oleks-netizen.github.io/product-images/L87229-137/006.jpg,https://oleks-netizen.github.io/product-images/L87229-137/007.jpg,https://oleks-netizen.github.io/product-images/L87229-137/008.jpg,https://oleks-netizen.github.io/product-images/L87229-137/009.jpg</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>L87251-5</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87251-5/001.jpg,https://oleks-netizen.github.io/product-images/L87251-5/003.jpg,https://oleks-netizen.github.io/product-images/L87251-5/004.jpg,https://oleks-netizen.github.io/product-images/L87251-5/005.jpg,https://oleks-netizen.github.io/product-images/L87251-5/006.jpg,https://oleks-netizen.github.io/product-images/L87251-5/007.jpg,https://oleks-netizen.github.io/product-images/L87251-5/008.jpg</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>L87274-58</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87274-58/001.jpg,https://oleks-netizen.github.io/product-images/L87274-58/003.jpg,https://oleks-netizen.github.io/product-images/L87274-58/004.jpg,https://oleks-netizen.github.io/product-images/L87274-58/005.jpg,https://oleks-netizen.github.io/product-images/L87274-58/006.jpg,https://oleks-netizen.github.io/product-images/L87274-58/007.jpg,https://oleks-netizen.github.io/product-images/L87274-58/008.jpg,https://oleks-netizen.github.io/product-images/L87274-58/009.jpg</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>L87309-7</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87309-7/001.jpg,https://oleks-netizen.github.io/product-images/L87309-7/003.jpg,https://oleks-netizen.github.io/product-images/L87309-7/004.jpg,https://oleks-netizen.github.io/product-images/L87309-7/005.jpg,https://oleks-netizen.github.io/product-images/L87309-7/006.jpg,https://oleks-netizen.github.io/product-images/L87309-7/007.jpg,https://oleks-netizen.github.io/product-images/L87309-7/008.jpg,https://oleks-netizen.github.io/product-images/L87309-7/009.jpg</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>L87341-171</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87341-171/001.jpg,https://oleks-netizen.github.io/product-images/L87341-171/003.jpg,https://oleks-netizen.github.io/product-images/L87341-171/004.jpg,https://oleks-netizen.github.io/product-images/L87341-171/005.jpg,https://oleks-netizen.github.io/product-images/L87341-171/006.jpg,https://oleks-netizen.github.io/product-images/L87341-171/007.jpg,https://oleks-netizen.github.io/product-images/L87341-171/008.jpg,https://oleks-netizen.github.io/product-images/L87341-171/009.jpg</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>L87341-22</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87341-22/001.jpg,https://oleks-netizen.github.io/product-images/L87341-22/003.jpg,https://oleks-netizen.github.io/product-images/L87341-22/004.jpg,https://oleks-netizen.github.io/product-images/L87341-22/005.jpg,https://oleks-netizen.github.io/product-images/L87341-22/006.jpg,https://oleks-netizen.github.io/product-images/L87341-22/007.jpg,https://oleks-netizen.github.io/product-images/L87341-22/008.jpg,https://oleks-netizen.github.io/product-images/L87341-22/009.jpg</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>L87480-1X</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87480-1X/001.jpg,https://oleks-netizen.github.io/product-images/L87480-1X/003.jpg,https://oleks-netizen.github.io/product-images/L87480-1X/004.jpg,https://oleks-netizen.github.io/product-images/L87480-1X/005.jpg,https://oleks-netizen.github.io/product-images/L87480-1X/006.jpg,https://oleks-netizen.github.io/product-images/L87480-1X/007.jpg,https://oleks-netizen.github.io/product-images/L87480-1X/008.jpg,https://oleks-netizen.github.io/product-images/L87480-1X/009.jpg,https://oleks-netizen.github.io/product-images/L87480-1X/010.jpg</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>L87480-94X</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87480-94X/001.jpg,https://oleks-netizen.github.io/product-images/L87480-94X/003.jpg,https://oleks-netizen.github.io/product-images/L87480-94X/004.jpg,https://oleks-netizen.github.io/product-images/L87480-94X/005.jpg,https://oleks-netizen.github.io/product-images/L87480-94X/006.jpg,https://oleks-netizen.github.io/product-images/L87480-94X/007.jpg,https://oleks-netizen.github.io/product-images/L87480-94X/008.jpg,https://oleks-netizen.github.io/product-images/L87480-94X/009.jpg,https://oleks-netizen.github.io/product-images/L87480-94X/010.jpg</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>L87483-1</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87483-1/001.jpg,https://oleks-netizen.github.io/product-images/L87483-1/003.jpg,https://oleks-netizen.github.io/product-images/L87483-1/004.jpg,https://oleks-netizen.github.io/product-images/L87483-1/005.jpg,https://oleks-netizen.github.io/product-images/L87483-1/006.jpg,https://oleks-netizen.github.io/product-images/L87483-1/007.jpg,https://oleks-netizen.github.io/product-images/L87483-1/008.jpg,https://oleks-netizen.github.io/product-images/L87483-1/009.jpg,https://oleks-netizen.github.io/product-images/L87483-1/010.jpg</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>L87501-161</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87501-161/001.jpg,https://oleks-netizen.github.io/product-images/L87501-161/003.jpg,https://oleks-netizen.github.io/product-images/L87501-161/004.jpg,https://oleks-netizen.github.io/product-images/L87501-161/005.jpg,https://oleks-netizen.github.io/product-images/L87501-161/006.jpg,https://oleks-netizen.github.io/product-images/L87501-161/007.jpg,https://oleks-netizen.github.io/product-images/L87501-161/008.jpg,https://oleks-netizen.github.io/product-images/L87501-161/009.jpg</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>L87501-163</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87501-163/001.jpg,https://oleks-netizen.github.io/product-images/L87501-163/003.jpg,https://oleks-netizen.github.io/product-images/L87501-163/004.jpg,https://oleks-netizen.github.io/product-images/L87501-163/005.jpg,https://oleks-netizen.github.io/product-images/L87501-163/006.jpg,https://oleks-netizen.github.io/product-images/L87501-163/007.jpg,https://oleks-netizen.github.io/product-images/L87501-163/008.jpg,https://oleks-netizen.github.io/product-images/L87501-163/009.jpg</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>L87501-92</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87501-92/001.jpg,https://oleks-netizen.github.io/product-images/L87501-92/003.jpg,https://oleks-netizen.github.io/product-images/L87501-92/004.jpg,https://oleks-netizen.github.io/product-images/L87501-92/005.jpg,https://oleks-netizen.github.io/product-images/L87501-92/006.jpg,https://oleks-netizen.github.io/product-images/L87501-92/007.jpg,https://oleks-netizen.github.io/product-images/L87501-92/008.jpg,https://oleks-netizen.github.io/product-images/L87501-92/009.jpg</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>L87503-1</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87503-1/001.jpg,https://oleks-netizen.github.io/product-images/L87503-1/003.jpg,https://oleks-netizen.github.io/product-images/L87503-1/004.jpg,https://oleks-netizen.github.io/product-images/L87503-1/005.jpg,https://oleks-netizen.github.io/product-images/L87503-1/006.jpg,https://oleks-netizen.github.io/product-images/L87503-1/007.jpg,https://oleks-netizen.github.io/product-images/L87503-1/008.jpg,https://oleks-netizen.github.io/product-images/L87503-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>L87505-162</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87505-162/001.jpg,https://oleks-netizen.github.io/product-images/L87505-162/003.jpg,https://oleks-netizen.github.io/product-images/L87505-162/004.jpg,https://oleks-netizen.github.io/product-images/L87505-162/005.jpg,https://oleks-netizen.github.io/product-images/L87505-162/006.jpg,https://oleks-netizen.github.io/product-images/L87505-162/007.jpg,https://oleks-netizen.github.io/product-images/L87505-162/008.jpg,https://oleks-netizen.github.io/product-images/L87505-162/009.jpg,https://oleks-netizen.github.io/product-images/L87505-162/010.jpg</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>L87505-163</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87505-163/001.jpg,https://oleks-netizen.github.io/product-images/L87505-163/003.jpg,https://oleks-netizen.github.io/product-images/L87505-163/004.jpg,https://oleks-netizen.github.io/product-images/L87505-163/005.jpg,https://oleks-netizen.github.io/product-images/L87505-163/006.jpg,https://oleks-netizen.github.io/product-images/L87505-163/007.jpg,https://oleks-netizen.github.io/product-images/L87505-163/008.jpg,https://oleks-netizen.github.io/product-images/L87505-163/009.jpg,https://oleks-netizen.github.io/product-images/L87505-163/010.jpg</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>L87511-1</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87511-1/001.jpg,https://oleks-netizen.github.io/product-images/L87511-1/003.jpg,https://oleks-netizen.github.io/product-images/L87511-1/004.jpg,https://oleks-netizen.github.io/product-images/L87511-1/005.jpg,https://oleks-netizen.github.io/product-images/L87511-1/006.jpg,https://oleks-netizen.github.io/product-images/L87511-1/007.jpg,https://oleks-netizen.github.io/product-images/L87511-1/008.jpg,https://oleks-netizen.github.io/product-images/L87511-1/009.jpg</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>L87518-01</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87518-01/001.jpg,https://oleks-netizen.github.io/product-images/L87518-01/003.jpg,https://oleks-netizen.github.io/product-images/L87518-01/004.jpg,https://oleks-netizen.github.io/product-images/L87518-01/005.jpg,https://oleks-netizen.github.io/product-images/L87518-01/006.jpg,https://oleks-netizen.github.io/product-images/L87518-01/007.jpg,https://oleks-netizen.github.io/product-images/L87518-01/008.jpg,https://oleks-netizen.github.io/product-images/L87518-01/009.jpg</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>L87535-94X</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87535-94X/001.jpg,https://oleks-netizen.github.io/product-images/L87535-94X/003.jpg,https://oleks-netizen.github.io/product-images/L87535-94X/004.jpg,https://oleks-netizen.github.io/product-images/L87535-94X/005.jpg,https://oleks-netizen.github.io/product-images/L87535-94X/006.jpg,https://oleks-netizen.github.io/product-images/L87535-94X/007.jpg,https://oleks-netizen.github.io/product-images/L87535-94X/008.jpg,https://oleks-netizen.github.io/product-images/L87535-94X/009.jpg,https://oleks-netizen.github.io/product-images/L87535-94X/010.jpg</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>L87606-1X</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87606-1X/001.jpg,https://oleks-netizen.github.io/product-images/L87606-1X/003.jpg,https://oleks-netizen.github.io/product-images/L87606-1X/004.jpg,https://oleks-netizen.github.io/product-images/L87606-1X/005.jpg,https://oleks-netizen.github.io/product-images/L87606-1X/006.jpg,https://oleks-netizen.github.io/product-images/L87606-1X/007.jpg,https://oleks-netizen.github.io/product-images/L87606-1X/008.jpg,https://oleks-netizen.github.io/product-images/L87606-1X/009.jpg,https://oleks-netizen.github.io/product-images/L87606-1X/010.jpg,https://oleks-netizen.github.io/product-images/L87606-1X/011.jpg</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>L87606-70</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87606-70/001.jpg,https://oleks-netizen.github.io/product-images/L87606-70/003.jpg,https://oleks-netizen.github.io/product-images/L87606-70/004.jpg,https://oleks-netizen.github.io/product-images/L87606-70/005.jpg,https://oleks-netizen.github.io/product-images/L87606-70/006.jpg,https://oleks-netizen.github.io/product-images/L87606-70/007.jpg,https://oleks-netizen.github.io/product-images/L87606-70/008.jpg,https://oleks-netizen.github.io/product-images/L87606-70/009.jpg,https://oleks-netizen.github.io/product-images/L87606-70/010.jpg,https://oleks-netizen.github.io/product-images/L87606-70/011.jpg</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>L87891-1X</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L87891-1X/001.jpg,https://oleks-netizen.github.io/product-images/L87891-1X/003.jpg,https://oleks-netizen.github.io/product-images/L87891-1X/004.jpg,https://oleks-netizen.github.io/product-images/L87891-1X/005.jpg,https://oleks-netizen.github.io/product-images/L87891-1X/006.jpg,https://oleks-netizen.github.io/product-images/L87891-1X/007.jpg,https://oleks-netizen.github.io/product-images/L87891-1X/008.jpg,https://oleks-netizen.github.io/product-images/L87891-1X/009.jpg,https://oleks-netizen.github.io/product-images/L87891-1X/010.jpg</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>L88005-211</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L88005-211/001.jpg,https://oleks-netizen.github.io/product-images/L88005-211/003.jpg,https://oleks-netizen.github.io/product-images/L88005-211/004.jpg,https://oleks-netizen.github.io/product-images/L88005-211/005.jpg,https://oleks-netizen.github.io/product-images/L88005-211/006.jpg,https://oleks-netizen.github.io/product-images/L88005-211/007.jpg,https://oleks-netizen.github.io/product-images/L88005-211/008.jpg,https://oleks-netizen.github.io/product-images/L88005-211/009.jpg</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>L88015-66</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L88015-66/001.jpg,https://oleks-netizen.github.io/product-images/L88015-66/003.jpg,https://oleks-netizen.github.io/product-images/L88015-66/004.jpg,https://oleks-netizen.github.io/product-images/L88015-66/005.jpg,https://oleks-netizen.github.io/product-images/L88015-66/006.jpg,https://oleks-netizen.github.io/product-images/L88015-66/007.jpg,https://oleks-netizen.github.io/product-images/L88015-66/008.jpg,https://oleks-netizen.github.io/product-images/L88015-66/009.jpg</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>L88542-32</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L88542-32/001.jpg,https://oleks-netizen.github.io/product-images/L88542-32/003.jpg,https://oleks-netizen.github.io/product-images/L88542-32/004.jpg,https://oleks-netizen.github.io/product-images/L88542-32/005.jpg,https://oleks-netizen.github.io/product-images/L88542-32/006.jpg,https://oleks-netizen.github.io/product-images/L88542-32/007.jpg,https://oleks-netizen.github.io/product-images/L88542-32/008.jpg,https://oleks-netizen.github.io/product-images/L88542-32/009.jpg</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>L88542-65</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L88542-65/001.jpg,https://oleks-netizen.github.io/product-images/L88542-65/003.jpg,https://oleks-netizen.github.io/product-images/L88542-65/004.jpg,https://oleks-netizen.github.io/product-images/L88542-65/005.jpg,https://oleks-netizen.github.io/product-images/L88542-65/006.jpg,https://oleks-netizen.github.io/product-images/L88542-65/007.jpg,https://oleks-netizen.github.io/product-images/L88542-65/008.jpg,https://oleks-netizen.github.io/product-images/L88542-65/009.jpg</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>L88801-201</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L88801-201/001.jpg,https://oleks-netizen.github.io/product-images/L88801-201/003.jpg,https://oleks-netizen.github.io/product-images/L88801-201/004.jpg,https://oleks-netizen.github.io/product-images/L88801-201/005.jpg,https://oleks-netizen.github.io/product-images/L88801-201/006.jpg,https://oleks-netizen.github.io/product-images/L88801-201/007.jpg,https://oleks-netizen.github.io/product-images/L88801-201/008.jpg,https://oleks-netizen.github.io/product-images/L88801-201/009.jpg</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>L88801-216</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L88801-216/001.jpg,https://oleks-netizen.github.io/product-images/L88801-216/003.jpg,https://oleks-netizen.github.io/product-images/L88801-216/004.jpg,https://oleks-netizen.github.io/product-images/L88801-216/005.jpg,https://oleks-netizen.github.io/product-images/L88801-216/006.jpg,https://oleks-netizen.github.io/product-images/L88801-216/007.jpg,https://oleks-netizen.github.io/product-images/L88801-216/008.jpg,https://oleks-netizen.github.io/product-images/L88801-216/009.jpg</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>S31001-11</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31001-11/001.jpg,https://oleks-netizen.github.io/product-images/S31001-11/003.jpg,https://oleks-netizen.github.io/product-images/S31001-11/004.jpg,https://oleks-netizen.github.io/product-images/S31001-11/005.jpg,https://oleks-netizen.github.io/product-images/S31001-11/006.jpg,https://oleks-netizen.github.io/product-images/S31001-11/007.jpg,https://oleks-netizen.github.io/product-images/S31001-11/008.jpg</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>S31001-2</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31001-2/001.jpg,https://oleks-netizen.github.io/product-images/S31001-2/003.jpg,https://oleks-netizen.github.io/product-images/S31001-2/004.jpg,https://oleks-netizen.github.io/product-images/S31001-2/005.jpg,https://oleks-netizen.github.io/product-images/S31001-2/006.jpg,https://oleks-netizen.github.io/product-images/S31001-2/007.jpg,https://oleks-netizen.github.io/product-images/S31001-2/008.jpg</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>S31011-11</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31011-11/001.jpg,https://oleks-netizen.github.io/product-images/S31011-11/003.jpg,https://oleks-netizen.github.io/product-images/S31011-11/004.jpg,https://oleks-netizen.github.io/product-images/S31011-11/005.jpg,https://oleks-netizen.github.io/product-images/S31011-11/006.jpg,https://oleks-netizen.github.io/product-images/S31011-11/007.jpg</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>S31011-3</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31011-3/001.jpg,https://oleks-netizen.github.io/product-images/S31011-3/003.jpg,https://oleks-netizen.github.io/product-images/S31011-3/004.jpg,https://oleks-netizen.github.io/product-images/S31011-3/005.jpg,https://oleks-netizen.github.io/product-images/S31011-3/006.jpg,https://oleks-netizen.github.io/product-images/S31011-3/007.jpg</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>S31307-1</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31307-1/001.jpg,https://oleks-netizen.github.io/product-images/S31307-1/003.jpg,https://oleks-netizen.github.io/product-images/S31307-1/004.jpg,https://oleks-netizen.github.io/product-images/S31307-1/005.jpg,https://oleks-netizen.github.io/product-images/S31307-1/006.jpg,https://oleks-netizen.github.io/product-images/S31307-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>S31512-11</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31512-11/001.jpg,https://oleks-netizen.github.io/product-images/S31512-11/003.jpg,https://oleks-netizen.github.io/product-images/S31512-11/004.jpg,https://oleks-netizen.github.io/product-images/S31512-11/005.jpg,https://oleks-netizen.github.io/product-images/S31512-11/006.jpg,https://oleks-netizen.github.io/product-images/S31512-11/007.jpg</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>S31512-9</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31512-9/001.jpg,https://oleks-netizen.github.io/product-images/S31512-9/003.jpg,https://oleks-netizen.github.io/product-images/S31512-9/004.jpg,https://oleks-netizen.github.io/product-images/S31512-9/005.jpg,https://oleks-netizen.github.io/product-images/S31512-9/006.jpg,https://oleks-netizen.github.io/product-images/S31512-9/007.jpg</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>S31533-1</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31533-1/001.jpg,https://oleks-netizen.github.io/product-images/S31533-1/003.jpg,https://oleks-netizen.github.io/product-images/S31533-1/004.jpg,https://oleks-netizen.github.io/product-images/S31533-1/005.jpg,https://oleks-netizen.github.io/product-images/S31533-1/006.jpg,https://oleks-netizen.github.io/product-images/S31533-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>S31543-1</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31543-1/001.jpg,https://oleks-netizen.github.io/product-images/S31543-1/003.jpg,https://oleks-netizen.github.io/product-images/S31543-1/004.jpg,https://oleks-netizen.github.io/product-images/S31543-1/005.jpg,https://oleks-netizen.github.io/product-images/S31543-1/006.jpg,https://oleks-netizen.github.io/product-images/S31543-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>S31578-1</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31578-1/001.jpg,https://oleks-netizen.github.io/product-images/S31578-1/003.jpg,https://oleks-netizen.github.io/product-images/S31578-1/004.jpg,https://oleks-netizen.github.io/product-images/S31578-1/005.jpg,https://oleks-netizen.github.io/product-images/S31578-1/006.jpg,https://oleks-netizen.github.io/product-images/S31578-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>S31583-1</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31583-1/001.jpg,https://oleks-netizen.github.io/product-images/S31583-1/003.jpg,https://oleks-netizen.github.io/product-images/S31583-1/004.jpg,https://oleks-netizen.github.io/product-images/S31583-1/005.jpg,https://oleks-netizen.github.io/product-images/S31583-1/006.jpg,https://oleks-netizen.github.io/product-images/S31583-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>S31586-1</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31586-1/001.jpg,https://oleks-netizen.github.io/product-images/S31586-1/003.jpg,https://oleks-netizen.github.io/product-images/S31586-1/004.jpg,https://oleks-netizen.github.io/product-images/S31586-1/005.jpg,https://oleks-netizen.github.io/product-images/S31586-1/006.jpg,https://oleks-netizen.github.io/product-images/S31586-1/007.jpg</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>S31598-11</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31598-11/001.jpg,https://oleks-netizen.github.io/product-images/S31598-11/003.jpg,https://oleks-netizen.github.io/product-images/S31598-11/004.jpg,https://oleks-netizen.github.io/product-images/S31598-11/005.jpg,https://oleks-netizen.github.io/product-images/S31598-11/006.jpg,https://oleks-netizen.github.io/product-images/S31598-11/007.jpg,https://oleks-netizen.github.io/product-images/S31598-11/008.jpg</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>S31598-4</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31598-4/001.jpg,https://oleks-netizen.github.io/product-images/S31598-4/003.jpg,https://oleks-netizen.github.io/product-images/S31598-4/004.jpg,https://oleks-netizen.github.io/product-images/S31598-4/005.jpg,https://oleks-netizen.github.io/product-images/S31598-4/006.jpg,https://oleks-netizen.github.io/product-images/S31598-4/007.jpg,https://oleks-netizen.github.io/product-images/S31598-4/008.jpg</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>S31598-9</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31598-9/001.jpg,https://oleks-netizen.github.io/product-images/S31598-9/003.jpg,https://oleks-netizen.github.io/product-images/S31598-9/004.jpg,https://oleks-netizen.github.io/product-images/S31598-9/005.jpg,https://oleks-netizen.github.io/product-images/S31598-9/006.jpg,https://oleks-netizen.github.io/product-images/S31598-9/007.jpg,https://oleks-netizen.github.io/product-images/S31598-9/008.jpg</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>S31805-2</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/S31805-2/001.jpg,https://oleks-netizen.github.io/product-images/S31805-2/003.jpg,https://oleks-netizen.github.io/product-images/S31805-2/004.jpg,https://oleks-netizen.github.io/product-images/S31805-2/005.jpg,https://oleks-netizen.github.io/product-images/S31805-2/006.jpg,https://oleks-netizen.github.io/product-images/S31805-2/007.jpg</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-08-07 10:26:56
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,706 +436,361 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1092519939</t>
+          <t>336201100</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1092519939/001.jpg,https://oleks-netizen.github.io/product-images/1092519939/002.jpg,https://oleks-netizen.github.io/product-images/1092519939/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/336201100/001.jpg,https://oleks-netizen.github.io/product-images/336201100/002.jpg,https://oleks-netizen.github.io/product-images/336201100/003.jpg,https://oleks-netizen.github.io/product-images/336201100/004.jpg,https://oleks-netizen.github.io/product-images/336201100/005.jpg,https://oleks-netizen.github.io/product-images/336201100/006.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1113320509</t>
+          <t>410011208</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1113320509/001.jpg,https://oleks-netizen.github.io/product-images/1113320509/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/410011208/001.jpg,https://oleks-netizen.github.io/product-images/410011208/002.jpg,https://oleks-netizen.github.io/product-images/410011208/003.jpg,https://oleks-netizen.github.io/product-images/410011208/004.jpg,https://oleks-netizen.github.io/product-images/410011208/005.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1113320510</t>
+          <t>410011508</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1113320510/001.jpg,https://oleks-netizen.github.io/product-images/1113320510/002.jpg,https://oleks-netizen.github.io/product-images/1113320510/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/410011508/001.jpg,https://oleks-netizen.github.io/product-images/410011508/002.jpg,https://oleks-netizen.github.io/product-images/410011508/003.jpg,https://oleks-netizen.github.io/product-images/410011508/004.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1113320511</t>
+          <t>410413701</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1113320511/001.jpg,https://oleks-netizen.github.io/product-images/1113320511/002.jpg,https://oleks-netizen.github.io/product-images/1113320511/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/410413701/001.jpg,https://oleks-netizen.github.io/product-images/410413701/002.jpg,https://oleks-netizen.github.io/product-images/410413701/003.jpg,https://oleks-netizen.github.io/product-images/410413701/004.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1113320512</t>
+          <t>415011208</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1113320512/001.jpg,https://oleks-netizen.github.io/product-images/1113320512/002.jpg,https://oleks-netizen.github.io/product-images/1113320512/003.jpg,https://oleks-netizen.github.io/product-images/1113320512/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/415011208/001.jpg,https://oleks-netizen.github.io/product-images/415011208/002.jpg,https://oleks-netizen.github.io/product-images/415011208/003.jpg,https://oleks-netizen.github.io/product-images/415011208/004.jpg,https://oleks-netizen.github.io/product-images/415011208/005.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1121620882</t>
+          <t>457011208</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1121620882/001.jpg,https://oleks-netizen.github.io/product-images/1121620882/002.jpg,https://oleks-netizen.github.io/product-images/1121620882/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/457011208/001.jpg,https://oleks-netizen.github.io/product-images/457011208/002.jpg,https://oleks-netizen.github.io/product-images/457011208/003.jpg,https://oleks-netizen.github.io/product-images/457011208/004.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1140321759</t>
+          <t>51110700108</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1140321759/001.jpg,https://oleks-netizen.github.io/product-images/1140321759/003.jpg,https://oleks-netizen.github.io/product-images/1140321759/004.jpg,https://oleks-netizen.github.io/product-images/1140321759/005.jpg,https://oleks-netizen.github.io/product-images/1140321759/006.jpg,https://oleks-netizen.github.io/product-images/1140321759/007.jpg,https://oleks-netizen.github.io/product-images/1140321759/008.jpg,https://oleks-netizen.github.io/product-images/1140321759/009.jpg,https://oleks-netizen.github.io/product-images/1140321759/010.jpg,https://oleks-netizen.github.io/product-images/1140321759/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51110700108/001.jpg,https://oleks-netizen.github.io/product-images/51110700108/002.jpg,https://oleks-netizen.github.io/product-images/51110700108/003.jpg,https://oleks-netizen.github.io/product-images/51110700108/004.jpg,https://oleks-netizen.github.io/product-images/51110700108/005.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1140421761</t>
+          <t>512107001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1140421761/001.jpg,https://oleks-netizen.github.io/product-images/1140421761/002.jpg,https://oleks-netizen.github.io/product-images/1140421761/003.jpg,https://oleks-netizen.github.io/product-images/1140421761/004.jpg,https://oleks-netizen.github.io/product-images/1140421761/005.jpg,https://oleks-netizen.github.io/product-images/1140421761/006.jpg,https://oleks-netizen.github.io/product-images/1140421761/007.jpg,https://oleks-netizen.github.io/product-images/1140421761/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/512107001/001.jpg,https://oleks-netizen.github.io/product-images/512107001/002.jpg,https://oleks-netizen.github.io/product-images/512107001/003.jpg,https://oleks-netizen.github.io/product-images/512107001/004.jpg,https://oleks-netizen.github.io/product-images/512107001/005.jpg,https://oleks-netizen.github.io/product-images/512107001/006.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1140422416</t>
+          <t>tur-1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1140422416/001.jpg,https://oleks-netizen.github.io/product-images/1140422416/002.jpg,https://oleks-netizen.github.io/product-images/1140422416/003.jpg,https://oleks-netizen.github.io/product-images/1140422416/004.jpg,https://oleks-netizen.github.io/product-images/1140422416/005.jpg,https://oleks-netizen.github.io/product-images/1140422416/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/tur-1/001.jpg,https://oleks-netizen.github.io/product-images/tur-1/002.jpg,https://oleks-netizen.github.io/product-images/tur-1/003.jpg,https://oleks-netizen.github.io/product-images/tur-1/004.jpg,https://oleks-netizen.github.io/product-images/tur-1/005.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1214323810</t>
+          <t>tur-2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1214323810/001.jpg,https://oleks-netizen.github.io/product-images/1214323810/003.jpg,https://oleks-netizen.github.io/product-images/1214323810/004.jpg,https://oleks-netizen.github.io/product-images/1214323810/005.jpg,https://oleks-netizen.github.io/product-images/1214323810/006.jpg,https://oleks-netizen.github.io/product-images/1214323810/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/tur-2/001.jpg,https://oleks-netizen.github.io/product-images/tur-2/002.jpg,https://oleks-netizen.github.io/product-images/tur-2/003.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1214323811</t>
+          <t>tur-3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/1214323811/001.jpg,https://oleks-netizen.github.io/product-images/1214323811/003.jpg,https://oleks-netizen.github.io/product-images/1214323811/004.jpg,https://oleks-netizen.github.io/product-images/1214323811/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/tur-3/001.jpg,https://oleks-netizen.github.io/product-images/tur-3/002.jpg,https://oleks-netizen.github.io/product-images/tur-3/003.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>54650009</t>
+          <t>ua-avtmt-35k-10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/54650009/001.jpg,https://oleks-netizen.github.io/product-images/54650009/002.jpg,https://oleks-netizen.github.io/product-images/54650009/003.jpg,https://oleks-netizen.github.io/product-images/54650009/004.jpg,https://oleks-netizen.github.io/product-images/54650009/005.jpg,https://oleks-netizen.github.io/product-images/54650009/006.jpg,https://oleks-netizen.github.io/product-images/54650009/007.jpg,https://oleks-netizen.github.io/product-images/54650009/008.jpg,https://oleks-netizen.github.io/product-images/54650009/010.jpg,https://oleks-netizen.github.io/product-images/54650009/011.jpg,https://oleks-netizen.github.io/product-images/54650009/012.jpg,https://oleks-netizen.github.io/product-images/54650009/013.jpg,https://oleks-netizen.github.io/product-images/54650009/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-10/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-10/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-10/003.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>702702</t>
+          <t>ua-avtmt-35k-11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/702702/001.jpg,https://oleks-netizen.github.io/product-images/702702/003.jpg,https://oleks-netizen.github.io/product-images/702702/004.jpg,https://oleks-netizen.github.io/product-images/702702/005.jpg,https://oleks-netizen.github.io/product-images/702702/006.jpg,https://oleks-netizen.github.io/product-images/702702/007.jpg,https://oleks-netizen.github.io/product-images/702702/008.jpg,https://oleks-netizen.github.io/product-images/702702/009.jpg,https://oleks-netizen.github.io/product-images/702702/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-11/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-11/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-11/003.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>74541705</t>
+          <t>ua-avtmt-35k-12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/74541705/001.jpg,https://oleks-netizen.github.io/product-images/74541705/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-12/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-12/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-12/003.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-12/004.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>75621811</t>
+          <t>ua-avtmt-35k-13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/75621811/001.jpg,https://oleks-netizen.github.io/product-images/75621811/002.jpg,https://oleks-netizen.github.io/product-images/75621811/004.jpg,https://oleks-netizen.github.io/product-images/75621811/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-13/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-13/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-13/003.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>76771928</t>
+          <t>ua-avtmt-35k-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/76771928/001.jpg,https://oleks-netizen.github.io/product-images/76771928/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-14/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-14/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-14/003.jpg</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>76781929</t>
+          <t>ua-avtmt-35k-15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/76781929/001.jpg,https://oleks-netizen.github.io/product-images/76781929/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-15/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-15/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-15/003.jpg</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>76781933</t>
+          <t>ua-avtmt-35k-16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/76781933/001.jpg,https://oleks-netizen.github.io/product-images/76781933/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-16/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-16/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-16/003.jpg</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>76781934</t>
+          <t>ua-avtmt-35k-17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/76781934/001.jpg,https://oleks-netizen.github.io/product-images/76781934/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-17/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-17/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-17/003.jpg</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>80341064</t>
+          <t>ua-avtmt-35k-18</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80341064/001.jpg,https://oleks-netizen.github.io/product-images/80341064/002.jpg,https://oleks-netizen.github.io/product-images/80341064/003.jpg,https://oleks-netizen.github.io/product-images/80341064/004.jpg,https://oleks-netizen.github.io/product-images/80341064/006.jpg,https://oleks-netizen.github.io/product-images/80341064/007.jpg,https://oleks-netizen.github.io/product-images/80341064/008.jpg,https://oleks-netizen.github.io/product-images/80341064/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-18/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-18/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-18/003.jpg</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>80341510</t>
+          <t>ua-avtmt-35k-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80341510/001.jpg,https://oleks-netizen.github.io/product-images/80341510/002.jpg,https://oleks-netizen.github.io/product-images/80341510/004.jpg,https://oleks-netizen.github.io/product-images/80341510/005.jpg,https://oleks-netizen.github.io/product-images/80341510/006.jpg,https://oleks-netizen.github.io/product-images/80341510/007.jpg,https://oleks-netizen.github.io/product-images/80341510/008.jpg,https://oleks-netizen.github.io/product-images/80341510/009.jpg,https://oleks-netizen.github.io/product-images/80341510/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-19/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-19/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-19/003.jpg</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>80341515</t>
+          <t>ua-avtmt-35k-20</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80341515/001.jpg,https://oleks-netizen.github.io/product-images/80341515/003.jpg,https://oleks-netizen.github.io/product-images/80341515/004.jpg,https://oleks-netizen.github.io/product-images/80341515/005.jpg,https://oleks-netizen.github.io/product-images/80341515/006.jpg,https://oleks-netizen.github.io/product-images/80341515/007.jpg,https://oleks-netizen.github.io/product-images/80341515/008.jpg,https://oleks-netizen.github.io/product-images/80341515/009.jpg,https://oleks-netizen.github.io/product-images/80341515/010.jpg,https://oleks-netizen.github.io/product-images/80341515/011.jpg,https://oleks-netizen.github.io/product-images/80341515/012.jpg,https://oleks-netizen.github.io/product-images/80341515/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-20/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-20/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-20/003.jpg</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>80411725</t>
+          <t>ua-avtmt-35k-21</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/80411725/001.jpg,https://oleks-netizen.github.io/product-images/80411725/002.jpg,https://oleks-netizen.github.io/product-images/80411725/004.jpg,https://oleks-netizen.github.io/product-images/80411725/005.jpg,https://oleks-netizen.github.io/product-images/80411725/006.jpg,https://oleks-netizen.github.io/product-images/80411725/007.jpg,https://oleks-netizen.github.io/product-images/80411725/008.jpg,https://oleks-netizen.github.io/product-images/80411725/009.jpg,https://oleks-netizen.github.io/product-images/80411725/010.jpg,https://oleks-netizen.github.io/product-images/80411725/011.jpg,https://oleks-netizen.github.io/product-images/80411725/012.jpg,https://oleks-netizen.github.io/product-images/80411725/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-21/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-21/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-21/003.jpg</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>81204057</t>
+          <t>ua-avtmt-35k-22</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/81204057/001.jpg,https://oleks-netizen.github.io/product-images/81204057/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-22/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-22/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-22/003.jpg</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>81714241</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/81714241/001.jpg,https://oleks-netizen.github.io/product-images/81714241/002.jpg,https://oleks-netizen.github.io/product-images/81714241/003.jpg,https://oleks-netizen.github.io/product-images/81714241/004.jpg</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>85351101</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/85351101/001.jpg,https://oleks-netizen.github.io/product-images/85351101/002.jpg,https://oleks-netizen.github.io/product-images/85351101/003.jpg,https://oleks-netizen.github.io/product-images/85351101/005.jpg,https://oleks-netizen.github.io/product-images/85351101/006.jpg,https://oleks-netizen.github.io/product-images/85351101/007.jpg,https://oleks-netizen.github.io/product-images/85351101/008.jpg,https://oleks-netizen.github.io/product-images/85351101/009.jpg,https://oleks-netizen.github.io/product-images/85351101/010.jpg,https://oleks-netizen.github.io/product-images/85351101/011.jpg,https://oleks-netizen.github.io/product-images/85351101/012.jpg,https://oleks-netizen.github.io/product-images/85351101/013.jpg,https://oleks-netizen.github.io/product-images/85351101/014.jpg</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>85351120</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/85351120/001.jpg,https://oleks-netizen.github.io/product-images/85351120/002.jpg,https://oleks-netizen.github.io/product-images/85351120/003.jpg,https://oleks-netizen.github.io/product-images/85351120/004.jpg,https://oleks-netizen.github.io/product-images/85351120/005.jpg,https://oleks-netizen.github.io/product-images/85351120/006.jpg,https://oleks-netizen.github.io/product-images/85351120/007.jpg,https://oleks-netizen.github.io/product-images/85351120/008.jpg,https://oleks-netizen.github.io/product-images/85351120/010.jpg,https://oleks-netizen.github.io/product-images/85351120/011.jpg</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>85351130</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/85351130/001.jpg,https://oleks-netizen.github.io/product-images/85351130/002.jpg,https://oleks-netizen.github.io/product-images/85351130/003.jpg,https://oleks-netizen.github.io/product-images/85351130/005.jpg,https://oleks-netizen.github.io/product-images/85351130/006.jpg,https://oleks-netizen.github.io/product-images/85351130/007.jpg,https://oleks-netizen.github.io/product-images/85351130/008.jpg,https://oleks-netizen.github.io/product-images/85351130/009.jpg,https://oleks-netizen.github.io/product-images/85351130/010.jpg,https://oleks-netizen.github.io/product-images/85351130/011.jpg,https://oleks-netizen.github.io/product-images/85351130/012.jpg,https://oleks-netizen.github.io/product-images/85351130/013.jpg</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>90521001</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/90521001/001.jpg,https://oleks-netizen.github.io/product-images/90521001/003.jpg,https://oleks-netizen.github.io/product-images/90521001/004.jpg,https://oleks-netizen.github.io/product-images/90521001/005.jpg,https://oleks-netizen.github.io/product-images/90521001/006.jpg,https://oleks-netizen.github.io/product-images/90521001/007.jpg,https://oleks-netizen.github.io/product-images/90521001/008.jpg,https://oleks-netizen.github.io/product-images/90521001/009.jpg,https://oleks-netizen.github.io/product-images/90521001/010.jpg,https://oleks-netizen.github.io/product-images/90521001/011.jpg,https://oleks-netizen.github.io/product-images/90521001/012.jpg,https://oleks-netizen.github.io/product-images/90521001/013.jpg,https://oleks-netizen.github.io/product-images/90521001/014.jpg</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>90521506</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/90521506/001.jpg,https://oleks-netizen.github.io/product-images/90521506/003.jpg,https://oleks-netizen.github.io/product-images/90521506/004.jpg,https://oleks-netizen.github.io/product-images/90521506/005.jpg,https://oleks-netizen.github.io/product-images/90521506/006.jpg,https://oleks-netizen.github.io/product-images/90521506/007.jpg,https://oleks-netizen.github.io/product-images/90521506/008.jpg,https://oleks-netizen.github.io/product-images/90521506/009.jpg,https://oleks-netizen.github.io/product-images/90521506/010.jpg,https://oleks-netizen.github.io/product-images/90521506/011.jpg,https://oleks-netizen.github.io/product-images/90521506/012.jpg</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>952120541</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/952120541/001.jpg,https://oleks-netizen.github.io/product-images/952120541/002.jpg,https://oleks-netizen.github.io/product-images/952120541/003.jpg,https://oleks-netizen.github.io/product-images/952120541/004.jpg,https://oleks-netizen.github.io/product-images/952120541/006.jpg</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>952120542</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/952120542/001.jpg,https://oleks-netizen.github.io/product-images/952120542/002.jpg,https://oleks-netizen.github.io/product-images/952120542/003.jpg,https://oleks-netizen.github.io/product-images/952120542/004.jpg,https://oleks-netizen.github.io/product-images/952120542/006.jpg</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>C53 TAN</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/C53 TAN/001.jpg,https://oleks-netizen.github.io/product-images/C53 TAN/002.jpg,https://oleks-netizen.github.io/product-images/C53 TAN/003.jpg,https://oleks-netizen.github.io/product-images/C53 TAN/004.jpg,https://oleks-netizen.github.io/product-images/C53 TAN/005.jpg</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>D102 NAVY</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/D102 NAVY/001.jpg,https://oleks-netizen.github.io/product-images/D102 NAVY/002.jpg,https://oleks-netizen.github.io/product-images/D102 NAVY/003.jpg,https://oleks-netizen.github.io/product-images/D102 NAVY/004.jpg</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>FA-232-3md</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/FA-232-3md/001.jpg,https://oleks-netizen.github.io/product-images/FA-232-3md/002.jpg,https://oleks-netizen.github.io/product-images/FA-232-3md/003.jpg,https://oleks-netizen.github.io/product-images/FA-232-3md/004.jpg,https://oleks-netizen.github.io/product-images/FA-232-3md/005.jpg,https://oleks-netizen.github.io/product-images/FA-232-3md/006.jpg</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Q42 BLK</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/Q42 BLK/001.jpg,https://oleks-netizen.github.io/product-images/Q42 BLK/002.jpg,https://oleks-netizen.github.io/product-images/Q42 BLK/003.jpg,https://oleks-netizen.github.io/product-images/Q42 BLK/004.jpg</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Q42 CHESTNUT</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/Q42 CHESTNUT/001.jpg,https://oleks-netizen.github.io/product-images/Q42 CHESTNUT/002.jpg,https://oleks-netizen.github.io/product-images/Q42 CHESTNUT/003.jpg,https://oleks-netizen.github.io/product-images/Q42 CHESTNUT/004.jpg</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>RB-3107-4lx</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/RB-3107-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RB-3107-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RB-3107-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RB-3107-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RB-3107-4lx/005.jpg</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>RC-0324-4lx</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/RC-0324-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RC-0324-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RC-0324-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RC-0324-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RC-0324-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RC-0324-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RC-0324-4lx/008.jpg,https://oleks-netizen.github.io/product-images/RC-0324-4lx/009.jpg,https://oleks-netizen.github.io/product-images/RC-0324-4lx/010.jpg</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>RCv-232-3md</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/RCv-232-3md/001.jpg,https://oleks-netizen.github.io/product-images/RCv-232-3md/002.jpg,https://oleks-netizen.github.io/product-images/RCv-232-3md/003.jpg,https://oleks-netizen.github.io/product-images/RCv-232-3md/004.jpg,https://oleks-netizen.github.io/product-images/RCv-232-3md/005.jpg,https://oleks-netizen.github.io/product-images/RCv-232-3md/006.jpg,https://oleks-netizen.github.io/product-images/RCv-232-3md/007.jpg</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>RЕ-0604-3md</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/RЕ-0604-3md/001.jpg,https://oleks-netizen.github.io/product-images/RЕ-0604-3md/002.jpg,https://oleks-netizen.github.io/product-images/RЕ-0604-3md/004.jpg,https://oleks-netizen.github.io/product-images/RЕ-0604-3md/005.jpg,https://oleks-netizen.github.io/product-images/RЕ-0604-3md/006.jpg,https://oleks-netizen.github.io/product-images/RЕ-0604-3md/007.jpg,https://oleks-netizen.github.io/product-images/RЕ-0604-3md/008.jpg,https://oleks-netizen.github.io/product-images/RЕ-0604-3md/009.jpg</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>S4 BLUE</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/S4 BLUE/001.jpg,https://oleks-netizen.github.io/product-images/S4 BLUE/003.jpg,https://oleks-netizen.github.io/product-images/S4 BLUE/004.jpg,https://oleks-netizen.github.io/product-images/S4 BLUE/005.jpg,https://oleks-netizen.github.io/product-images/S4 BLUE/006.jpg,https://oleks-netizen.github.io/product-images/S4 BLUE/007.jpg,https://oleks-netizen.github.io/product-images/S4 BLUE/008.jpg,https://oleks-netizen.github.io/product-images/S4 BLUE/009.jpg</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>WELL-11992</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-11992/001.jpg,https://oleks-netizen.github.io/product-images/WELL-11992/002.jpg</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>WELL-72319</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-72319/001.jpg,https://oleks-netizen.github.io/product-images/WELL-72319/003.jpg,https://oleks-netizen.github.io/product-images/WELL-72319/004.jpg,https://oleks-netizen.github.io/product-images/WELL-72319/005.jpg,https://oleks-netizen.github.io/product-images/WELL-72319/006.jpg</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>WELL-72324</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-72324/001.jpg,https://oleks-netizen.github.io/product-images/WELL-72324/002.jpg,https://oleks-netizen.github.io/product-images/WELL-72324/003.jpg,https://oleks-netizen.github.io/product-images/WELL-72324/004.jpg,https://oleks-netizen.github.io/product-images/WELL-72324/005.jpg</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>WELL-72326</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-72326/001.jpg,https://oleks-netizen.github.io/product-images/WELL-72326/002.jpg,https://oleks-netizen.github.io/product-images/WELL-72326/004.jpg,https://oleks-netizen.github.io/product-images/WELL-72326/005.jpg,https://oleks-netizen.github.io/product-images/WELL-72326/006.jpg</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>WELL-K76519</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/WELL-K76519/001.jpg,https://oleks-netizen.github.io/product-images/WELL-K76519/003.jpg,https://oleks-netizen.github.io/product-images/WELL-K76519/004.jpg,https://oleks-netizen.github.io/product-images/WELL-K76519/005.jpg,https://oleks-netizen.github.io/product-images/WELL-K76519/006.jpg</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-08-12 15:48:52
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,117 +436,117 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>336201100</t>
+          <t>2222-05-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/336201100/001.jpg,https://oleks-netizen.github.io/product-images/336201100/002.jpg,https://oleks-netizen.github.io/product-images/336201100/003.jpg,https://oleks-netizen.github.io/product-images/336201100/004.jpg,https://oleks-netizen.github.io/product-images/336201100/005.jpg,https://oleks-netizen.github.io/product-images/336201100/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/2222-05-31/001.jpg,https://oleks-netizen.github.io/product-images/2222-05-31/002.jpg,https://oleks-netizen.github.io/product-images/2222-05-31/003.jpg,https://oleks-netizen.github.io/product-images/2222-05-31/004.jpg,https://oleks-netizen.github.io/product-images/2222-05-31/006.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>410011208</t>
+          <t>51311301s</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/410011208/001.jpg,https://oleks-netizen.github.io/product-images/410011208/002.jpg,https://oleks-netizen.github.io/product-images/410011208/003.jpg,https://oleks-netizen.github.io/product-images/410011208/004.jpg,https://oleks-netizen.github.io/product-images/410011208/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51311301s/001.jpg,https://oleks-netizen.github.io/product-images/51311301s/002.jpg,https://oleks-netizen.github.io/product-images/51311301s/003.jpg,https://oleks-netizen.github.io/product-images/51311301s/005.jpg,https://oleks-netizen.github.io/product-images/51311301s/006.jpg,https://oleks-netizen.github.io/product-images/51311301s/007.jpg,https://oleks-netizen.github.io/product-images/51311301s/008.jpg,https://oleks-netizen.github.io/product-images/51311301s/009.jpg,https://oleks-netizen.github.io/product-images/51311301s/010.jpg,https://oleks-netizen.github.io/product-images/51311301s/011.jpg,https://oleks-netizen.github.io/product-images/51311301s/012.jpg,https://oleks-netizen.github.io/product-images/51311301s/013.jpg,https://oleks-netizen.github.io/product-images/51311301s/014.jpg,https://oleks-netizen.github.io/product-images/51311301s/015.jpg,https://oleks-netizen.github.io/product-images/51311301s/016.jpg,https://oleks-netizen.github.io/product-images/51311301s/017.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>410011508</t>
+          <t>51411010s</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/410011508/001.jpg,https://oleks-netizen.github.io/product-images/410011508/002.jpg,https://oleks-netizen.github.io/product-images/410011508/003.jpg,https://oleks-netizen.github.io/product-images/410011508/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411010s/001.jpg,https://oleks-netizen.github.io/product-images/51411010s/002.jpg,https://oleks-netizen.github.io/product-images/51411010s/003.jpg,https://oleks-netizen.github.io/product-images/51411010s/005.jpg,https://oleks-netizen.github.io/product-images/51411010s/006.jpg,https://oleks-netizen.github.io/product-images/51411010s/007.jpg,https://oleks-netizen.github.io/product-images/51411010s/008.jpg,https://oleks-netizen.github.io/product-images/51411010s/009.jpg,https://oleks-netizen.github.io/product-images/51411010s/010.jpg,https://oleks-netizen.github.io/product-images/51411010s/011.jpg,https://oleks-netizen.github.io/product-images/51411010s/012.jpg,https://oleks-netizen.github.io/product-images/51411010s/013.jpg,https://oleks-netizen.github.io/product-images/51411010s/014.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>410413701</t>
+          <t>51411215s</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/410413701/001.jpg,https://oleks-netizen.github.io/product-images/410413701/002.jpg,https://oleks-netizen.github.io/product-images/410413701/003.jpg,https://oleks-netizen.github.io/product-images/410413701/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411215s/001.jpg,https://oleks-netizen.github.io/product-images/51411215s/002.jpg,https://oleks-netizen.github.io/product-images/51411215s/003.jpg,https://oleks-netizen.github.io/product-images/51411215s/004.jpg,https://oleks-netizen.github.io/product-images/51411215s/006.jpg,https://oleks-netizen.github.io/product-images/51411215s/007.jpg,https://oleks-netizen.github.io/product-images/51411215s/008.jpg,https://oleks-netizen.github.io/product-images/51411215s/009.jpg,https://oleks-netizen.github.io/product-images/51411215s/010.jpg,https://oleks-netizen.github.io/product-images/51411215s/011.jpg,https://oleks-netizen.github.io/product-images/51411215s/012.jpg,https://oleks-netizen.github.io/product-images/51411215s/013.jpg,https://oleks-netizen.github.io/product-images/51411215s/014.jpg,https://oleks-netizen.github.io/product-images/51411215s/015.jpg,https://oleks-netizen.github.io/product-images/51411215s/016.jpg,https://oleks-netizen.github.io/product-images/51411215s/017.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>415011208</t>
+          <t>51411264s</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/415011208/001.jpg,https://oleks-netizen.github.io/product-images/415011208/002.jpg,https://oleks-netizen.github.io/product-images/415011208/003.jpg,https://oleks-netizen.github.io/product-images/415011208/004.jpg,https://oleks-netizen.github.io/product-images/415011208/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/51411264s/001.jpg,https://oleks-netizen.github.io/product-images/51411264s/002.jpg,https://oleks-netizen.github.io/product-images/51411264s/003.jpg,https://oleks-netizen.github.io/product-images/51411264s/005.jpg,https://oleks-netizen.github.io/product-images/51411264s/006.jpg,https://oleks-netizen.github.io/product-images/51411264s/007.jpg,https://oleks-netizen.github.io/product-images/51411264s/008.jpg,https://oleks-netizen.github.io/product-images/51411264s/009.jpg,https://oleks-netizen.github.io/product-images/51411264s/010.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>457011208</t>
+          <t>BN-BAG-62-caramel</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/457011208/001.jpg,https://oleks-netizen.github.io/product-images/457011208/002.jpg,https://oleks-netizen.github.io/product-images/457011208/003.jpg,https://oleks-netizen.github.io/product-images/457011208/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-BAG-62-caramel/001.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-caramel/002.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-caramel/003.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-caramel/004.jpg,https://oleks-netizen.github.io/product-images/BN-BAG-62-caramel/006.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>51110700108</t>
+          <t>FA-0324-4lx</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/51110700108/001.jpg,https://oleks-netizen.github.io/product-images/51110700108/002.jpg,https://oleks-netizen.github.io/product-images/51110700108/003.jpg,https://oleks-netizen.github.io/product-images/51110700108/004.jpg,https://oleks-netizen.github.io/product-images/51110700108/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/FA-0324-4lx/001.jpg,https://oleks-netizen.github.io/product-images/FA-0324-4lx/002.jpg,https://oleks-netizen.github.io/product-images/FA-0324-4lx/004.jpg,https://oleks-netizen.github.io/product-images/FA-0324-4lx/005.jpg,https://oleks-netizen.github.io/product-images/FA-0324-4lx/006.jpg,https://oleks-netizen.github.io/product-images/FA-0324-4lx/007.jpg,https://oleks-netizen.github.io/product-images/FA-0324-4lx/008.jpg,https://oleks-netizen.github.io/product-images/FA-0324-4lx/009.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>512107001</t>
+          <t>GARETH VT BLK</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/512107001/001.jpg,https://oleks-netizen.github.io/product-images/512107001/002.jpg,https://oleks-netizen.github.io/product-images/512107001/003.jpg,https://oleks-netizen.github.io/product-images/512107001/004.jpg,https://oleks-netizen.github.io/product-images/512107001/005.jpg,https://oleks-netizen.github.io/product-images/512107001/006.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/GARETH VT BLK/001.jpg,https://oleks-netizen.github.io/product-images/GARETH VT BLK/002.jpg,https://oleks-netizen.github.io/product-images/GARETH VT BLK/003.jpg,https://oleks-netizen.github.io/product-images/GARETH VT BLK/004.jpg,https://oleks-netizen.github.io/product-images/GARETH VT BLK/005.jpg,https://oleks-netizen.github.io/product-images/GARETH VT BLK/006.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -556,241 +556,106 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tur-1</t>
+          <t>RA-3107-4lx</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/tur-1/001.jpg,https://oleks-netizen.github.io/product-images/tur-1/002.jpg,https://oleks-netizen.github.io/product-images/tur-1/003.jpg,https://oleks-netizen.github.io/product-images/tur-1/004.jpg,https://oleks-netizen.github.io/product-images/tur-1/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/RA-3107-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RA-3107-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RA-3107-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RA-3107-4lx/005.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tur-2</t>
+          <t>RC-0001-4lx</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/tur-2/001.jpg,https://oleks-netizen.github.io/product-images/tur-2/002.jpg,https://oleks-netizen.github.io/product-images/tur-2/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/RC-0001-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RC-0001-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RC-0001-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RC-0001-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RC-0001-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RC-0001-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RC-0001-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RC-0001-4lx/008.jpg,https://oleks-netizen.github.io/product-images/RC-0001-4lx/009.jpg,https://oleks-netizen.github.io/product-images/RC-0001-4lx/010.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tur-3</t>
+          <t>RC-3107-4lx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/tur-3/001.jpg,https://oleks-netizen.github.io/product-images/tur-3/002.jpg,https://oleks-netizen.github.io/product-images/tur-3/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/RC-3107-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RC-3107-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RC-3107-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RC-3107-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RC-3107-4lx/005.jpg</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ua-avtmt-35k-10</t>
+          <t>RC-8839-4lx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-10/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-10/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-10/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/RC-8839-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RC-8839-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RC-8839-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RC-8839-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RC-8839-4lx/006.jpg,https://oleks-netizen.github.io/product-images/RC-8839-4lx/007.jpg,https://oleks-netizen.github.io/product-images/RC-8839-4lx/008.jpg,https://oleks-netizen.github.io/product-images/RC-8839-4lx/009.jpg,https://oleks-netizen.github.io/product-images/RC-8839-4lx/010.jpg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ua-avtmt-35k-11</t>
+          <t>RE-3107-4lx</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-11/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-11/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-11/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/RE-3107-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RE-3107-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RE-3107-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RE-3107-4lx/005.jpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ua-avtmt-35k-12</t>
+          <t>RE-3107-4lx-96888</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-12/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-12/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-12/003.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-12/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/RE-3107-4lx-96888/001.jpg,https://oleks-netizen.github.io/product-images/RE-3107-4lx-96888/002.jpg,https://oleks-netizen.github.io/product-images/RE-3107-4lx-96888/004.jpg,https://oleks-netizen.github.io/product-images/RE-3107-4lx-96888/005.jpg,https://oleks-netizen.github.io/product-images/RE-3107-4lx-96888/006.jpg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ua-avtmt-35k-13</t>
+          <t>RYv-3107-4lx</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-13/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-13/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-13/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/RYv-3107-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RYv-3107-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RYv-3107-4lx/004.jpg,https://oleks-netizen.github.io/product-images/RYv-3107-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RYv-3107-4lx/006.jpg</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>ua-avtmt-35k-14</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-14/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-14/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-14/003.jpg</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>ua-avtmt-35k-15</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-15/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-15/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-15/003.jpg</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>ua-avtmt-35k-16</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-16/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-16/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-16/003.jpg</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>ua-avtmt-35k-17</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-17/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-17/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-17/003.jpg</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>ua-avtmt-35k-18</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-18/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-18/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-18/003.jpg</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>ua-avtmt-35k-19</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-19/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-19/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-19/003.jpg</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>ua-avtmt-35k-20</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-20/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-20/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-20/003.jpg</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>ua-avtmt-35k-21</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-21/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-21/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-21/003.jpg</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>ua-avtmt-35k-22</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/ua-avtmt-35k-22/001.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-22/002.jpg,https://oleks-netizen.github.io/product-images/ua-avtmt-35k-22/003.jpg</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>